<commit_message>
Refactor framework to Page Object Model (POM)
</commit_message>
<xml_diff>
--- a/sqa-testing-report/Data/DataTest.xlsx
+++ b/sqa-testing-report/Data/DataTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\sqa-testing-report\sqa-testing-report\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1982713C-B533-4DE7-A7B0-0D972C5CBC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C69B56A-177D-45FB-B754-1C00B7A1660F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
     <x:workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="664" firstSheet="0" activeTab="3" xr2:uid="{DC4DB269-603C-4B5B-A498-B166C8A18B92}"/>
   </x:bookViews>
@@ -7770,7 +7770,7 @@
     <x:t>Hiển thị danh sách khu vực.</x:t>
   </x:si>
   <x:si>
-    <x:t>Đã hiển thị đầy đủ danh sách rạp, sắp xếp theo khu vực/thành phố thành công.</x:t>
+    <x:t>Hệ thống đã hiển thị đầy đủ danh sách khu vực.</x:t>
   </x:si>
   <x:si>
     <x:t>Click vào khu vực [Khu vực]</x:t>
@@ -7782,6 +7782,9 @@
     <x:t>Hiển thị danh sách rạp thuộc [Bến Tre].</x:t>
   </x:si>
   <x:si>
+    <x:t>Đã hiển thị danh sách rạp thuộc khu vực [Bến Tre].</x:t>
+  </x:si>
+  <x:si>
     <x:t>Kiểm tra truy cập rạp không tồn tại qua URL.</x:t>
   </x:si>
   <x:si>
@@ -7842,19 +7845,13 @@
     <x:t>Đã chuyển hướng đến trang chi tiết rạp Galaxy Bến Tre.</x:t>
   </x:si>
   <x:si>
-    <x:t>Fail</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Data/Screenshots/TC_CINEMA_09.png</x:t>
-  </x:si>
-  <x:si>
     <x:t>Cuộn màn hình đến phần danh sách phim ("Movies").</x:t>
   </x:si>
   <x:si>
     <x:t>Hiển thị tiêu đề "Movies" và danh sách các phim đang có lịch chiếu.</x:t>
   </x:si>
   <x:si>
-    <x:t>Lỗi: CỐ TÌNH LÀM FAIL TẠI BƯỚC 2: Kiểm tra tính năng chụp ảnh màn hình và lưu file Excel.</x:t>
+    <x:t>Đã cuộn đến danh sách phim và chọn thành công Tab ngày 10/04/2026.</x:t>
   </x:si>
   <x:si>
     <x:t>Kiểm tra vị trí hiển thị của các suất chiếu (08:00, 11:00).</x:t>
@@ -7863,7 +7860,7 @@
     <x:t>Các suất chiếu được hiển thị nằm gọn bên dưới tên phim tương ứng (VD: phim "Khá").</x:t>
   </x:si>
   <x:si>
-    <x:t>Đánh giá Fail do bước trước đó đã thất bại.</x:t>
+    <x:t>Các suất chiếu nằm gọn dưới tên phim Khá. Đã nhấn vào suất chiếu thành công.</x:t>
   </x:si>
   <x:si>
     <x:t>Click chọn suất chiếu bất kỳ.</x:t>
@@ -48183,41 +48180,41 @@
   </x:mergeCells>
   <x:phoneticPr fontId="16" type="noConversion"/>
   <x:hyperlinks>
-    <x:hyperlink ref="H382" r:id="rId79"/>
-    <x:hyperlink ref="H388" r:id="rId80"/>
-    <x:hyperlink ref="H396" r:id="rId81"/>
-    <x:hyperlink ref="H397" r:id="rId82"/>
-    <x:hyperlink ref="H415" r:id="rId83"/>
-    <x:hyperlink ref="H418" r:id="rId84"/>
-    <x:hyperlink ref="H420" r:id="rId85"/>
-    <x:hyperlink ref="H421" r:id="rId86"/>
-    <x:hyperlink ref="H423" r:id="rId87"/>
-    <x:hyperlink ref="H424" r:id="rId88"/>
-    <x:hyperlink ref="H53" r:id="rId89"/>
-    <x:hyperlink ref="H61" r:id="rId90"/>
-    <x:hyperlink ref="H65" r:id="rId91"/>
-    <x:hyperlink ref="H69" r:id="rId92"/>
-    <x:hyperlink ref="H73" r:id="rId93"/>
-    <x:hyperlink ref="H77" r:id="rId94"/>
-    <x:hyperlink ref="H81" r:id="rId95"/>
-    <x:hyperlink ref="H112" r:id="rId96"/>
-    <x:hyperlink ref="H115" r:id="rId97"/>
-    <x:hyperlink ref="H118" r:id="rId98"/>
-    <x:hyperlink ref="H399" r:id="rId99"/>
-    <x:hyperlink ref="H402" r:id="rId100"/>
-    <x:hyperlink ref="H405" r:id="rId101"/>
-    <x:hyperlink ref="H408" r:id="rId167"/>
-    <x:hyperlink ref="H411" r:id="rId168"/>
-    <x:hyperlink ref="H400" r:id="rId169"/>
-    <x:hyperlink ref="H403" r:id="rId170"/>
-    <x:hyperlink ref="H406" r:id="rId171"/>
-    <x:hyperlink ref="H409" r:id="rId172"/>
-    <x:hyperlink ref="H412" r:id="rId173"/>
-    <x:hyperlink ref="H1075" r:id="rId174"/>
-    <x:hyperlink ref="H1081" r:id="rId175"/>
-    <x:hyperlink ref="H1087" r:id="rId176"/>
-    <x:hyperlink ref="H1093" r:id="rId177"/>
-    <x:hyperlink ref="H1099" r:id="rId178"/>
+    <x:hyperlink ref="H382" r:id="rId102"/>
+    <x:hyperlink ref="H388" r:id="rId103"/>
+    <x:hyperlink ref="H396" r:id="rId104"/>
+    <x:hyperlink ref="H397" r:id="rId105"/>
+    <x:hyperlink ref="H415" r:id="rId106"/>
+    <x:hyperlink ref="H418" r:id="rId107"/>
+    <x:hyperlink ref="H420" r:id="rId108"/>
+    <x:hyperlink ref="H421" r:id="rId109"/>
+    <x:hyperlink ref="H423" r:id="rId110"/>
+    <x:hyperlink ref="H424" r:id="rId111"/>
+    <x:hyperlink ref="H53" r:id="rId112"/>
+    <x:hyperlink ref="H61" r:id="rId113"/>
+    <x:hyperlink ref="H65" r:id="rId114"/>
+    <x:hyperlink ref="H69" r:id="rId115"/>
+    <x:hyperlink ref="H73" r:id="rId116"/>
+    <x:hyperlink ref="H77" r:id="rId117"/>
+    <x:hyperlink ref="H81" r:id="rId118"/>
+    <x:hyperlink ref="H112" r:id="rId119"/>
+    <x:hyperlink ref="H115" r:id="rId120"/>
+    <x:hyperlink ref="H118" r:id="rId121"/>
+    <x:hyperlink ref="H399" r:id="rId122"/>
+    <x:hyperlink ref="H402" r:id="rId123"/>
+    <x:hyperlink ref="H405" r:id="rId124"/>
+    <x:hyperlink ref="H408" r:id="rId125"/>
+    <x:hyperlink ref="H411" r:id="rId126"/>
+    <x:hyperlink ref="H400" r:id="rId127"/>
+    <x:hyperlink ref="H403" r:id="rId128"/>
+    <x:hyperlink ref="H406" r:id="rId129"/>
+    <x:hyperlink ref="H409" r:id="rId130"/>
+    <x:hyperlink ref="H412" r:id="rId131"/>
+    <x:hyperlink ref="H1075" r:id="rId132"/>
+    <x:hyperlink ref="H1081" r:id="rId133"/>
+    <x:hyperlink ref="H1087" r:id="rId134"/>
+    <x:hyperlink ref="H1093" r:id="rId135"/>
+    <x:hyperlink ref="H1099" r:id="rId136"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51594,7 +51591,7 @@
       <x:c r="K154" s="134" t="s">
         <x:v>2007</x:v>
       </x:c>
-      <x:c r="L154" s="134"/>
+      <x:c r="L154" s="134" t="s"/>
     </x:row>
     <x:row r="155" spans="1:12" ht="27.6" customHeight="1">
       <x:c r="A155" s="140"/>
@@ -51615,7 +51612,7 @@
         <x:v>2035</x:v>
       </x:c>
       <x:c r="J155" s="134" t="s">
-        <x:v>2032</x:v>
+        <x:v>2036</x:v>
       </x:c>
       <x:c r="K155" s="134"/>
       <x:c r="L155" s="134"/>
@@ -51631,7 +51628,7 @@
         <x:v>626</x:v>
       </x:c>
       <x:c r="D156" s="140" t="s">
-        <x:v>2036</x:v>
+        <x:v>2037</x:v>
       </x:c>
       <x:c r="E156" s="140" t="s">
         <x:v>616</x:v>
@@ -51640,13 +51637,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G156" s="138" t="s">
-        <x:v>2037</x:v>
+        <x:v>2038</x:v>
       </x:c>
       <x:c r="H156" s="140" t="s">
-        <x:v>2038</x:v>
+        <x:v>2039</x:v>
       </x:c>
       <x:c r="I156" s="138" t="s">
-        <x:v>2039</x:v>
+        <x:v>2040</x:v>
       </x:c>
       <x:c r="J156" s="134"/>
       <x:c r="K156" s="134"/>
@@ -51672,21 +51669,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G157" s="138" t="s">
-        <x:v>2040</x:v>
+        <x:v>2041</x:v>
       </x:c>
       <x:c r="H157" s="140" t="s">
-        <x:v>2041</x:v>
+        <x:v>2042</x:v>
       </x:c>
       <x:c r="I157" s="138" t="s">
-        <x:v>2042</x:v>
+        <x:v>2043</x:v>
       </x:c>
       <x:c r="J157" s="134" t="s">
-        <x:v>2043</x:v>
+        <x:v>2044</x:v>
       </x:c>
       <x:c r="K157" s="134" t="s">
         <x:v>2007</x:v>
       </x:c>
-      <x:c r="L157" s="134"/>
+      <x:c r="L157" s="134" t="s"/>
     </x:row>
     <x:row r="158" spans="1:12" ht="41.4" customHeight="1">
       <x:c r="A158" s="140"/>
@@ -51698,14 +51695,14 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G158" s="138" t="s">
-        <x:v>2044</x:v>
+        <x:v>2045</x:v>
       </x:c>
       <x:c r="H158" s="140"/>
       <x:c r="I158" s="138" t="s">
-        <x:v>2045</x:v>
+        <x:v>2046</x:v>
       </x:c>
       <x:c r="J158" s="134" t="s">
-        <x:v>2046</x:v>
+        <x:v>2047</x:v>
       </x:c>
       <x:c r="K158" s="134"/>
       <x:c r="L158" s="134"/>
@@ -51720,14 +51717,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G159" s="138" t="s">
-        <x:v>2047</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="H159" s="140"/>
       <x:c r="I159" s="138" t="s">
-        <x:v>2048</x:v>
+        <x:v>2049</x:v>
       </x:c>
       <x:c r="J159" s="134" t="s">
-        <x:v>2049</x:v>
+        <x:v>2050</x:v>
       </x:c>
       <x:c r="K159" s="134"/>
       <x:c r="L159" s="134"/>
@@ -51752,13 +51749,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G160" s="138" t="s">
-        <x:v>2040</x:v>
+        <x:v>2041</x:v>
       </x:c>
       <x:c r="H160" s="140" t="s">
-        <x:v>2041</x:v>
+        <x:v>2042</x:v>
       </x:c>
       <x:c r="I160" s="138" t="s">
-        <x:v>2050</x:v>
+        <x:v>2051</x:v>
       </x:c>
       <x:c r="J160" s="134"/>
       <x:c r="K160" s="134"/>
@@ -51774,7 +51771,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G161" s="138" t="s">
-        <x:v>2051</x:v>
+        <x:v>2052</x:v>
       </x:c>
       <x:c r="H161" s="313">
         <x:v>46109</x:v>
@@ -51795,32 +51792,30 @@
         <x:v>644</x:v>
       </x:c>
       <x:c r="D162" s="116" t="s">
-        <x:v>2052</x:v>
+        <x:v>2053</x:v>
       </x:c>
       <x:c r="E162" s="116" t="s">
-        <x:v>2053</x:v>
+        <x:v>2054</x:v>
       </x:c>
       <x:c r="F162" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G162" s="320" t="s">
-        <x:v>2054</x:v>
+        <x:v>2055</x:v>
       </x:c>
       <x:c r="H162" s="116" t="s">
-        <x:v>2041</x:v>
+        <x:v>2042</x:v>
       </x:c>
       <x:c r="I162" s="320" t="s">
-        <x:v>2042</x:v>
+        <x:v>2043</x:v>
       </x:c>
       <x:c r="J162" s="134" t="s">
-        <x:v>2055</x:v>
+        <x:v>2056</x:v>
       </x:c>
       <x:c r="K162" s="134" t="s">
-        <x:v>2056</x:v>
-      </x:c>
-      <x:c r="L162" s="134" t="s">
-        <x:v>2057</x:v>
-      </x:c>
+        <x:v>2007</x:v>
+      </x:c>
+      <x:c r="L162" s="134"/>
     </x:row>
     <x:row r="163" spans="1:12" ht="54" customHeight="1">
       <x:c r="A163" s="116"/>
@@ -51832,14 +51827,14 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G163" s="320" t="s">
-        <x:v>2058</x:v>
+        <x:v>2057</x:v>
       </x:c>
       <x:c r="H163" s="116"/>
       <x:c r="I163" s="320" t="s">
+        <x:v>2058</x:v>
+      </x:c>
+      <x:c r="J163" s="134" t="s">
         <x:v>2059</x:v>
-      </x:c>
-      <x:c r="J163" s="134" t="s">
-        <x:v>2060</x:v>
       </x:c>
       <x:c r="K163" s="134"/>
       <x:c r="L163" s="134"/>
@@ -51854,14 +51849,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G164" s="320" t="s">
-        <x:v>2061</x:v>
+        <x:v>2060</x:v>
       </x:c>
       <x:c r="H164" s="116"/>
       <x:c r="I164" s="320" t="s">
+        <x:v>2061</x:v>
+      </x:c>
+      <x:c r="J164" s="134" t="s">
         <x:v>2062</x:v>
-      </x:c>
-      <x:c r="J164" s="134" t="s">
-        <x:v>2063</x:v>
       </x:c>
       <x:c r="K164" s="134"/>
       <x:c r="L164" s="134"/>
@@ -51886,13 +51881,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G165" s="320" t="s">
-        <x:v>2064</x:v>
+        <x:v>2063</x:v>
       </x:c>
       <x:c r="H165" s="318">
         <x:v>0.333333333333333</x:v>
       </x:c>
       <x:c r="I165" s="320" t="s">
-        <x:v>2065</x:v>
+        <x:v>2064</x:v>
       </x:c>
       <x:c r="J165" s="134"/>
       <x:c r="K165" s="134"/>
@@ -51908,13 +51903,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G166" s="320" t="s">
+        <x:v>2065</x:v>
+      </x:c>
+      <x:c r="H166" s="116" t="s">
         <x:v>2066</x:v>
       </x:c>
-      <x:c r="H166" s="116" t="s">
+      <x:c r="I166" s="320" t="s">
         <x:v>2067</x:v>
-      </x:c>
-      <x:c r="I166" s="320" t="s">
-        <x:v>2068</x:v>
       </x:c>
       <x:c r="J166" s="134"/>
       <x:c r="K166" s="134"/>
@@ -51930,13 +51925,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G167" s="320" t="s">
+        <x:v>2068</x:v>
+      </x:c>
+      <x:c r="H167" s="116" t="s">
         <x:v>2069</x:v>
       </x:c>
-      <x:c r="H167" s="116" t="s">
+      <x:c r="I167" s="320" t="s">
         <x:v>2070</x:v>
-      </x:c>
-      <x:c r="I167" s="320" t="s">
-        <x:v>2071</x:v>
       </x:c>
       <x:c r="J167" s="134"/>
       <x:c r="K167" s="134"/>
@@ -51952,11 +51947,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G168" s="320" t="s">
-        <x:v>2072</x:v>
+        <x:v>2071</x:v>
       </x:c>
       <x:c r="H168" s="116"/>
       <x:c r="I168" s="320" t="s">
-        <x:v>2073</x:v>
+        <x:v>2072</x:v>
       </x:c>
       <x:c r="J168" s="134"/>
       <x:c r="K168" s="134"/>
@@ -51973,22 +51968,22 @@
         <x:v>658</x:v>
       </x:c>
       <x:c r="D169" s="116" t="s">
+        <x:v>2073</x:v>
+      </x:c>
+      <x:c r="E169" s="116" t="s">
         <x:v>2074</x:v>
-      </x:c>
-      <x:c r="E169" s="116" t="s">
-        <x:v>2075</x:v>
       </x:c>
       <x:c r="F169" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G169" s="320" t="s">
+        <x:v>2075</x:v>
+      </x:c>
+      <x:c r="H169" s="116" t="s">
         <x:v>2076</x:v>
       </x:c>
-      <x:c r="H169" s="116" t="s">
+      <x:c r="I169" s="320" t="s">
         <x:v>2077</x:v>
-      </x:c>
-      <x:c r="I169" s="320" t="s">
-        <x:v>2078</x:v>
       </x:c>
       <x:c r="J169" s="134"/>
       <x:c r="K169" s="134"/>
@@ -52004,11 +51999,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G170" s="320" t="s">
-        <x:v>2079</x:v>
+        <x:v>2078</x:v>
       </x:c>
       <x:c r="H170" s="116"/>
       <x:c r="I170" s="320" t="s">
-        <x:v>2080</x:v>
+        <x:v>2079</x:v>
       </x:c>
       <x:c r="J170" s="134"/>
       <x:c r="K170" s="134"/>
@@ -52024,11 +52019,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G171" s="320" t="s">
-        <x:v>2081</x:v>
+        <x:v>2080</x:v>
       </x:c>
       <x:c r="H171" s="116"/>
       <x:c r="I171" s="320" t="s">
-        <x:v>2082</x:v>
+        <x:v>2081</x:v>
       </x:c>
       <x:c r="J171" s="134"/>
       <x:c r="K171" s="134"/>
@@ -52054,13 +52049,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G172" s="320" t="s">
-        <x:v>2083</x:v>
+        <x:v>2082</x:v>
       </x:c>
       <x:c r="H172" s="116" t="s">
+        <x:v>2076</x:v>
+      </x:c>
+      <x:c r="I172" s="320" t="s">
         <x:v>2077</x:v>
-      </x:c>
-      <x:c r="I172" s="320" t="s">
-        <x:v>2078</x:v>
       </x:c>
       <x:c r="J172" s="134"/>
       <x:c r="K172" s="134"/>
@@ -52076,11 +52071,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G173" s="320" t="s">
-        <x:v>2084</x:v>
+        <x:v>2083</x:v>
       </x:c>
       <x:c r="H173" s="116"/>
       <x:c r="I173" s="320" t="s">
-        <x:v>2085</x:v>
+        <x:v>2084</x:v>
       </x:c>
       <x:c r="J173" s="134"/>
       <x:c r="K173" s="134"/>
@@ -52106,13 +52101,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G174" s="320" t="s">
+        <x:v>2085</x:v>
+      </x:c>
+      <x:c r="H174" s="116" t="s">
+        <x:v>2076</x:v>
+      </x:c>
+      <x:c r="I174" s="320" t="s">
         <x:v>2086</x:v>
-      </x:c>
-      <x:c r="H174" s="116" t="s">
-        <x:v>2077</x:v>
-      </x:c>
-      <x:c r="I174" s="320" t="s">
-        <x:v>2087</x:v>
       </x:c>
       <x:c r="J174" s="134"/>
       <x:c r="K174" s="134"/>
@@ -52128,11 +52123,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G175" s="320" t="s">
-        <x:v>2088</x:v>
+        <x:v>2087</x:v>
       </x:c>
       <x:c r="H175" s="116"/>
       <x:c r="I175" s="320" t="s">
-        <x:v>2078</x:v>
+        <x:v>2077</x:v>
       </x:c>
       <x:c r="J175" s="134"/>
       <x:c r="K175" s="134"/>
@@ -52148,11 +52143,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G176" s="320" t="s">
-        <x:v>2089</x:v>
+        <x:v>2088</x:v>
       </x:c>
       <x:c r="H176" s="116"/>
       <x:c r="I176" s="320" t="s">
-        <x:v>2090</x:v>
+        <x:v>2089</x:v>
       </x:c>
       <x:c r="J176" s="134"/>
       <x:c r="K176" s="134"/>
@@ -52169,20 +52164,20 @@
         <x:v>674</x:v>
       </x:c>
       <x:c r="D177" s="116" t="s">
+        <x:v>2090</x:v>
+      </x:c>
+      <x:c r="E177" s="116" t="s">
         <x:v>2091</x:v>
-      </x:c>
-      <x:c r="E177" s="116" t="s">
-        <x:v>2092</x:v>
       </x:c>
       <x:c r="F177" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G177" s="320" t="s">
-        <x:v>2093</x:v>
+        <x:v>2092</x:v>
       </x:c>
       <x:c r="H177" s="116"/>
       <x:c r="I177" s="320" t="s">
-        <x:v>2094</x:v>
+        <x:v>2093</x:v>
       </x:c>
       <x:c r="J177" s="134"/>
       <x:c r="K177" s="134"/>
@@ -52198,11 +52193,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G178" s="320" t="s">
-        <x:v>2095</x:v>
+        <x:v>2094</x:v>
       </x:c>
       <x:c r="H178" s="116"/>
       <x:c r="I178" s="320" t="s">
-        <x:v>2096</x:v>
+        <x:v>2095</x:v>
       </x:c>
       <x:c r="J178" s="134"/>
       <x:c r="K178" s="134"/>
@@ -52219,22 +52214,22 @@
         <x:v>677</x:v>
       </x:c>
       <x:c r="D179" s="116" t="s">
+        <x:v>2096</x:v>
+      </x:c>
+      <x:c r="E179" s="116" t="s">
         <x:v>2097</x:v>
-      </x:c>
-      <x:c r="E179" s="116" t="s">
-        <x:v>2098</x:v>
       </x:c>
       <x:c r="F179" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G179" s="320" t="s">
-        <x:v>2099</x:v>
+        <x:v>2098</x:v>
       </x:c>
       <x:c r="H179" s="116" t="s">
         <x:v>681</x:v>
       </x:c>
       <x:c r="I179" s="320" t="s">
-        <x:v>2100</x:v>
+        <x:v>2099</x:v>
       </x:c>
       <x:c r="J179" s="116"/>
       <x:c r="K179" s="134"/>
@@ -52250,13 +52245,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G180" s="321" t="s">
+        <x:v>2100</x:v>
+      </x:c>
+      <x:c r="H180" s="115" t="s">
         <x:v>2101</x:v>
       </x:c>
-      <x:c r="H180" s="115" t="s">
+      <x:c r="I180" s="321" t="s">
         <x:v>2102</x:v>
-      </x:c>
-      <x:c r="I180" s="321" t="s">
-        <x:v>2103</x:v>
       </x:c>
       <x:c r="J180" s="115"/>
       <x:c r="K180" s="137"/>
@@ -52273,22 +52268,22 @@
         <x:v>686</x:v>
       </x:c>
       <x:c r="D181" s="116" t="s">
+        <x:v>2103</x:v>
+      </x:c>
+      <x:c r="E181" s="116" t="s">
         <x:v>2104</x:v>
-      </x:c>
-      <x:c r="E181" s="116" t="s">
-        <x:v>2105</x:v>
       </x:c>
       <x:c r="F181" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G181" s="320" t="s">
+        <x:v>2105</x:v>
+      </x:c>
+      <x:c r="H181" s="116" t="s">
         <x:v>2106</x:v>
       </x:c>
-      <x:c r="H181" s="116" t="s">
+      <x:c r="I181" s="320" t="s">
         <x:v>2107</x:v>
-      </x:c>
-      <x:c r="I181" s="320" t="s">
-        <x:v>2108</x:v>
       </x:c>
       <x:c r="J181" s="134"/>
       <x:c r="K181" s="134"/>
@@ -52304,13 +52299,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G182" s="320" t="s">
+        <x:v>2108</x:v>
+      </x:c>
+      <x:c r="H182" s="116" t="s">
         <x:v>2109</x:v>
       </x:c>
-      <x:c r="H182" s="116" t="s">
+      <x:c r="I182" s="320" t="s">
         <x:v>2110</x:v>
-      </x:c>
-      <x:c r="I182" s="320" t="s">
-        <x:v>2111</x:v>
       </x:c>
       <x:c r="J182" s="134"/>
       <x:c r="K182" s="134"/>
@@ -52326,11 +52321,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G183" s="320" t="s">
-        <x:v>2112</x:v>
+        <x:v>2111</x:v>
       </x:c>
       <x:c r="H183" s="116"/>
       <x:c r="I183" s="320" t="s">
-        <x:v>2113</x:v>
+        <x:v>2112</x:v>
       </x:c>
       <x:c r="J183" s="134"/>
       <x:c r="K183" s="134"/>
@@ -52347,20 +52342,20 @@
         <x:v>696</x:v>
       </x:c>
       <x:c r="D184" s="116" t="s">
+        <x:v>2113</x:v>
+      </x:c>
+      <x:c r="E184" s="116" t="s">
         <x:v>2114</x:v>
-      </x:c>
-      <x:c r="E184" s="116" t="s">
-        <x:v>2115</x:v>
       </x:c>
       <x:c r="F184" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G184" s="320" t="s">
-        <x:v>2116</x:v>
+        <x:v>2115</x:v>
       </x:c>
       <x:c r="H184" s="116"/>
       <x:c r="I184" s="320" t="s">
-        <x:v>2117</x:v>
+        <x:v>2116</x:v>
       </x:c>
       <x:c r="J184" s="134"/>
       <x:c r="K184" s="134"/>
@@ -52376,13 +52371,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G185" s="320" t="s">
+        <x:v>2117</x:v>
+      </x:c>
+      <x:c r="H185" s="116" t="s">
         <x:v>2118</x:v>
       </x:c>
-      <x:c r="H185" s="116" t="s">
+      <x:c r="I185" s="320" t="s">
         <x:v>2119</x:v>
-      </x:c>
-      <x:c r="I185" s="320" t="s">
-        <x:v>2120</x:v>
       </x:c>
       <x:c r="J185" s="134"/>
       <x:c r="K185" s="134"/>
@@ -52398,11 +52393,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G186" s="320" t="s">
-        <x:v>2121</x:v>
+        <x:v>2120</x:v>
       </x:c>
       <x:c r="H186" s="116"/>
       <x:c r="I186" s="320" t="s">
-        <x:v>2122</x:v>
+        <x:v>2121</x:v>
       </x:c>
       <x:c r="J186" s="134"/>
       <x:c r="K186" s="134"/>
@@ -52418,11 +52413,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G187" s="320" t="s">
-        <x:v>2123</x:v>
+        <x:v>2122</x:v>
       </x:c>
       <x:c r="H187" s="116"/>
       <x:c r="I187" s="320" t="s">
-        <x:v>2124</x:v>
+        <x:v>2123</x:v>
       </x:c>
       <x:c r="J187" s="134"/>
       <x:c r="K187" s="134"/>
@@ -52439,22 +52434,22 @@
         <x:v>932</x:v>
       </x:c>
       <x:c r="D188" s="114" t="s">
+        <x:v>2124</x:v>
+      </x:c>
+      <x:c r="E188" s="114" t="s">
         <x:v>2125</x:v>
-      </x:c>
-      <x:c r="E188" s="114" t="s">
-        <x:v>2126</x:v>
       </x:c>
       <x:c r="F188" s="329">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G188" s="324" t="s">
+        <x:v>2126</x:v>
+      </x:c>
+      <x:c r="H188" s="324" t="s">
         <x:v>2127</x:v>
       </x:c>
-      <x:c r="H188" s="324" t="s">
+      <x:c r="I188" s="325" t="s">
         <x:v>2128</x:v>
-      </x:c>
-      <x:c r="I188" s="325" t="s">
-        <x:v>2129</x:v>
       </x:c>
       <x:c r="J188" s="61"/>
       <x:c r="K188" s="133"/>
@@ -52470,13 +52465,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G189" s="324" t="s">
+        <x:v>2129</x:v>
+      </x:c>
+      <x:c r="H189" s="324" t="s">
         <x:v>2130</x:v>
       </x:c>
-      <x:c r="H189" s="324" t="s">
+      <x:c r="I189" s="325" t="s">
         <x:v>2131</x:v>
-      </x:c>
-      <x:c r="I189" s="325" t="s">
-        <x:v>2132</x:v>
       </x:c>
       <x:c r="J189" s="61"/>
       <x:c r="K189" s="124"/>
@@ -52492,11 +52487,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G190" s="324" t="s">
-        <x:v>2133</x:v>
+        <x:v>2132</x:v>
       </x:c>
       <x:c r="H190" s="324"/>
       <x:c r="I190" s="325" t="s">
-        <x:v>2134</x:v>
+        <x:v>2133</x:v>
       </x:c>
       <x:c r="J190" s="61"/>
       <x:c r="K190" s="111"/>
@@ -52513,20 +52508,20 @@
         <x:v>947</x:v>
       </x:c>
       <x:c r="D191" s="114" t="s">
+        <x:v>2134</x:v>
+      </x:c>
+      <x:c r="E191" s="114" t="s">
         <x:v>2135</x:v>
-      </x:c>
-      <x:c r="E191" s="114" t="s">
-        <x:v>2136</x:v>
       </x:c>
       <x:c r="F191" s="329">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G191" s="324" t="s">
-        <x:v>2137</x:v>
+        <x:v>2136</x:v>
       </x:c>
       <x:c r="H191" s="324"/>
       <x:c r="I191" s="325" t="s">
-        <x:v>2138</x:v>
+        <x:v>2137</x:v>
       </x:c>
       <x:c r="J191" s="61"/>
       <x:c r="K191" s="133"/>
@@ -52542,11 +52537,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G192" s="324" t="s">
-        <x:v>2139</x:v>
+        <x:v>2138</x:v>
       </x:c>
       <x:c r="H192" s="324"/>
       <x:c r="I192" s="325" t="s">
-        <x:v>2140</x:v>
+        <x:v>2139</x:v>
       </x:c>
       <x:c r="J192" s="61"/>
       <x:c r="K192" s="124"/>
@@ -52562,13 +52557,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G193" s="324" t="s">
+        <x:v>2140</x:v>
+      </x:c>
+      <x:c r="H193" s="324" t="s">
         <x:v>2141</x:v>
       </x:c>
-      <x:c r="H193" s="324" t="s">
+      <x:c r="I193" s="325" t="s">
         <x:v>2142</x:v>
-      </x:c>
-      <x:c r="I193" s="325" t="s">
-        <x:v>2143</x:v>
       </x:c>
       <x:c r="J193" s="61"/>
       <x:c r="K193" s="111"/>
@@ -52913,13 +52908,13 @@
     <x:mergeCell ref="L191:L193"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H49" r:id="rId179"/>
-    <x:hyperlink ref="H67" r:id="rId180"/>
-    <x:hyperlink ref="H76" r:id="rId181"/>
-    <x:hyperlink ref="H85" r:id="rId182"/>
-    <x:hyperlink ref="H94" r:id="rId183"/>
-    <x:hyperlink ref="H103" r:id="rId184"/>
-    <x:hyperlink ref="H112" r:id="rId185"/>
+    <x:hyperlink ref="H49" r:id="rId137"/>
+    <x:hyperlink ref="H67" r:id="rId138"/>
+    <x:hyperlink ref="H76" r:id="rId139"/>
+    <x:hyperlink ref="H85" r:id="rId140"/>
+    <x:hyperlink ref="H94" r:id="rId141"/>
+    <x:hyperlink ref="H103" r:id="rId142"/>
+    <x:hyperlink ref="H112" r:id="rId143"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -53012,7 +53007,7 @@
         <x:v>1270</x:v>
       </x:c>
       <x:c r="H2" s="288" t="s">
-        <x:v>2144</x:v>
+        <x:v>2143</x:v>
       </x:c>
       <x:c r="I2" s="134" t="s">
         <x:v>1272</x:v>
@@ -53059,7 +53054,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="297" t="s">
-        <x:v>2145</x:v>
+        <x:v>2144</x:v>
       </x:c>
       <x:c r="H4" s="297" t="s">
         <x:v>1277</x:v>
@@ -53139,7 +53134,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="297" t="s">
-        <x:v>2146</x:v>
+        <x:v>2145</x:v>
       </x:c>
       <x:c r="H7" s="297"/>
       <x:c r="I7" s="298" t="s">
@@ -53172,7 +53167,7 @@
         <x:v>1297</x:v>
       </x:c>
       <x:c r="H8" s="297" t="s">
-        <x:v>2147</x:v>
+        <x:v>2146</x:v>
       </x:c>
       <x:c r="I8" s="134" t="s">
         <x:v>1299</x:v>
@@ -53191,7 +53186,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G9" s="319" t="s">
-        <x:v>2148</x:v>
+        <x:v>2147</x:v>
       </x:c>
       <x:c r="H9" s="297"/>
       <x:c r="I9" s="134"/>
@@ -53280,7 +53275,7 @@
         <x:v>1297</x:v>
       </x:c>
       <x:c r="H13" s="297" t="s">
-        <x:v>2149</x:v>
+        <x:v>2148</x:v>
       </x:c>
       <x:c r="I13" s="134" t="s">
         <x:v>1307</x:v>
@@ -53299,7 +53294,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="319" t="s">
-        <x:v>2148</x:v>
+        <x:v>2147</x:v>
       </x:c>
       <x:c r="H14" s="297"/>
       <x:c r="I14" s="134"/>
@@ -53385,7 +53380,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="61" t="s">
-        <x:v>2150</x:v>
+        <x:v>2149</x:v>
       </x:c>
       <x:c r="H18" s="140"/>
       <x:c r="I18" s="140" t="s">
@@ -53405,7 +53400,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="61" t="s">
-        <x:v>2151</x:v>
+        <x:v>2150</x:v>
       </x:c>
       <x:c r="H19" s="140" t="s">
         <x:v>965</x:v>
@@ -53425,7 +53420,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="61" t="s">
-        <x:v>2152</x:v>
+        <x:v>2151</x:v>
       </x:c>
       <x:c r="H20" s="140"/>
       <x:c r="I20" s="140"/>
@@ -53443,7 +53438,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G21" s="61" t="s">
-        <x:v>2153</x:v>
+        <x:v>2152</x:v>
       </x:c>
       <x:c r="H21" s="140" t="s">
         <x:v>968</x:v>
@@ -53463,7 +53458,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G22" s="61" t="s">
-        <x:v>2154</x:v>
+        <x:v>2153</x:v>
       </x:c>
       <x:c r="H22" s="314" t="s">
         <x:v>970</x:v>
@@ -53483,7 +53478,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G23" s="61" t="s">
-        <x:v>2155</x:v>
+        <x:v>2154</x:v>
       </x:c>
       <x:c r="H23" s="140">
         <x:v>1</x:v>
@@ -53503,7 +53498,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G24" s="61" t="s">
-        <x:v>2156</x:v>
+        <x:v>2155</x:v>
       </x:c>
       <x:c r="H24" s="140" t="s">
         <x:v>973</x:v>
@@ -53523,7 +53518,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G25" s="61" t="s">
-        <x:v>2157</x:v>
+        <x:v>2156</x:v>
       </x:c>
       <x:c r="H25" s="140"/>
       <x:c r="I25" s="140"/>
@@ -53551,7 +53546,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G26" s="61" t="s">
-        <x:v>2158</x:v>
+        <x:v>2157</x:v>
       </x:c>
       <x:c r="H26" s="140"/>
       <x:c r="I26" s="133" t="s">
@@ -53591,7 +53586,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G28" s="61" t="s">
-        <x:v>2159</x:v>
+        <x:v>2158</x:v>
       </x:c>
       <x:c r="H28" s="239" t="s">
         <x:v>970</x:v>
@@ -53611,7 +53606,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G29" s="61" t="s">
-        <x:v>2160</x:v>
+        <x:v>2159</x:v>
       </x:c>
       <x:c r="H29" s="140">
         <x:v>1</x:v>
@@ -53631,7 +53626,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G30" s="61" t="s">
-        <x:v>2161</x:v>
+        <x:v>2160</x:v>
       </x:c>
       <x:c r="H30" s="140"/>
       <x:c r="I30" s="111"/>
@@ -53659,7 +53654,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="61" t="s">
-        <x:v>2162</x:v>
+        <x:v>2161</x:v>
       </x:c>
       <x:c r="H31" s="140"/>
       <x:c r="I31" s="133" t="s">
@@ -53758,7 +53753,7 @@
         <x:v>1309</x:v>
       </x:c>
       <x:c r="D36" s="134" t="s">
-        <x:v>2163</x:v>
+        <x:v>2162</x:v>
       </x:c>
       <x:c r="E36" s="134" t="s">
         <x:v>1311</x:v>
@@ -53770,7 +53765,7 @@
         <x:v>988</x:v>
       </x:c>
       <x:c r="H36" s="297" t="s">
-        <x:v>2164</x:v>
+        <x:v>2163</x:v>
       </x:c>
       <x:c r="I36" s="134" t="s">
         <x:v>1312</x:v>
@@ -53792,7 +53787,7 @@
         <x:v>990</x:v>
       </x:c>
       <x:c r="H37" s="314" t="s">
-        <x:v>2165</x:v>
+        <x:v>2164</x:v>
       </x:c>
       <x:c r="I37" s="134"/>
       <x:c r="J37" s="9"/>
@@ -53828,7 +53823,7 @@
         <x:v>1314</x:v>
       </x:c>
       <x:c r="D39" s="134" t="s">
-        <x:v>2166</x:v>
+        <x:v>2165</x:v>
       </x:c>
       <x:c r="E39" s="134" t="s">
         <x:v>1311</x:v>
@@ -53837,10 +53832,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G39" s="319" t="s">
+        <x:v>2166</x:v>
+      </x:c>
+      <x:c r="H39" s="297" t="s">
         <x:v>2167</x:v>
-      </x:c>
-      <x:c r="H39" s="297" t="s">
-        <x:v>2168</x:v>
       </x:c>
       <x:c r="I39" s="134" t="s">
         <x:v>1317</x:v>
@@ -53862,7 +53857,7 @@
         <x:v>990</x:v>
       </x:c>
       <x:c r="H40" s="314" t="s">
-        <x:v>2165</x:v>
+        <x:v>2164</x:v>
       </x:c>
       <x:c r="I40" s="134"/>
       <x:c r="J40" s="9"/>
@@ -56798,17 +56793,17 @@
     <x:mergeCell ref="J168:J171"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H22" r:id="rId186"/>
-    <x:hyperlink ref="H28" r:id="rId187"/>
-    <x:hyperlink ref="H11" r:id="rId188"/>
-    <x:hyperlink ref="H16" r:id="rId189"/>
-    <x:hyperlink ref="H37" r:id="rId190"/>
-    <x:hyperlink ref="H40" r:id="rId191"/>
-    <x:hyperlink ref="H130" r:id="rId192"/>
-    <x:hyperlink ref="H136" r:id="rId193"/>
-    <x:hyperlink ref="H142" r:id="rId194"/>
-    <x:hyperlink ref="H148" r:id="rId195"/>
-    <x:hyperlink ref="H154" r:id="rId196"/>
+    <x:hyperlink ref="H22" r:id="rId144"/>
+    <x:hyperlink ref="H28" r:id="rId145"/>
+    <x:hyperlink ref="H11" r:id="rId146"/>
+    <x:hyperlink ref="H16" r:id="rId147"/>
+    <x:hyperlink ref="H37" r:id="rId148"/>
+    <x:hyperlink ref="H40" r:id="rId149"/>
+    <x:hyperlink ref="H130" r:id="rId150"/>
+    <x:hyperlink ref="H136" r:id="rId151"/>
+    <x:hyperlink ref="H142" r:id="rId152"/>
+    <x:hyperlink ref="H148" r:id="rId153"/>
+    <x:hyperlink ref="H154" r:id="rId154"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -56893,19 +56888,19 @@
         <x:v>705</x:v>
       </x:c>
       <x:c r="E2" s="116" t="s">
-        <x:v>2169</x:v>
+        <x:v>2168</x:v>
       </x:c>
       <x:c r="F2" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G2" s="327" t="s">
+        <x:v>2169</x:v>
+      </x:c>
+      <x:c r="H2" s="116" t="s">
         <x:v>2170</x:v>
       </x:c>
-      <x:c r="H2" s="116" t="s">
+      <x:c r="I2" s="289" t="s">
         <x:v>2171</x:v>
-      </x:c>
-      <x:c r="I2" s="289" t="s">
-        <x:v>2172</x:v>
       </x:c>
       <x:c r="J2" s="1"/>
       <x:c r="K2" s="1"/>
@@ -56921,11 +56916,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G3" s="327" t="s">
-        <x:v>2173</x:v>
+        <x:v>2172</x:v>
       </x:c>
       <x:c r="H3" s="116"/>
       <x:c r="I3" s="289" t="s">
-        <x:v>2174</x:v>
+        <x:v>2173</x:v>
       </x:c>
       <x:c r="J3" s="1"/>
       <x:c r="K3" s="1"/>
@@ -56945,19 +56940,19 @@
         <x:v>707</x:v>
       </x:c>
       <x:c r="E4" s="116" t="s">
-        <x:v>2169</x:v>
+        <x:v>2168</x:v>
       </x:c>
       <x:c r="F4" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="327" t="s">
+        <x:v>2174</x:v>
+      </x:c>
+      <x:c r="H4" s="116" t="s">
         <x:v>2175</x:v>
       </x:c>
-      <x:c r="H4" s="116" t="s">
+      <x:c r="I4" s="289" t="s">
         <x:v>2176</x:v>
-      </x:c>
-      <x:c r="I4" s="289" t="s">
-        <x:v>2177</x:v>
       </x:c>
       <x:c r="J4" s="61"/>
       <x:c r="K4" s="1"/>
@@ -56973,11 +56968,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G5" s="327" t="s">
-        <x:v>2178</x:v>
+        <x:v>2177</x:v>
       </x:c>
       <x:c r="H5" s="116"/>
       <x:c r="I5" s="289" t="s">
-        <x:v>2179</x:v>
+        <x:v>2178</x:v>
       </x:c>
       <x:c r="J5" s="61"/>
       <x:c r="K5" s="1"/>
@@ -56993,11 +56988,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G6" s="327" t="s">
-        <x:v>2072</x:v>
+        <x:v>2071</x:v>
       </x:c>
       <x:c r="H6" s="116"/>
       <x:c r="I6" s="289" t="s">
-        <x:v>2180</x:v>
+        <x:v>2179</x:v>
       </x:c>
       <x:c r="J6" s="61"/>
       <x:c r="K6" s="1"/>
@@ -57017,19 +57012,19 @@
         <x:v>709</x:v>
       </x:c>
       <x:c r="E7" s="116" t="s">
-        <x:v>2181</x:v>
+        <x:v>2180</x:v>
       </x:c>
       <x:c r="F7" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="327" t="s">
+        <x:v>2181</x:v>
+      </x:c>
+      <x:c r="H7" s="116" t="s">
         <x:v>2182</x:v>
       </x:c>
-      <x:c r="H7" s="116" t="s">
+      <x:c r="I7" s="289" t="s">
         <x:v>2183</x:v>
-      </x:c>
-      <x:c r="I7" s="289" t="s">
-        <x:v>2184</x:v>
       </x:c>
       <x:c r="J7" s="61"/>
       <x:c r="K7" s="1"/>
@@ -57045,11 +57040,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G8" s="327" t="s">
-        <x:v>2072</x:v>
+        <x:v>2071</x:v>
       </x:c>
       <x:c r="H8" s="116"/>
       <x:c r="I8" s="289" t="s">
-        <x:v>2185</x:v>
+        <x:v>2184</x:v>
       </x:c>
       <x:c r="J8" s="61"/>
       <x:c r="K8" s="1"/>
@@ -57065,11 +57060,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G9" s="327" t="s">
-        <x:v>2186</x:v>
+        <x:v>2185</x:v>
       </x:c>
       <x:c r="H9" s="116"/>
       <x:c r="I9" s="289" t="s">
-        <x:v>2187</x:v>
+        <x:v>2186</x:v>
       </x:c>
       <x:c r="J9" s="61"/>
       <x:c r="K9" s="1"/>
@@ -57086,20 +57081,20 @@
         <x:v>717</x:v>
       </x:c>
       <x:c r="D10" s="116" t="s">
+        <x:v>2187</x:v>
+      </x:c>
+      <x:c r="E10" s="116" t="s">
         <x:v>2188</x:v>
-      </x:c>
-      <x:c r="E10" s="116" t="s">
-        <x:v>2189</x:v>
       </x:c>
       <x:c r="F10" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="327" t="s">
-        <x:v>2093</x:v>
+        <x:v>2092</x:v>
       </x:c>
       <x:c r="H10" s="116"/>
       <x:c r="I10" s="289" t="s">
-        <x:v>2190</x:v>
+        <x:v>2189</x:v>
       </x:c>
       <x:c r="J10" s="61"/>
       <x:c r="K10" s="1"/>
@@ -57115,11 +57110,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G11" s="327" t="s">
-        <x:v>2191</x:v>
+        <x:v>2190</x:v>
       </x:c>
       <x:c r="H11" s="116"/>
       <x:c r="I11" s="289" t="s">
-        <x:v>2192</x:v>
+        <x:v>2191</x:v>
       </x:c>
       <x:c r="J11" s="61"/>
       <x:c r="K11" s="1"/>
@@ -57135,11 +57130,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G12" s="327" t="s">
-        <x:v>2193</x:v>
+        <x:v>2192</x:v>
       </x:c>
       <x:c r="H12" s="116"/>
       <x:c r="I12" s="289" t="s">
-        <x:v>2194</x:v>
+        <x:v>2193</x:v>
       </x:c>
       <x:c r="J12" s="61"/>
       <x:c r="K12" s="1"/>
@@ -57156,20 +57151,20 @@
         <x:v>722</x:v>
       </x:c>
       <x:c r="D13" s="116" t="s">
+        <x:v>2194</x:v>
+      </x:c>
+      <x:c r="E13" s="116" t="s">
         <x:v>2195</x:v>
-      </x:c>
-      <x:c r="E13" s="116" t="s">
-        <x:v>2196</x:v>
       </x:c>
       <x:c r="F13" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="327" t="s">
-        <x:v>2072</x:v>
+        <x:v>2071</x:v>
       </x:c>
       <x:c r="H13" s="116"/>
       <x:c r="I13" s="289" t="s">
-        <x:v>2197</x:v>
+        <x:v>2196</x:v>
       </x:c>
       <x:c r="J13" s="61"/>
       <x:c r="K13" s="1"/>
@@ -57185,11 +57180,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="327" t="s">
-        <x:v>2198</x:v>
+        <x:v>2197</x:v>
       </x:c>
       <x:c r="H14" s="116"/>
       <x:c r="I14" s="289" t="s">
-        <x:v>2199</x:v>
+        <x:v>2198</x:v>
       </x:c>
       <x:c r="J14" s="61"/>
       <x:c r="K14" s="1"/>
@@ -57206,22 +57201,22 @@
         <x:v>724</x:v>
       </x:c>
       <x:c r="D15" s="116" t="s">
+        <x:v>2199</x:v>
+      </x:c>
+      <x:c r="E15" s="116" t="s">
         <x:v>2200</x:v>
-      </x:c>
-      <x:c r="E15" s="116" t="s">
-        <x:v>2201</x:v>
       </x:c>
       <x:c r="F15" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G15" s="327" t="s">
+        <x:v>2201</x:v>
+      </x:c>
+      <x:c r="H15" s="116" t="s">
         <x:v>2202</x:v>
       </x:c>
-      <x:c r="H15" s="116" t="s">
+      <x:c r="I15" s="289" t="s">
         <x:v>2203</x:v>
-      </x:c>
-      <x:c r="I15" s="289" t="s">
-        <x:v>2204</x:v>
       </x:c>
       <x:c r="J15" s="61"/>
       <x:c r="K15" s="1"/>
@@ -57237,11 +57232,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G16" s="327" t="s">
-        <x:v>2205</x:v>
+        <x:v>2204</x:v>
       </x:c>
       <x:c r="H16" s="116"/>
       <x:c r="I16" s="289" t="s">
-        <x:v>2206</x:v>
+        <x:v>2205</x:v>
       </x:c>
       <x:c r="J16" s="61"/>
       <x:c r="K16" s="1"/>
@@ -57257,11 +57252,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G17" s="327" t="s">
-        <x:v>2207</x:v>
+        <x:v>2206</x:v>
       </x:c>
       <x:c r="H17" s="116"/>
       <x:c r="I17" s="289" t="s">
-        <x:v>2208</x:v>
+        <x:v>2207</x:v>
       </x:c>
       <x:c r="J17" s="61"/>
       <x:c r="K17" s="1"/>
@@ -57278,20 +57273,20 @@
         <x:v>726</x:v>
       </x:c>
       <x:c r="D18" s="116" t="s">
+        <x:v>2208</x:v>
+      </x:c>
+      <x:c r="E18" s="116" t="s">
         <x:v>2209</x:v>
-      </x:c>
-      <x:c r="E18" s="116" t="s">
-        <x:v>2210</x:v>
       </x:c>
       <x:c r="F18" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="327" t="s">
-        <x:v>2211</x:v>
+        <x:v>2210</x:v>
       </x:c>
       <x:c r="H18" s="116"/>
       <x:c r="I18" s="289" t="s">
-        <x:v>2212</x:v>
+        <x:v>2211</x:v>
       </x:c>
       <x:c r="J18" s="61"/>
       <x:c r="K18" s="1"/>
@@ -57307,13 +57302,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="327" t="s">
+        <x:v>2212</x:v>
+      </x:c>
+      <x:c r="H19" s="116" t="s">
         <x:v>2213</x:v>
       </x:c>
-      <x:c r="H19" s="116" t="s">
+      <x:c r="I19" s="289" t="s">
         <x:v>2214</x:v>
-      </x:c>
-      <x:c r="I19" s="289" t="s">
-        <x:v>2215</x:v>
       </x:c>
       <x:c r="J19" s="61"/>
       <x:c r="K19" s="1"/>
@@ -57329,11 +57324,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="327" t="s">
-        <x:v>2216</x:v>
+        <x:v>2215</x:v>
       </x:c>
       <x:c r="H20" s="116"/>
       <x:c r="I20" s="289" t="s">
-        <x:v>2217</x:v>
+        <x:v>2216</x:v>
       </x:c>
       <x:c r="J20" s="61"/>
       <x:c r="K20" s="1"/>
@@ -57344,7 +57339,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B21" s="116" t="s">
-        <x:v>2218</x:v>
+        <x:v>2217</x:v>
       </x:c>
       <x:c r="C21" s="116" t="s">
         <x:v>732</x:v>
@@ -57353,19 +57348,19 @@
         <x:v>733</x:v>
       </x:c>
       <x:c r="E21" s="116" t="s">
-        <x:v>2219</x:v>
+        <x:v>2218</x:v>
       </x:c>
       <x:c r="F21" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G21" s="327" t="s">
-        <x:v>2220</x:v>
+        <x:v>2219</x:v>
       </x:c>
       <x:c r="H21" s="116" t="s">
         <x:v>741</x:v>
       </x:c>
       <x:c r="I21" s="289" t="s">
-        <x:v>2221</x:v>
+        <x:v>2220</x:v>
       </x:c>
       <x:c r="J21" s="61"/>
       <x:c r="K21" s="1"/>
@@ -57381,11 +57376,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G22" s="327" t="s">
-        <x:v>2222</x:v>
+        <x:v>2221</x:v>
       </x:c>
       <x:c r="H22" s="116"/>
       <x:c r="I22" s="289" t="s">
-        <x:v>2223</x:v>
+        <x:v>2222</x:v>
       </x:c>
       <x:c r="J22" s="61"/>
       <x:c r="K22" s="1"/>
@@ -57401,11 +57396,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G23" s="327" t="s">
-        <x:v>2224</x:v>
+        <x:v>2223</x:v>
       </x:c>
       <x:c r="H23" s="116"/>
       <x:c r="I23" s="289" t="s">
-        <x:v>2225</x:v>
+        <x:v>2224</x:v>
       </x:c>
       <x:c r="J23" s="61"/>
       <x:c r="K23" s="1"/>
@@ -57422,20 +57417,20 @@
         <x:v>737</x:v>
       </x:c>
       <x:c r="D24" s="116" t="s">
+        <x:v>2225</x:v>
+      </x:c>
+      <x:c r="E24" s="116" t="s">
         <x:v>2226</x:v>
-      </x:c>
-      <x:c r="E24" s="116" t="s">
-        <x:v>2227</x:v>
       </x:c>
       <x:c r="F24" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G24" s="327" t="s">
-        <x:v>2228</x:v>
+        <x:v>2227</x:v>
       </x:c>
       <x:c r="H24" s="116"/>
       <x:c r="I24" s="289" t="s">
-        <x:v>2229</x:v>
+        <x:v>2228</x:v>
       </x:c>
       <x:c r="J24" s="61"/>
       <x:c r="K24" s="35"/>
@@ -57451,11 +57446,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G25" s="327" t="s">
-        <x:v>2230</x:v>
+        <x:v>2229</x:v>
       </x:c>
       <x:c r="H25" s="116"/>
       <x:c r="I25" s="289" t="s">
-        <x:v>2231</x:v>
+        <x:v>2230</x:v>
       </x:c>
       <x:c r="J25" s="61"/>
       <x:c r="K25" s="35"/>
@@ -57471,11 +57466,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G26" s="327" t="s">
-        <x:v>2123</x:v>
+        <x:v>2122</x:v>
       </x:c>
       <x:c r="H26" s="116"/>
       <x:c r="I26" s="289" t="s">
-        <x:v>2232</x:v>
+        <x:v>2231</x:v>
       </x:c>
       <x:c r="J26" s="61"/>
       <x:c r="K26" s="35"/>
@@ -57492,20 +57487,20 @@
         <x:v>751</x:v>
       </x:c>
       <x:c r="D27" s="116" t="s">
+        <x:v>2232</x:v>
+      </x:c>
+      <x:c r="E27" s="116" t="s">
         <x:v>2233</x:v>
-      </x:c>
-      <x:c r="E27" s="116" t="s">
-        <x:v>2234</x:v>
       </x:c>
       <x:c r="F27" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G27" s="327" t="s">
-        <x:v>2235</x:v>
+        <x:v>2234</x:v>
       </x:c>
       <x:c r="H27" s="116"/>
       <x:c r="I27" s="327" t="s">
-        <x:v>2078</x:v>
+        <x:v>2077</x:v>
       </x:c>
       <x:c r="J27" s="61"/>
       <x:c r="K27" s="35"/>
@@ -57521,11 +57516,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G28" s="327" t="s">
-        <x:v>2236</x:v>
+        <x:v>2235</x:v>
       </x:c>
       <x:c r="H28" s="116"/>
       <x:c r="I28" s="289" t="s">
-        <x:v>2237</x:v>
+        <x:v>2236</x:v>
       </x:c>
       <x:c r="J28" s="61"/>
       <x:c r="K28" s="35"/>
@@ -57542,20 +57537,20 @@
         <x:v>753</x:v>
       </x:c>
       <x:c r="D29" s="116" t="s">
-        <x:v>2238</x:v>
+        <x:v>2237</x:v>
       </x:c>
       <x:c r="E29" s="116" t="s">
-        <x:v>2234</x:v>
+        <x:v>2233</x:v>
       </x:c>
       <x:c r="F29" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G29" s="327" t="s">
-        <x:v>2239</x:v>
+        <x:v>2238</x:v>
       </x:c>
       <x:c r="H29" s="116"/>
       <x:c r="I29" s="327" t="s">
-        <x:v>2078</x:v>
+        <x:v>2077</x:v>
       </x:c>
       <x:c r="J29" s="61"/>
       <x:c r="K29" s="35"/>
@@ -57571,11 +57566,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G30" s="327" t="s">
-        <x:v>2240</x:v>
+        <x:v>2239</x:v>
       </x:c>
       <x:c r="H30" s="116"/>
       <x:c r="I30" s="289" t="s">
-        <x:v>2241</x:v>
+        <x:v>2240</x:v>
       </x:c>
       <x:c r="J30" s="61"/>
       <x:c r="K30" s="35"/>
@@ -57595,19 +57590,19 @@
         <x:v>793</x:v>
       </x:c>
       <x:c r="E31" s="116" t="s">
-        <x:v>2242</x:v>
+        <x:v>2241</x:v>
       </x:c>
       <x:c r="F31" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="327" t="s">
+        <x:v>2242</x:v>
+      </x:c>
+      <x:c r="H31" s="116" t="s">
         <x:v>2243</x:v>
       </x:c>
-      <x:c r="H31" s="116" t="s">
+      <x:c r="I31" s="289" t="s">
         <x:v>2244</x:v>
-      </x:c>
-      <x:c r="I31" s="289" t="s">
-        <x:v>2245</x:v>
       </x:c>
       <x:c r="J31" s="61"/>
       <x:c r="K31" s="35"/>
@@ -57623,11 +57618,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G32" s="327" t="s">
-        <x:v>2246</x:v>
+        <x:v>2245</x:v>
       </x:c>
       <x:c r="H32" s="116"/>
       <x:c r="I32" s="289" t="s">
-        <x:v>2247</x:v>
+        <x:v>2246</x:v>
       </x:c>
       <x:c r="J32" s="61"/>
       <x:c r="K32" s="35"/>
@@ -57647,19 +57642,19 @@
         <x:v>798</x:v>
       </x:c>
       <x:c r="E33" s="116" t="s">
-        <x:v>2248</x:v>
+        <x:v>2247</x:v>
       </x:c>
       <x:c r="F33" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G33" s="327" t="s">
-        <x:v>2249</x:v>
+        <x:v>2248</x:v>
       </x:c>
       <x:c r="H33" s="116" t="s">
-        <x:v>2244</x:v>
+        <x:v>2243</x:v>
       </x:c>
       <x:c r="I33" s="327" t="s">
-        <x:v>2078</x:v>
+        <x:v>2077</x:v>
       </x:c>
       <x:c r="J33" s="61"/>
       <x:c r="K33" s="35"/>
@@ -57675,11 +57670,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G34" s="327" t="s">
-        <x:v>2250</x:v>
+        <x:v>2249</x:v>
       </x:c>
       <x:c r="H34" s="116"/>
       <x:c r="I34" s="289" t="s">
-        <x:v>2251</x:v>
+        <x:v>2250</x:v>
       </x:c>
       <x:c r="J34" s="292"/>
       <x:c r="K34" s="35"/>
@@ -57696,20 +57691,20 @@
         <x:v>802</x:v>
       </x:c>
       <x:c r="D35" s="116" t="s">
+        <x:v>2251</x:v>
+      </x:c>
+      <x:c r="E35" s="116" t="s">
         <x:v>2252</x:v>
-      </x:c>
-      <x:c r="E35" s="116" t="s">
-        <x:v>2253</x:v>
       </x:c>
       <x:c r="F35" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G35" s="327" t="s">
-        <x:v>2254</x:v>
+        <x:v>2253</x:v>
       </x:c>
       <x:c r="H35" s="116"/>
       <x:c r="I35" s="289" t="s">
-        <x:v>2255</x:v>
+        <x:v>2254</x:v>
       </x:c>
       <x:c r="J35" s="61"/>
       <x:c r="K35" s="35"/>
@@ -57725,11 +57720,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G36" s="327" t="s">
-        <x:v>2256</x:v>
+        <x:v>2255</x:v>
       </x:c>
       <x:c r="H36" s="116"/>
       <x:c r="I36" s="289" t="s">
-        <x:v>2257</x:v>
+        <x:v>2256</x:v>
       </x:c>
       <x:c r="J36" s="61"/>
       <x:c r="K36" s="35"/>
@@ -57745,13 +57740,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G37" s="327" t="s">
+        <x:v>2257</x:v>
+      </x:c>
+      <x:c r="H37" s="116" t="s">
         <x:v>2258</x:v>
       </x:c>
-      <x:c r="H37" s="116" t="s">
+      <x:c r="I37" s="289" t="s">
         <x:v>2259</x:v>
-      </x:c>
-      <x:c r="I37" s="289" t="s">
-        <x:v>2260</x:v>
       </x:c>
       <x:c r="J37" s="61"/>
       <x:c r="K37" s="35"/>
@@ -57768,20 +57763,20 @@
         <x:v>814</x:v>
       </x:c>
       <x:c r="D38" s="116" t="s">
+        <x:v>2260</x:v>
+      </x:c>
+      <x:c r="E38" s="116" t="s">
         <x:v>2261</x:v>
-      </x:c>
-      <x:c r="E38" s="116" t="s">
-        <x:v>2262</x:v>
       </x:c>
       <x:c r="F38" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G38" s="327" t="s">
-        <x:v>2263</x:v>
+        <x:v>2262</x:v>
       </x:c>
       <x:c r="H38" s="116"/>
       <x:c r="I38" s="289" t="s">
-        <x:v>2264</x:v>
+        <x:v>2263</x:v>
       </x:c>
       <x:c r="J38" s="61"/>
       <x:c r="K38" s="35"/>
@@ -57797,11 +57792,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G39" s="327" t="s">
-        <x:v>2265</x:v>
+        <x:v>2264</x:v>
       </x:c>
       <x:c r="H39" s="116"/>
       <x:c r="I39" s="289" t="s">
-        <x:v>2266</x:v>
+        <x:v>2265</x:v>
       </x:c>
       <x:c r="J39" s="61"/>
       <x:c r="K39" s="35"/>
@@ -57817,13 +57812,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G40" s="327" t="s">
+        <x:v>2266</x:v>
+      </x:c>
+      <x:c r="H40" s="116" t="s">
+        <x:v>2258</x:v>
+      </x:c>
+      <x:c r="I40" s="289" t="s">
         <x:v>2267</x:v>
-      </x:c>
-      <x:c r="H40" s="116" t="s">
-        <x:v>2259</x:v>
-      </x:c>
-      <x:c r="I40" s="289" t="s">
-        <x:v>2268</x:v>
       </x:c>
       <x:c r="J40" s="61"/>
       <x:c r="K40" s="35"/>
@@ -57839,11 +57834,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G41" s="327" t="s">
-        <x:v>2269</x:v>
+        <x:v>2268</x:v>
       </x:c>
       <x:c r="H41" s="116"/>
       <x:c r="I41" s="289" t="s">
-        <x:v>2270</x:v>
+        <x:v>2269</x:v>
       </x:c>
       <x:c r="J41" s="61"/>
       <x:c r="K41" s="35"/>
@@ -57860,20 +57855,20 @@
         <x:v>824</x:v>
       </x:c>
       <x:c r="D42" s="116" t="s">
+        <x:v>2270</x:v>
+      </x:c>
+      <x:c r="E42" s="116" t="s">
         <x:v>2271</x:v>
-      </x:c>
-      <x:c r="E42" s="116" t="s">
-        <x:v>2272</x:v>
       </x:c>
       <x:c r="F42" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G42" s="327" t="s">
-        <x:v>2273</x:v>
+        <x:v>2272</x:v>
       </x:c>
       <x:c r="H42" s="116"/>
       <x:c r="I42" s="289" t="s">
-        <x:v>2274</x:v>
+        <x:v>2273</x:v>
       </x:c>
       <x:c r="J42" s="61"/>
       <x:c r="K42" s="35"/>
@@ -57889,11 +57884,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G43" s="327" t="s">
-        <x:v>2275</x:v>
+        <x:v>2274</x:v>
       </x:c>
       <x:c r="H43" s="116"/>
       <x:c r="I43" s="289" t="s">
-        <x:v>2276</x:v>
+        <x:v>2275</x:v>
       </x:c>
       <x:c r="J43" s="61"/>
       <x:c r="K43" s="35"/>
@@ -57909,11 +57904,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G44" s="327" t="s">
-        <x:v>2277</x:v>
+        <x:v>2276</x:v>
       </x:c>
       <x:c r="H44" s="116"/>
       <x:c r="I44" s="289" t="s">
-        <x:v>2278</x:v>
+        <x:v>2277</x:v>
       </x:c>
       <x:c r="J44" s="61"/>
       <x:c r="K44" s="35"/>
@@ -57929,11 +57924,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G45" s="327" t="s">
-        <x:v>2279</x:v>
+        <x:v>2278</x:v>
       </x:c>
       <x:c r="H45" s="116"/>
       <x:c r="I45" s="289" t="s">
-        <x:v>2280</x:v>
+        <x:v>2279</x:v>
       </x:c>
       <x:c r="J45" s="61"/>
       <x:c r="K45" s="35"/>
@@ -57950,20 +57945,20 @@
         <x:v>835</x:v>
       </x:c>
       <x:c r="D46" s="116" t="s">
+        <x:v>2280</x:v>
+      </x:c>
+      <x:c r="E46" s="116" t="s">
         <x:v>2281</x:v>
-      </x:c>
-      <x:c r="E46" s="116" t="s">
-        <x:v>2282</x:v>
       </x:c>
       <x:c r="F46" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G46" s="327" t="s">
-        <x:v>2273</x:v>
+        <x:v>2272</x:v>
       </x:c>
       <x:c r="H46" s="116"/>
       <x:c r="I46" s="289" t="s">
-        <x:v>2283</x:v>
+        <x:v>2282</x:v>
       </x:c>
       <x:c r="J46" s="61"/>
       <x:c r="K46" s="35"/>
@@ -57979,13 +57974,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G47" s="327" t="s">
+        <x:v>2283</x:v>
+      </x:c>
+      <x:c r="H47" s="116" t="s">
+        <x:v>2258</x:v>
+      </x:c>
+      <x:c r="I47" s="289" t="s">
         <x:v>2284</x:v>
-      </x:c>
-      <x:c r="H47" s="116" t="s">
-        <x:v>2259</x:v>
-      </x:c>
-      <x:c r="I47" s="289" t="s">
-        <x:v>2285</x:v>
       </x:c>
       <x:c r="J47" s="61"/>
       <x:c r="K47" s="35"/>
@@ -58001,11 +57996,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G48" s="327" t="s">
-        <x:v>2286</x:v>
+        <x:v>2285</x:v>
       </x:c>
       <x:c r="H48" s="116"/>
       <x:c r="I48" s="289" t="s">
-        <x:v>2287</x:v>
+        <x:v>2286</x:v>
       </x:c>
       <x:c r="J48" s="61"/>
       <x:c r="K48" s="35"/>
@@ -58104,10 +58099,10 @@
         <x:v>999</x:v>
       </x:c>
       <x:c r="H52" s="334" t="s">
+        <x:v>2287</x:v>
+      </x:c>
+      <x:c r="I52" s="51" t="s">
         <x:v>2288</x:v>
-      </x:c>
-      <x:c r="I52" s="51" t="s">
-        <x:v>2289</x:v>
       </x:c>
       <x:c r="J52" s="51"/>
       <x:c r="K52" s="35"/>
@@ -58126,7 +58121,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H53" s="314" t="s">
-        <x:v>2290</x:v>
+        <x:v>2289</x:v>
       </x:c>
       <x:c r="I53" s="51"/>
       <x:c r="J53" s="51"/>
@@ -58177,7 +58172,7 @@
         <x:v>1000</x:v>
       </x:c>
       <x:c r="I55" s="51" t="s">
-        <x:v>2291</x:v>
+        <x:v>2290</x:v>
       </x:c>
       <x:c r="J55" s="51"/>
       <x:c r="K55" s="35"/>
@@ -58196,7 +58191,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H56" s="314" t="s">
-        <x:v>2292</x:v>
+        <x:v>2291</x:v>
       </x:c>
       <x:c r="I56" s="51"/>
       <x:c r="J56" s="51"/>
@@ -58315,7 +58310,7 @@
         <x:v>422</x:v>
       </x:c>
       <x:c r="I61" s="51" t="s">
-        <x:v>2293</x:v>
+        <x:v>2292</x:v>
       </x:c>
       <x:c r="J61" s="51"/>
       <x:c r="K61" s="35"/>
@@ -58613,7 +58608,7 @@
         <x:v>1037</x:v>
       </x:c>
       <x:c r="I74" s="51" t="s">
-        <x:v>2294</x:v>
+        <x:v>2293</x:v>
       </x:c>
       <x:c r="J74" s="51"/>
       <x:c r="K74" s="35"/>
@@ -59309,19 +59304,19 @@
         <x:v>843</x:v>
       </x:c>
       <x:c r="E106" s="116" t="s">
-        <x:v>2295</x:v>
+        <x:v>2294</x:v>
       </x:c>
       <x:c r="F106" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G106" s="327" t="s">
+        <x:v>2295</x:v>
+      </x:c>
+      <x:c r="H106" s="116" t="s">
         <x:v>2296</x:v>
       </x:c>
-      <x:c r="H106" s="116" t="s">
+      <x:c r="I106" s="289" t="s">
         <x:v>2297</x:v>
-      </x:c>
-      <x:c r="I106" s="289" t="s">
-        <x:v>2298</x:v>
       </x:c>
       <x:c r="J106" s="61"/>
       <x:c r="K106" s="140"/>
@@ -59337,11 +59332,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G107" s="327" t="s">
-        <x:v>2299</x:v>
+        <x:v>2298</x:v>
       </x:c>
       <x:c r="H107" s="116"/>
       <x:c r="I107" s="289" t="s">
-        <x:v>2300</x:v>
+        <x:v>2299</x:v>
       </x:c>
       <x:c r="J107" s="61"/>
       <x:c r="K107" s="140"/>
@@ -59357,13 +59352,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G108" s="327" t="s">
+        <x:v>2300</x:v>
+      </x:c>
+      <x:c r="H108" s="116" t="s">
         <x:v>2301</x:v>
       </x:c>
-      <x:c r="H108" s="116" t="s">
+      <x:c r="I108" s="289" t="s">
         <x:v>2302</x:v>
-      </x:c>
-      <x:c r="I108" s="289" t="s">
-        <x:v>2303</x:v>
       </x:c>
       <x:c r="J108" s="61"/>
       <x:c r="K108" s="140"/>
@@ -59379,11 +59374,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G109" s="327" t="s">
-        <x:v>2304</x:v>
+        <x:v>2303</x:v>
       </x:c>
       <x:c r="H109" s="116"/>
       <x:c r="I109" s="289" t="s">
-        <x:v>2305</x:v>
+        <x:v>2304</x:v>
       </x:c>
       <x:c r="J109" s="61"/>
       <x:c r="K109" s="140"/>
@@ -59403,19 +59398,19 @@
         <x:v>854</x:v>
       </x:c>
       <x:c r="E110" s="116" t="s">
-        <x:v>2306</x:v>
+        <x:v>2305</x:v>
       </x:c>
       <x:c r="F110" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G110" s="327" t="s">
+        <x:v>2306</x:v>
+      </x:c>
+      <x:c r="H110" s="116" t="s">
         <x:v>2307</x:v>
       </x:c>
-      <x:c r="H110" s="116" t="s">
+      <x:c r="I110" s="289" t="s">
         <x:v>2308</x:v>
-      </x:c>
-      <x:c r="I110" s="289" t="s">
-        <x:v>2309</x:v>
       </x:c>
       <x:c r="J110" s="61"/>
       <x:c r="K110" s="140"/>
@@ -59431,11 +59426,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G111" s="327" t="s">
-        <x:v>2299</x:v>
+        <x:v>2298</x:v>
       </x:c>
       <x:c r="H111" s="116"/>
       <x:c r="I111" s="289" t="s">
-        <x:v>2310</x:v>
+        <x:v>2309</x:v>
       </x:c>
       <x:c r="J111" s="61"/>
       <x:c r="K111" s="140"/>
@@ -59451,13 +59446,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G112" s="327" t="s">
+        <x:v>2310</x:v>
+      </x:c>
+      <x:c r="H112" s="116" t="s">
         <x:v>2311</x:v>
       </x:c>
-      <x:c r="H112" s="116" t="s">
+      <x:c r="I112" s="289" t="s">
         <x:v>2312</x:v>
-      </x:c>
-      <x:c r="I112" s="289" t="s">
-        <x:v>2313</x:v>
       </x:c>
       <x:c r="J112" s="61"/>
       <x:c r="K112" s="140"/>
@@ -59473,11 +59468,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G113" s="327" t="s">
-        <x:v>2314</x:v>
+        <x:v>2313</x:v>
       </x:c>
       <x:c r="H113" s="116"/>
       <x:c r="I113" s="289" t="s">
-        <x:v>2315</x:v>
+        <x:v>2314</x:v>
       </x:c>
       <x:c r="J113" s="61"/>
       <x:c r="K113" s="140"/>
@@ -59494,7 +59489,7 @@
         <x:v>863</x:v>
       </x:c>
       <x:c r="D114" s="140" t="s">
-        <x:v>2316</x:v>
+        <x:v>2315</x:v>
       </x:c>
       <x:c r="E114" s="140" t="s">
         <x:v>865</x:v>
@@ -59503,7 +59498,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G114" s="61" t="s">
-        <x:v>2317</x:v>
+        <x:v>2316</x:v>
       </x:c>
       <x:c r="H114" s="140"/>
       <x:c r="I114" s="61" t="s">
@@ -59523,7 +59518,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G115" s="61" t="s">
-        <x:v>2318</x:v>
+        <x:v>2317</x:v>
       </x:c>
       <x:c r="H115" s="140"/>
       <x:c r="I115" s="61" t="s">
@@ -59543,10 +59538,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G116" s="61" t="s">
+        <x:v>2318</x:v>
+      </x:c>
+      <x:c r="H116" s="140" t="s">
         <x:v>2319</x:v>
-      </x:c>
-      <x:c r="H116" s="140" t="s">
-        <x:v>2320</x:v>
       </x:c>
       <x:c r="I116" s="61"/>
       <x:c r="J116" s="140"/>
@@ -59563,10 +59558,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G117" s="61" t="s">
+        <x:v>2320</x:v>
+      </x:c>
+      <x:c r="H117" s="140" t="s">
         <x:v>2321</x:v>
-      </x:c>
-      <x:c r="H117" s="140" t="s">
-        <x:v>2322</x:v>
       </x:c>
       <x:c r="I117" s="61"/>
       <x:c r="J117" s="140"/>
@@ -59601,7 +59596,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G119" s="61" t="s">
-        <x:v>2323</x:v>
+        <x:v>2322</x:v>
       </x:c>
       <x:c r="H119" s="140" t="s">
         <x:v>877</x:v>
@@ -59621,7 +59616,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G120" s="61" t="s">
-        <x:v>2324</x:v>
+        <x:v>2323</x:v>
       </x:c>
       <x:c r="H120" s="251">
         <x:v>0.375</x:v>
@@ -59641,7 +59636,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G121" s="61" t="s">
-        <x:v>2325</x:v>
+        <x:v>2324</x:v>
       </x:c>
       <x:c r="H121" s="140">
         <x:v>100000</x:v>
@@ -59661,7 +59656,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="G122" s="61" t="s">
-        <x:v>2326</x:v>
+        <x:v>2325</x:v>
       </x:c>
       <x:c r="H122" s="140">
         <x:v>1</x:v>
@@ -59681,7 +59676,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G123" s="61" t="s">
-        <x:v>2327</x:v>
+        <x:v>2326</x:v>
       </x:c>
       <x:c r="H123" s="140"/>
       <x:c r="I123" s="61" t="s">
@@ -59702,7 +59697,7 @@
         <x:v>884</x:v>
       </x:c>
       <x:c r="D124" s="140" t="s">
-        <x:v>2328</x:v>
+        <x:v>2327</x:v>
       </x:c>
       <x:c r="E124" s="140" t="s">
         <x:v>886</x:v>
@@ -59711,7 +59706,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G124" s="61" t="s">
-        <x:v>2329</x:v>
+        <x:v>2328</x:v>
       </x:c>
       <x:c r="H124" s="140"/>
       <x:c r="I124" s="140" t="s">
@@ -59731,7 +59726,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G125" s="61" t="s">
-        <x:v>2330</x:v>
+        <x:v>2329</x:v>
       </x:c>
       <x:c r="H125" s="140"/>
       <x:c r="I125" s="140"/>
@@ -59749,10 +59744,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G126" s="61" t="s">
+        <x:v>2330</x:v>
+      </x:c>
+      <x:c r="H126" s="140" t="s">
         <x:v>2331</x:v>
-      </x:c>
-      <x:c r="H126" s="140" t="s">
-        <x:v>2332</x:v>
       </x:c>
       <x:c r="I126" s="140"/>
       <x:c r="J126" s="140"/>
@@ -59769,10 +59764,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G127" s="61" t="s">
+        <x:v>2332</x:v>
+      </x:c>
+      <x:c r="H127" s="140" t="s">
         <x:v>2333</x:v>
-      </x:c>
-      <x:c r="H127" s="140" t="s">
-        <x:v>2334</x:v>
       </x:c>
       <x:c r="I127" s="140"/>
       <x:c r="J127" s="140"/>
@@ -59789,7 +59784,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G128" s="61" t="s">
-        <x:v>2335</x:v>
+        <x:v>2334</x:v>
       </x:c>
       <x:c r="H128" s="140" t="s">
         <x:v>877</x:v>
@@ -59827,7 +59822,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G130" s="61" t="s">
-        <x:v>2336</x:v>
+        <x:v>2335</x:v>
       </x:c>
       <x:c r="H130" s="140">
         <x:v>100000</x:v>
@@ -59847,7 +59842,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="G131" s="61" t="s">
-        <x:v>2337</x:v>
+        <x:v>2336</x:v>
       </x:c>
       <x:c r="H131" s="140">
         <x:v>1</x:v>
@@ -59867,7 +59862,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G132" s="61" t="s">
-        <x:v>2338</x:v>
+        <x:v>2337</x:v>
       </x:c>
       <x:c r="H132" s="140"/>
       <x:c r="I132" s="140"/>
@@ -59886,7 +59881,7 @@
         <x:v>900</x:v>
       </x:c>
       <x:c r="D133" s="140" t="s">
-        <x:v>2339</x:v>
+        <x:v>2338</x:v>
       </x:c>
       <x:c r="E133" s="140" t="s">
         <x:v>886</x:v>
@@ -59895,7 +59890,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G133" s="61" t="s">
-        <x:v>2340</x:v>
+        <x:v>2339</x:v>
       </x:c>
       <x:c r="H133" s="140"/>
       <x:c r="I133" s="140" t="s">
@@ -59915,7 +59910,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G134" s="61" t="s">
-        <x:v>2341</x:v>
+        <x:v>2340</x:v>
       </x:c>
       <x:c r="H134" s="140"/>
       <x:c r="I134" s="140"/>
@@ -59933,7 +59928,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G135" s="61" t="s">
-        <x:v>2342</x:v>
+        <x:v>2341</x:v>
       </x:c>
       <x:c r="H135" s="140" t="s">
         <x:v>891</x:v>
@@ -60011,7 +60006,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G139" s="61" t="s">
-        <x:v>2343</x:v>
+        <x:v>2342</x:v>
       </x:c>
       <x:c r="H139" s="140">
         <x:f>1</x:f>
@@ -60031,7 +60026,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G140" s="61" t="s">
-        <x:v>2344</x:v>
+        <x:v>2343</x:v>
       </x:c>
       <x:c r="H140" s="140"/>
       <x:c r="I140" s="140"/>
@@ -60050,7 +60045,7 @@
         <x:v>911</x:v>
       </x:c>
       <x:c r="D141" s="140" t="s">
-        <x:v>2345</x:v>
+        <x:v>2344</x:v>
       </x:c>
       <x:c r="E141" s="140" t="s">
         <x:v>886</x:v>
@@ -60059,7 +60054,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G141" s="61" t="s">
-        <x:v>2346</x:v>
+        <x:v>2345</x:v>
       </x:c>
       <x:c r="H141" s="140"/>
       <x:c r="I141" s="140" t="s">
@@ -60079,7 +60074,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G142" s="61" t="s">
-        <x:v>2347</x:v>
+        <x:v>2346</x:v>
       </x:c>
       <x:c r="H142" s="140"/>
       <x:c r="I142" s="140"/>
@@ -60097,7 +60092,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G143" s="61" t="s">
-        <x:v>2348</x:v>
+        <x:v>2347</x:v>
       </x:c>
       <x:c r="H143" s="140" t="s">
         <x:v>891</x:v>
@@ -60195,7 +60190,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G148" s="61" t="s">
-        <x:v>2349</x:v>
+        <x:v>2348</x:v>
       </x:c>
       <x:c r="H148" s="140"/>
       <x:c r="I148" s="140"/>
@@ -60214,22 +60209,22 @@
         <x:v>921</x:v>
       </x:c>
       <x:c r="D149" s="116" t="s">
+        <x:v>2349</x:v>
+      </x:c>
+      <x:c r="E149" s="116" t="s">
         <x:v>2350</x:v>
-      </x:c>
-      <x:c r="E149" s="116" t="s">
-        <x:v>2351</x:v>
       </x:c>
       <x:c r="F149" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G149" s="327" t="s">
+        <x:v>2351</x:v>
+      </x:c>
+      <x:c r="H149" s="116" t="s">
         <x:v>2352</x:v>
       </x:c>
-      <x:c r="H149" s="116" t="s">
+      <x:c r="I149" s="289" t="s">
         <x:v>2353</x:v>
-      </x:c>
-      <x:c r="I149" s="289" t="s">
-        <x:v>2354</x:v>
       </x:c>
       <x:c r="J149" s="61"/>
       <x:c r="K149" s="140"/>
@@ -60245,11 +60240,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G150" s="327" t="s">
-        <x:v>2355</x:v>
+        <x:v>2354</x:v>
       </x:c>
       <x:c r="H150" s="116"/>
       <x:c r="I150" s="289" t="s">
-        <x:v>2356</x:v>
+        <x:v>2355</x:v>
       </x:c>
       <x:c r="J150" s="61"/>
       <x:c r="K150" s="140"/>
@@ -60265,13 +60260,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G151" s="327" t="s">
+        <x:v>2356</x:v>
+      </x:c>
+      <x:c r="H151" s="116" t="s">
         <x:v>2357</x:v>
       </x:c>
-      <x:c r="H151" s="116" t="s">
+      <x:c r="I151" s="289" t="s">
         <x:v>2358</x:v>
-      </x:c>
-      <x:c r="I151" s="289" t="s">
-        <x:v>2359</x:v>
       </x:c>
       <x:c r="J151" s="61"/>
       <x:c r="K151" s="140"/>
@@ -60287,11 +60282,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G152" s="327" t="s">
-        <x:v>2360</x:v>
+        <x:v>2359</x:v>
       </x:c>
       <x:c r="H152" s="116"/>
       <x:c r="I152" s="289" t="s">
-        <x:v>2361</x:v>
+        <x:v>2360</x:v>
       </x:c>
       <x:c r="J152" s="61"/>
       <x:c r="K152" s="140"/>
@@ -60307,11 +60302,11 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G153" s="327" t="s">
-        <x:v>2362</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H153" s="116"/>
       <x:c r="I153" s="289" t="s">
-        <x:v>2363</x:v>
+        <x:v>2362</x:v>
       </x:c>
       <x:c r="J153" s="61"/>
       <x:c r="K153" s="140"/>
@@ -60648,17 +60643,17 @@
     <x:mergeCell ref="L149:L153"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H49" r:id="rId197"/>
-    <x:hyperlink ref="H50" r:id="rId198"/>
-    <x:hyperlink ref="H55" r:id="rId199"/>
-    <x:hyperlink ref="H56" r:id="rId200"/>
-    <x:hyperlink ref="H59" r:id="rId201"/>
-    <x:hyperlink ref="H64" r:id="rId202"/>
-    <x:hyperlink ref="H65" r:id="rId203"/>
-    <x:hyperlink ref="H67" r:id="rId204"/>
-    <x:hyperlink ref="H68" r:id="rId205"/>
-    <x:hyperlink ref="H52" r:id="rId206"/>
-    <x:hyperlink ref="H61" r:id="rId207"/>
+    <x:hyperlink ref="H49" r:id="rId155"/>
+    <x:hyperlink ref="H50" r:id="rId156"/>
+    <x:hyperlink ref="H55" r:id="rId157"/>
+    <x:hyperlink ref="H56" r:id="rId158"/>
+    <x:hyperlink ref="H59" r:id="rId159"/>
+    <x:hyperlink ref="H64" r:id="rId160"/>
+    <x:hyperlink ref="H65" r:id="rId161"/>
+    <x:hyperlink ref="H67" r:id="rId162"/>
+    <x:hyperlink ref="H68" r:id="rId163"/>
+    <x:hyperlink ref="H52" r:id="rId164"/>
+    <x:hyperlink ref="H61" r:id="rId165"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -60752,7 +60747,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H2" s="340" t="s">
-        <x:v>2364</x:v>
+        <x:v>2363</x:v>
       </x:c>
       <x:c r="I2" s="51" t="s">
         <x:v>1102</x:v>
@@ -60991,7 +60986,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G14" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H14" s="292"/>
       <x:c r="I14" s="51"/>
@@ -61261,7 +61256,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G27" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H27" s="292"/>
       <x:c r="I27" s="51"/>
@@ -61292,7 +61287,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H28" s="340" t="s">
-        <x:v>2366</x:v>
+        <x:v>2365</x:v>
       </x:c>
       <x:c r="I28" s="51" t="s">
         <x:v>1127</x:v>
@@ -61531,7 +61526,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G40" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H40" s="292"/>
       <x:c r="I40" s="51"/>
@@ -61562,7 +61557,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H41" s="340" t="s">
-        <x:v>2367</x:v>
+        <x:v>2366</x:v>
       </x:c>
       <x:c r="I41" s="51" t="s">
         <x:v>1130</x:v>
@@ -61801,7 +61796,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G53" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H53" s="292"/>
       <x:c r="I53" s="51"/>
@@ -61832,7 +61827,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H54" s="340" t="s">
-        <x:v>2368</x:v>
+        <x:v>2367</x:v>
       </x:c>
       <x:c r="I54" s="51" t="s">
         <x:v>1134</x:v>
@@ -62071,7 +62066,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G66" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H66" s="292"/>
       <x:c r="I66" s="51"/>
@@ -62102,7 +62097,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H67" s="340" t="s">
-        <x:v>2369</x:v>
+        <x:v>2368</x:v>
       </x:c>
       <x:c r="I67" s="51" t="s">
         <x:v>1138</x:v>
@@ -62341,7 +62336,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G79" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H79" s="292"/>
       <x:c r="I79" s="51"/>
@@ -62372,7 +62367,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H80" s="340" t="s">
-        <x:v>2370</x:v>
+        <x:v>2369</x:v>
       </x:c>
       <x:c r="I80" s="51" t="s">
         <x:v>1141</x:v>
@@ -62611,7 +62606,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G92" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H92" s="292"/>
       <x:c r="I92" s="51"/>
@@ -62642,7 +62637,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H93" s="340" t="s">
-        <x:v>2371</x:v>
+        <x:v>2370</x:v>
       </x:c>
       <x:c r="I93" s="51" t="s">
         <x:v>1145</x:v>
@@ -62881,7 +62876,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G105" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H105" s="292"/>
       <x:c r="I105" s="51"/>
@@ -62912,7 +62907,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H106" s="340" t="s">
-        <x:v>2371</x:v>
+        <x:v>2370</x:v>
       </x:c>
       <x:c r="I106" s="51" t="s">
         <x:v>1149</x:v>
@@ -63151,7 +63146,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G118" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H118" s="292"/>
       <x:c r="I118" s="51"/>
@@ -63182,7 +63177,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H119" s="340" t="s">
-        <x:v>2372</x:v>
+        <x:v>2371</x:v>
       </x:c>
       <x:c r="I119" s="51" t="s">
         <x:v>1149</x:v>
@@ -63421,7 +63416,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G131" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H131" s="292"/>
       <x:c r="I131" s="51"/>
@@ -63452,7 +63447,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H132" s="340" t="s">
-        <x:v>2373</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="I132" s="51" t="s">
         <x:v>1160</x:v>
@@ -63691,7 +63686,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G144" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H144" s="292"/>
       <x:c r="I144" s="51"/>
@@ -63722,7 +63717,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H145" s="340" t="s">
-        <x:v>2374</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="I145" s="51" t="s">
         <x:v>1160</x:v>
@@ -63961,7 +63956,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G157" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H157" s="292"/>
       <x:c r="I157" s="51"/>
@@ -63992,7 +63987,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H158" s="340" t="s">
-        <x:v>2375</x:v>
+        <x:v>2374</x:v>
       </x:c>
       <x:c r="I158" s="51" t="s">
         <x:v>1160</x:v>
@@ -64231,7 +64226,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G170" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H170" s="292"/>
       <x:c r="I170" s="51"/>
@@ -64262,7 +64257,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H171" s="340" t="s">
-        <x:v>2376</x:v>
+        <x:v>2375</x:v>
       </x:c>
       <x:c r="I171" s="51" t="s">
         <x:v>1160</x:v>
@@ -64501,7 +64496,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G183" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H183" s="292"/>
       <x:c r="I183" s="51"/>
@@ -64771,7 +64766,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G196" s="292" t="s">
-        <x:v>2365</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H196" s="340"/>
       <x:c r="I196" s="51"/>
@@ -64802,7 +64797,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H197" s="340" t="s">
-        <x:v>2377</x:v>
+        <x:v>2376</x:v>
       </x:c>
       <x:c r="I197" s="134" t="s">
         <x:v>1178</x:v>
@@ -65072,7 +65067,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H210" s="340" t="s">
-        <x:v>2378</x:v>
+        <x:v>2377</x:v>
       </x:c>
       <x:c r="I210" s="134" t="s">
         <x:v>1187</x:v>
@@ -65330,7 +65325,7 @@
         <x:v>1189</x:v>
       </x:c>
       <x:c r="D223" s="134" t="s">
-        <x:v>2379</x:v>
+        <x:v>2378</x:v>
       </x:c>
       <x:c r="E223" s="35" t="s">
         <x:v>1176</x:v>
@@ -65342,7 +65337,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H223" s="340" t="s">
-        <x:v>2380</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="I223" s="10" t="s">
         <x:v>1192</x:v>
@@ -65612,7 +65607,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H236" s="340" t="s">
-        <x:v>2381</x:v>
+        <x:v>2380</x:v>
       </x:c>
       <x:c r="I236" s="10" t="s">
         <x:v>1197</x:v>
@@ -65882,7 +65877,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H249" s="340" t="s">
-        <x:v>2382</x:v>
+        <x:v>2381</x:v>
       </x:c>
       <x:c r="I249" s="10" t="s">
         <x:v>1203</x:v>
@@ -66064,7 +66059,7 @@
         <x:v>1115</x:v>
       </x:c>
       <x:c r="H258" s="292" t="s">
-        <x:v>2383</x:v>
+        <x:v>2382</x:v>
       </x:c>
       <x:c r="I258" s="9"/>
       <x:c r="J258" s="9"/>
@@ -66410,7 +66405,7 @@
         <x:v>1212</x:v>
       </x:c>
       <x:c r="D275" s="35" t="s">
-        <x:v>2384</x:v>
+        <x:v>2383</x:v>
       </x:c>
       <x:c r="E275" s="35" t="s">
         <x:v>1214</x:v>
@@ -66419,10 +66414,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G275" s="297" t="s">
+        <x:v>2384</x:v>
+      </x:c>
+      <x:c r="I275" s="10" t="s">
         <x:v>2385</x:v>
-      </x:c>
-      <x:c r="I275" s="10" t="s">
-        <x:v>2386</x:v>
       </x:c>
       <x:c r="J275" s="10"/>
       <x:c r="K275" s="35"/>
@@ -66438,7 +66433,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G276" s="297" t="s">
-        <x:v>2387</x:v>
+        <x:v>2386</x:v>
       </x:c>
       <x:c r="I276" s="9"/>
       <x:c r="J276" s="9"/>
@@ -66455,10 +66450,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G277" s="297" t="s">
+        <x:v>2387</x:v>
+      </x:c>
+      <x:c r="H277" s="297" t="s">
         <x:v>2388</x:v>
-      </x:c>
-      <x:c r="H277" s="297" t="s">
-        <x:v>2389</x:v>
       </x:c>
       <x:c r="I277" s="9"/>
       <x:c r="J277" s="9"/>
@@ -66497,13 +66492,13 @@
         <x:v>1220</x:v>
       </x:c>
       <x:c r="E279" s="35" t="s">
-        <x:v>2390</x:v>
+        <x:v>2389</x:v>
       </x:c>
       <x:c r="F279" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G279" s="297" t="s">
-        <x:v>2385</x:v>
+        <x:v>2384</x:v>
       </x:c>
       <x:c r="I279" s="10" t="s">
         <x:v>1223</x:v>
@@ -66522,7 +66517,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G280" s="297" t="s">
-        <x:v>2391</x:v>
+        <x:v>2390</x:v>
       </x:c>
       <x:c r="H280" s="297" t="s">
         <x:v>1117</x:v>
@@ -66564,17 +66559,17 @@
         <x:v>1226</x:v>
       </x:c>
       <x:c r="E282" s="35" t="s">
-        <x:v>2392</x:v>
+        <x:v>2391</x:v>
       </x:c>
       <x:c r="F282" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G282" s="297" t="s">
-        <x:v>2385</x:v>
+        <x:v>2384</x:v>
       </x:c>
       <x:c r="H282" s="297"/>
       <x:c r="I282" s="10" t="s">
-        <x:v>2393</x:v>
+        <x:v>2392</x:v>
       </x:c>
       <x:c r="J282" s="10"/>
       <x:c r="K282" s="35"/>
@@ -66590,7 +66585,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G283" s="297" t="s">
-        <x:v>2387</x:v>
+        <x:v>2386</x:v>
       </x:c>
       <x:c r="H283" s="297"/>
       <x:c r="I283" s="9"/>
@@ -66608,10 +66603,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G284" s="297" t="s">
+        <x:v>2393</x:v>
+      </x:c>
+      <x:c r="H284" s="323" t="s">
         <x:v>2394</x:v>
-      </x:c>
-      <x:c r="H284" s="323" t="s">
-        <x:v>2395</x:v>
       </x:c>
       <x:c r="I284" s="9"/>
       <x:c r="J284" s="9"/>
@@ -66650,17 +66645,17 @@
         <x:v>1233</x:v>
       </x:c>
       <x:c r="E286" s="35" t="s">
-        <x:v>2392</x:v>
+        <x:v>2391</x:v>
       </x:c>
       <x:c r="F286" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G286" s="297" t="s">
-        <x:v>2385</x:v>
+        <x:v>2384</x:v>
       </x:c>
       <x:c r="H286" s="297"/>
       <x:c r="I286" s="10" t="s">
-        <x:v>2393</x:v>
+        <x:v>2392</x:v>
       </x:c>
       <x:c r="J286" s="10"/>
       <x:c r="K286" s="35"/>
@@ -66676,7 +66671,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G287" s="297" t="s">
-        <x:v>2387</x:v>
+        <x:v>2386</x:v>
       </x:c>
       <x:c r="H287" s="297"/>
       <x:c r="I287" s="9"/>
@@ -66694,10 +66689,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G288" s="297" t="s">
+        <x:v>2395</x:v>
+      </x:c>
+      <x:c r="H288" s="297" t="s">
         <x:v>2396</x:v>
-      </x:c>
-      <x:c r="H288" s="297" t="s">
-        <x:v>2397</x:v>
       </x:c>
       <x:c r="I288" s="9"/>
       <x:c r="J288" s="9"/>
@@ -66745,7 +66740,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H290" s="340" t="s">
-        <x:v>2398</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I290" s="51" t="s">
         <x:v>1102</x:v>
@@ -66824,7 +66819,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G294" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H294" s="312" t="s">
         <x:v>1117</x:v>
@@ -66844,7 +66839,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G295" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H295" s="312">
         <x:v>45758</x:v>
@@ -66964,7 +66959,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G301" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="H301" s="297"/>
       <x:c r="I301" s="51"/>
@@ -67074,7 +67069,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G306" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H306" s="312" t="s">
         <x:v>1117</x:v>
@@ -67094,7 +67089,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G307" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H307" s="312">
         <x:v>45758</x:v>
@@ -67214,7 +67209,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G313" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I313" s="51"/>
       <x:c r="J313" s="48"/>
@@ -67244,7 +67239,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H314" s="340" t="s">
-        <x:v>2402</x:v>
+        <x:v>2401</x:v>
       </x:c>
       <x:c r="I314" s="51" t="s">
         <x:v>1127</x:v>
@@ -67321,7 +67316,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G318" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H318" s="312" t="s">
         <x:v>1117</x:v>
@@ -67341,7 +67336,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G319" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H319" s="312">
         <x:v>45758</x:v>
@@ -67461,7 +67456,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G325" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I325" s="51"/>
       <x:c r="J325" s="48"/>
@@ -67491,7 +67486,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H326" s="340" t="s">
-        <x:v>2403</x:v>
+        <x:v>2402</x:v>
       </x:c>
       <x:c r="I326" s="51" t="s">
         <x:v>1130</x:v>
@@ -67568,7 +67563,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G330" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H330" s="312" t="s">
         <x:v>1117</x:v>
@@ -67588,7 +67583,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G331" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H331" s="312">
         <x:v>45758</x:v>
@@ -67708,7 +67703,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G337" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I337" s="51"/>
       <x:c r="J337" s="48"/>
@@ -67738,7 +67733,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H338" s="340" t="s">
-        <x:v>2404</x:v>
+        <x:v>2403</x:v>
       </x:c>
       <x:c r="I338" s="51" t="s">
         <x:v>1134</x:v>
@@ -67817,7 +67812,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G342" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H342" s="312"/>
       <x:c r="I342" s="51"/>
@@ -67835,7 +67830,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G343" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H343" s="312">
         <x:v>45758</x:v>
@@ -67955,7 +67950,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G349" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I349" s="51"/>
       <x:c r="J349" s="48"/>
@@ -67985,7 +67980,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H350" s="340" t="s">
-        <x:v>2404</x:v>
+        <x:v>2403</x:v>
       </x:c>
       <x:c r="I350" s="51" t="s">
         <x:v>1138</x:v>
@@ -68064,7 +68059,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G354" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H354" s="312" t="s">
         <x:v>1117</x:v>
@@ -68084,7 +68079,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G355" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H355" s="312"/>
       <x:c r="I355" s="51"/>
@@ -68202,7 +68197,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G361" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I361" s="51"/>
       <x:c r="J361" s="48"/>
@@ -68220,7 +68215,7 @@
         <x:v>1254</x:v>
       </x:c>
       <x:c r="D362" s="51" t="s">
-        <x:v>2405</x:v>
+        <x:v>2404</x:v>
       </x:c>
       <x:c r="E362" s="51" t="s">
         <x:v>1099</x:v>
@@ -68232,10 +68227,10 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H362" s="340" t="s">
+        <x:v>2405</x:v>
+      </x:c>
+      <x:c r="I362" s="51" t="s">
         <x:v>2406</x:v>
-      </x:c>
-      <x:c r="I362" s="51" t="s">
-        <x:v>2407</x:v>
       </x:c>
       <x:c r="J362" s="50"/>
       <x:c r="K362" s="51"/>
@@ -68309,7 +68304,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G366" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H366" s="312" t="s">
         <x:v>1117</x:v>
@@ -68329,7 +68324,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G367" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H367" s="312">
         <x:v>49410</x:v>
@@ -68447,7 +68442,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G373" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="H373" s="292"/>
       <x:c r="I373" s="51"/>
@@ -68478,7 +68473,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H374" s="340" t="s">
-        <x:v>2408</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="I374" s="51" t="s">
         <x:v>1145</x:v>
@@ -68557,7 +68552,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G378" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H378" s="312" t="s">
         <x:v>1117</x:v>
@@ -68577,7 +68572,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G379" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H379" s="312">
         <x:v>45758</x:v>
@@ -68695,7 +68690,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G385" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I385" s="51"/>
       <x:c r="J385" s="48"/>
@@ -68725,7 +68720,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H386" s="340" t="s">
-        <x:v>2409</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I386" s="51" t="s">
         <x:v>1149</x:v>
@@ -68804,7 +68799,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G390" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H390" s="312" t="s">
         <x:v>1117</x:v>
@@ -68824,7 +68819,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G391" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H391" s="312">
         <x:v>45758</x:v>
@@ -68942,7 +68937,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G397" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I397" s="51"/>
       <x:c r="J397" s="48"/>
@@ -68972,7 +68967,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H398" s="340" t="s">
-        <x:v>2410</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I398" s="51" t="s">
         <x:v>1149</x:v>
@@ -69049,7 +69044,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G402" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H402" s="312" t="s">
         <x:v>1117</x:v>
@@ -69069,7 +69064,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G403" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H403" s="312">
         <x:v>45758</x:v>
@@ -69189,7 +69184,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G409" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I409" s="51"/>
       <x:c r="J409" s="48"/>
@@ -69219,7 +69214,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H410" s="340" t="s">
-        <x:v>2411</x:v>
+        <x:v>2410</x:v>
       </x:c>
       <x:c r="I410" s="51" t="s">
         <x:v>1160</x:v>
@@ -69298,7 +69293,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G414" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H414" s="312" t="s">
         <x:v>1117</x:v>
@@ -69318,7 +69313,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G415" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H415" s="312">
         <x:v>45758</x:v>
@@ -69436,7 +69431,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G421" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I421" s="51"/>
       <x:c r="J421" s="48"/>
@@ -69454,7 +69449,7 @@
         <x:v>1260</x:v>
       </x:c>
       <x:c r="D422" s="51" t="s">
-        <x:v>2412</x:v>
+        <x:v>2411</x:v>
       </x:c>
       <x:c r="E422" s="51" t="s">
         <x:v>1099</x:v>
@@ -69466,10 +69461,10 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H422" s="340" t="s">
+        <x:v>2412</x:v>
+      </x:c>
+      <x:c r="I422" s="51" t="s">
         <x:v>2413</x:v>
-      </x:c>
-      <x:c r="I422" s="51" t="s">
-        <x:v>2414</x:v>
       </x:c>
       <x:c r="J422" s="50"/>
       <x:c r="K422" s="51"/>
@@ -69545,7 +69540,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G426" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H426" s="312" t="s">
         <x:v>1117</x:v>
@@ -69565,7 +69560,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G427" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H427" s="312">
         <x:v>45758</x:v>
@@ -69685,7 +69680,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G433" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I433" s="51"/>
       <x:c r="J433" s="48"/>
@@ -69715,7 +69710,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H434" s="340" t="s">
-        <x:v>2415</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="I434" s="51" t="s">
         <x:v>1160</x:v>
@@ -69794,7 +69789,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G438" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H438" s="312" t="s">
         <x:v>1117</x:v>
@@ -69814,7 +69809,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G439" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H439" s="312">
         <x:v>45758</x:v>
@@ -69932,7 +69927,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G445" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I445" s="51"/>
       <x:c r="J445" s="48"/>
@@ -69962,7 +69957,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H446" s="340" t="s">
-        <x:v>2416</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I446" s="51" t="s">
         <x:v>1160</x:v>
@@ -70041,7 +70036,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G450" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H450" s="312" t="s">
         <x:v>1117</x:v>
@@ -70061,7 +70056,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G451" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H451" s="312">
         <x:v>45758</x:v>
@@ -70179,7 +70174,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G457" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I457" s="51"/>
       <x:c r="J457" s="48"/>
@@ -70288,7 +70283,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G462" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H462" s="340" t="s">
         <x:v>437</x:v>
@@ -70308,7 +70303,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G463" s="292" t="s">
-        <x:v>2400</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H463" s="340" t="s">
         <x:v>437</x:v>
@@ -70428,7 +70423,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G469" s="288" t="s">
-        <x:v>2401</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="H469" s="340" t="s">
         <x:v>437</x:v>
@@ -70762,7 +70757,7 @@
     <x:mergeCell ref="K458:K469"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H284" r:id="rId208"/>
+    <x:hyperlink ref="H284" r:id="rId166"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -70786,13 +70781,13 @@
   <x:sheetData>
     <x:row r="2" spans="1:7">
       <x:c r="A2" s="196" t="s">
-        <x:v>2417</x:v>
+        <x:v>2416</x:v>
       </x:c>
       <x:c r="D2" s="196" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="G2" s="196" t="s">
-        <x:v>2418</x:v>
+        <x:v>2417</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
@@ -70800,7 +70795,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>2419</x:v>
+        <x:v>2418</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
         <x:v>244</x:v>
@@ -70811,7 +70806,7 @@
         <x:v>245</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>2420</x:v>
+        <x:v>2419</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
         <x:v>234</x:v>
@@ -70819,10 +70814,10 @@
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="A5" s="0" t="s">
+        <x:v>2420</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
         <x:v>2421</x:v>
-      </x:c>
-      <x:c r="D5" s="0" t="s">
-        <x:v>2422</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
         <x:v>239</x:v>

</xml_diff>

<commit_message>
chore: update test results and clean up workspace after merge
</commit_message>
<xml_diff>
--- a/sqa-testing-report/Data/DataTest.xlsx
+++ b/sqa-testing-report/Data/DataTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\sqa-testing-report\sqa-testing-report\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C69B56A-177D-45FB-B754-1C00B7A1660F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62CFFD6C-B776-4998-B290-C03700EB1126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
     <x:workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="664" firstSheet="0" activeTab="3" xr2:uid="{DC4DB269-603C-4B5B-A498-B166C8A18B92}"/>
   </x:bookViews>
@@ -7692,85 +7692,76 @@
     <x:t>Screenshots</x:t>
   </x:si>
   <x:si>
-    <x:t>Đã kiểm tra: OK</x:t>
+    <x:t>Kiểm tra đăng ký với mật khẩu chứa ký tự đặc biệt gây lỗi (SQL Injection).</x:t>
+  </x:si>
+  <x:si>
+    <x:t>' OR 1=1 --</x:t>
+  </x:si>
+  <x:si>
+    <x:t>chuỗi &gt; 255 kí tự</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0376808424B</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hiển thị lỗi: "Email hoặc mật khẩu không chính xác."</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hiển thị thông báo "Tài khoản của bạn đã bị khóa tạm thời trong 15 phút do nhập sai quá nhiều lần. Vui lòng thử lại sau."</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Đăng nhập thành công.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> OR 1=1 --</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hiển thị lỗi "Email hoặc mật khẩu không chính xác."</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Đăng nhập thành công</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nhấn vào "Thay đổi" tại mục Mật khẩu.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hiển thị lỗi: "Mật khẩu cũ không chính xác"</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nhập "Mật khẩu cũ"</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Khoa@999</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nhập "Mật khẩu mới"</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Moi@45678</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nhập lại mật khẩu mới trùng khớp vào ô "Nhập lại mật khẩu mới"</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nhấn nút "XÁC NHẬN".</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Chuyển đến trang chi tiết phim tương ứng</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hiển thị đầy đủ: tên phim, thể loại, quốc gia, đạo diễn, diễn viên, thời lượng, ngày công chiếu</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Có nội dung phim và danh sách lịch chiếu rõ ràng</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hiển thị danh sách khu vực.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hệ thống đã hiển thị đầy đủ danh sách khu vực.</x:t>
   </x:si>
   <x:si>
     <x:t>Pass</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Data/Screenshots/screenshot_20260327_154116_d62378ca.png</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hiển thị đúng lỗi: Hiển thị lỗi “Vui lòng nhập họ và tên.”</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Kiểm tra đăng ký với mật khẩu chứa ký tự đặc biệt gây lỗi (SQL Injection).</x:t>
-  </x:si>
-  <x:si>
-    <x:t>' OR 1=1 --</x:t>
-  </x:si>
-  <x:si>
-    <x:t>chuỗi &gt; 255 kí tự</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0376808424B</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hiển thị lỗi: "Email hoặc mật khẩu không chính xác."</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hiển thị thông báo "Tài khoản của bạn đã bị khóa tạm thời trong 15 phút do nhập sai quá nhiều lần. Vui lòng thử lại sau."</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Đăng nhập thành công.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> OR 1=1 --</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hiển thị lỗi "Email hoặc mật khẩu không chính xác."</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Đăng nhập thành công</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Nhấn vào "Thay đổi" tại mục Mật khẩu.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hiển thị lỗi: "Mật khẩu cũ không chính xác"</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Nhập "Mật khẩu cũ"</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Khoa@999</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Nhập "Mật khẩu mới"</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Moi@45678</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Nhập lại mật khẩu mới trùng khớp vào ô "Nhập lại mật khẩu mới"</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Nhấn nút "XÁC NHẬN".</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Chuyển đến trang chi tiết phim tương ứng</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hiển thị đầy đủ: tên phim, thể loại, quốc gia, đạo diễn, diễn viên, thời lượng, ngày công chiếu</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Có nội dung phim và danh sách lịch chiếu rõ ràng</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hiển thị danh sách khu vực.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hệ thống đã hiển thị đầy đủ danh sách khu vực.</x:t>
   </x:si>
   <x:si>
     <x:t>Click vào khu vực [Khu vực]</x:t>
@@ -48180,41 +48171,41 @@
   </x:mergeCells>
   <x:phoneticPr fontId="16" type="noConversion"/>
   <x:hyperlinks>
-    <x:hyperlink ref="H382" r:id="rId102"/>
-    <x:hyperlink ref="H388" r:id="rId103"/>
-    <x:hyperlink ref="H396" r:id="rId104"/>
-    <x:hyperlink ref="H397" r:id="rId105"/>
-    <x:hyperlink ref="H415" r:id="rId106"/>
-    <x:hyperlink ref="H418" r:id="rId107"/>
-    <x:hyperlink ref="H420" r:id="rId108"/>
-    <x:hyperlink ref="H421" r:id="rId109"/>
-    <x:hyperlink ref="H423" r:id="rId110"/>
-    <x:hyperlink ref="H424" r:id="rId111"/>
-    <x:hyperlink ref="H53" r:id="rId112"/>
-    <x:hyperlink ref="H61" r:id="rId113"/>
-    <x:hyperlink ref="H65" r:id="rId114"/>
-    <x:hyperlink ref="H69" r:id="rId115"/>
-    <x:hyperlink ref="H73" r:id="rId116"/>
-    <x:hyperlink ref="H77" r:id="rId117"/>
-    <x:hyperlink ref="H81" r:id="rId118"/>
-    <x:hyperlink ref="H112" r:id="rId119"/>
-    <x:hyperlink ref="H115" r:id="rId120"/>
-    <x:hyperlink ref="H118" r:id="rId121"/>
-    <x:hyperlink ref="H399" r:id="rId122"/>
-    <x:hyperlink ref="H402" r:id="rId123"/>
-    <x:hyperlink ref="H405" r:id="rId124"/>
-    <x:hyperlink ref="H408" r:id="rId125"/>
-    <x:hyperlink ref="H411" r:id="rId126"/>
-    <x:hyperlink ref="H400" r:id="rId127"/>
-    <x:hyperlink ref="H403" r:id="rId128"/>
-    <x:hyperlink ref="H406" r:id="rId129"/>
-    <x:hyperlink ref="H409" r:id="rId130"/>
-    <x:hyperlink ref="H412" r:id="rId131"/>
-    <x:hyperlink ref="H1075" r:id="rId132"/>
-    <x:hyperlink ref="H1081" r:id="rId133"/>
-    <x:hyperlink ref="H1087" r:id="rId134"/>
-    <x:hyperlink ref="H1093" r:id="rId135"/>
-    <x:hyperlink ref="H1099" r:id="rId136"/>
+    <x:hyperlink ref="H382" r:id="rId79"/>
+    <x:hyperlink ref="H388" r:id="rId80"/>
+    <x:hyperlink ref="H396" r:id="rId81"/>
+    <x:hyperlink ref="H397" r:id="rId82"/>
+    <x:hyperlink ref="H415" r:id="rId83"/>
+    <x:hyperlink ref="H418" r:id="rId84"/>
+    <x:hyperlink ref="H420" r:id="rId85"/>
+    <x:hyperlink ref="H421" r:id="rId86"/>
+    <x:hyperlink ref="H423" r:id="rId87"/>
+    <x:hyperlink ref="H424" r:id="rId88"/>
+    <x:hyperlink ref="H53" r:id="rId89"/>
+    <x:hyperlink ref="H61" r:id="rId90"/>
+    <x:hyperlink ref="H65" r:id="rId91"/>
+    <x:hyperlink ref="H69" r:id="rId92"/>
+    <x:hyperlink ref="H73" r:id="rId93"/>
+    <x:hyperlink ref="H77" r:id="rId94"/>
+    <x:hyperlink ref="H81" r:id="rId95"/>
+    <x:hyperlink ref="H112" r:id="rId96"/>
+    <x:hyperlink ref="H115" r:id="rId97"/>
+    <x:hyperlink ref="H118" r:id="rId98"/>
+    <x:hyperlink ref="H399" r:id="rId99"/>
+    <x:hyperlink ref="H402" r:id="rId100"/>
+    <x:hyperlink ref="H405" r:id="rId101"/>
+    <x:hyperlink ref="H408" r:id="rId167"/>
+    <x:hyperlink ref="H411" r:id="rId168"/>
+    <x:hyperlink ref="H400" r:id="rId169"/>
+    <x:hyperlink ref="H403" r:id="rId170"/>
+    <x:hyperlink ref="H406" r:id="rId171"/>
+    <x:hyperlink ref="H409" r:id="rId172"/>
+    <x:hyperlink ref="H412" r:id="rId173"/>
+    <x:hyperlink ref="H1075" r:id="rId174"/>
+    <x:hyperlink ref="H1081" r:id="rId175"/>
+    <x:hyperlink ref="H1087" r:id="rId176"/>
+    <x:hyperlink ref="H1093" r:id="rId177"/>
+    <x:hyperlink ref="H1099" r:id="rId178"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -48311,15 +48302,9 @@
       <x:c r="I2" s="138" t="s">
         <x:v>417</x:v>
       </x:c>
-      <x:c r="J2" s="137" t="s">
-        <x:v>2006</x:v>
-      </x:c>
-      <x:c r="K2" s="137" t="s">
-        <x:v>2007</x:v>
-      </x:c>
-      <x:c r="L2" s="137" t="s">
-        <x:v>2008</x:v>
-      </x:c>
+      <x:c r="J2" s="137"/>
+      <x:c r="K2" s="137"/>
+      <x:c r="L2" s="137"/>
     </x:row>
     <x:row r="3" spans="1:12">
       <x:c r="A3" s="140"/>
@@ -48505,12 +48490,8 @@
       <x:c r="I11" s="138" t="s">
         <x:v>438</x:v>
       </x:c>
-      <x:c r="J11" s="137" t="s">
-        <x:v>2009</x:v>
-      </x:c>
-      <x:c r="K11" s="137" t="s">
-        <x:v>2007</x:v>
-      </x:c>
+      <x:c r="J11" s="137"/>
+      <x:c r="K11" s="137"/>
       <x:c r="L11" s="137"/>
     </x:row>
     <x:row r="12" spans="1:12">
@@ -49996,7 +49977,7 @@
         <x:v>468</x:v>
       </x:c>
       <x:c r="D83" s="140" t="s">
-        <x:v>2010</x:v>
+        <x:v>2006</x:v>
       </x:c>
       <x:c r="E83" s="140" t="s">
         <x:v>434</x:v>
@@ -50128,7 +50109,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H89" s="25" t="s">
-        <x:v>2011</x:v>
+        <x:v>2007</x:v>
       </x:c>
       <x:c r="I89" s="138"/>
       <x:c r="J89" s="136"/>
@@ -50148,7 +50129,7 @@
         <x:v>445</x:v>
       </x:c>
       <x:c r="H90" s="25" t="s">
-        <x:v>2011</x:v>
+        <x:v>2007</x:v>
       </x:c>
       <x:c r="I90" s="138"/>
       <x:c r="J90" s="136"/>
@@ -50216,7 +50197,7 @@
         <x:v>419</x:v>
       </x:c>
       <x:c r="H93" s="140" t="s">
-        <x:v>2012</x:v>
+        <x:v>2008</x:v>
       </x:c>
       <x:c r="I93" s="138"/>
       <x:c r="J93" s="136"/>
@@ -50444,7 +50425,7 @@
         <x:v>439</x:v>
       </x:c>
       <x:c r="H104" s="139" t="s">
-        <x:v>2013</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I104" s="138"/>
       <x:c r="J104" s="134"/>
@@ -51009,7 +50990,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I129" s="138" t="s">
-        <x:v>2014</x:v>
+        <x:v>2010</x:v>
       </x:c>
       <x:c r="J129" s="134"/>
       <x:c r="K129" s="134"/>
@@ -51079,7 +51060,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I132" s="123" t="s">
-        <x:v>2015</x:v>
+        <x:v>2011</x:v>
       </x:c>
       <x:c r="J132" s="134"/>
       <x:c r="K132" s="134"/>
@@ -51149,7 +51130,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I135" s="138" t="s">
-        <x:v>2016</x:v>
+        <x:v>2012</x:v>
       </x:c>
       <x:c r="J135" s="134"/>
       <x:c r="K135" s="134"/>
@@ -51216,10 +51197,10 @@
         <x:v>480</x:v>
       </x:c>
       <x:c r="H138" s="316" t="s">
-        <x:v>2017</x:v>
+        <x:v>2013</x:v>
       </x:c>
       <x:c r="I138" s="120" t="s">
-        <x:v>2018</x:v>
+        <x:v>2014</x:v>
       </x:c>
       <x:c r="J138" s="134"/>
       <x:c r="K138" s="134"/>
@@ -51289,7 +51270,7 @@
         <x:v>422</x:v>
       </x:c>
       <x:c r="I141" s="138" t="s">
-        <x:v>2019</x:v>
+        <x:v>2015</x:v>
       </x:c>
       <x:c r="J141" s="118"/>
       <x:c r="K141" s="134"/>
@@ -51353,11 +51334,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G144" s="138" t="s">
-        <x:v>2020</x:v>
+        <x:v>2016</x:v>
       </x:c>
       <x:c r="H144" s="140"/>
       <x:c r="I144" s="138" t="s">
-        <x:v>2021</x:v>
+        <x:v>2017</x:v>
       </x:c>
       <x:c r="J144" s="134"/>
       <x:c r="K144" s="134"/>
@@ -51373,10 +51354,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G145" s="319" t="s">
-        <x:v>2022</x:v>
+        <x:v>2018</x:v>
       </x:c>
       <x:c r="H145" s="134" t="s">
-        <x:v>2023</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="I145" s="138"/>
       <x:c r="J145" s="134"/>
@@ -51393,10 +51374,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G146" s="138" t="s">
-        <x:v>2024</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="H146" s="317" t="s">
-        <x:v>2025</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="I146" s="138"/>
       <x:c r="J146" s="134"/>
@@ -51413,10 +51394,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G147" s="138" t="s">
-        <x:v>2026</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="H147" s="134" t="s">
-        <x:v>2025</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="I147" s="138"/>
       <x:c r="J147" s="134"/>
@@ -51433,7 +51414,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G148" s="138" t="s">
-        <x:v>2027</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="H148" s="134"/>
       <x:c r="I148" s="138"/>
@@ -51467,7 +51448,7 @@
         <x:v>590</x:v>
       </x:c>
       <x:c r="I149" s="138" t="s">
-        <x:v>2028</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="J149" s="298"/>
       <x:c r="K149" s="134"/>
@@ -51487,7 +51468,7 @@
       </x:c>
       <x:c r="H150" s="140"/>
       <x:c r="I150" s="138" t="s">
-        <x:v>2029</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="J150" s="298"/>
       <x:c r="K150" s="134"/>
@@ -51507,7 +51488,7 @@
       </x:c>
       <x:c r="H151" s="140"/>
       <x:c r="I151" s="138" t="s">
-        <x:v>2030</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="J151" s="298"/>
       <x:c r="K151" s="134"/>
@@ -51583,13 +51564,13 @@
       </x:c>
       <x:c r="H154" s="140"/>
       <x:c r="I154" s="138" t="s">
-        <x:v>2031</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="J154" s="134" t="s">
-        <x:v>2032</x:v>
+        <x:v>2028</x:v>
       </x:c>
       <x:c r="K154" s="134" t="s">
-        <x:v>2007</x:v>
+        <x:v>2029</x:v>
       </x:c>
       <x:c r="L154" s="134" t="s"/>
     </x:row>
@@ -51603,16 +51584,16 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G155" s="138" t="s">
+        <x:v>2030</x:v>
+      </x:c>
+      <x:c r="H155" s="140" t="s">
+        <x:v>2031</x:v>
+      </x:c>
+      <x:c r="I155" s="138" t="s">
+        <x:v>2032</x:v>
+      </x:c>
+      <x:c r="J155" s="134" t="s">
         <x:v>2033</x:v>
-      </x:c>
-      <x:c r="H155" s="140" t="s">
-        <x:v>2034</x:v>
-      </x:c>
-      <x:c r="I155" s="138" t="s">
-        <x:v>2035</x:v>
-      </x:c>
-      <x:c r="J155" s="134" t="s">
-        <x:v>2036</x:v>
       </x:c>
       <x:c r="K155" s="134"/>
       <x:c r="L155" s="134"/>
@@ -51628,7 +51609,7 @@
         <x:v>626</x:v>
       </x:c>
       <x:c r="D156" s="140" t="s">
-        <x:v>2037</x:v>
+        <x:v>2034</x:v>
       </x:c>
       <x:c r="E156" s="140" t="s">
         <x:v>616</x:v>
@@ -51637,13 +51618,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G156" s="138" t="s">
-        <x:v>2038</x:v>
+        <x:v>2035</x:v>
       </x:c>
       <x:c r="H156" s="140" t="s">
-        <x:v>2039</x:v>
+        <x:v>2036</x:v>
       </x:c>
       <x:c r="I156" s="138" t="s">
-        <x:v>2040</x:v>
+        <x:v>2037</x:v>
       </x:c>
       <x:c r="J156" s="134"/>
       <x:c r="K156" s="134"/>
@@ -51669,19 +51650,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G157" s="138" t="s">
+        <x:v>2038</x:v>
+      </x:c>
+      <x:c r="H157" s="140" t="s">
+        <x:v>2039</x:v>
+      </x:c>
+      <x:c r="I157" s="138" t="s">
+        <x:v>2040</x:v>
+      </x:c>
+      <x:c r="J157" s="134" t="s">
         <x:v>2041</x:v>
       </x:c>
-      <x:c r="H157" s="140" t="s">
-        <x:v>2042</x:v>
-      </x:c>
-      <x:c r="I157" s="138" t="s">
-        <x:v>2043</x:v>
-      </x:c>
-      <x:c r="J157" s="134" t="s">
-        <x:v>2044</x:v>
-      </x:c>
       <x:c r="K157" s="134" t="s">
-        <x:v>2007</x:v>
+        <x:v>2029</x:v>
       </x:c>
       <x:c r="L157" s="134" t="s"/>
     </x:row>
@@ -51695,14 +51676,14 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G158" s="138" t="s">
-        <x:v>2045</x:v>
+        <x:v>2042</x:v>
       </x:c>
       <x:c r="H158" s="140"/>
       <x:c r="I158" s="138" t="s">
-        <x:v>2046</x:v>
+        <x:v>2043</x:v>
       </x:c>
       <x:c r="J158" s="134" t="s">
-        <x:v>2047</x:v>
+        <x:v>2044</x:v>
       </x:c>
       <x:c r="K158" s="134"/>
       <x:c r="L158" s="134"/>
@@ -51717,14 +51698,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G159" s="138" t="s">
-        <x:v>2048</x:v>
+        <x:v>2045</x:v>
       </x:c>
       <x:c r="H159" s="140"/>
       <x:c r="I159" s="138" t="s">
-        <x:v>2049</x:v>
+        <x:v>2046</x:v>
       </x:c>
       <x:c r="J159" s="134" t="s">
-        <x:v>2050</x:v>
+        <x:v>2047</x:v>
       </x:c>
       <x:c r="K159" s="134"/>
       <x:c r="L159" s="134"/>
@@ -51749,13 +51730,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G160" s="138" t="s">
-        <x:v>2041</x:v>
+        <x:v>2038</x:v>
       </x:c>
       <x:c r="H160" s="140" t="s">
-        <x:v>2042</x:v>
+        <x:v>2039</x:v>
       </x:c>
       <x:c r="I160" s="138" t="s">
-        <x:v>2051</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="J160" s="134"/>
       <x:c r="K160" s="134"/>
@@ -51771,7 +51752,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G161" s="138" t="s">
-        <x:v>2052</x:v>
+        <x:v>2049</x:v>
       </x:c>
       <x:c r="H161" s="313">
         <x:v>46109</x:v>
@@ -51792,30 +51773,30 @@
         <x:v>644</x:v>
       </x:c>
       <x:c r="D162" s="116" t="s">
-        <x:v>2053</x:v>
+        <x:v>2050</x:v>
       </x:c>
       <x:c r="E162" s="116" t="s">
-        <x:v>2054</x:v>
+        <x:v>2051</x:v>
       </x:c>
       <x:c r="F162" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G162" s="320" t="s">
-        <x:v>2055</x:v>
+        <x:v>2052</x:v>
       </x:c>
       <x:c r="H162" s="116" t="s">
-        <x:v>2042</x:v>
+        <x:v>2039</x:v>
       </x:c>
       <x:c r="I162" s="320" t="s">
-        <x:v>2043</x:v>
+        <x:v>2040</x:v>
       </x:c>
       <x:c r="J162" s="134" t="s">
-        <x:v>2056</x:v>
+        <x:v>2053</x:v>
       </x:c>
       <x:c r="K162" s="134" t="s">
-        <x:v>2007</x:v>
-      </x:c>
-      <x:c r="L162" s="134"/>
+        <x:v>2029</x:v>
+      </x:c>
+      <x:c r="L162" s="134" t="s"/>
     </x:row>
     <x:row r="163" spans="1:12" ht="54" customHeight="1">
       <x:c r="A163" s="116"/>
@@ -51827,14 +51808,14 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G163" s="320" t="s">
-        <x:v>2057</x:v>
+        <x:v>2054</x:v>
       </x:c>
       <x:c r="H163" s="116"/>
       <x:c r="I163" s="320" t="s">
-        <x:v>2058</x:v>
+        <x:v>2055</x:v>
       </x:c>
       <x:c r="J163" s="134" t="s">
-        <x:v>2059</x:v>
+        <x:v>2056</x:v>
       </x:c>
       <x:c r="K163" s="134"/>
       <x:c r="L163" s="134"/>
@@ -51849,14 +51830,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G164" s="320" t="s">
-        <x:v>2060</x:v>
+        <x:v>2057</x:v>
       </x:c>
       <x:c r="H164" s="116"/>
       <x:c r="I164" s="320" t="s">
-        <x:v>2061</x:v>
+        <x:v>2058</x:v>
       </x:c>
       <x:c r="J164" s="134" t="s">
-        <x:v>2062</x:v>
+        <x:v>2059</x:v>
       </x:c>
       <x:c r="K164" s="134"/>
       <x:c r="L164" s="134"/>
@@ -51881,13 +51862,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G165" s="320" t="s">
-        <x:v>2063</x:v>
+        <x:v>2060</x:v>
       </x:c>
       <x:c r="H165" s="318">
         <x:v>0.333333333333333</x:v>
       </x:c>
       <x:c r="I165" s="320" t="s">
-        <x:v>2064</x:v>
+        <x:v>2061</x:v>
       </x:c>
       <x:c r="J165" s="134"/>
       <x:c r="K165" s="134"/>
@@ -51903,13 +51884,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G166" s="320" t="s">
-        <x:v>2065</x:v>
+        <x:v>2062</x:v>
       </x:c>
       <x:c r="H166" s="116" t="s">
-        <x:v>2066</x:v>
+        <x:v>2063</x:v>
       </x:c>
       <x:c r="I166" s="320" t="s">
-        <x:v>2067</x:v>
+        <x:v>2064</x:v>
       </x:c>
       <x:c r="J166" s="134"/>
       <x:c r="K166" s="134"/>
@@ -51925,13 +51906,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G167" s="320" t="s">
-        <x:v>2068</x:v>
+        <x:v>2065</x:v>
       </x:c>
       <x:c r="H167" s="116" t="s">
-        <x:v>2069</x:v>
+        <x:v>2066</x:v>
       </x:c>
       <x:c r="I167" s="320" t="s">
-        <x:v>2070</x:v>
+        <x:v>2067</x:v>
       </x:c>
       <x:c r="J167" s="134"/>
       <x:c r="K167" s="134"/>
@@ -51947,11 +51928,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G168" s="320" t="s">
-        <x:v>2071</x:v>
+        <x:v>2068</x:v>
       </x:c>
       <x:c r="H168" s="116"/>
       <x:c r="I168" s="320" t="s">
-        <x:v>2072</x:v>
+        <x:v>2069</x:v>
       </x:c>
       <x:c r="J168" s="134"/>
       <x:c r="K168" s="134"/>
@@ -51968,22 +51949,22 @@
         <x:v>658</x:v>
       </x:c>
       <x:c r="D169" s="116" t="s">
-        <x:v>2073</x:v>
+        <x:v>2070</x:v>
       </x:c>
       <x:c r="E169" s="116" t="s">
-        <x:v>2074</x:v>
+        <x:v>2071</x:v>
       </x:c>
       <x:c r="F169" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G169" s="320" t="s">
-        <x:v>2075</x:v>
+        <x:v>2072</x:v>
       </x:c>
       <x:c r="H169" s="116" t="s">
-        <x:v>2076</x:v>
+        <x:v>2073</x:v>
       </x:c>
       <x:c r="I169" s="320" t="s">
-        <x:v>2077</x:v>
+        <x:v>2074</x:v>
       </x:c>
       <x:c r="J169" s="134"/>
       <x:c r="K169" s="134"/>
@@ -51999,11 +51980,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G170" s="320" t="s">
-        <x:v>2078</x:v>
+        <x:v>2075</x:v>
       </x:c>
       <x:c r="H170" s="116"/>
       <x:c r="I170" s="320" t="s">
-        <x:v>2079</x:v>
+        <x:v>2076</x:v>
       </x:c>
       <x:c r="J170" s="134"/>
       <x:c r="K170" s="134"/>
@@ -52019,11 +52000,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G171" s="320" t="s">
-        <x:v>2080</x:v>
+        <x:v>2077</x:v>
       </x:c>
       <x:c r="H171" s="116"/>
       <x:c r="I171" s="320" t="s">
-        <x:v>2081</x:v>
+        <x:v>2078</x:v>
       </x:c>
       <x:c r="J171" s="134"/>
       <x:c r="K171" s="134"/>
@@ -52049,13 +52030,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G172" s="320" t="s">
-        <x:v>2082</x:v>
+        <x:v>2079</x:v>
       </x:c>
       <x:c r="H172" s="116" t="s">
-        <x:v>2076</x:v>
+        <x:v>2073</x:v>
       </x:c>
       <x:c r="I172" s="320" t="s">
-        <x:v>2077</x:v>
+        <x:v>2074</x:v>
       </x:c>
       <x:c r="J172" s="134"/>
       <x:c r="K172" s="134"/>
@@ -52071,11 +52052,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G173" s="320" t="s">
-        <x:v>2083</x:v>
+        <x:v>2080</x:v>
       </x:c>
       <x:c r="H173" s="116"/>
       <x:c r="I173" s="320" t="s">
-        <x:v>2084</x:v>
+        <x:v>2081</x:v>
       </x:c>
       <x:c r="J173" s="134"/>
       <x:c r="K173" s="134"/>
@@ -52101,13 +52082,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G174" s="320" t="s">
-        <x:v>2085</x:v>
+        <x:v>2082</x:v>
       </x:c>
       <x:c r="H174" s="116" t="s">
-        <x:v>2076</x:v>
+        <x:v>2073</x:v>
       </x:c>
       <x:c r="I174" s="320" t="s">
-        <x:v>2086</x:v>
+        <x:v>2083</x:v>
       </x:c>
       <x:c r="J174" s="134"/>
       <x:c r="K174" s="134"/>
@@ -52123,11 +52104,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G175" s="320" t="s">
-        <x:v>2087</x:v>
+        <x:v>2084</x:v>
       </x:c>
       <x:c r="H175" s="116"/>
       <x:c r="I175" s="320" t="s">
-        <x:v>2077</x:v>
+        <x:v>2074</x:v>
       </x:c>
       <x:c r="J175" s="134"/>
       <x:c r="K175" s="134"/>
@@ -52143,11 +52124,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G176" s="320" t="s">
-        <x:v>2088</x:v>
+        <x:v>2085</x:v>
       </x:c>
       <x:c r="H176" s="116"/>
       <x:c r="I176" s="320" t="s">
-        <x:v>2089</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="J176" s="134"/>
       <x:c r="K176" s="134"/>
@@ -52164,20 +52145,20 @@
         <x:v>674</x:v>
       </x:c>
       <x:c r="D177" s="116" t="s">
-        <x:v>2090</x:v>
+        <x:v>2087</x:v>
       </x:c>
       <x:c r="E177" s="116" t="s">
-        <x:v>2091</x:v>
+        <x:v>2088</x:v>
       </x:c>
       <x:c r="F177" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G177" s="320" t="s">
-        <x:v>2092</x:v>
+        <x:v>2089</x:v>
       </x:c>
       <x:c r="H177" s="116"/>
       <x:c r="I177" s="320" t="s">
-        <x:v>2093</x:v>
+        <x:v>2090</x:v>
       </x:c>
       <x:c r="J177" s="134"/>
       <x:c r="K177" s="134"/>
@@ -52193,11 +52174,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G178" s="320" t="s">
-        <x:v>2094</x:v>
+        <x:v>2091</x:v>
       </x:c>
       <x:c r="H178" s="116"/>
       <x:c r="I178" s="320" t="s">
-        <x:v>2095</x:v>
+        <x:v>2092</x:v>
       </x:c>
       <x:c r="J178" s="134"/>
       <x:c r="K178" s="134"/>
@@ -52214,22 +52195,22 @@
         <x:v>677</x:v>
       </x:c>
       <x:c r="D179" s="116" t="s">
-        <x:v>2096</x:v>
+        <x:v>2093</x:v>
       </x:c>
       <x:c r="E179" s="116" t="s">
-        <x:v>2097</x:v>
+        <x:v>2094</x:v>
       </x:c>
       <x:c r="F179" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G179" s="320" t="s">
-        <x:v>2098</x:v>
+        <x:v>2095</x:v>
       </x:c>
       <x:c r="H179" s="116" t="s">
         <x:v>681</x:v>
       </x:c>
       <x:c r="I179" s="320" t="s">
-        <x:v>2099</x:v>
+        <x:v>2096</x:v>
       </x:c>
       <x:c r="J179" s="116"/>
       <x:c r="K179" s="134"/>
@@ -52245,13 +52226,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G180" s="321" t="s">
-        <x:v>2100</x:v>
+        <x:v>2097</x:v>
       </x:c>
       <x:c r="H180" s="115" t="s">
-        <x:v>2101</x:v>
+        <x:v>2098</x:v>
       </x:c>
       <x:c r="I180" s="321" t="s">
-        <x:v>2102</x:v>
+        <x:v>2099</x:v>
       </x:c>
       <x:c r="J180" s="115"/>
       <x:c r="K180" s="137"/>
@@ -52268,22 +52249,22 @@
         <x:v>686</x:v>
       </x:c>
       <x:c r="D181" s="116" t="s">
-        <x:v>2103</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="E181" s="116" t="s">
-        <x:v>2104</x:v>
+        <x:v>2101</x:v>
       </x:c>
       <x:c r="F181" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G181" s="320" t="s">
-        <x:v>2105</x:v>
+        <x:v>2102</x:v>
       </x:c>
       <x:c r="H181" s="116" t="s">
-        <x:v>2106</x:v>
+        <x:v>2103</x:v>
       </x:c>
       <x:c r="I181" s="320" t="s">
-        <x:v>2107</x:v>
+        <x:v>2104</x:v>
       </x:c>
       <x:c r="J181" s="134"/>
       <x:c r="K181" s="134"/>
@@ -52299,13 +52280,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G182" s="320" t="s">
-        <x:v>2108</x:v>
+        <x:v>2105</x:v>
       </x:c>
       <x:c r="H182" s="116" t="s">
-        <x:v>2109</x:v>
+        <x:v>2106</x:v>
       </x:c>
       <x:c r="I182" s="320" t="s">
-        <x:v>2110</x:v>
+        <x:v>2107</x:v>
       </x:c>
       <x:c r="J182" s="134"/>
       <x:c r="K182" s="134"/>
@@ -52321,11 +52302,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G183" s="320" t="s">
-        <x:v>2111</x:v>
+        <x:v>2108</x:v>
       </x:c>
       <x:c r="H183" s="116"/>
       <x:c r="I183" s="320" t="s">
-        <x:v>2112</x:v>
+        <x:v>2109</x:v>
       </x:c>
       <x:c r="J183" s="134"/>
       <x:c r="K183" s="134"/>
@@ -52342,20 +52323,20 @@
         <x:v>696</x:v>
       </x:c>
       <x:c r="D184" s="116" t="s">
-        <x:v>2113</x:v>
+        <x:v>2110</x:v>
       </x:c>
       <x:c r="E184" s="116" t="s">
-        <x:v>2114</x:v>
+        <x:v>2111</x:v>
       </x:c>
       <x:c r="F184" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G184" s="320" t="s">
-        <x:v>2115</x:v>
+        <x:v>2112</x:v>
       </x:c>
       <x:c r="H184" s="116"/>
       <x:c r="I184" s="320" t="s">
-        <x:v>2116</x:v>
+        <x:v>2113</x:v>
       </x:c>
       <x:c r="J184" s="134"/>
       <x:c r="K184" s="134"/>
@@ -52371,13 +52352,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G185" s="320" t="s">
-        <x:v>2117</x:v>
+        <x:v>2114</x:v>
       </x:c>
       <x:c r="H185" s="116" t="s">
-        <x:v>2118</x:v>
+        <x:v>2115</x:v>
       </x:c>
       <x:c r="I185" s="320" t="s">
-        <x:v>2119</x:v>
+        <x:v>2116</x:v>
       </x:c>
       <x:c r="J185" s="134"/>
       <x:c r="K185" s="134"/>
@@ -52393,11 +52374,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G186" s="320" t="s">
-        <x:v>2120</x:v>
+        <x:v>2117</x:v>
       </x:c>
       <x:c r="H186" s="116"/>
       <x:c r="I186" s="320" t="s">
-        <x:v>2121</x:v>
+        <x:v>2118</x:v>
       </x:c>
       <x:c r="J186" s="134"/>
       <x:c r="K186" s="134"/>
@@ -52413,11 +52394,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G187" s="320" t="s">
-        <x:v>2122</x:v>
+        <x:v>2119</x:v>
       </x:c>
       <x:c r="H187" s="116"/>
       <x:c r="I187" s="320" t="s">
-        <x:v>2123</x:v>
+        <x:v>2120</x:v>
       </x:c>
       <x:c r="J187" s="134"/>
       <x:c r="K187" s="134"/>
@@ -52434,22 +52415,22 @@
         <x:v>932</x:v>
       </x:c>
       <x:c r="D188" s="114" t="s">
-        <x:v>2124</x:v>
+        <x:v>2121</x:v>
       </x:c>
       <x:c r="E188" s="114" t="s">
-        <x:v>2125</x:v>
+        <x:v>2122</x:v>
       </x:c>
       <x:c r="F188" s="329">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G188" s="324" t="s">
-        <x:v>2126</x:v>
+        <x:v>2123</x:v>
       </x:c>
       <x:c r="H188" s="324" t="s">
-        <x:v>2127</x:v>
+        <x:v>2124</x:v>
       </x:c>
       <x:c r="I188" s="325" t="s">
-        <x:v>2128</x:v>
+        <x:v>2125</x:v>
       </x:c>
       <x:c r="J188" s="61"/>
       <x:c r="K188" s="133"/>
@@ -52465,13 +52446,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G189" s="324" t="s">
-        <x:v>2129</x:v>
+        <x:v>2126</x:v>
       </x:c>
       <x:c r="H189" s="324" t="s">
-        <x:v>2130</x:v>
+        <x:v>2127</x:v>
       </x:c>
       <x:c r="I189" s="325" t="s">
-        <x:v>2131</x:v>
+        <x:v>2128</x:v>
       </x:c>
       <x:c r="J189" s="61"/>
       <x:c r="K189" s="124"/>
@@ -52487,11 +52468,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G190" s="324" t="s">
-        <x:v>2132</x:v>
+        <x:v>2129</x:v>
       </x:c>
       <x:c r="H190" s="324"/>
       <x:c r="I190" s="325" t="s">
-        <x:v>2133</x:v>
+        <x:v>2130</x:v>
       </x:c>
       <x:c r="J190" s="61"/>
       <x:c r="K190" s="111"/>
@@ -52508,20 +52489,20 @@
         <x:v>947</x:v>
       </x:c>
       <x:c r="D191" s="114" t="s">
-        <x:v>2134</x:v>
+        <x:v>2131</x:v>
       </x:c>
       <x:c r="E191" s="114" t="s">
-        <x:v>2135</x:v>
+        <x:v>2132</x:v>
       </x:c>
       <x:c r="F191" s="329">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G191" s="324" t="s">
-        <x:v>2136</x:v>
+        <x:v>2133</x:v>
       </x:c>
       <x:c r="H191" s="324"/>
       <x:c r="I191" s="325" t="s">
-        <x:v>2137</x:v>
+        <x:v>2134</x:v>
       </x:c>
       <x:c r="J191" s="61"/>
       <x:c r="K191" s="133"/>
@@ -52537,11 +52518,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G192" s="324" t="s">
-        <x:v>2138</x:v>
+        <x:v>2135</x:v>
       </x:c>
       <x:c r="H192" s="324"/>
       <x:c r="I192" s="325" t="s">
-        <x:v>2139</x:v>
+        <x:v>2136</x:v>
       </x:c>
       <x:c r="J192" s="61"/>
       <x:c r="K192" s="124"/>
@@ -52557,13 +52538,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G193" s="324" t="s">
-        <x:v>2140</x:v>
+        <x:v>2137</x:v>
       </x:c>
       <x:c r="H193" s="324" t="s">
-        <x:v>2141</x:v>
+        <x:v>2138</x:v>
       </x:c>
       <x:c r="I193" s="325" t="s">
-        <x:v>2142</x:v>
+        <x:v>2139</x:v>
       </x:c>
       <x:c r="J193" s="61"/>
       <x:c r="K193" s="111"/>
@@ -52908,13 +52889,13 @@
     <x:mergeCell ref="L191:L193"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H49" r:id="rId137"/>
-    <x:hyperlink ref="H67" r:id="rId138"/>
-    <x:hyperlink ref="H76" r:id="rId139"/>
-    <x:hyperlink ref="H85" r:id="rId140"/>
-    <x:hyperlink ref="H94" r:id="rId141"/>
-    <x:hyperlink ref="H103" r:id="rId142"/>
-    <x:hyperlink ref="H112" r:id="rId143"/>
+    <x:hyperlink ref="H49" r:id="rId179"/>
+    <x:hyperlink ref="H67" r:id="rId180"/>
+    <x:hyperlink ref="H76" r:id="rId181"/>
+    <x:hyperlink ref="H85" r:id="rId182"/>
+    <x:hyperlink ref="H94" r:id="rId183"/>
+    <x:hyperlink ref="H103" r:id="rId184"/>
+    <x:hyperlink ref="H112" r:id="rId185"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -53007,7 +52988,7 @@
         <x:v>1270</x:v>
       </x:c>
       <x:c r="H2" s="288" t="s">
-        <x:v>2143</x:v>
+        <x:v>2140</x:v>
       </x:c>
       <x:c r="I2" s="134" t="s">
         <x:v>1272</x:v>
@@ -53054,7 +53035,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="297" t="s">
-        <x:v>2144</x:v>
+        <x:v>2141</x:v>
       </x:c>
       <x:c r="H4" s="297" t="s">
         <x:v>1277</x:v>
@@ -53134,7 +53115,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="297" t="s">
-        <x:v>2145</x:v>
+        <x:v>2142</x:v>
       </x:c>
       <x:c r="H7" s="297"/>
       <x:c r="I7" s="298" t="s">
@@ -53167,7 +53148,7 @@
         <x:v>1297</x:v>
       </x:c>
       <x:c r="H8" s="297" t="s">
-        <x:v>2146</x:v>
+        <x:v>2143</x:v>
       </x:c>
       <x:c r="I8" s="134" t="s">
         <x:v>1299</x:v>
@@ -53186,7 +53167,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G9" s="319" t="s">
-        <x:v>2147</x:v>
+        <x:v>2144</x:v>
       </x:c>
       <x:c r="H9" s="297"/>
       <x:c r="I9" s="134"/>
@@ -53275,7 +53256,7 @@
         <x:v>1297</x:v>
       </x:c>
       <x:c r="H13" s="297" t="s">
-        <x:v>2148</x:v>
+        <x:v>2145</x:v>
       </x:c>
       <x:c r="I13" s="134" t="s">
         <x:v>1307</x:v>
@@ -53294,7 +53275,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="319" t="s">
-        <x:v>2147</x:v>
+        <x:v>2144</x:v>
       </x:c>
       <x:c r="H14" s="297"/>
       <x:c r="I14" s="134"/>
@@ -53380,7 +53361,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="61" t="s">
-        <x:v>2149</x:v>
+        <x:v>2146</x:v>
       </x:c>
       <x:c r="H18" s="140"/>
       <x:c r="I18" s="140" t="s">
@@ -53400,7 +53381,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="61" t="s">
-        <x:v>2150</x:v>
+        <x:v>2147</x:v>
       </x:c>
       <x:c r="H19" s="140" t="s">
         <x:v>965</x:v>
@@ -53420,7 +53401,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="61" t="s">
-        <x:v>2151</x:v>
+        <x:v>2148</x:v>
       </x:c>
       <x:c r="H20" s="140"/>
       <x:c r="I20" s="140"/>
@@ -53438,7 +53419,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G21" s="61" t="s">
-        <x:v>2152</x:v>
+        <x:v>2149</x:v>
       </x:c>
       <x:c r="H21" s="140" t="s">
         <x:v>968</x:v>
@@ -53458,7 +53439,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G22" s="61" t="s">
-        <x:v>2153</x:v>
+        <x:v>2150</x:v>
       </x:c>
       <x:c r="H22" s="314" t="s">
         <x:v>970</x:v>
@@ -53478,7 +53459,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G23" s="61" t="s">
-        <x:v>2154</x:v>
+        <x:v>2151</x:v>
       </x:c>
       <x:c r="H23" s="140">
         <x:v>1</x:v>
@@ -53498,7 +53479,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G24" s="61" t="s">
-        <x:v>2155</x:v>
+        <x:v>2152</x:v>
       </x:c>
       <x:c r="H24" s="140" t="s">
         <x:v>973</x:v>
@@ -53518,7 +53499,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G25" s="61" t="s">
-        <x:v>2156</x:v>
+        <x:v>2153</x:v>
       </x:c>
       <x:c r="H25" s="140"/>
       <x:c r="I25" s="140"/>
@@ -53546,7 +53527,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G26" s="61" t="s">
-        <x:v>2157</x:v>
+        <x:v>2154</x:v>
       </x:c>
       <x:c r="H26" s="140"/>
       <x:c r="I26" s="133" t="s">
@@ -53586,7 +53567,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G28" s="61" t="s">
-        <x:v>2158</x:v>
+        <x:v>2155</x:v>
       </x:c>
       <x:c r="H28" s="239" t="s">
         <x:v>970</x:v>
@@ -53606,7 +53587,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G29" s="61" t="s">
-        <x:v>2159</x:v>
+        <x:v>2156</x:v>
       </x:c>
       <x:c r="H29" s="140">
         <x:v>1</x:v>
@@ -53626,7 +53607,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G30" s="61" t="s">
-        <x:v>2160</x:v>
+        <x:v>2157</x:v>
       </x:c>
       <x:c r="H30" s="140"/>
       <x:c r="I30" s="111"/>
@@ -53654,7 +53635,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="61" t="s">
-        <x:v>2161</x:v>
+        <x:v>2158</x:v>
       </x:c>
       <x:c r="H31" s="140"/>
       <x:c r="I31" s="133" t="s">
@@ -53753,7 +53734,7 @@
         <x:v>1309</x:v>
       </x:c>
       <x:c r="D36" s="134" t="s">
-        <x:v>2162</x:v>
+        <x:v>2159</x:v>
       </x:c>
       <x:c r="E36" s="134" t="s">
         <x:v>1311</x:v>
@@ -53765,7 +53746,7 @@
         <x:v>988</x:v>
       </x:c>
       <x:c r="H36" s="297" t="s">
-        <x:v>2163</x:v>
+        <x:v>2160</x:v>
       </x:c>
       <x:c r="I36" s="134" t="s">
         <x:v>1312</x:v>
@@ -53787,7 +53768,7 @@
         <x:v>990</x:v>
       </x:c>
       <x:c r="H37" s="314" t="s">
-        <x:v>2164</x:v>
+        <x:v>2161</x:v>
       </x:c>
       <x:c r="I37" s="134"/>
       <x:c r="J37" s="9"/>
@@ -53823,7 +53804,7 @@
         <x:v>1314</x:v>
       </x:c>
       <x:c r="D39" s="134" t="s">
-        <x:v>2165</x:v>
+        <x:v>2162</x:v>
       </x:c>
       <x:c r="E39" s="134" t="s">
         <x:v>1311</x:v>
@@ -53832,10 +53813,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G39" s="319" t="s">
-        <x:v>2166</x:v>
+        <x:v>2163</x:v>
       </x:c>
       <x:c r="H39" s="297" t="s">
-        <x:v>2167</x:v>
+        <x:v>2164</x:v>
       </x:c>
       <x:c r="I39" s="134" t="s">
         <x:v>1317</x:v>
@@ -53857,7 +53838,7 @@
         <x:v>990</x:v>
       </x:c>
       <x:c r="H40" s="314" t="s">
-        <x:v>2164</x:v>
+        <x:v>2161</x:v>
       </x:c>
       <x:c r="I40" s="134"/>
       <x:c r="J40" s="9"/>
@@ -56793,17 +56774,17 @@
     <x:mergeCell ref="J168:J171"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H22" r:id="rId144"/>
-    <x:hyperlink ref="H28" r:id="rId145"/>
-    <x:hyperlink ref="H11" r:id="rId146"/>
-    <x:hyperlink ref="H16" r:id="rId147"/>
-    <x:hyperlink ref="H37" r:id="rId148"/>
-    <x:hyperlink ref="H40" r:id="rId149"/>
-    <x:hyperlink ref="H130" r:id="rId150"/>
-    <x:hyperlink ref="H136" r:id="rId151"/>
-    <x:hyperlink ref="H142" r:id="rId152"/>
-    <x:hyperlink ref="H148" r:id="rId153"/>
-    <x:hyperlink ref="H154" r:id="rId154"/>
+    <x:hyperlink ref="H22" r:id="rId186"/>
+    <x:hyperlink ref="H28" r:id="rId187"/>
+    <x:hyperlink ref="H11" r:id="rId188"/>
+    <x:hyperlink ref="H16" r:id="rId189"/>
+    <x:hyperlink ref="H37" r:id="rId190"/>
+    <x:hyperlink ref="H40" r:id="rId191"/>
+    <x:hyperlink ref="H130" r:id="rId192"/>
+    <x:hyperlink ref="H136" r:id="rId193"/>
+    <x:hyperlink ref="H142" r:id="rId194"/>
+    <x:hyperlink ref="H148" r:id="rId195"/>
+    <x:hyperlink ref="H154" r:id="rId196"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -56888,19 +56869,19 @@
         <x:v>705</x:v>
       </x:c>
       <x:c r="E2" s="116" t="s">
-        <x:v>2168</x:v>
+        <x:v>2165</x:v>
       </x:c>
       <x:c r="F2" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G2" s="327" t="s">
-        <x:v>2169</x:v>
+        <x:v>2166</x:v>
       </x:c>
       <x:c r="H2" s="116" t="s">
-        <x:v>2170</x:v>
+        <x:v>2167</x:v>
       </x:c>
       <x:c r="I2" s="289" t="s">
-        <x:v>2171</x:v>
+        <x:v>2168</x:v>
       </x:c>
       <x:c r="J2" s="1"/>
       <x:c r="K2" s="1"/>
@@ -56916,11 +56897,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G3" s="327" t="s">
-        <x:v>2172</x:v>
+        <x:v>2169</x:v>
       </x:c>
       <x:c r="H3" s="116"/>
       <x:c r="I3" s="289" t="s">
-        <x:v>2173</x:v>
+        <x:v>2170</x:v>
       </x:c>
       <x:c r="J3" s="1"/>
       <x:c r="K3" s="1"/>
@@ -56940,19 +56921,19 @@
         <x:v>707</x:v>
       </x:c>
       <x:c r="E4" s="116" t="s">
-        <x:v>2168</x:v>
+        <x:v>2165</x:v>
       </x:c>
       <x:c r="F4" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="327" t="s">
-        <x:v>2174</x:v>
+        <x:v>2171</x:v>
       </x:c>
       <x:c r="H4" s="116" t="s">
-        <x:v>2175</x:v>
+        <x:v>2172</x:v>
       </x:c>
       <x:c r="I4" s="289" t="s">
-        <x:v>2176</x:v>
+        <x:v>2173</x:v>
       </x:c>
       <x:c r="J4" s="61"/>
       <x:c r="K4" s="1"/>
@@ -56968,11 +56949,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G5" s="327" t="s">
-        <x:v>2177</x:v>
+        <x:v>2174</x:v>
       </x:c>
       <x:c r="H5" s="116"/>
       <x:c r="I5" s="289" t="s">
-        <x:v>2178</x:v>
+        <x:v>2175</x:v>
       </x:c>
       <x:c r="J5" s="61"/>
       <x:c r="K5" s="1"/>
@@ -56988,11 +56969,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G6" s="327" t="s">
-        <x:v>2071</x:v>
+        <x:v>2068</x:v>
       </x:c>
       <x:c r="H6" s="116"/>
       <x:c r="I6" s="289" t="s">
-        <x:v>2179</x:v>
+        <x:v>2176</x:v>
       </x:c>
       <x:c r="J6" s="61"/>
       <x:c r="K6" s="1"/>
@@ -57012,19 +56993,19 @@
         <x:v>709</x:v>
       </x:c>
       <x:c r="E7" s="116" t="s">
-        <x:v>2180</x:v>
+        <x:v>2177</x:v>
       </x:c>
       <x:c r="F7" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="327" t="s">
-        <x:v>2181</x:v>
+        <x:v>2178</x:v>
       </x:c>
       <x:c r="H7" s="116" t="s">
-        <x:v>2182</x:v>
+        <x:v>2179</x:v>
       </x:c>
       <x:c r="I7" s="289" t="s">
-        <x:v>2183</x:v>
+        <x:v>2180</x:v>
       </x:c>
       <x:c r="J7" s="61"/>
       <x:c r="K7" s="1"/>
@@ -57040,11 +57021,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G8" s="327" t="s">
-        <x:v>2071</x:v>
+        <x:v>2068</x:v>
       </x:c>
       <x:c r="H8" s="116"/>
       <x:c r="I8" s="289" t="s">
-        <x:v>2184</x:v>
+        <x:v>2181</x:v>
       </x:c>
       <x:c r="J8" s="61"/>
       <x:c r="K8" s="1"/>
@@ -57060,11 +57041,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G9" s="327" t="s">
-        <x:v>2185</x:v>
+        <x:v>2182</x:v>
       </x:c>
       <x:c r="H9" s="116"/>
       <x:c r="I9" s="289" t="s">
-        <x:v>2186</x:v>
+        <x:v>2183</x:v>
       </x:c>
       <x:c r="J9" s="61"/>
       <x:c r="K9" s="1"/>
@@ -57081,20 +57062,20 @@
         <x:v>717</x:v>
       </x:c>
       <x:c r="D10" s="116" t="s">
-        <x:v>2187</x:v>
+        <x:v>2184</x:v>
       </x:c>
       <x:c r="E10" s="116" t="s">
-        <x:v>2188</x:v>
+        <x:v>2185</x:v>
       </x:c>
       <x:c r="F10" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="327" t="s">
-        <x:v>2092</x:v>
+        <x:v>2089</x:v>
       </x:c>
       <x:c r="H10" s="116"/>
       <x:c r="I10" s="289" t="s">
-        <x:v>2189</x:v>
+        <x:v>2186</x:v>
       </x:c>
       <x:c r="J10" s="61"/>
       <x:c r="K10" s="1"/>
@@ -57110,11 +57091,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G11" s="327" t="s">
-        <x:v>2190</x:v>
+        <x:v>2187</x:v>
       </x:c>
       <x:c r="H11" s="116"/>
       <x:c r="I11" s="289" t="s">
-        <x:v>2191</x:v>
+        <x:v>2188</x:v>
       </x:c>
       <x:c r="J11" s="61"/>
       <x:c r="K11" s="1"/>
@@ -57130,11 +57111,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G12" s="327" t="s">
-        <x:v>2192</x:v>
+        <x:v>2189</x:v>
       </x:c>
       <x:c r="H12" s="116"/>
       <x:c r="I12" s="289" t="s">
-        <x:v>2193</x:v>
+        <x:v>2190</x:v>
       </x:c>
       <x:c r="J12" s="61"/>
       <x:c r="K12" s="1"/>
@@ -57151,20 +57132,20 @@
         <x:v>722</x:v>
       </x:c>
       <x:c r="D13" s="116" t="s">
-        <x:v>2194</x:v>
+        <x:v>2191</x:v>
       </x:c>
       <x:c r="E13" s="116" t="s">
-        <x:v>2195</x:v>
+        <x:v>2192</x:v>
       </x:c>
       <x:c r="F13" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="327" t="s">
-        <x:v>2071</x:v>
+        <x:v>2068</x:v>
       </x:c>
       <x:c r="H13" s="116"/>
       <x:c r="I13" s="289" t="s">
-        <x:v>2196</x:v>
+        <x:v>2193</x:v>
       </x:c>
       <x:c r="J13" s="61"/>
       <x:c r="K13" s="1"/>
@@ -57180,11 +57161,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="327" t="s">
-        <x:v>2197</x:v>
+        <x:v>2194</x:v>
       </x:c>
       <x:c r="H14" s="116"/>
       <x:c r="I14" s="289" t="s">
-        <x:v>2198</x:v>
+        <x:v>2195</x:v>
       </x:c>
       <x:c r="J14" s="61"/>
       <x:c r="K14" s="1"/>
@@ -57201,22 +57182,22 @@
         <x:v>724</x:v>
       </x:c>
       <x:c r="D15" s="116" t="s">
-        <x:v>2199</x:v>
+        <x:v>2196</x:v>
       </x:c>
       <x:c r="E15" s="116" t="s">
-        <x:v>2200</x:v>
+        <x:v>2197</x:v>
       </x:c>
       <x:c r="F15" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G15" s="327" t="s">
-        <x:v>2201</x:v>
+        <x:v>2198</x:v>
       </x:c>
       <x:c r="H15" s="116" t="s">
-        <x:v>2202</x:v>
+        <x:v>2199</x:v>
       </x:c>
       <x:c r="I15" s="289" t="s">
-        <x:v>2203</x:v>
+        <x:v>2200</x:v>
       </x:c>
       <x:c r="J15" s="61"/>
       <x:c r="K15" s="1"/>
@@ -57232,11 +57213,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G16" s="327" t="s">
-        <x:v>2204</x:v>
+        <x:v>2201</x:v>
       </x:c>
       <x:c r="H16" s="116"/>
       <x:c r="I16" s="289" t="s">
-        <x:v>2205</x:v>
+        <x:v>2202</x:v>
       </x:c>
       <x:c r="J16" s="61"/>
       <x:c r="K16" s="1"/>
@@ -57252,11 +57233,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G17" s="327" t="s">
-        <x:v>2206</x:v>
+        <x:v>2203</x:v>
       </x:c>
       <x:c r="H17" s="116"/>
       <x:c r="I17" s="289" t="s">
-        <x:v>2207</x:v>
+        <x:v>2204</x:v>
       </x:c>
       <x:c r="J17" s="61"/>
       <x:c r="K17" s="1"/>
@@ -57273,20 +57254,20 @@
         <x:v>726</x:v>
       </x:c>
       <x:c r="D18" s="116" t="s">
-        <x:v>2208</x:v>
+        <x:v>2205</x:v>
       </x:c>
       <x:c r="E18" s="116" t="s">
-        <x:v>2209</x:v>
+        <x:v>2206</x:v>
       </x:c>
       <x:c r="F18" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="327" t="s">
-        <x:v>2210</x:v>
+        <x:v>2207</x:v>
       </x:c>
       <x:c r="H18" s="116"/>
       <x:c r="I18" s="289" t="s">
-        <x:v>2211</x:v>
+        <x:v>2208</x:v>
       </x:c>
       <x:c r="J18" s="61"/>
       <x:c r="K18" s="1"/>
@@ -57302,13 +57283,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="327" t="s">
-        <x:v>2212</x:v>
+        <x:v>2209</x:v>
       </x:c>
       <x:c r="H19" s="116" t="s">
-        <x:v>2213</x:v>
+        <x:v>2210</x:v>
       </x:c>
       <x:c r="I19" s="289" t="s">
-        <x:v>2214</x:v>
+        <x:v>2211</x:v>
       </x:c>
       <x:c r="J19" s="61"/>
       <x:c r="K19" s="1"/>
@@ -57324,11 +57305,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="327" t="s">
-        <x:v>2215</x:v>
+        <x:v>2212</x:v>
       </x:c>
       <x:c r="H20" s="116"/>
       <x:c r="I20" s="289" t="s">
-        <x:v>2216</x:v>
+        <x:v>2213</x:v>
       </x:c>
       <x:c r="J20" s="61"/>
       <x:c r="K20" s="1"/>
@@ -57339,7 +57320,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B21" s="116" t="s">
-        <x:v>2217</x:v>
+        <x:v>2214</x:v>
       </x:c>
       <x:c r="C21" s="116" t="s">
         <x:v>732</x:v>
@@ -57348,19 +57329,19 @@
         <x:v>733</x:v>
       </x:c>
       <x:c r="E21" s="116" t="s">
-        <x:v>2218</x:v>
+        <x:v>2215</x:v>
       </x:c>
       <x:c r="F21" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G21" s="327" t="s">
-        <x:v>2219</x:v>
+        <x:v>2216</x:v>
       </x:c>
       <x:c r="H21" s="116" t="s">
         <x:v>741</x:v>
       </x:c>
       <x:c r="I21" s="289" t="s">
-        <x:v>2220</x:v>
+        <x:v>2217</x:v>
       </x:c>
       <x:c r="J21" s="61"/>
       <x:c r="K21" s="1"/>
@@ -57376,11 +57357,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G22" s="327" t="s">
-        <x:v>2221</x:v>
+        <x:v>2218</x:v>
       </x:c>
       <x:c r="H22" s="116"/>
       <x:c r="I22" s="289" t="s">
-        <x:v>2222</x:v>
+        <x:v>2219</x:v>
       </x:c>
       <x:c r="J22" s="61"/>
       <x:c r="K22" s="1"/>
@@ -57396,11 +57377,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G23" s="327" t="s">
-        <x:v>2223</x:v>
+        <x:v>2220</x:v>
       </x:c>
       <x:c r="H23" s="116"/>
       <x:c r="I23" s="289" t="s">
-        <x:v>2224</x:v>
+        <x:v>2221</x:v>
       </x:c>
       <x:c r="J23" s="61"/>
       <x:c r="K23" s="1"/>
@@ -57417,20 +57398,20 @@
         <x:v>737</x:v>
       </x:c>
       <x:c r="D24" s="116" t="s">
-        <x:v>2225</x:v>
+        <x:v>2222</x:v>
       </x:c>
       <x:c r="E24" s="116" t="s">
-        <x:v>2226</x:v>
+        <x:v>2223</x:v>
       </x:c>
       <x:c r="F24" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G24" s="327" t="s">
-        <x:v>2227</x:v>
+        <x:v>2224</x:v>
       </x:c>
       <x:c r="H24" s="116"/>
       <x:c r="I24" s="289" t="s">
-        <x:v>2228</x:v>
+        <x:v>2225</x:v>
       </x:c>
       <x:c r="J24" s="61"/>
       <x:c r="K24" s="35"/>
@@ -57446,11 +57427,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G25" s="327" t="s">
-        <x:v>2229</x:v>
+        <x:v>2226</x:v>
       </x:c>
       <x:c r="H25" s="116"/>
       <x:c r="I25" s="289" t="s">
-        <x:v>2230</x:v>
+        <x:v>2227</x:v>
       </x:c>
       <x:c r="J25" s="61"/>
       <x:c r="K25" s="35"/>
@@ -57466,11 +57447,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G26" s="327" t="s">
-        <x:v>2122</x:v>
+        <x:v>2119</x:v>
       </x:c>
       <x:c r="H26" s="116"/>
       <x:c r="I26" s="289" t="s">
-        <x:v>2231</x:v>
+        <x:v>2228</x:v>
       </x:c>
       <x:c r="J26" s="61"/>
       <x:c r="K26" s="35"/>
@@ -57487,20 +57468,20 @@
         <x:v>751</x:v>
       </x:c>
       <x:c r="D27" s="116" t="s">
-        <x:v>2232</x:v>
+        <x:v>2229</x:v>
       </x:c>
       <x:c r="E27" s="116" t="s">
-        <x:v>2233</x:v>
+        <x:v>2230</x:v>
       </x:c>
       <x:c r="F27" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G27" s="327" t="s">
-        <x:v>2234</x:v>
+        <x:v>2231</x:v>
       </x:c>
       <x:c r="H27" s="116"/>
       <x:c r="I27" s="327" t="s">
-        <x:v>2077</x:v>
+        <x:v>2074</x:v>
       </x:c>
       <x:c r="J27" s="61"/>
       <x:c r="K27" s="35"/>
@@ -57516,11 +57497,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G28" s="327" t="s">
-        <x:v>2235</x:v>
+        <x:v>2232</x:v>
       </x:c>
       <x:c r="H28" s="116"/>
       <x:c r="I28" s="289" t="s">
-        <x:v>2236</x:v>
+        <x:v>2233</x:v>
       </x:c>
       <x:c r="J28" s="61"/>
       <x:c r="K28" s="35"/>
@@ -57537,20 +57518,20 @@
         <x:v>753</x:v>
       </x:c>
       <x:c r="D29" s="116" t="s">
-        <x:v>2237</x:v>
+        <x:v>2234</x:v>
       </x:c>
       <x:c r="E29" s="116" t="s">
-        <x:v>2233</x:v>
+        <x:v>2230</x:v>
       </x:c>
       <x:c r="F29" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G29" s="327" t="s">
-        <x:v>2238</x:v>
+        <x:v>2235</x:v>
       </x:c>
       <x:c r="H29" s="116"/>
       <x:c r="I29" s="327" t="s">
-        <x:v>2077</x:v>
+        <x:v>2074</x:v>
       </x:c>
       <x:c r="J29" s="61"/>
       <x:c r="K29" s="35"/>
@@ -57566,11 +57547,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G30" s="327" t="s">
-        <x:v>2239</x:v>
+        <x:v>2236</x:v>
       </x:c>
       <x:c r="H30" s="116"/>
       <x:c r="I30" s="289" t="s">
-        <x:v>2240</x:v>
+        <x:v>2237</x:v>
       </x:c>
       <x:c r="J30" s="61"/>
       <x:c r="K30" s="35"/>
@@ -57590,19 +57571,19 @@
         <x:v>793</x:v>
       </x:c>
       <x:c r="E31" s="116" t="s">
-        <x:v>2241</x:v>
+        <x:v>2238</x:v>
       </x:c>
       <x:c r="F31" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="327" t="s">
-        <x:v>2242</x:v>
+        <x:v>2239</x:v>
       </x:c>
       <x:c r="H31" s="116" t="s">
-        <x:v>2243</x:v>
+        <x:v>2240</x:v>
       </x:c>
       <x:c r="I31" s="289" t="s">
-        <x:v>2244</x:v>
+        <x:v>2241</x:v>
       </x:c>
       <x:c r="J31" s="61"/>
       <x:c r="K31" s="35"/>
@@ -57618,11 +57599,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G32" s="327" t="s">
-        <x:v>2245</x:v>
+        <x:v>2242</x:v>
       </x:c>
       <x:c r="H32" s="116"/>
       <x:c r="I32" s="289" t="s">
-        <x:v>2246</x:v>
+        <x:v>2243</x:v>
       </x:c>
       <x:c r="J32" s="61"/>
       <x:c r="K32" s="35"/>
@@ -57642,19 +57623,19 @@
         <x:v>798</x:v>
       </x:c>
       <x:c r="E33" s="116" t="s">
-        <x:v>2247</x:v>
+        <x:v>2244</x:v>
       </x:c>
       <x:c r="F33" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G33" s="327" t="s">
-        <x:v>2248</x:v>
+        <x:v>2245</x:v>
       </x:c>
       <x:c r="H33" s="116" t="s">
-        <x:v>2243</x:v>
+        <x:v>2240</x:v>
       </x:c>
       <x:c r="I33" s="327" t="s">
-        <x:v>2077</x:v>
+        <x:v>2074</x:v>
       </x:c>
       <x:c r="J33" s="61"/>
       <x:c r="K33" s="35"/>
@@ -57670,11 +57651,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G34" s="327" t="s">
-        <x:v>2249</x:v>
+        <x:v>2246</x:v>
       </x:c>
       <x:c r="H34" s="116"/>
       <x:c r="I34" s="289" t="s">
-        <x:v>2250</x:v>
+        <x:v>2247</x:v>
       </x:c>
       <x:c r="J34" s="292"/>
       <x:c r="K34" s="35"/>
@@ -57691,20 +57672,20 @@
         <x:v>802</x:v>
       </x:c>
       <x:c r="D35" s="116" t="s">
-        <x:v>2251</x:v>
+        <x:v>2248</x:v>
       </x:c>
       <x:c r="E35" s="116" t="s">
-        <x:v>2252</x:v>
+        <x:v>2249</x:v>
       </x:c>
       <x:c r="F35" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G35" s="327" t="s">
-        <x:v>2253</x:v>
+        <x:v>2250</x:v>
       </x:c>
       <x:c r="H35" s="116"/>
       <x:c r="I35" s="289" t="s">
-        <x:v>2254</x:v>
+        <x:v>2251</x:v>
       </x:c>
       <x:c r="J35" s="61"/>
       <x:c r="K35" s="35"/>
@@ -57720,11 +57701,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G36" s="327" t="s">
-        <x:v>2255</x:v>
+        <x:v>2252</x:v>
       </x:c>
       <x:c r="H36" s="116"/>
       <x:c r="I36" s="289" t="s">
-        <x:v>2256</x:v>
+        <x:v>2253</x:v>
       </x:c>
       <x:c r="J36" s="61"/>
       <x:c r="K36" s="35"/>
@@ -57740,13 +57721,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G37" s="327" t="s">
-        <x:v>2257</x:v>
+        <x:v>2254</x:v>
       </x:c>
       <x:c r="H37" s="116" t="s">
-        <x:v>2258</x:v>
+        <x:v>2255</x:v>
       </x:c>
       <x:c r="I37" s="289" t="s">
-        <x:v>2259</x:v>
+        <x:v>2256</x:v>
       </x:c>
       <x:c r="J37" s="61"/>
       <x:c r="K37" s="35"/>
@@ -57763,20 +57744,20 @@
         <x:v>814</x:v>
       </x:c>
       <x:c r="D38" s="116" t="s">
-        <x:v>2260</x:v>
+        <x:v>2257</x:v>
       </x:c>
       <x:c r="E38" s="116" t="s">
-        <x:v>2261</x:v>
+        <x:v>2258</x:v>
       </x:c>
       <x:c r="F38" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G38" s="327" t="s">
-        <x:v>2262</x:v>
+        <x:v>2259</x:v>
       </x:c>
       <x:c r="H38" s="116"/>
       <x:c r="I38" s="289" t="s">
-        <x:v>2263</x:v>
+        <x:v>2260</x:v>
       </x:c>
       <x:c r="J38" s="61"/>
       <x:c r="K38" s="35"/>
@@ -57792,11 +57773,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G39" s="327" t="s">
-        <x:v>2264</x:v>
+        <x:v>2261</x:v>
       </x:c>
       <x:c r="H39" s="116"/>
       <x:c r="I39" s="289" t="s">
-        <x:v>2265</x:v>
+        <x:v>2262</x:v>
       </x:c>
       <x:c r="J39" s="61"/>
       <x:c r="K39" s="35"/>
@@ -57812,13 +57793,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G40" s="327" t="s">
-        <x:v>2266</x:v>
+        <x:v>2263</x:v>
       </x:c>
       <x:c r="H40" s="116" t="s">
-        <x:v>2258</x:v>
+        <x:v>2255</x:v>
       </x:c>
       <x:c r="I40" s="289" t="s">
-        <x:v>2267</x:v>
+        <x:v>2264</x:v>
       </x:c>
       <x:c r="J40" s="61"/>
       <x:c r="K40" s="35"/>
@@ -57834,11 +57815,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G41" s="327" t="s">
-        <x:v>2268</x:v>
+        <x:v>2265</x:v>
       </x:c>
       <x:c r="H41" s="116"/>
       <x:c r="I41" s="289" t="s">
-        <x:v>2269</x:v>
+        <x:v>2266</x:v>
       </x:c>
       <x:c r="J41" s="61"/>
       <x:c r="K41" s="35"/>
@@ -57855,20 +57836,20 @@
         <x:v>824</x:v>
       </x:c>
       <x:c r="D42" s="116" t="s">
-        <x:v>2270</x:v>
+        <x:v>2267</x:v>
       </x:c>
       <x:c r="E42" s="116" t="s">
-        <x:v>2271</x:v>
+        <x:v>2268</x:v>
       </x:c>
       <x:c r="F42" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G42" s="327" t="s">
-        <x:v>2272</x:v>
+        <x:v>2269</x:v>
       </x:c>
       <x:c r="H42" s="116"/>
       <x:c r="I42" s="289" t="s">
-        <x:v>2273</x:v>
+        <x:v>2270</x:v>
       </x:c>
       <x:c r="J42" s="61"/>
       <x:c r="K42" s="35"/>
@@ -57884,11 +57865,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G43" s="327" t="s">
-        <x:v>2274</x:v>
+        <x:v>2271</x:v>
       </x:c>
       <x:c r="H43" s="116"/>
       <x:c r="I43" s="289" t="s">
-        <x:v>2275</x:v>
+        <x:v>2272</x:v>
       </x:c>
       <x:c r="J43" s="61"/>
       <x:c r="K43" s="35"/>
@@ -57904,11 +57885,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G44" s="327" t="s">
-        <x:v>2276</x:v>
+        <x:v>2273</x:v>
       </x:c>
       <x:c r="H44" s="116"/>
       <x:c r="I44" s="289" t="s">
-        <x:v>2277</x:v>
+        <x:v>2274</x:v>
       </x:c>
       <x:c r="J44" s="61"/>
       <x:c r="K44" s="35"/>
@@ -57924,11 +57905,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G45" s="327" t="s">
-        <x:v>2278</x:v>
+        <x:v>2275</x:v>
       </x:c>
       <x:c r="H45" s="116"/>
       <x:c r="I45" s="289" t="s">
-        <x:v>2279</x:v>
+        <x:v>2276</x:v>
       </x:c>
       <x:c r="J45" s="61"/>
       <x:c r="K45" s="35"/>
@@ -57945,20 +57926,20 @@
         <x:v>835</x:v>
       </x:c>
       <x:c r="D46" s="116" t="s">
-        <x:v>2280</x:v>
+        <x:v>2277</x:v>
       </x:c>
       <x:c r="E46" s="116" t="s">
-        <x:v>2281</x:v>
+        <x:v>2278</x:v>
       </x:c>
       <x:c r="F46" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G46" s="327" t="s">
-        <x:v>2272</x:v>
+        <x:v>2269</x:v>
       </x:c>
       <x:c r="H46" s="116"/>
       <x:c r="I46" s="289" t="s">
-        <x:v>2282</x:v>
+        <x:v>2279</x:v>
       </x:c>
       <x:c r="J46" s="61"/>
       <x:c r="K46" s="35"/>
@@ -57974,13 +57955,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G47" s="327" t="s">
-        <x:v>2283</x:v>
+        <x:v>2280</x:v>
       </x:c>
       <x:c r="H47" s="116" t="s">
-        <x:v>2258</x:v>
+        <x:v>2255</x:v>
       </x:c>
       <x:c r="I47" s="289" t="s">
-        <x:v>2284</x:v>
+        <x:v>2281</x:v>
       </x:c>
       <x:c r="J47" s="61"/>
       <x:c r="K47" s="35"/>
@@ -57996,11 +57977,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G48" s="327" t="s">
-        <x:v>2285</x:v>
+        <x:v>2282</x:v>
       </x:c>
       <x:c r="H48" s="116"/>
       <x:c r="I48" s="289" t="s">
-        <x:v>2286</x:v>
+        <x:v>2283</x:v>
       </x:c>
       <x:c r="J48" s="61"/>
       <x:c r="K48" s="35"/>
@@ -58099,10 +58080,10 @@
         <x:v>999</x:v>
       </x:c>
       <x:c r="H52" s="334" t="s">
-        <x:v>2287</x:v>
+        <x:v>2284</x:v>
       </x:c>
       <x:c r="I52" s="51" t="s">
-        <x:v>2288</x:v>
+        <x:v>2285</x:v>
       </x:c>
       <x:c r="J52" s="51"/>
       <x:c r="K52" s="35"/>
@@ -58121,7 +58102,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H53" s="314" t="s">
-        <x:v>2289</x:v>
+        <x:v>2286</x:v>
       </x:c>
       <x:c r="I53" s="51"/>
       <x:c r="J53" s="51"/>
@@ -58172,7 +58153,7 @@
         <x:v>1000</x:v>
       </x:c>
       <x:c r="I55" s="51" t="s">
-        <x:v>2290</x:v>
+        <x:v>2287</x:v>
       </x:c>
       <x:c r="J55" s="51"/>
       <x:c r="K55" s="35"/>
@@ -58191,7 +58172,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H56" s="314" t="s">
-        <x:v>2291</x:v>
+        <x:v>2288</x:v>
       </x:c>
       <x:c r="I56" s="51"/>
       <x:c r="J56" s="51"/>
@@ -58310,7 +58291,7 @@
         <x:v>422</x:v>
       </x:c>
       <x:c r="I61" s="51" t="s">
-        <x:v>2292</x:v>
+        <x:v>2289</x:v>
       </x:c>
       <x:c r="J61" s="51"/>
       <x:c r="K61" s="35"/>
@@ -58608,7 +58589,7 @@
         <x:v>1037</x:v>
       </x:c>
       <x:c r="I74" s="51" t="s">
-        <x:v>2293</x:v>
+        <x:v>2290</x:v>
       </x:c>
       <x:c r="J74" s="51"/>
       <x:c r="K74" s="35"/>
@@ -59304,19 +59285,19 @@
         <x:v>843</x:v>
       </x:c>
       <x:c r="E106" s="116" t="s">
-        <x:v>2294</x:v>
+        <x:v>2291</x:v>
       </x:c>
       <x:c r="F106" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G106" s="327" t="s">
-        <x:v>2295</x:v>
+        <x:v>2292</x:v>
       </x:c>
       <x:c r="H106" s="116" t="s">
-        <x:v>2296</x:v>
+        <x:v>2293</x:v>
       </x:c>
       <x:c r="I106" s="289" t="s">
-        <x:v>2297</x:v>
+        <x:v>2294</x:v>
       </x:c>
       <x:c r="J106" s="61"/>
       <x:c r="K106" s="140"/>
@@ -59332,11 +59313,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G107" s="327" t="s">
-        <x:v>2298</x:v>
+        <x:v>2295</x:v>
       </x:c>
       <x:c r="H107" s="116"/>
       <x:c r="I107" s="289" t="s">
-        <x:v>2299</x:v>
+        <x:v>2296</x:v>
       </x:c>
       <x:c r="J107" s="61"/>
       <x:c r="K107" s="140"/>
@@ -59352,13 +59333,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G108" s="327" t="s">
-        <x:v>2300</x:v>
+        <x:v>2297</x:v>
       </x:c>
       <x:c r="H108" s="116" t="s">
-        <x:v>2301</x:v>
+        <x:v>2298</x:v>
       </x:c>
       <x:c r="I108" s="289" t="s">
-        <x:v>2302</x:v>
+        <x:v>2299</x:v>
       </x:c>
       <x:c r="J108" s="61"/>
       <x:c r="K108" s="140"/>
@@ -59374,11 +59355,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G109" s="327" t="s">
-        <x:v>2303</x:v>
+        <x:v>2300</x:v>
       </x:c>
       <x:c r="H109" s="116"/>
       <x:c r="I109" s="289" t="s">
-        <x:v>2304</x:v>
+        <x:v>2301</x:v>
       </x:c>
       <x:c r="J109" s="61"/>
       <x:c r="K109" s="140"/>
@@ -59398,19 +59379,19 @@
         <x:v>854</x:v>
       </x:c>
       <x:c r="E110" s="116" t="s">
-        <x:v>2305</x:v>
+        <x:v>2302</x:v>
       </x:c>
       <x:c r="F110" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G110" s="327" t="s">
-        <x:v>2306</x:v>
+        <x:v>2303</x:v>
       </x:c>
       <x:c r="H110" s="116" t="s">
-        <x:v>2307</x:v>
+        <x:v>2304</x:v>
       </x:c>
       <x:c r="I110" s="289" t="s">
-        <x:v>2308</x:v>
+        <x:v>2305</x:v>
       </x:c>
       <x:c r="J110" s="61"/>
       <x:c r="K110" s="140"/>
@@ -59426,11 +59407,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G111" s="327" t="s">
-        <x:v>2298</x:v>
+        <x:v>2295</x:v>
       </x:c>
       <x:c r="H111" s="116"/>
       <x:c r="I111" s="289" t="s">
-        <x:v>2309</x:v>
+        <x:v>2306</x:v>
       </x:c>
       <x:c r="J111" s="61"/>
       <x:c r="K111" s="140"/>
@@ -59446,13 +59427,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G112" s="327" t="s">
-        <x:v>2310</x:v>
+        <x:v>2307</x:v>
       </x:c>
       <x:c r="H112" s="116" t="s">
-        <x:v>2311</x:v>
+        <x:v>2308</x:v>
       </x:c>
       <x:c r="I112" s="289" t="s">
-        <x:v>2312</x:v>
+        <x:v>2309</x:v>
       </x:c>
       <x:c r="J112" s="61"/>
       <x:c r="K112" s="140"/>
@@ -59468,11 +59449,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G113" s="327" t="s">
-        <x:v>2313</x:v>
+        <x:v>2310</x:v>
       </x:c>
       <x:c r="H113" s="116"/>
       <x:c r="I113" s="289" t="s">
-        <x:v>2314</x:v>
+        <x:v>2311</x:v>
       </x:c>
       <x:c r="J113" s="61"/>
       <x:c r="K113" s="140"/>
@@ -59489,7 +59470,7 @@
         <x:v>863</x:v>
       </x:c>
       <x:c r="D114" s="140" t="s">
-        <x:v>2315</x:v>
+        <x:v>2312</x:v>
       </x:c>
       <x:c r="E114" s="140" t="s">
         <x:v>865</x:v>
@@ -59498,7 +59479,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G114" s="61" t="s">
-        <x:v>2316</x:v>
+        <x:v>2313</x:v>
       </x:c>
       <x:c r="H114" s="140"/>
       <x:c r="I114" s="61" t="s">
@@ -59518,7 +59499,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G115" s="61" t="s">
-        <x:v>2317</x:v>
+        <x:v>2314</x:v>
       </x:c>
       <x:c r="H115" s="140"/>
       <x:c r="I115" s="61" t="s">
@@ -59538,10 +59519,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G116" s="61" t="s">
-        <x:v>2318</x:v>
+        <x:v>2315</x:v>
       </x:c>
       <x:c r="H116" s="140" t="s">
-        <x:v>2319</x:v>
+        <x:v>2316</x:v>
       </x:c>
       <x:c r="I116" s="61"/>
       <x:c r="J116" s="140"/>
@@ -59558,10 +59539,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G117" s="61" t="s">
-        <x:v>2320</x:v>
+        <x:v>2317</x:v>
       </x:c>
       <x:c r="H117" s="140" t="s">
-        <x:v>2321</x:v>
+        <x:v>2318</x:v>
       </x:c>
       <x:c r="I117" s="61"/>
       <x:c r="J117" s="140"/>
@@ -59596,7 +59577,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G119" s="61" t="s">
-        <x:v>2322</x:v>
+        <x:v>2319</x:v>
       </x:c>
       <x:c r="H119" s="140" t="s">
         <x:v>877</x:v>
@@ -59616,7 +59597,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G120" s="61" t="s">
-        <x:v>2323</x:v>
+        <x:v>2320</x:v>
       </x:c>
       <x:c r="H120" s="251">
         <x:v>0.375</x:v>
@@ -59636,7 +59617,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G121" s="61" t="s">
-        <x:v>2324</x:v>
+        <x:v>2321</x:v>
       </x:c>
       <x:c r="H121" s="140">
         <x:v>100000</x:v>
@@ -59656,7 +59637,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="G122" s="61" t="s">
-        <x:v>2325</x:v>
+        <x:v>2322</x:v>
       </x:c>
       <x:c r="H122" s="140">
         <x:v>1</x:v>
@@ -59676,7 +59657,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G123" s="61" t="s">
-        <x:v>2326</x:v>
+        <x:v>2323</x:v>
       </x:c>
       <x:c r="H123" s="140"/>
       <x:c r="I123" s="61" t="s">
@@ -59697,7 +59678,7 @@
         <x:v>884</x:v>
       </x:c>
       <x:c r="D124" s="140" t="s">
-        <x:v>2327</x:v>
+        <x:v>2324</x:v>
       </x:c>
       <x:c r="E124" s="140" t="s">
         <x:v>886</x:v>
@@ -59706,7 +59687,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G124" s="61" t="s">
-        <x:v>2328</x:v>
+        <x:v>2325</x:v>
       </x:c>
       <x:c r="H124" s="140"/>
       <x:c r="I124" s="140" t="s">
@@ -59726,7 +59707,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G125" s="61" t="s">
-        <x:v>2329</x:v>
+        <x:v>2326</x:v>
       </x:c>
       <x:c r="H125" s="140"/>
       <x:c r="I125" s="140"/>
@@ -59744,10 +59725,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G126" s="61" t="s">
-        <x:v>2330</x:v>
+        <x:v>2327</x:v>
       </x:c>
       <x:c r="H126" s="140" t="s">
-        <x:v>2331</x:v>
+        <x:v>2328</x:v>
       </x:c>
       <x:c r="I126" s="140"/>
       <x:c r="J126" s="140"/>
@@ -59764,10 +59745,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G127" s="61" t="s">
-        <x:v>2332</x:v>
+        <x:v>2329</x:v>
       </x:c>
       <x:c r="H127" s="140" t="s">
-        <x:v>2333</x:v>
+        <x:v>2330</x:v>
       </x:c>
       <x:c r="I127" s="140"/>
       <x:c r="J127" s="140"/>
@@ -59784,7 +59765,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G128" s="61" t="s">
-        <x:v>2334</x:v>
+        <x:v>2331</x:v>
       </x:c>
       <x:c r="H128" s="140" t="s">
         <x:v>877</x:v>
@@ -59822,7 +59803,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G130" s="61" t="s">
-        <x:v>2335</x:v>
+        <x:v>2332</x:v>
       </x:c>
       <x:c r="H130" s="140">
         <x:v>100000</x:v>
@@ -59842,7 +59823,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="G131" s="61" t="s">
-        <x:v>2336</x:v>
+        <x:v>2333</x:v>
       </x:c>
       <x:c r="H131" s="140">
         <x:v>1</x:v>
@@ -59862,7 +59843,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G132" s="61" t="s">
-        <x:v>2337</x:v>
+        <x:v>2334</x:v>
       </x:c>
       <x:c r="H132" s="140"/>
       <x:c r="I132" s="140"/>
@@ -59881,7 +59862,7 @@
         <x:v>900</x:v>
       </x:c>
       <x:c r="D133" s="140" t="s">
-        <x:v>2338</x:v>
+        <x:v>2335</x:v>
       </x:c>
       <x:c r="E133" s="140" t="s">
         <x:v>886</x:v>
@@ -59890,7 +59871,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G133" s="61" t="s">
-        <x:v>2339</x:v>
+        <x:v>2336</x:v>
       </x:c>
       <x:c r="H133" s="140"/>
       <x:c r="I133" s="140" t="s">
@@ -59910,7 +59891,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G134" s="61" t="s">
-        <x:v>2340</x:v>
+        <x:v>2337</x:v>
       </x:c>
       <x:c r="H134" s="140"/>
       <x:c r="I134" s="140"/>
@@ -59928,7 +59909,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G135" s="61" t="s">
-        <x:v>2341</x:v>
+        <x:v>2338</x:v>
       </x:c>
       <x:c r="H135" s="140" t="s">
         <x:v>891</x:v>
@@ -60006,7 +59987,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G139" s="61" t="s">
-        <x:v>2342</x:v>
+        <x:v>2339</x:v>
       </x:c>
       <x:c r="H139" s="140">
         <x:f>1</x:f>
@@ -60026,7 +60007,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G140" s="61" t="s">
-        <x:v>2343</x:v>
+        <x:v>2340</x:v>
       </x:c>
       <x:c r="H140" s="140"/>
       <x:c r="I140" s="140"/>
@@ -60045,7 +60026,7 @@
         <x:v>911</x:v>
       </x:c>
       <x:c r="D141" s="140" t="s">
-        <x:v>2344</x:v>
+        <x:v>2341</x:v>
       </x:c>
       <x:c r="E141" s="140" t="s">
         <x:v>886</x:v>
@@ -60054,7 +60035,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G141" s="61" t="s">
-        <x:v>2345</x:v>
+        <x:v>2342</x:v>
       </x:c>
       <x:c r="H141" s="140"/>
       <x:c r="I141" s="140" t="s">
@@ -60074,7 +60055,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G142" s="61" t="s">
-        <x:v>2346</x:v>
+        <x:v>2343</x:v>
       </x:c>
       <x:c r="H142" s="140"/>
       <x:c r="I142" s="140"/>
@@ -60092,7 +60073,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G143" s="61" t="s">
-        <x:v>2347</x:v>
+        <x:v>2344</x:v>
       </x:c>
       <x:c r="H143" s="140" t="s">
         <x:v>891</x:v>
@@ -60190,7 +60171,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G148" s="61" t="s">
-        <x:v>2348</x:v>
+        <x:v>2345</x:v>
       </x:c>
       <x:c r="H148" s="140"/>
       <x:c r="I148" s="140"/>
@@ -60209,22 +60190,22 @@
         <x:v>921</x:v>
       </x:c>
       <x:c r="D149" s="116" t="s">
-        <x:v>2349</x:v>
+        <x:v>2346</x:v>
       </x:c>
       <x:c r="E149" s="116" t="s">
-        <x:v>2350</x:v>
+        <x:v>2347</x:v>
       </x:c>
       <x:c r="F149" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G149" s="327" t="s">
-        <x:v>2351</x:v>
+        <x:v>2348</x:v>
       </x:c>
       <x:c r="H149" s="116" t="s">
-        <x:v>2352</x:v>
+        <x:v>2349</x:v>
       </x:c>
       <x:c r="I149" s="289" t="s">
-        <x:v>2353</x:v>
+        <x:v>2350</x:v>
       </x:c>
       <x:c r="J149" s="61"/>
       <x:c r="K149" s="140"/>
@@ -60240,11 +60221,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G150" s="327" t="s">
-        <x:v>2354</x:v>
+        <x:v>2351</x:v>
       </x:c>
       <x:c r="H150" s="116"/>
       <x:c r="I150" s="289" t="s">
-        <x:v>2355</x:v>
+        <x:v>2352</x:v>
       </x:c>
       <x:c r="J150" s="61"/>
       <x:c r="K150" s="140"/>
@@ -60260,13 +60241,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G151" s="327" t="s">
-        <x:v>2356</x:v>
+        <x:v>2353</x:v>
       </x:c>
       <x:c r="H151" s="116" t="s">
-        <x:v>2357</x:v>
+        <x:v>2354</x:v>
       </x:c>
       <x:c r="I151" s="289" t="s">
-        <x:v>2358</x:v>
+        <x:v>2355</x:v>
       </x:c>
       <x:c r="J151" s="61"/>
       <x:c r="K151" s="140"/>
@@ -60282,11 +60263,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G152" s="327" t="s">
-        <x:v>2359</x:v>
+        <x:v>2356</x:v>
       </x:c>
       <x:c r="H152" s="116"/>
       <x:c r="I152" s="289" t="s">
-        <x:v>2360</x:v>
+        <x:v>2357</x:v>
       </x:c>
       <x:c r="J152" s="61"/>
       <x:c r="K152" s="140"/>
@@ -60302,11 +60283,11 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G153" s="327" t="s">
-        <x:v>2361</x:v>
+        <x:v>2358</x:v>
       </x:c>
       <x:c r="H153" s="116"/>
       <x:c r="I153" s="289" t="s">
-        <x:v>2362</x:v>
+        <x:v>2359</x:v>
       </x:c>
       <x:c r="J153" s="61"/>
       <x:c r="K153" s="140"/>
@@ -60643,17 +60624,17 @@
     <x:mergeCell ref="L149:L153"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H49" r:id="rId155"/>
-    <x:hyperlink ref="H50" r:id="rId156"/>
-    <x:hyperlink ref="H55" r:id="rId157"/>
-    <x:hyperlink ref="H56" r:id="rId158"/>
-    <x:hyperlink ref="H59" r:id="rId159"/>
-    <x:hyperlink ref="H64" r:id="rId160"/>
-    <x:hyperlink ref="H65" r:id="rId161"/>
-    <x:hyperlink ref="H67" r:id="rId162"/>
-    <x:hyperlink ref="H68" r:id="rId163"/>
-    <x:hyperlink ref="H52" r:id="rId164"/>
-    <x:hyperlink ref="H61" r:id="rId165"/>
+    <x:hyperlink ref="H49" r:id="rId197"/>
+    <x:hyperlink ref="H50" r:id="rId198"/>
+    <x:hyperlink ref="H55" r:id="rId199"/>
+    <x:hyperlink ref="H56" r:id="rId200"/>
+    <x:hyperlink ref="H59" r:id="rId201"/>
+    <x:hyperlink ref="H64" r:id="rId202"/>
+    <x:hyperlink ref="H65" r:id="rId203"/>
+    <x:hyperlink ref="H67" r:id="rId204"/>
+    <x:hyperlink ref="H68" r:id="rId205"/>
+    <x:hyperlink ref="H52" r:id="rId206"/>
+    <x:hyperlink ref="H61" r:id="rId207"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -60747,7 +60728,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H2" s="340" t="s">
-        <x:v>2363</x:v>
+        <x:v>2360</x:v>
       </x:c>
       <x:c r="I2" s="51" t="s">
         <x:v>1102</x:v>
@@ -60986,7 +60967,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G14" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H14" s="292"/>
       <x:c r="I14" s="51"/>
@@ -61256,7 +61237,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G27" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H27" s="292"/>
       <x:c r="I27" s="51"/>
@@ -61287,7 +61268,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H28" s="340" t="s">
-        <x:v>2365</x:v>
+        <x:v>2362</x:v>
       </x:c>
       <x:c r="I28" s="51" t="s">
         <x:v>1127</x:v>
@@ -61526,7 +61507,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G40" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H40" s="292"/>
       <x:c r="I40" s="51"/>
@@ -61557,7 +61538,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H41" s="340" t="s">
-        <x:v>2366</x:v>
+        <x:v>2363</x:v>
       </x:c>
       <x:c r="I41" s="51" t="s">
         <x:v>1130</x:v>
@@ -61796,7 +61777,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G53" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H53" s="292"/>
       <x:c r="I53" s="51"/>
@@ -61827,7 +61808,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H54" s="340" t="s">
-        <x:v>2367</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="I54" s="51" t="s">
         <x:v>1134</x:v>
@@ -62066,7 +62047,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G66" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H66" s="292"/>
       <x:c r="I66" s="51"/>
@@ -62097,7 +62078,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H67" s="340" t="s">
-        <x:v>2368</x:v>
+        <x:v>2365</x:v>
       </x:c>
       <x:c r="I67" s="51" t="s">
         <x:v>1138</x:v>
@@ -62336,7 +62317,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G79" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H79" s="292"/>
       <x:c r="I79" s="51"/>
@@ -62367,7 +62348,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H80" s="340" t="s">
-        <x:v>2369</x:v>
+        <x:v>2366</x:v>
       </x:c>
       <x:c r="I80" s="51" t="s">
         <x:v>1141</x:v>
@@ -62606,7 +62587,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G92" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H92" s="292"/>
       <x:c r="I92" s="51"/>
@@ -62637,7 +62618,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H93" s="340" t="s">
-        <x:v>2370</x:v>
+        <x:v>2367</x:v>
       </x:c>
       <x:c r="I93" s="51" t="s">
         <x:v>1145</x:v>
@@ -62876,7 +62857,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G105" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H105" s="292"/>
       <x:c r="I105" s="51"/>
@@ -62907,7 +62888,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H106" s="340" t="s">
-        <x:v>2370</x:v>
+        <x:v>2367</x:v>
       </x:c>
       <x:c r="I106" s="51" t="s">
         <x:v>1149</x:v>
@@ -63146,7 +63127,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G118" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H118" s="292"/>
       <x:c r="I118" s="51"/>
@@ -63177,7 +63158,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H119" s="340" t="s">
-        <x:v>2371</x:v>
+        <x:v>2368</x:v>
       </x:c>
       <x:c r="I119" s="51" t="s">
         <x:v>1149</x:v>
@@ -63416,7 +63397,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G131" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H131" s="292"/>
       <x:c r="I131" s="51"/>
@@ -63447,7 +63428,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H132" s="340" t="s">
-        <x:v>2372</x:v>
+        <x:v>2369</x:v>
       </x:c>
       <x:c r="I132" s="51" t="s">
         <x:v>1160</x:v>
@@ -63686,7 +63667,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G144" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H144" s="292"/>
       <x:c r="I144" s="51"/>
@@ -63717,7 +63698,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H145" s="340" t="s">
-        <x:v>2373</x:v>
+        <x:v>2370</x:v>
       </x:c>
       <x:c r="I145" s="51" t="s">
         <x:v>1160</x:v>
@@ -63956,7 +63937,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G157" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H157" s="292"/>
       <x:c r="I157" s="51"/>
@@ -63987,7 +63968,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H158" s="340" t="s">
-        <x:v>2374</x:v>
+        <x:v>2371</x:v>
       </x:c>
       <x:c r="I158" s="51" t="s">
         <x:v>1160</x:v>
@@ -64226,7 +64207,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G170" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H170" s="292"/>
       <x:c r="I170" s="51"/>
@@ -64257,7 +64238,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H171" s="340" t="s">
-        <x:v>2375</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="I171" s="51" t="s">
         <x:v>1160</x:v>
@@ -64496,7 +64477,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G183" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H183" s="292"/>
       <x:c r="I183" s="51"/>
@@ -64766,7 +64747,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G196" s="292" t="s">
-        <x:v>2364</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H196" s="340"/>
       <x:c r="I196" s="51"/>
@@ -64797,7 +64778,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H197" s="340" t="s">
-        <x:v>2376</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="I197" s="134" t="s">
         <x:v>1178</x:v>
@@ -65067,7 +65048,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H210" s="340" t="s">
-        <x:v>2377</x:v>
+        <x:v>2374</x:v>
       </x:c>
       <x:c r="I210" s="134" t="s">
         <x:v>1187</x:v>
@@ -65325,7 +65306,7 @@
         <x:v>1189</x:v>
       </x:c>
       <x:c r="D223" s="134" t="s">
-        <x:v>2378</x:v>
+        <x:v>2375</x:v>
       </x:c>
       <x:c r="E223" s="35" t="s">
         <x:v>1176</x:v>
@@ -65337,7 +65318,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H223" s="340" t="s">
-        <x:v>2379</x:v>
+        <x:v>2376</x:v>
       </x:c>
       <x:c r="I223" s="10" t="s">
         <x:v>1192</x:v>
@@ -65607,7 +65588,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H236" s="340" t="s">
-        <x:v>2380</x:v>
+        <x:v>2377</x:v>
       </x:c>
       <x:c r="I236" s="10" t="s">
         <x:v>1197</x:v>
@@ -65877,7 +65858,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H249" s="340" t="s">
-        <x:v>2381</x:v>
+        <x:v>2378</x:v>
       </x:c>
       <x:c r="I249" s="10" t="s">
         <x:v>1203</x:v>
@@ -66059,7 +66040,7 @@
         <x:v>1115</x:v>
       </x:c>
       <x:c r="H258" s="292" t="s">
-        <x:v>2382</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="I258" s="9"/>
       <x:c r="J258" s="9"/>
@@ -66405,7 +66386,7 @@
         <x:v>1212</x:v>
       </x:c>
       <x:c r="D275" s="35" t="s">
-        <x:v>2383</x:v>
+        <x:v>2380</x:v>
       </x:c>
       <x:c r="E275" s="35" t="s">
         <x:v>1214</x:v>
@@ -66414,10 +66395,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G275" s="297" t="s">
-        <x:v>2384</x:v>
+        <x:v>2381</x:v>
       </x:c>
       <x:c r="I275" s="10" t="s">
-        <x:v>2385</x:v>
+        <x:v>2382</x:v>
       </x:c>
       <x:c r="J275" s="10"/>
       <x:c r="K275" s="35"/>
@@ -66433,7 +66414,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G276" s="297" t="s">
-        <x:v>2386</x:v>
+        <x:v>2383</x:v>
       </x:c>
       <x:c r="I276" s="9"/>
       <x:c r="J276" s="9"/>
@@ -66450,10 +66431,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G277" s="297" t="s">
-        <x:v>2387</x:v>
+        <x:v>2384</x:v>
       </x:c>
       <x:c r="H277" s="297" t="s">
-        <x:v>2388</x:v>
+        <x:v>2385</x:v>
       </x:c>
       <x:c r="I277" s="9"/>
       <x:c r="J277" s="9"/>
@@ -66492,13 +66473,13 @@
         <x:v>1220</x:v>
       </x:c>
       <x:c r="E279" s="35" t="s">
-        <x:v>2389</x:v>
+        <x:v>2386</x:v>
       </x:c>
       <x:c r="F279" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G279" s="297" t="s">
-        <x:v>2384</x:v>
+        <x:v>2381</x:v>
       </x:c>
       <x:c r="I279" s="10" t="s">
         <x:v>1223</x:v>
@@ -66517,7 +66498,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G280" s="297" t="s">
-        <x:v>2390</x:v>
+        <x:v>2387</x:v>
       </x:c>
       <x:c r="H280" s="297" t="s">
         <x:v>1117</x:v>
@@ -66559,17 +66540,17 @@
         <x:v>1226</x:v>
       </x:c>
       <x:c r="E282" s="35" t="s">
-        <x:v>2391</x:v>
+        <x:v>2388</x:v>
       </x:c>
       <x:c r="F282" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G282" s="297" t="s">
-        <x:v>2384</x:v>
+        <x:v>2381</x:v>
       </x:c>
       <x:c r="H282" s="297"/>
       <x:c r="I282" s="10" t="s">
-        <x:v>2392</x:v>
+        <x:v>2389</x:v>
       </x:c>
       <x:c r="J282" s="10"/>
       <x:c r="K282" s="35"/>
@@ -66585,7 +66566,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G283" s="297" t="s">
-        <x:v>2386</x:v>
+        <x:v>2383</x:v>
       </x:c>
       <x:c r="H283" s="297"/>
       <x:c r="I283" s="9"/>
@@ -66603,10 +66584,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G284" s="297" t="s">
-        <x:v>2393</x:v>
+        <x:v>2390</x:v>
       </x:c>
       <x:c r="H284" s="323" t="s">
-        <x:v>2394</x:v>
+        <x:v>2391</x:v>
       </x:c>
       <x:c r="I284" s="9"/>
       <x:c r="J284" s="9"/>
@@ -66645,17 +66626,17 @@
         <x:v>1233</x:v>
       </x:c>
       <x:c r="E286" s="35" t="s">
-        <x:v>2391</x:v>
+        <x:v>2388</x:v>
       </x:c>
       <x:c r="F286" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G286" s="297" t="s">
-        <x:v>2384</x:v>
+        <x:v>2381</x:v>
       </x:c>
       <x:c r="H286" s="297"/>
       <x:c r="I286" s="10" t="s">
-        <x:v>2392</x:v>
+        <x:v>2389</x:v>
       </x:c>
       <x:c r="J286" s="10"/>
       <x:c r="K286" s="35"/>
@@ -66671,7 +66652,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G287" s="297" t="s">
-        <x:v>2386</x:v>
+        <x:v>2383</x:v>
       </x:c>
       <x:c r="H287" s="297"/>
       <x:c r="I287" s="9"/>
@@ -66689,10 +66670,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G288" s="297" t="s">
-        <x:v>2395</x:v>
+        <x:v>2392</x:v>
       </x:c>
       <x:c r="H288" s="297" t="s">
-        <x:v>2396</x:v>
+        <x:v>2393</x:v>
       </x:c>
       <x:c r="I288" s="9"/>
       <x:c r="J288" s="9"/>
@@ -66740,7 +66721,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H290" s="340" t="s">
-        <x:v>2397</x:v>
+        <x:v>2394</x:v>
       </x:c>
       <x:c r="I290" s="51" t="s">
         <x:v>1102</x:v>
@@ -66819,7 +66800,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G294" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H294" s="312" t="s">
         <x:v>1117</x:v>
@@ -66839,7 +66820,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G295" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H295" s="312">
         <x:v>45758</x:v>
@@ -66959,7 +66940,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G301" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="H301" s="297"/>
       <x:c r="I301" s="51"/>
@@ -67069,7 +67050,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G306" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H306" s="312" t="s">
         <x:v>1117</x:v>
@@ -67089,7 +67070,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G307" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H307" s="312">
         <x:v>45758</x:v>
@@ -67209,7 +67190,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G313" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I313" s="51"/>
       <x:c r="J313" s="48"/>
@@ -67239,7 +67220,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H314" s="340" t="s">
-        <x:v>2401</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="I314" s="51" t="s">
         <x:v>1127</x:v>
@@ -67316,7 +67297,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G318" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H318" s="312" t="s">
         <x:v>1117</x:v>
@@ -67336,7 +67317,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G319" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H319" s="312">
         <x:v>45758</x:v>
@@ -67456,7 +67437,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G325" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I325" s="51"/>
       <x:c r="J325" s="48"/>
@@ -67486,7 +67467,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H326" s="340" t="s">
-        <x:v>2402</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="I326" s="51" t="s">
         <x:v>1130</x:v>
@@ -67563,7 +67544,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G330" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H330" s="312" t="s">
         <x:v>1117</x:v>
@@ -67583,7 +67564,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G331" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H331" s="312">
         <x:v>45758</x:v>
@@ -67703,7 +67684,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G337" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I337" s="51"/>
       <x:c r="J337" s="48"/>
@@ -67733,7 +67714,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H338" s="340" t="s">
-        <x:v>2403</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I338" s="51" t="s">
         <x:v>1134</x:v>
@@ -67812,7 +67793,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G342" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H342" s="312"/>
       <x:c r="I342" s="51"/>
@@ -67830,7 +67811,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G343" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H343" s="312">
         <x:v>45758</x:v>
@@ -67950,7 +67931,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G349" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I349" s="51"/>
       <x:c r="J349" s="48"/>
@@ -67980,7 +67961,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H350" s="340" t="s">
-        <x:v>2403</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="I350" s="51" t="s">
         <x:v>1138</x:v>
@@ -68059,7 +68040,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G354" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H354" s="312" t="s">
         <x:v>1117</x:v>
@@ -68079,7 +68060,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G355" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H355" s="312"/>
       <x:c r="I355" s="51"/>
@@ -68197,7 +68178,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G361" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I361" s="51"/>
       <x:c r="J361" s="48"/>
@@ -68215,7 +68196,7 @@
         <x:v>1254</x:v>
       </x:c>
       <x:c r="D362" s="51" t="s">
-        <x:v>2404</x:v>
+        <x:v>2401</x:v>
       </x:c>
       <x:c r="E362" s="51" t="s">
         <x:v>1099</x:v>
@@ -68227,10 +68208,10 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H362" s="340" t="s">
-        <x:v>2405</x:v>
+        <x:v>2402</x:v>
       </x:c>
       <x:c r="I362" s="51" t="s">
-        <x:v>2406</x:v>
+        <x:v>2403</x:v>
       </x:c>
       <x:c r="J362" s="50"/>
       <x:c r="K362" s="51"/>
@@ -68304,7 +68285,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G366" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H366" s="312" t="s">
         <x:v>1117</x:v>
@@ -68324,7 +68305,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G367" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H367" s="312">
         <x:v>49410</x:v>
@@ -68442,7 +68423,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G373" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="H373" s="292"/>
       <x:c r="I373" s="51"/>
@@ -68473,7 +68454,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H374" s="340" t="s">
-        <x:v>2407</x:v>
+        <x:v>2404</x:v>
       </x:c>
       <x:c r="I374" s="51" t="s">
         <x:v>1145</x:v>
@@ -68552,7 +68533,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G378" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H378" s="312" t="s">
         <x:v>1117</x:v>
@@ -68572,7 +68553,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G379" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H379" s="312">
         <x:v>45758</x:v>
@@ -68690,7 +68671,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G385" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I385" s="51"/>
       <x:c r="J385" s="48"/>
@@ -68720,7 +68701,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H386" s="340" t="s">
-        <x:v>2408</x:v>
+        <x:v>2405</x:v>
       </x:c>
       <x:c r="I386" s="51" t="s">
         <x:v>1149</x:v>
@@ -68799,7 +68780,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G390" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H390" s="312" t="s">
         <x:v>1117</x:v>
@@ -68819,7 +68800,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G391" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H391" s="312">
         <x:v>45758</x:v>
@@ -68937,7 +68918,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G397" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I397" s="51"/>
       <x:c r="J397" s="48"/>
@@ -68967,7 +68948,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H398" s="340" t="s">
-        <x:v>2409</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="I398" s="51" t="s">
         <x:v>1149</x:v>
@@ -69044,7 +69025,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G402" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H402" s="312" t="s">
         <x:v>1117</x:v>
@@ -69064,7 +69045,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G403" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H403" s="312">
         <x:v>45758</x:v>
@@ -69184,7 +69165,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G409" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I409" s="51"/>
       <x:c r="J409" s="48"/>
@@ -69214,7 +69195,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H410" s="340" t="s">
-        <x:v>2410</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="I410" s="51" t="s">
         <x:v>1160</x:v>
@@ -69293,7 +69274,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G414" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H414" s="312" t="s">
         <x:v>1117</x:v>
@@ -69313,7 +69294,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G415" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H415" s="312">
         <x:v>45758</x:v>
@@ -69431,7 +69412,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G421" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I421" s="51"/>
       <x:c r="J421" s="48"/>
@@ -69449,7 +69430,7 @@
         <x:v>1260</x:v>
       </x:c>
       <x:c r="D422" s="51" t="s">
-        <x:v>2411</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="E422" s="51" t="s">
         <x:v>1099</x:v>
@@ -69461,10 +69442,10 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H422" s="340" t="s">
-        <x:v>2412</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I422" s="51" t="s">
-        <x:v>2413</x:v>
+        <x:v>2410</x:v>
       </x:c>
       <x:c r="J422" s="50"/>
       <x:c r="K422" s="51"/>
@@ -69540,7 +69521,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G426" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H426" s="312" t="s">
         <x:v>1117</x:v>
@@ -69560,7 +69541,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G427" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H427" s="312">
         <x:v>45758</x:v>
@@ -69680,7 +69661,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G433" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I433" s="51"/>
       <x:c r="J433" s="48"/>
@@ -69710,7 +69691,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H434" s="340" t="s">
-        <x:v>2414</x:v>
+        <x:v>2411</x:v>
       </x:c>
       <x:c r="I434" s="51" t="s">
         <x:v>1160</x:v>
@@ -69789,7 +69770,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G438" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H438" s="312" t="s">
         <x:v>1117</x:v>
@@ -69809,7 +69790,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G439" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H439" s="312">
         <x:v>45758</x:v>
@@ -69927,7 +69908,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G445" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I445" s="51"/>
       <x:c r="J445" s="48"/>
@@ -69957,7 +69938,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H446" s="340" t="s">
-        <x:v>2415</x:v>
+        <x:v>2412</x:v>
       </x:c>
       <x:c r="I446" s="51" t="s">
         <x:v>1160</x:v>
@@ -70036,7 +70017,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G450" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H450" s="312" t="s">
         <x:v>1117</x:v>
@@ -70056,7 +70037,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G451" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H451" s="312">
         <x:v>45758</x:v>
@@ -70174,7 +70155,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G457" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I457" s="51"/>
       <x:c r="J457" s="48"/>
@@ -70283,7 +70264,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G462" s="292" t="s">
-        <x:v>2398</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H462" s="340" t="s">
         <x:v>437</x:v>
@@ -70303,7 +70284,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G463" s="292" t="s">
-        <x:v>2399</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H463" s="340" t="s">
         <x:v>437</x:v>
@@ -70423,7 +70404,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G469" s="288" t="s">
-        <x:v>2400</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="H469" s="340" t="s">
         <x:v>437</x:v>
@@ -70757,7 +70738,7 @@
     <x:mergeCell ref="K458:K469"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H284" r:id="rId166"/>
+    <x:hyperlink ref="H284" r:id="rId208"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -70781,13 +70762,13 @@
   <x:sheetData>
     <x:row r="2" spans="1:7">
       <x:c r="A2" s="196" t="s">
-        <x:v>2416</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="D2" s="196" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="G2" s="196" t="s">
-        <x:v>2417</x:v>
+        <x:v>2414</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
@@ -70795,7 +70776,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>2418</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
         <x:v>244</x:v>
@@ -70806,7 +70787,7 @@
         <x:v>245</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>2419</x:v>
+        <x:v>2416</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
         <x:v>234</x:v>
@@ -70814,10 +70795,10 @@
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="A5" s="0" t="s">
-        <x:v>2420</x:v>
+        <x:v>2417</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>2421</x:v>
+        <x:v>2418</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
         <x:v>239</x:v>

</xml_diff>

<commit_message>
Test: Optimizing dynamic data generation and Admin check flow for TC_REG_01 to TC_REG_06
</commit_message>
<xml_diff>
--- a/sqa-testing-report/Data/DataTest.xlsx
+++ b/sqa-testing-report/Data/DataTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\sqa-testing-report\sqa-testing-report\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB4F84E-53EB-4513-AFFB-0ED1A466C8C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B3991C-E6A1-4458-8027-922AF348F1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
     <x:workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="664" firstSheet="0" activeTab="3" xr2:uid="{DC4DB269-603C-4B5B-A498-B166C8A18B92}"/>
   </x:bookViews>
@@ -7692,6 +7692,9 @@
     <x:t>Screenshots</x:t>
   </x:si>
   <x:si>
+    <x:t>hệ thống báo Đăng ký thành công</x:t>
+  </x:si>
+  <x:si>
     <x:t>Hệ thống báo: Đăng ký thành công!</x:t>
   </x:si>
   <x:si>
@@ -7713,10 +7716,8 @@
     <x:t>Hệ thống báo lỗi mật khẩu không đúng định dạng thành công.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Lỗi:   Lỗi thực tế: Đăng ký thành công!
-  Expected: True
-  But was:  False
-</x:t>
+    <x:t>Lỗi: invalid argument: No dialog is showing
+  (Session info: chrome=146.0.7680.165)</x:t>
   </x:si>
   <x:si>
     <x:t>Fail</x:t>
@@ -11771,7 +11772,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="398">
+  <x:cellXfs count="399">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -12779,6 +12780,9 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="2" borderId="31" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -13320,31 +13324,31 @@
   <x:sheetData>
     <x:row r="1" spans="1:5" ht="10.5" customHeight="1"/>
     <x:row r="2" spans="1:5" ht="35.25" customHeight="1">
-      <x:c r="B2" s="347" t="s">
+      <x:c r="B2" s="348" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C2" s="347"/>
-      <x:c r="D2" s="347"/>
-      <x:c r="E2" s="347"/>
+      <x:c r="C2" s="348"/>
+      <x:c r="D2" s="348"/>
+      <x:c r="E2" s="348"/>
     </x:row>
     <x:row r="3" spans="1:5" ht="31.5" customHeight="1">
-      <x:c r="B3" s="348" t="s">
+      <x:c r="B3" s="349" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C3" s="348"/>
-      <x:c r="D3" s="348"/>
-      <x:c r="E3" s="348"/>
+      <x:c r="C3" s="349"/>
+      <x:c r="D3" s="349"/>
+      <x:c r="E3" s="349"/>
     </x:row>
     <x:row r="4" spans="1:5" ht="18.75" customHeight="1">
       <x:c r="B4" s="184"/>
     </x:row>
     <x:row r="5" spans="1:5" ht="23.25" customHeight="1">
-      <x:c r="B5" s="349" t="s">
+      <x:c r="B5" s="350" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C5" s="350"/>
-      <x:c r="D5" s="350"/>
-      <x:c r="E5" s="351"/>
+      <x:c r="C5" s="351"/>
+      <x:c r="D5" s="351"/>
+      <x:c r="E5" s="352"/>
     </x:row>
     <x:row r="6" spans="1:5" ht="18.75" customHeight="1">
       <x:c r="B6" s="190" t="s">
@@ -13391,32 +13395,32 @@
       <x:c r="E11" s="186"/>
     </x:row>
     <x:row r="12" spans="1:5" ht="18.75" customHeight="1">
-      <x:c r="B12" s="352" t="s">
+      <x:c r="B12" s="353" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C12" s="353"/>
-      <x:c r="D12" s="353"/>
-      <x:c r="E12" s="354"/>
+      <x:c r="C12" s="354"/>
+      <x:c r="D12" s="354"/>
+      <x:c r="E12" s="355"/>
     </x:row>
     <x:row r="14" spans="1:5" ht="18.75" customHeight="1">
-      <x:c r="B14" s="349" t="s">
+      <x:c r="B14" s="350" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="C14" s="350"/>
-      <x:c r="D14" s="350"/>
-      <x:c r="E14" s="351"/>
+      <x:c r="C14" s="351"/>
+      <x:c r="D14" s="351"/>
+      <x:c r="E14" s="352"/>
     </x:row>
     <x:row r="15" spans="1:5" ht="18.75" customHeight="1">
-      <x:c r="B15" s="355" t="s">
+      <x:c r="B15" s="356" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C15" s="356" t="s">
+      <x:c r="C15" s="357" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D15" s="357" t="s">
+      <x:c r="D15" s="358" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E15" s="358"/>
+      <x:c r="E15" s="359"/>
     </x:row>
     <x:row r="16" spans="1:5" ht="18.75" customHeight="1">
       <x:c r="B16" s="187" t="s">
@@ -13447,10 +13451,10 @@
       <x:c r="E19" s="98"/>
     </x:row>
     <x:row r="20" spans="1:5" ht="18.75" customHeight="1">
-      <x:c r="B20" s="352"/>
-      <x:c r="C20" s="353"/>
-      <x:c r="D20" s="353"/>
-      <x:c r="E20" s="354"/>
+      <x:c r="B20" s="353"/>
+      <x:c r="C20" s="354"/>
+      <x:c r="D20" s="354"/>
+      <x:c r="E20" s="355"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells count="11">
@@ -13511,16 +13515,16 @@
       <x:c r="J1" s="97"/>
     </x:row>
     <x:row r="2" spans="1:11" ht="14.4" customHeight="1">
-      <x:c r="A2" s="359" t="s">
+      <x:c r="A2" s="360" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B2" s="360"/>
+      <x:c r="B2" s="361"/>
       <x:c r="C2" s="94" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="D2" s="93"/>
       <x:c r="E2" s="92"/>
-      <x:c r="F2" s="361" t="s">
+      <x:c r="F2" s="362" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="G2" s="94" t="s">
@@ -13531,14 +13535,14 @@
       <x:c r="J2" s="91"/>
     </x:row>
     <x:row r="3" spans="1:11" ht="14.4" customHeight="1">
-      <x:c r="A3" s="362" t="s">
+      <x:c r="A3" s="363" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B3" s="363"/>
+      <x:c r="B3" s="364"/>
       <x:c r="C3" s="88"/>
       <x:c r="D3" s="87"/>
       <x:c r="E3" s="86"/>
-      <x:c r="F3" s="364" t="s">
+      <x:c r="F3" s="365" t="s">
         <x:v>18</x:v>
       </x:c>
       <x:c r="G3" s="88"/>
@@ -13547,14 +13551,14 @@
       <x:c r="J3" s="85"/>
     </x:row>
     <x:row r="4" spans="1:11" ht="15" customHeight="1">
-      <x:c r="A4" s="365" t="s">
+      <x:c r="A4" s="366" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B4" s="366"/>
+      <x:c r="B4" s="367"/>
       <x:c r="C4" s="82"/>
       <x:c r="D4" s="81"/>
       <x:c r="E4" s="80"/>
-      <x:c r="F4" s="367" t="s">
+      <x:c r="F4" s="368" t="s">
         <x:v>20</x:v>
       </x:c>
       <x:c r="G4" s="79" t="s">
@@ -13579,50 +13583,50 @@
       <x:c r="J7" s="77"/>
     </x:row>
     <x:row r="8" spans="1:11" ht="28.2" customHeight="1">
-      <x:c r="A8" s="368" t="s">
+      <x:c r="A8" s="369" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B8" s="369" t="s">
+      <x:c r="B8" s="370" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="C8" s="369" t="s">
+      <x:c r="C8" s="370" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="D8" s="369" t="s">
+      <x:c r="D8" s="370" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="E8" s="369" t="s">
+      <x:c r="E8" s="370" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="F8" s="369" t="s">
+      <x:c r="F8" s="370" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="G8" s="369" t="s">
+      <x:c r="G8" s="370" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="H8" s="370" t="s">
+      <x:c r="H8" s="371" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="I8" s="370" t="s">
+      <x:c r="I8" s="371" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="J8" s="371" t="s">
+      <x:c r="J8" s="372" t="s">
         <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:11" ht="14.4" customHeight="1">
-      <x:c r="A9" s="372" t="s">
+      <x:c r="A9" s="373" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B9" s="373"/>
-      <x:c r="C9" s="373"/>
-      <x:c r="D9" s="373"/>
-      <x:c r="E9" s="373"/>
-      <x:c r="F9" s="373"/>
-      <x:c r="G9" s="373"/>
-      <x:c r="H9" s="373"/>
-      <x:c r="I9" s="373"/>
-      <x:c r="J9" s="374"/>
+      <x:c r="B9" s="374"/>
+      <x:c r="C9" s="374"/>
+      <x:c r="D9" s="374"/>
+      <x:c r="E9" s="374"/>
+      <x:c r="F9" s="374"/>
+      <x:c r="G9" s="374"/>
+      <x:c r="H9" s="374"/>
+      <x:c r="I9" s="374"/>
+      <x:c r="J9" s="375"/>
     </x:row>
     <x:row r="10" spans="1:11" ht="16.8" customHeight="1">
       <x:c r="A10" s="260">
@@ -14913,18 +14917,18 @@
       <x:c r="J55" s="267"/>
     </x:row>
     <x:row r="56" spans="1:11" ht="14.25" customHeight="1">
-      <x:c r="A56" s="375" t="s">
+      <x:c r="A56" s="376" t="s">
         <x:v>224</x:v>
       </x:c>
-      <x:c r="B56" s="376"/>
-      <x:c r="C56" s="376"/>
-      <x:c r="D56" s="376"/>
-      <x:c r="E56" s="376"/>
-      <x:c r="F56" s="376"/>
-      <x:c r="G56" s="376"/>
-      <x:c r="H56" s="376"/>
-      <x:c r="I56" s="376"/>
-      <x:c r="J56" s="377"/>
+      <x:c r="B56" s="377"/>
+      <x:c r="C56" s="377"/>
+      <x:c r="D56" s="377"/>
+      <x:c r="E56" s="377"/>
+      <x:c r="F56" s="377"/>
+      <x:c r="G56" s="377"/>
+      <x:c r="H56" s="377"/>
+      <x:c r="I56" s="377"/>
+      <x:c r="J56" s="378"/>
     </x:row>
     <x:row r="57" spans="1:11" ht="16.8" customHeight="1">
       <x:c r="A57" s="221">
@@ -16180,19 +16184,19 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:14" ht="25.2" customHeight="1">
-      <x:c r="A1" s="378" t="s">
+      <x:c r="A1" s="379" t="s">
         <x:v>402</x:v>
       </x:c>
-      <x:c r="B1" s="378"/>
-      <x:c r="C1" s="378"/>
-      <x:c r="D1" s="378"/>
-      <x:c r="E1" s="378"/>
-      <x:c r="F1" s="378"/>
-      <x:c r="G1" s="378"/>
-      <x:c r="H1" s="378"/>
-      <x:c r="I1" s="378"/>
-      <x:c r="J1" s="378"/>
-      <x:c r="K1" s="378"/>
+      <x:c r="B1" s="379"/>
+      <x:c r="C1" s="379"/>
+      <x:c r="D1" s="379"/>
+      <x:c r="E1" s="379"/>
+      <x:c r="F1" s="379"/>
+      <x:c r="G1" s="379"/>
+      <x:c r="H1" s="379"/>
+      <x:c r="I1" s="379"/>
+      <x:c r="J1" s="379"/>
+      <x:c r="K1" s="379"/>
     </x:row>
     <x:row r="2" spans="1:14" ht="13.8" customHeight="1">
       <x:c r="C2" s="236"/>
@@ -16201,37 +16205,37 @@
       <x:c r="F2" s="236"/>
     </x:row>
     <x:row r="3" spans="1:14" ht="28.2" customHeight="1">
-      <x:c r="A3" s="379" t="s">
+      <x:c r="A3" s="380" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B3" s="380" t="s">
+      <x:c r="B3" s="381" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="C3" s="381" t="s">
+      <x:c r="C3" s="382" t="s">
         <x:v>403</x:v>
       </x:c>
-      <x:c r="D3" s="381" t="s">
+      <x:c r="D3" s="382" t="s">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="E3" s="381" t="s">
+      <x:c r="E3" s="382" t="s">
         <x:v>405</x:v>
       </x:c>
-      <x:c r="F3" s="382" t="s">
+      <x:c r="F3" s="383" t="s">
         <x:v>406</x:v>
       </x:c>
-      <x:c r="G3" s="381" t="s">
+      <x:c r="G3" s="382" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="H3" s="381" t="s">
+      <x:c r="H3" s="382" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="I3" s="381" t="s">
+      <x:c r="I3" s="382" t="s">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="J3" s="383" t="s">
+      <x:c r="J3" s="384" t="s">
         <x:v>410</x:v>
       </x:c>
-      <x:c r="K3" s="384" t="s">
+      <x:c r="K3" s="385" t="s">
         <x:v>411</x:v>
       </x:c>
       <x:c r="L3" s="253"/>
@@ -16239,37 +16243,37 @@
       <x:c r="N3" s="253"/>
     </x:row>
     <x:row r="4" spans="1:14" ht="14.4" customHeight="1">
-      <x:c r="A4" s="385" t="s">
+      <x:c r="A4" s="386" t="s">
         <x:v>412</x:v>
       </x:c>
-      <x:c r="B4" s="385"/>
-      <x:c r="C4" s="385"/>
-      <x:c r="D4" s="385"/>
-      <x:c r="E4" s="385"/>
-      <x:c r="F4" s="385"/>
-      <x:c r="G4" s="385"/>
-      <x:c r="H4" s="385"/>
-      <x:c r="I4" s="385"/>
-      <x:c r="J4" s="385"/>
-      <x:c r="K4" s="385"/>
+      <x:c r="B4" s="386"/>
+      <x:c r="C4" s="386"/>
+      <x:c r="D4" s="386"/>
+      <x:c r="E4" s="386"/>
+      <x:c r="F4" s="386"/>
+      <x:c r="G4" s="386"/>
+      <x:c r="H4" s="386"/>
+      <x:c r="I4" s="386"/>
+      <x:c r="J4" s="386"/>
+      <x:c r="K4" s="386"/>
       <x:c r="L4" s="253"/>
       <x:c r="M4" s="253"/>
       <x:c r="N4" s="253"/>
     </x:row>
     <x:row r="5" spans="1:14" ht="14.4" customHeight="1">
-      <x:c r="A5" s="386" t="s">
+      <x:c r="A5" s="387" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B5" s="386"/>
-      <x:c r="C5" s="386"/>
-      <x:c r="D5" s="386"/>
-      <x:c r="E5" s="386"/>
-      <x:c r="F5" s="386"/>
-      <x:c r="G5" s="386"/>
-      <x:c r="H5" s="386"/>
-      <x:c r="I5" s="386"/>
-      <x:c r="J5" s="386"/>
-      <x:c r="K5" s="386"/>
+      <x:c r="B5" s="387"/>
+      <x:c r="C5" s="387"/>
+      <x:c r="D5" s="387"/>
+      <x:c r="E5" s="387"/>
+      <x:c r="F5" s="387"/>
+      <x:c r="G5" s="387"/>
+      <x:c r="H5" s="387"/>
+      <x:c r="I5" s="387"/>
+      <x:c r="J5" s="387"/>
+      <x:c r="K5" s="387"/>
       <x:c r="L5" s="253"/>
       <x:c r="M5" s="253"/>
       <x:c r="N5" s="253"/>
@@ -24493,19 +24497,19 @@
       <x:c r="N319" s="253"/>
     </x:row>
     <x:row r="320" spans="1:14" ht="14.4" customHeight="1">
-      <x:c r="A320" s="387" t="s">
+      <x:c r="A320" s="388" t="s">
         <x:v>224</x:v>
       </x:c>
-      <x:c r="B320" s="388"/>
-      <x:c r="C320" s="388"/>
-      <x:c r="D320" s="388"/>
-      <x:c r="E320" s="388"/>
-      <x:c r="F320" s="388"/>
-      <x:c r="G320" s="388"/>
-      <x:c r="H320" s="388"/>
-      <x:c r="I320" s="388"/>
-      <x:c r="J320" s="388"/>
-      <x:c r="K320" s="389"/>
+      <x:c r="B320" s="389"/>
+      <x:c r="C320" s="389"/>
+      <x:c r="D320" s="389"/>
+      <x:c r="E320" s="389"/>
+      <x:c r="F320" s="389"/>
+      <x:c r="G320" s="389"/>
+      <x:c r="H320" s="389"/>
+      <x:c r="I320" s="389"/>
+      <x:c r="J320" s="389"/>
+      <x:c r="K320" s="390"/>
       <x:c r="L320" s="253"/>
       <x:c r="M320" s="253"/>
       <x:c r="N320" s="253"/>
@@ -43698,34 +43702,34 @@
     </x:row>
     <x:row r="1146" spans="1:14" ht="13.8" customHeight="1"/>
     <x:row r="1147" spans="1:14" ht="14.4" customHeight="1">
-      <x:c r="A1147" s="390" t="s">
+      <x:c r="A1147" s="391" t="s">
         <x:v>1630</x:v>
       </x:c>
-      <x:c r="B1147" s="390"/>
-      <x:c r="C1147" s="390"/>
-      <x:c r="D1147" s="390"/>
-      <x:c r="E1147" s="390"/>
-      <x:c r="F1147" s="390"/>
-      <x:c r="G1147" s="390"/>
-      <x:c r="H1147" s="390"/>
-      <x:c r="I1147" s="390"/>
-      <x:c r="J1147" s="390"/>
-      <x:c r="K1147" s="391"/>
+      <x:c r="B1147" s="391"/>
+      <x:c r="C1147" s="391"/>
+      <x:c r="D1147" s="391"/>
+      <x:c r="E1147" s="391"/>
+      <x:c r="F1147" s="391"/>
+      <x:c r="G1147" s="391"/>
+      <x:c r="H1147" s="391"/>
+      <x:c r="I1147" s="391"/>
+      <x:c r="J1147" s="391"/>
+      <x:c r="K1147" s="392"/>
     </x:row>
     <x:row r="1148" spans="1:14" ht="14.4" customHeight="1">
-      <x:c r="A1148" s="386" t="s">
+      <x:c r="A1148" s="387" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B1148" s="386"/>
-      <x:c r="C1148" s="386"/>
-      <x:c r="D1148" s="386"/>
-      <x:c r="E1148" s="386"/>
-      <x:c r="F1148" s="386"/>
-      <x:c r="G1148" s="386"/>
-      <x:c r="H1148" s="386"/>
-      <x:c r="I1148" s="386"/>
-      <x:c r="J1148" s="386"/>
-      <x:c r="K1148" s="392"/>
+      <x:c r="B1148" s="387"/>
+      <x:c r="C1148" s="387"/>
+      <x:c r="D1148" s="387"/>
+      <x:c r="E1148" s="387"/>
+      <x:c r="F1148" s="387"/>
+      <x:c r="G1148" s="387"/>
+      <x:c r="H1148" s="387"/>
+      <x:c r="I1148" s="387"/>
+      <x:c r="J1148" s="387"/>
+      <x:c r="K1148" s="393"/>
     </x:row>
     <x:row r="1149" spans="1:14" ht="42" customHeight="1">
       <x:c r="A1149" s="248">
@@ -44922,19 +44926,19 @@
       <x:c r="K1204" s="59"/>
     </x:row>
     <x:row r="1205" spans="1:14">
-      <x:c r="A1205" s="393" t="s">
+      <x:c r="A1205" s="394" t="s">
         <x:v>224</x:v>
       </x:c>
-      <x:c r="B1205" s="394"/>
-      <x:c r="C1205" s="394"/>
-      <x:c r="D1205" s="394"/>
-      <x:c r="E1205" s="394"/>
-      <x:c r="F1205" s="394"/>
-      <x:c r="G1205" s="394"/>
-      <x:c r="H1205" s="394"/>
-      <x:c r="I1205" s="394"/>
-      <x:c r="J1205" s="394"/>
-      <x:c r="K1205" s="395"/>
+      <x:c r="B1205" s="395"/>
+      <x:c r="C1205" s="395"/>
+      <x:c r="D1205" s="395"/>
+      <x:c r="E1205" s="395"/>
+      <x:c r="F1205" s="395"/>
+      <x:c r="G1205" s="395"/>
+      <x:c r="H1205" s="395"/>
+      <x:c r="I1205" s="395"/>
+      <x:c r="J1205" s="395"/>
+      <x:c r="K1205" s="396"/>
     </x:row>
     <x:row r="1206" spans="1:14" ht="27.6" customHeight="1">
       <x:c r="A1206" s="128">
@@ -48204,41 +48208,41 @@
   </x:mergeCells>
   <x:phoneticPr fontId="16" type="noConversion"/>
   <x:hyperlinks>
-    <x:hyperlink ref="H382" r:id="rId104"/>
-    <x:hyperlink ref="H388" r:id="rId105"/>
-    <x:hyperlink ref="H396" r:id="rId106"/>
-    <x:hyperlink ref="H397" r:id="rId107"/>
-    <x:hyperlink ref="H415" r:id="rId108"/>
-    <x:hyperlink ref="H418" r:id="rId109"/>
-    <x:hyperlink ref="H420" r:id="rId110"/>
-    <x:hyperlink ref="H421" r:id="rId111"/>
-    <x:hyperlink ref="H423" r:id="rId112"/>
-    <x:hyperlink ref="H424" r:id="rId113"/>
-    <x:hyperlink ref="H53" r:id="rId114"/>
-    <x:hyperlink ref="H61" r:id="rId115"/>
-    <x:hyperlink ref="H65" r:id="rId116"/>
-    <x:hyperlink ref="H69" r:id="rId117"/>
-    <x:hyperlink ref="H73" r:id="rId118"/>
-    <x:hyperlink ref="H77" r:id="rId119"/>
-    <x:hyperlink ref="H81" r:id="rId120"/>
-    <x:hyperlink ref="H112" r:id="rId121"/>
-    <x:hyperlink ref="H115" r:id="rId122"/>
-    <x:hyperlink ref="H118" r:id="rId123"/>
-    <x:hyperlink ref="H399" r:id="rId124"/>
-    <x:hyperlink ref="H402" r:id="rId125"/>
-    <x:hyperlink ref="H405" r:id="rId126"/>
-    <x:hyperlink ref="H408" r:id="rId127"/>
-    <x:hyperlink ref="H411" r:id="rId128"/>
-    <x:hyperlink ref="H400" r:id="rId129"/>
-    <x:hyperlink ref="H403" r:id="rId130"/>
-    <x:hyperlink ref="H406" r:id="rId131"/>
-    <x:hyperlink ref="H409" r:id="rId132"/>
-    <x:hyperlink ref="H412" r:id="rId133"/>
-    <x:hyperlink ref="H1075" r:id="rId134"/>
-    <x:hyperlink ref="H1081" r:id="rId135"/>
-    <x:hyperlink ref="H1087" r:id="rId136"/>
-    <x:hyperlink ref="H1093" r:id="rId137"/>
-    <x:hyperlink ref="H1099" r:id="rId138"/>
+    <x:hyperlink ref="H382" r:id="rId105"/>
+    <x:hyperlink ref="H388" r:id="rId106"/>
+    <x:hyperlink ref="H396" r:id="rId107"/>
+    <x:hyperlink ref="H397" r:id="rId108"/>
+    <x:hyperlink ref="H415" r:id="rId109"/>
+    <x:hyperlink ref="H418" r:id="rId110"/>
+    <x:hyperlink ref="H420" r:id="rId111"/>
+    <x:hyperlink ref="H421" r:id="rId112"/>
+    <x:hyperlink ref="H423" r:id="rId113"/>
+    <x:hyperlink ref="H424" r:id="rId114"/>
+    <x:hyperlink ref="H53" r:id="rId115"/>
+    <x:hyperlink ref="H61" r:id="rId116"/>
+    <x:hyperlink ref="H65" r:id="rId117"/>
+    <x:hyperlink ref="H69" r:id="rId118"/>
+    <x:hyperlink ref="H73" r:id="rId119"/>
+    <x:hyperlink ref="H77" r:id="rId120"/>
+    <x:hyperlink ref="H81" r:id="rId121"/>
+    <x:hyperlink ref="H112" r:id="rId122"/>
+    <x:hyperlink ref="H115" r:id="rId123"/>
+    <x:hyperlink ref="H118" r:id="rId124"/>
+    <x:hyperlink ref="H399" r:id="rId125"/>
+    <x:hyperlink ref="H402" r:id="rId126"/>
+    <x:hyperlink ref="H405" r:id="rId127"/>
+    <x:hyperlink ref="H408" r:id="rId128"/>
+    <x:hyperlink ref="H411" r:id="rId129"/>
+    <x:hyperlink ref="H400" r:id="rId130"/>
+    <x:hyperlink ref="H403" r:id="rId131"/>
+    <x:hyperlink ref="H406" r:id="rId132"/>
+    <x:hyperlink ref="H409" r:id="rId133"/>
+    <x:hyperlink ref="H412" r:id="rId134"/>
+    <x:hyperlink ref="H1075" r:id="rId135"/>
+    <x:hyperlink ref="H1081" r:id="rId136"/>
+    <x:hyperlink ref="H1087" r:id="rId137"/>
+    <x:hyperlink ref="H1093" r:id="rId138"/>
+    <x:hyperlink ref="H1099" r:id="rId139"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -48272,40 +48276,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:12">
-      <x:c r="A1" s="396" t="s">
+      <x:c r="A1" s="397" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B1" s="396" t="s">
+      <x:c r="B1" s="397" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="C1" s="396" t="s">
+      <x:c r="C1" s="397" t="s">
         <x:v>403</x:v>
       </x:c>
-      <x:c r="D1" s="396" t="s">
+      <x:c r="D1" s="397" t="s">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="E1" s="396" t="s">
+      <x:c r="E1" s="397" t="s">
         <x:v>405</x:v>
       </x:c>
-      <x:c r="F1" s="397" t="s">
+      <x:c r="F1" s="398" t="s">
         <x:v>406</x:v>
       </x:c>
-      <x:c r="G1" s="396" t="s">
+      <x:c r="G1" s="397" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="H1" s="396" t="s">
+      <x:c r="H1" s="397" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="I1" s="396" t="s">
+      <x:c r="I1" s="397" t="s">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="J1" s="396" t="s">
+      <x:c r="J1" s="397" t="s">
         <x:v>410</x:v>
       </x:c>
-      <x:c r="K1" s="396" t="s">
+      <x:c r="K1" s="397" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="L1" s="396" t="s">
+      <x:c r="L1" s="397" t="s">
         <x:v>2005</x:v>
       </x:c>
     </x:row>
@@ -48333,13 +48337,13 @@
       </x:c>
       <x:c r="H2" s="140"/>
       <x:c r="I2" s="138" t="s">
-        <x:v>417</x:v>
+        <x:v>2006</x:v>
       </x:c>
       <x:c r="J2" s="137" t="s">
-        <x:v>2006</x:v>
+        <x:v>2007</x:v>
       </x:c>
       <x:c r="K2" s="137" t="s">
-        <x:v>2007</x:v>
+        <x:v>2008</x:v>
       </x:c>
       <x:c r="L2" s="137" t="s"/>
     </x:row>
@@ -48376,7 +48380,7 @@
         <x:v>421</x:v>
       </x:c>
       <x:c r="H4" s="314" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I4" s="138"/>
       <x:c r="J4" s="136"/>
@@ -48528,10 +48532,10 @@
         <x:v>438</x:v>
       </x:c>
       <x:c r="J11" s="137" t="s">
-        <x:v>2009</x:v>
+        <x:v>2010</x:v>
       </x:c>
       <x:c r="K11" s="137" t="s">
-        <x:v>2007</x:v>
+        <x:v>2008</x:v>
       </x:c>
       <x:c r="L11" s="137" t="s"/>
     </x:row>
@@ -48566,7 +48570,7 @@
         <x:v>421</x:v>
       </x:c>
       <x:c r="H13" s="134" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I13" s="138"/>
       <x:c r="J13" s="136"/>
@@ -48718,10 +48722,10 @@
         <x:v>451</x:v>
       </x:c>
       <x:c r="J20" s="137" t="s">
-        <x:v>2010</x:v>
+        <x:v>2011</x:v>
       </x:c>
       <x:c r="K20" s="137" t="s">
-        <x:v>2007</x:v>
+        <x:v>2008</x:v>
       </x:c>
       <x:c r="L20" s="137" t="s"/>
     </x:row>
@@ -48910,10 +48914,10 @@
         <x:v>455</x:v>
       </x:c>
       <x:c r="J29" s="137" t="s">
-        <x:v>2011</x:v>
+        <x:v>2012</x:v>
       </x:c>
       <x:c r="K29" s="137" t="s">
-        <x:v>2007</x:v>
+        <x:v>2008</x:v>
       </x:c>
       <x:c r="L29" s="137" t="s"/>
     </x:row>
@@ -48950,7 +48954,7 @@
         <x:v>421</x:v>
       </x:c>
       <x:c r="H31" s="134" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I31" s="138"/>
       <x:c r="J31" s="136"/>
@@ -49102,10 +49106,10 @@
         <x:v>458</x:v>
       </x:c>
       <x:c r="J38" s="137" t="s">
-        <x:v>2012</x:v>
+        <x:v>2013</x:v>
       </x:c>
       <x:c r="K38" s="137" t="s">
-        <x:v>2007</x:v>
+        <x:v>2008</x:v>
       </x:c>
       <x:c r="L38" s="137" t="s"/>
     </x:row>
@@ -49142,7 +49146,7 @@
         <x:v>421</x:v>
       </x:c>
       <x:c r="H40" s="134" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I40" s="138"/>
       <x:c r="J40" s="136"/>
@@ -49294,13 +49298,13 @@
         <x:v>461</x:v>
       </x:c>
       <x:c r="J47" s="137" t="s">
-        <x:v>2013</x:v>
+        <x:v>2014</x:v>
       </x:c>
       <x:c r="K47" s="137" t="s">
-        <x:v>2014</x:v>
+        <x:v>2015</x:v>
       </x:c>
       <x:c r="L47" s="137" t="s">
-        <x:v>2015</x:v>
+        <x:v>2016</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:12">
@@ -49336,7 +49340,7 @@
         <x:v>421</x:v>
       </x:c>
       <x:c r="H49" s="314" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I49" s="138"/>
       <x:c r="J49" s="136"/>
@@ -49436,7 +49440,7 @@
         <x:v>445</x:v>
       </x:c>
       <x:c r="H54" s="314" t="s">
-        <x:v>2016</x:v>
+        <x:v>2017</x:v>
       </x:c>
       <x:c r="I54" s="138"/>
       <x:c r="J54" s="136"/>
@@ -49523,8 +49527,8 @@
       <x:c r="G58" s="138" t="s">
         <x:v>421</x:v>
       </x:c>
-      <x:c r="H58" s="25" t="s">
-        <x:v>2008</x:v>
+      <x:c r="H58" s="347" t="s">
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I58" s="138"/>
       <x:c r="J58" s="136"/>
@@ -49712,7 +49716,7 @@
         <x:v>421</x:v>
       </x:c>
       <x:c r="H67" s="314" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I67" s="138"/>
       <x:c r="J67" s="136"/>
@@ -49900,7 +49904,7 @@
         <x:v>421</x:v>
       </x:c>
       <x:c r="H76" s="314" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I76" s="138"/>
       <x:c r="J76" s="136"/>
@@ -50036,7 +50040,7 @@
         <x:v>468</x:v>
       </x:c>
       <x:c r="D83" s="140" t="s">
-        <x:v>2017</x:v>
+        <x:v>2018</x:v>
       </x:c>
       <x:c r="E83" s="140" t="s">
         <x:v>434</x:v>
@@ -50088,7 +50092,7 @@
         <x:v>421</x:v>
       </x:c>
       <x:c r="H85" s="314" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I85" s="138"/>
       <x:c r="J85" s="136"/>
@@ -50168,7 +50172,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H89" s="25" t="s">
-        <x:v>2018</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="I89" s="138"/>
       <x:c r="J89" s="136"/>
@@ -50188,7 +50192,7 @@
         <x:v>445</x:v>
       </x:c>
       <x:c r="H90" s="25" t="s">
-        <x:v>2018</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="I90" s="138"/>
       <x:c r="J90" s="136"/>
@@ -50256,7 +50260,7 @@
         <x:v>419</x:v>
       </x:c>
       <x:c r="H93" s="140" t="s">
-        <x:v>2019</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="I93" s="138"/>
       <x:c r="J93" s="136"/>
@@ -50276,7 +50280,7 @@
         <x:v>421</x:v>
       </x:c>
       <x:c r="H94" s="314" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I94" s="138"/>
       <x:c r="J94" s="136"/>
@@ -50464,7 +50468,7 @@
         <x:v>421</x:v>
       </x:c>
       <x:c r="H103" s="314" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I103" s="138"/>
       <x:c r="J103" s="134"/>
@@ -50484,7 +50488,7 @@
         <x:v>439</x:v>
       </x:c>
       <x:c r="H104" s="139" t="s">
-        <x:v>2020</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="I104" s="138"/>
       <x:c r="J104" s="134"/>
@@ -50632,7 +50636,7 @@
         <x:v>480</x:v>
       </x:c>
       <x:c r="H111" s="134" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I111" s="138"/>
       <x:c r="J111" s="134"/>
@@ -50838,7 +50842,7 @@
         <x:v>480</x:v>
       </x:c>
       <x:c r="H120" s="134" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I120" s="138" t="s">
         <x:v>496</x:v>
@@ -50908,7 +50912,7 @@
         <x:v>480</x:v>
       </x:c>
       <x:c r="H123" s="134" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I123" s="138" t="s">
         <x:v>500</x:v>
@@ -51049,7 +51053,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I129" s="138" t="s">
-        <x:v>2021</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="J129" s="134"/>
       <x:c r="K129" s="134"/>
@@ -51119,7 +51123,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I132" s="123" t="s">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="J132" s="134"/>
       <x:c r="K132" s="134"/>
@@ -51189,7 +51193,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I135" s="138" t="s">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="J135" s="134"/>
       <x:c r="K135" s="134"/>
@@ -51256,10 +51260,10 @@
         <x:v>480</x:v>
       </x:c>
       <x:c r="H138" s="316" t="s">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="I138" s="120" t="s">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="J138" s="134"/>
       <x:c r="K138" s="134"/>
@@ -51326,10 +51330,10 @@
         <x:v>480</x:v>
       </x:c>
       <x:c r="H141" s="315" t="s">
-        <x:v>2008</x:v>
+        <x:v>2009</x:v>
       </x:c>
       <x:c r="I141" s="138" t="s">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="J141" s="118"/>
       <x:c r="K141" s="134"/>
@@ -51393,11 +51397,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G144" s="138" t="s">
-        <x:v>2027</x:v>
+        <x:v>2028</x:v>
       </x:c>
       <x:c r="H144" s="140"/>
       <x:c r="I144" s="138" t="s">
-        <x:v>2028</x:v>
+        <x:v>2029</x:v>
       </x:c>
       <x:c r="J144" s="134"/>
       <x:c r="K144" s="134"/>
@@ -51413,10 +51417,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G145" s="319" t="s">
-        <x:v>2029</x:v>
+        <x:v>2030</x:v>
       </x:c>
       <x:c r="H145" s="134" t="s">
-        <x:v>2030</x:v>
+        <x:v>2031</x:v>
       </x:c>
       <x:c r="I145" s="138"/>
       <x:c r="J145" s="134"/>
@@ -51433,10 +51437,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G146" s="138" t="s">
-        <x:v>2031</x:v>
+        <x:v>2032</x:v>
       </x:c>
       <x:c r="H146" s="317" t="s">
-        <x:v>2032</x:v>
+        <x:v>2033</x:v>
       </x:c>
       <x:c r="I146" s="138"/>
       <x:c r="J146" s="134"/>
@@ -51453,10 +51457,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G147" s="138" t="s">
+        <x:v>2034</x:v>
+      </x:c>
+      <x:c r="H147" s="134" t="s">
         <x:v>2033</x:v>
-      </x:c>
-      <x:c r="H147" s="134" t="s">
-        <x:v>2032</x:v>
       </x:c>
       <x:c r="I147" s="138"/>
       <x:c r="J147" s="134"/>
@@ -51473,7 +51477,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G148" s="138" t="s">
-        <x:v>2034</x:v>
+        <x:v>2035</x:v>
       </x:c>
       <x:c r="H148" s="134"/>
       <x:c r="I148" s="138"/>
@@ -51507,7 +51511,7 @@
         <x:v>590</x:v>
       </x:c>
       <x:c r="I149" s="138" t="s">
-        <x:v>2035</x:v>
+        <x:v>2036</x:v>
       </x:c>
       <x:c r="J149" s="298"/>
       <x:c r="K149" s="134"/>
@@ -51527,7 +51531,7 @@
       </x:c>
       <x:c r="H150" s="140"/>
       <x:c r="I150" s="138" t="s">
-        <x:v>2036</x:v>
+        <x:v>2037</x:v>
       </x:c>
       <x:c r="J150" s="298"/>
       <x:c r="K150" s="134"/>
@@ -51547,7 +51551,7 @@
       </x:c>
       <x:c r="H151" s="140"/>
       <x:c r="I151" s="138" t="s">
-        <x:v>2037</x:v>
+        <x:v>2038</x:v>
       </x:c>
       <x:c r="J151" s="298"/>
       <x:c r="K151" s="134"/>
@@ -51623,13 +51627,13 @@
       </x:c>
       <x:c r="H154" s="140"/>
       <x:c r="I154" s="138" t="s">
-        <x:v>2038</x:v>
+        <x:v>2039</x:v>
       </x:c>
       <x:c r="J154" s="134" t="s">
-        <x:v>2039</x:v>
+        <x:v>2040</x:v>
       </x:c>
       <x:c r="K154" s="134" t="s">
-        <x:v>2007</x:v>
+        <x:v>2008</x:v>
       </x:c>
       <x:c r="L154" s="134"/>
     </x:row>
@@ -51643,16 +51647,16 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G155" s="138" t="s">
-        <x:v>2040</x:v>
+        <x:v>2041</x:v>
       </x:c>
       <x:c r="H155" s="140" t="s">
-        <x:v>2041</x:v>
+        <x:v>2042</x:v>
       </x:c>
       <x:c r="I155" s="138" t="s">
-        <x:v>2042</x:v>
+        <x:v>2043</x:v>
       </x:c>
       <x:c r="J155" s="134" t="s">
-        <x:v>2043</x:v>
+        <x:v>2044</x:v>
       </x:c>
       <x:c r="K155" s="134"/>
       <x:c r="L155" s="134"/>
@@ -51668,7 +51672,7 @@
         <x:v>626</x:v>
       </x:c>
       <x:c r="D156" s="140" t="s">
-        <x:v>2044</x:v>
+        <x:v>2045</x:v>
       </x:c>
       <x:c r="E156" s="140" t="s">
         <x:v>616</x:v>
@@ -51677,13 +51681,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G156" s="138" t="s">
-        <x:v>2045</x:v>
+        <x:v>2046</x:v>
       </x:c>
       <x:c r="H156" s="140" t="s">
-        <x:v>2046</x:v>
+        <x:v>2047</x:v>
       </x:c>
       <x:c r="I156" s="138" t="s">
-        <x:v>2047</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="J156" s="134"/>
       <x:c r="K156" s="134"/>
@@ -51709,19 +51713,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G157" s="138" t="s">
-        <x:v>2048</x:v>
+        <x:v>2049</x:v>
       </x:c>
       <x:c r="H157" s="140" t="s">
-        <x:v>2049</x:v>
+        <x:v>2050</x:v>
       </x:c>
       <x:c r="I157" s="138" t="s">
-        <x:v>2050</x:v>
+        <x:v>2051</x:v>
       </x:c>
       <x:c r="J157" s="134" t="s">
-        <x:v>2051</x:v>
+        <x:v>2052</x:v>
       </x:c>
       <x:c r="K157" s="134" t="s">
-        <x:v>2007</x:v>
+        <x:v>2008</x:v>
       </x:c>
       <x:c r="L157" s="134"/>
     </x:row>
@@ -51735,14 +51739,14 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G158" s="138" t="s">
-        <x:v>2052</x:v>
+        <x:v>2053</x:v>
       </x:c>
       <x:c r="H158" s="140"/>
       <x:c r="I158" s="138" t="s">
-        <x:v>2053</x:v>
+        <x:v>2054</x:v>
       </x:c>
       <x:c r="J158" s="134" t="s">
-        <x:v>2054</x:v>
+        <x:v>2055</x:v>
       </x:c>
       <x:c r="K158" s="134"/>
       <x:c r="L158" s="134"/>
@@ -51757,14 +51761,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G159" s="138" t="s">
-        <x:v>2055</x:v>
+        <x:v>2056</x:v>
       </x:c>
       <x:c r="H159" s="140"/>
       <x:c r="I159" s="138" t="s">
-        <x:v>2056</x:v>
+        <x:v>2057</x:v>
       </x:c>
       <x:c r="J159" s="134" t="s">
-        <x:v>2057</x:v>
+        <x:v>2058</x:v>
       </x:c>
       <x:c r="K159" s="134"/>
       <x:c r="L159" s="134"/>
@@ -51789,13 +51793,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G160" s="138" t="s">
-        <x:v>2048</x:v>
+        <x:v>2049</x:v>
       </x:c>
       <x:c r="H160" s="140" t="s">
-        <x:v>2049</x:v>
+        <x:v>2050</x:v>
       </x:c>
       <x:c r="I160" s="138" t="s">
-        <x:v>2058</x:v>
+        <x:v>2059</x:v>
       </x:c>
       <x:c r="J160" s="134"/>
       <x:c r="K160" s="134"/>
@@ -51811,7 +51815,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G161" s="138" t="s">
-        <x:v>2059</x:v>
+        <x:v>2060</x:v>
       </x:c>
       <x:c r="H161" s="313">
         <x:v>46109</x:v>
@@ -51832,28 +51836,28 @@
         <x:v>644</x:v>
       </x:c>
       <x:c r="D162" s="116" t="s">
-        <x:v>2060</x:v>
+        <x:v>2061</x:v>
       </x:c>
       <x:c r="E162" s="116" t="s">
-        <x:v>2061</x:v>
+        <x:v>2062</x:v>
       </x:c>
       <x:c r="F162" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G162" s="320" t="s">
-        <x:v>2062</x:v>
+        <x:v>2063</x:v>
       </x:c>
       <x:c r="H162" s="116" t="s">
-        <x:v>2049</x:v>
+        <x:v>2050</x:v>
       </x:c>
       <x:c r="I162" s="320" t="s">
-        <x:v>2050</x:v>
+        <x:v>2051</x:v>
       </x:c>
       <x:c r="J162" s="134" t="s">
-        <x:v>2063</x:v>
+        <x:v>2064</x:v>
       </x:c>
       <x:c r="K162" s="134" t="s">
-        <x:v>2007</x:v>
+        <x:v>2008</x:v>
       </x:c>
       <x:c r="L162" s="134"/>
     </x:row>
@@ -51867,14 +51871,14 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G163" s="320" t="s">
-        <x:v>2064</x:v>
+        <x:v>2065</x:v>
       </x:c>
       <x:c r="H163" s="116"/>
       <x:c r="I163" s="320" t="s">
-        <x:v>2065</x:v>
+        <x:v>2066</x:v>
       </x:c>
       <x:c r="J163" s="134" t="s">
-        <x:v>2066</x:v>
+        <x:v>2067</x:v>
       </x:c>
       <x:c r="K163" s="134"/>
       <x:c r="L163" s="134"/>
@@ -51889,14 +51893,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G164" s="320" t="s">
-        <x:v>2067</x:v>
+        <x:v>2068</x:v>
       </x:c>
       <x:c r="H164" s="116"/>
       <x:c r="I164" s="320" t="s">
-        <x:v>2068</x:v>
+        <x:v>2069</x:v>
       </x:c>
       <x:c r="J164" s="134" t="s">
-        <x:v>2069</x:v>
+        <x:v>2070</x:v>
       </x:c>
       <x:c r="K164" s="134"/>
       <x:c r="L164" s="134"/>
@@ -51921,13 +51925,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G165" s="320" t="s">
-        <x:v>2070</x:v>
+        <x:v>2071</x:v>
       </x:c>
       <x:c r="H165" s="318">
         <x:v>0.333333333333333</x:v>
       </x:c>
       <x:c r="I165" s="320" t="s">
-        <x:v>2071</x:v>
+        <x:v>2072</x:v>
       </x:c>
       <x:c r="J165" s="134"/>
       <x:c r="K165" s="134"/>
@@ -51943,13 +51947,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G166" s="320" t="s">
-        <x:v>2072</x:v>
+        <x:v>2073</x:v>
       </x:c>
       <x:c r="H166" s="116" t="s">
-        <x:v>2073</x:v>
+        <x:v>2074</x:v>
       </x:c>
       <x:c r="I166" s="320" t="s">
-        <x:v>2074</x:v>
+        <x:v>2075</x:v>
       </x:c>
       <x:c r="J166" s="134"/>
       <x:c r="K166" s="134"/>
@@ -51965,13 +51969,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G167" s="320" t="s">
-        <x:v>2075</x:v>
+        <x:v>2076</x:v>
       </x:c>
       <x:c r="H167" s="116" t="s">
-        <x:v>2076</x:v>
+        <x:v>2077</x:v>
       </x:c>
       <x:c r="I167" s="320" t="s">
-        <x:v>2077</x:v>
+        <x:v>2078</x:v>
       </x:c>
       <x:c r="J167" s="134"/>
       <x:c r="K167" s="134"/>
@@ -51987,11 +51991,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G168" s="320" t="s">
-        <x:v>2078</x:v>
+        <x:v>2079</x:v>
       </x:c>
       <x:c r="H168" s="116"/>
       <x:c r="I168" s="320" t="s">
-        <x:v>2079</x:v>
+        <x:v>2080</x:v>
       </x:c>
       <x:c r="J168" s="134"/>
       <x:c r="K168" s="134"/>
@@ -52008,22 +52012,22 @@
         <x:v>658</x:v>
       </x:c>
       <x:c r="D169" s="116" t="s">
-        <x:v>2080</x:v>
+        <x:v>2081</x:v>
       </x:c>
       <x:c r="E169" s="116" t="s">
-        <x:v>2081</x:v>
+        <x:v>2082</x:v>
       </x:c>
       <x:c r="F169" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G169" s="320" t="s">
-        <x:v>2082</x:v>
+        <x:v>2083</x:v>
       </x:c>
       <x:c r="H169" s="116" t="s">
-        <x:v>2083</x:v>
+        <x:v>2084</x:v>
       </x:c>
       <x:c r="I169" s="320" t="s">
-        <x:v>2084</x:v>
+        <x:v>2085</x:v>
       </x:c>
       <x:c r="J169" s="134"/>
       <x:c r="K169" s="134"/>
@@ -52039,11 +52043,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G170" s="320" t="s">
-        <x:v>2085</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="H170" s="116"/>
       <x:c r="I170" s="320" t="s">
-        <x:v>2086</x:v>
+        <x:v>2087</x:v>
       </x:c>
       <x:c r="J170" s="134"/>
       <x:c r="K170" s="134"/>
@@ -52059,11 +52063,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G171" s="320" t="s">
-        <x:v>2087</x:v>
+        <x:v>2088</x:v>
       </x:c>
       <x:c r="H171" s="116"/>
       <x:c r="I171" s="320" t="s">
-        <x:v>2088</x:v>
+        <x:v>2089</x:v>
       </x:c>
       <x:c r="J171" s="134"/>
       <x:c r="K171" s="134"/>
@@ -52089,13 +52093,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G172" s="320" t="s">
-        <x:v>2089</x:v>
+        <x:v>2090</x:v>
       </x:c>
       <x:c r="H172" s="116" t="s">
-        <x:v>2083</x:v>
+        <x:v>2084</x:v>
       </x:c>
       <x:c r="I172" s="320" t="s">
-        <x:v>2084</x:v>
+        <x:v>2085</x:v>
       </x:c>
       <x:c r="J172" s="134"/>
       <x:c r="K172" s="134"/>
@@ -52111,11 +52115,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G173" s="320" t="s">
-        <x:v>2090</x:v>
+        <x:v>2091</x:v>
       </x:c>
       <x:c r="H173" s="116"/>
       <x:c r="I173" s="320" t="s">
-        <x:v>2091</x:v>
+        <x:v>2092</x:v>
       </x:c>
       <x:c r="J173" s="134"/>
       <x:c r="K173" s="134"/>
@@ -52141,13 +52145,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G174" s="320" t="s">
-        <x:v>2092</x:v>
+        <x:v>2093</x:v>
       </x:c>
       <x:c r="H174" s="116" t="s">
-        <x:v>2083</x:v>
+        <x:v>2084</x:v>
       </x:c>
       <x:c r="I174" s="320" t="s">
-        <x:v>2093</x:v>
+        <x:v>2094</x:v>
       </x:c>
       <x:c r="J174" s="134"/>
       <x:c r="K174" s="134"/>
@@ -52163,11 +52167,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G175" s="320" t="s">
-        <x:v>2094</x:v>
+        <x:v>2095</x:v>
       </x:c>
       <x:c r="H175" s="116"/>
       <x:c r="I175" s="320" t="s">
-        <x:v>2084</x:v>
+        <x:v>2085</x:v>
       </x:c>
       <x:c r="J175" s="134"/>
       <x:c r="K175" s="134"/>
@@ -52183,11 +52187,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G176" s="320" t="s">
-        <x:v>2095</x:v>
+        <x:v>2096</x:v>
       </x:c>
       <x:c r="H176" s="116"/>
       <x:c r="I176" s="320" t="s">
-        <x:v>2096</x:v>
+        <x:v>2097</x:v>
       </x:c>
       <x:c r="J176" s="134"/>
       <x:c r="K176" s="134"/>
@@ -52204,20 +52208,20 @@
         <x:v>674</x:v>
       </x:c>
       <x:c r="D177" s="116" t="s">
-        <x:v>2097</x:v>
+        <x:v>2098</x:v>
       </x:c>
       <x:c r="E177" s="116" t="s">
-        <x:v>2098</x:v>
+        <x:v>2099</x:v>
       </x:c>
       <x:c r="F177" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G177" s="320" t="s">
-        <x:v>2099</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="H177" s="116"/>
       <x:c r="I177" s="320" t="s">
-        <x:v>2100</x:v>
+        <x:v>2101</x:v>
       </x:c>
       <x:c r="J177" s="134"/>
       <x:c r="K177" s="134"/>
@@ -52233,11 +52237,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G178" s="320" t="s">
-        <x:v>2101</x:v>
+        <x:v>2102</x:v>
       </x:c>
       <x:c r="H178" s="116"/>
       <x:c r="I178" s="320" t="s">
-        <x:v>2102</x:v>
+        <x:v>2103</x:v>
       </x:c>
       <x:c r="J178" s="134"/>
       <x:c r="K178" s="134"/>
@@ -52254,22 +52258,22 @@
         <x:v>677</x:v>
       </x:c>
       <x:c r="D179" s="116" t="s">
-        <x:v>2103</x:v>
+        <x:v>2104</x:v>
       </x:c>
       <x:c r="E179" s="116" t="s">
-        <x:v>2104</x:v>
+        <x:v>2105</x:v>
       </x:c>
       <x:c r="F179" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G179" s="320" t="s">
-        <x:v>2105</x:v>
+        <x:v>2106</x:v>
       </x:c>
       <x:c r="H179" s="116" t="s">
         <x:v>681</x:v>
       </x:c>
       <x:c r="I179" s="320" t="s">
-        <x:v>2106</x:v>
+        <x:v>2107</x:v>
       </x:c>
       <x:c r="J179" s="116"/>
       <x:c r="K179" s="134"/>
@@ -52285,13 +52289,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G180" s="321" t="s">
-        <x:v>2107</x:v>
+        <x:v>2108</x:v>
       </x:c>
       <x:c r="H180" s="115" t="s">
-        <x:v>2108</x:v>
+        <x:v>2109</x:v>
       </x:c>
       <x:c r="I180" s="321" t="s">
-        <x:v>2109</x:v>
+        <x:v>2110</x:v>
       </x:c>
       <x:c r="J180" s="115"/>
       <x:c r="K180" s="137"/>
@@ -52308,22 +52312,22 @@
         <x:v>686</x:v>
       </x:c>
       <x:c r="D181" s="116" t="s">
-        <x:v>2110</x:v>
+        <x:v>2111</x:v>
       </x:c>
       <x:c r="E181" s="116" t="s">
-        <x:v>2111</x:v>
+        <x:v>2112</x:v>
       </x:c>
       <x:c r="F181" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G181" s="320" t="s">
-        <x:v>2112</x:v>
+        <x:v>2113</x:v>
       </x:c>
       <x:c r="H181" s="116" t="s">
-        <x:v>2113</x:v>
+        <x:v>2114</x:v>
       </x:c>
       <x:c r="I181" s="320" t="s">
-        <x:v>2114</x:v>
+        <x:v>2115</x:v>
       </x:c>
       <x:c r="J181" s="134"/>
       <x:c r="K181" s="134"/>
@@ -52339,13 +52343,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G182" s="320" t="s">
-        <x:v>2115</x:v>
+        <x:v>2116</x:v>
       </x:c>
       <x:c r="H182" s="116" t="s">
-        <x:v>2116</x:v>
+        <x:v>2117</x:v>
       </x:c>
       <x:c r="I182" s="320" t="s">
-        <x:v>2117</x:v>
+        <x:v>2118</x:v>
       </x:c>
       <x:c r="J182" s="134"/>
       <x:c r="K182" s="134"/>
@@ -52361,11 +52365,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G183" s="320" t="s">
-        <x:v>2118</x:v>
+        <x:v>2119</x:v>
       </x:c>
       <x:c r="H183" s="116"/>
       <x:c r="I183" s="320" t="s">
-        <x:v>2119</x:v>
+        <x:v>2120</x:v>
       </x:c>
       <x:c r="J183" s="134"/>
       <x:c r="K183" s="134"/>
@@ -52382,20 +52386,20 @@
         <x:v>696</x:v>
       </x:c>
       <x:c r="D184" s="116" t="s">
-        <x:v>2120</x:v>
+        <x:v>2121</x:v>
       </x:c>
       <x:c r="E184" s="116" t="s">
-        <x:v>2121</x:v>
+        <x:v>2122</x:v>
       </x:c>
       <x:c r="F184" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G184" s="320" t="s">
-        <x:v>2122</x:v>
+        <x:v>2123</x:v>
       </x:c>
       <x:c r="H184" s="116"/>
       <x:c r="I184" s="320" t="s">
-        <x:v>2123</x:v>
+        <x:v>2124</x:v>
       </x:c>
       <x:c r="J184" s="134"/>
       <x:c r="K184" s="134"/>
@@ -52411,13 +52415,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G185" s="320" t="s">
-        <x:v>2124</x:v>
+        <x:v>2125</x:v>
       </x:c>
       <x:c r="H185" s="116" t="s">
-        <x:v>2125</x:v>
+        <x:v>2126</x:v>
       </x:c>
       <x:c r="I185" s="320" t="s">
-        <x:v>2126</x:v>
+        <x:v>2127</x:v>
       </x:c>
       <x:c r="J185" s="134"/>
       <x:c r="K185" s="134"/>
@@ -52433,11 +52437,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G186" s="320" t="s">
-        <x:v>2127</x:v>
+        <x:v>2128</x:v>
       </x:c>
       <x:c r="H186" s="116"/>
       <x:c r="I186" s="320" t="s">
-        <x:v>2128</x:v>
+        <x:v>2129</x:v>
       </x:c>
       <x:c r="J186" s="134"/>
       <x:c r="K186" s="134"/>
@@ -52453,11 +52457,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G187" s="320" t="s">
-        <x:v>2129</x:v>
+        <x:v>2130</x:v>
       </x:c>
       <x:c r="H187" s="116"/>
       <x:c r="I187" s="320" t="s">
-        <x:v>2130</x:v>
+        <x:v>2131</x:v>
       </x:c>
       <x:c r="J187" s="134"/>
       <x:c r="K187" s="134"/>
@@ -52474,22 +52478,22 @@
         <x:v>932</x:v>
       </x:c>
       <x:c r="D188" s="114" t="s">
-        <x:v>2131</x:v>
+        <x:v>2132</x:v>
       </x:c>
       <x:c r="E188" s="114" t="s">
-        <x:v>2132</x:v>
+        <x:v>2133</x:v>
       </x:c>
       <x:c r="F188" s="329">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G188" s="324" t="s">
-        <x:v>2133</x:v>
+        <x:v>2134</x:v>
       </x:c>
       <x:c r="H188" s="324" t="s">
-        <x:v>2134</x:v>
+        <x:v>2135</x:v>
       </x:c>
       <x:c r="I188" s="325" t="s">
-        <x:v>2135</x:v>
+        <x:v>2136</x:v>
       </x:c>
       <x:c r="J188" s="61"/>
       <x:c r="K188" s="133"/>
@@ -52505,13 +52509,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G189" s="324" t="s">
-        <x:v>2136</x:v>
+        <x:v>2137</x:v>
       </x:c>
       <x:c r="H189" s="324" t="s">
-        <x:v>2137</x:v>
+        <x:v>2138</x:v>
       </x:c>
       <x:c r="I189" s="325" t="s">
-        <x:v>2138</x:v>
+        <x:v>2139</x:v>
       </x:c>
       <x:c r="J189" s="61"/>
       <x:c r="K189" s="124"/>
@@ -52527,11 +52531,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G190" s="324" t="s">
-        <x:v>2139</x:v>
+        <x:v>2140</x:v>
       </x:c>
       <x:c r="H190" s="324"/>
       <x:c r="I190" s="325" t="s">
-        <x:v>2140</x:v>
+        <x:v>2141</x:v>
       </x:c>
       <x:c r="J190" s="61"/>
       <x:c r="K190" s="111"/>
@@ -52548,20 +52552,20 @@
         <x:v>947</x:v>
       </x:c>
       <x:c r="D191" s="114" t="s">
-        <x:v>2141</x:v>
+        <x:v>2142</x:v>
       </x:c>
       <x:c r="E191" s="114" t="s">
-        <x:v>2142</x:v>
+        <x:v>2143</x:v>
       </x:c>
       <x:c r="F191" s="329">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G191" s="324" t="s">
-        <x:v>2143</x:v>
+        <x:v>2144</x:v>
       </x:c>
       <x:c r="H191" s="324"/>
       <x:c r="I191" s="325" t="s">
-        <x:v>2144</x:v>
+        <x:v>2145</x:v>
       </x:c>
       <x:c r="J191" s="61"/>
       <x:c r="K191" s="133"/>
@@ -52577,11 +52581,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G192" s="324" t="s">
-        <x:v>2145</x:v>
+        <x:v>2146</x:v>
       </x:c>
       <x:c r="H192" s="324"/>
       <x:c r="I192" s="325" t="s">
-        <x:v>2146</x:v>
+        <x:v>2147</x:v>
       </x:c>
       <x:c r="J192" s="61"/>
       <x:c r="K192" s="124"/>
@@ -52597,13 +52601,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G193" s="324" t="s">
-        <x:v>2147</x:v>
+        <x:v>2148</x:v>
       </x:c>
       <x:c r="H193" s="324" t="s">
-        <x:v>2148</x:v>
+        <x:v>2149</x:v>
       </x:c>
       <x:c r="I193" s="325" t="s">
-        <x:v>2149</x:v>
+        <x:v>2150</x:v>
       </x:c>
       <x:c r="J193" s="61"/>
       <x:c r="K193" s="111"/>
@@ -52948,15 +52952,16 @@
     <x:mergeCell ref="L191:L193"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H49" r:id="rId139"/>
-    <x:hyperlink ref="H67" r:id="rId140"/>
-    <x:hyperlink ref="H76" r:id="rId141"/>
-    <x:hyperlink ref="H85" r:id="rId142"/>
-    <x:hyperlink ref="H94" r:id="rId143"/>
-    <x:hyperlink ref="H103" r:id="rId144"/>
-    <x:hyperlink ref="H112" r:id="rId145"/>
-    <x:hyperlink ref="H4" r:id="rId146"/>
-    <x:hyperlink ref="H54" r:id="rId147"/>
+    <x:hyperlink ref="H49" r:id="rId140"/>
+    <x:hyperlink ref="H67" r:id="rId141"/>
+    <x:hyperlink ref="H76" r:id="rId142"/>
+    <x:hyperlink ref="H85" r:id="rId143"/>
+    <x:hyperlink ref="H94" r:id="rId144"/>
+    <x:hyperlink ref="H103" r:id="rId145"/>
+    <x:hyperlink ref="H112" r:id="rId146"/>
+    <x:hyperlink ref="H4" r:id="rId147"/>
+    <x:hyperlink ref="H54" r:id="rId148"/>
+    <x:hyperlink ref="H58" r:id="rId149"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -52989,40 +52994,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:12" ht="27.6" customHeight="1">
-      <x:c r="A1" s="396" t="s">
+      <x:c r="A1" s="397" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B1" s="396" t="s">
+      <x:c r="B1" s="397" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="C1" s="396" t="s">
+      <x:c r="C1" s="397" t="s">
         <x:v>403</x:v>
       </x:c>
-      <x:c r="D1" s="396" t="s">
+      <x:c r="D1" s="397" t="s">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="E1" s="396" t="s">
+      <x:c r="E1" s="397" t="s">
         <x:v>405</x:v>
       </x:c>
-      <x:c r="F1" s="397" t="s">
+      <x:c r="F1" s="398" t="s">
         <x:v>406</x:v>
       </x:c>
-      <x:c r="G1" s="396" t="s">
+      <x:c r="G1" s="397" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="H1" s="396" t="s">
+      <x:c r="H1" s="397" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="I1" s="396" t="s">
+      <x:c r="I1" s="397" t="s">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="J1" s="396" t="s">
+      <x:c r="J1" s="397" t="s">
         <x:v>410</x:v>
       </x:c>
-      <x:c r="K1" s="396" t="s">
+      <x:c r="K1" s="397" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="L1" s="396" t="s">
+      <x:c r="L1" s="397" t="s">
         <x:v>2005</x:v>
       </x:c>
     </x:row>
@@ -53049,7 +53054,7 @@
         <x:v>1270</x:v>
       </x:c>
       <x:c r="H2" s="288" t="s">
-        <x:v>2150</x:v>
+        <x:v>2151</x:v>
       </x:c>
       <x:c r="I2" s="134" t="s">
         <x:v>1272</x:v>
@@ -53096,7 +53101,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="297" t="s">
-        <x:v>2151</x:v>
+        <x:v>2152</x:v>
       </x:c>
       <x:c r="H4" s="297" t="s">
         <x:v>1277</x:v>
@@ -53176,7 +53181,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="297" t="s">
-        <x:v>2152</x:v>
+        <x:v>2153</x:v>
       </x:c>
       <x:c r="H7" s="297"/>
       <x:c r="I7" s="298" t="s">
@@ -53209,7 +53214,7 @@
         <x:v>1297</x:v>
       </x:c>
       <x:c r="H8" s="297" t="s">
-        <x:v>2153</x:v>
+        <x:v>2154</x:v>
       </x:c>
       <x:c r="I8" s="134" t="s">
         <x:v>1299</x:v>
@@ -53228,7 +53233,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G9" s="319" t="s">
-        <x:v>2154</x:v>
+        <x:v>2155</x:v>
       </x:c>
       <x:c r="H9" s="297"/>
       <x:c r="I9" s="134"/>
@@ -53317,7 +53322,7 @@
         <x:v>1297</x:v>
       </x:c>
       <x:c r="H13" s="297" t="s">
-        <x:v>2155</x:v>
+        <x:v>2156</x:v>
       </x:c>
       <x:c r="I13" s="134" t="s">
         <x:v>1307</x:v>
@@ -53336,7 +53341,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="319" t="s">
-        <x:v>2154</x:v>
+        <x:v>2155</x:v>
       </x:c>
       <x:c r="H14" s="297"/>
       <x:c r="I14" s="134"/>
@@ -53422,7 +53427,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="61" t="s">
-        <x:v>2156</x:v>
+        <x:v>2157</x:v>
       </x:c>
       <x:c r="H18" s="140"/>
       <x:c r="I18" s="140" t="s">
@@ -53442,7 +53447,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="61" t="s">
-        <x:v>2157</x:v>
+        <x:v>2158</x:v>
       </x:c>
       <x:c r="H19" s="140" t="s">
         <x:v>965</x:v>
@@ -53462,7 +53467,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="61" t="s">
-        <x:v>2158</x:v>
+        <x:v>2159</x:v>
       </x:c>
       <x:c r="H20" s="140"/>
       <x:c r="I20" s="140"/>
@@ -53480,7 +53485,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G21" s="61" t="s">
-        <x:v>2159</x:v>
+        <x:v>2160</x:v>
       </x:c>
       <x:c r="H21" s="140" t="s">
         <x:v>968</x:v>
@@ -53500,7 +53505,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G22" s="61" t="s">
-        <x:v>2160</x:v>
+        <x:v>2161</x:v>
       </x:c>
       <x:c r="H22" s="314" t="s">
         <x:v>970</x:v>
@@ -53520,7 +53525,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G23" s="61" t="s">
-        <x:v>2161</x:v>
+        <x:v>2162</x:v>
       </x:c>
       <x:c r="H23" s="140">
         <x:v>1</x:v>
@@ -53540,7 +53545,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G24" s="61" t="s">
-        <x:v>2162</x:v>
+        <x:v>2163</x:v>
       </x:c>
       <x:c r="H24" s="140" t="s">
         <x:v>973</x:v>
@@ -53560,7 +53565,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G25" s="61" t="s">
-        <x:v>2163</x:v>
+        <x:v>2164</x:v>
       </x:c>
       <x:c r="H25" s="140"/>
       <x:c r="I25" s="140"/>
@@ -53588,7 +53593,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G26" s="61" t="s">
-        <x:v>2164</x:v>
+        <x:v>2165</x:v>
       </x:c>
       <x:c r="H26" s="140"/>
       <x:c r="I26" s="133" t="s">
@@ -53628,7 +53633,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G28" s="61" t="s">
-        <x:v>2165</x:v>
+        <x:v>2166</x:v>
       </x:c>
       <x:c r="H28" s="239" t="s">
         <x:v>970</x:v>
@@ -53648,7 +53653,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G29" s="61" t="s">
-        <x:v>2166</x:v>
+        <x:v>2167</x:v>
       </x:c>
       <x:c r="H29" s="140">
         <x:v>1</x:v>
@@ -53668,7 +53673,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G30" s="61" t="s">
-        <x:v>2167</x:v>
+        <x:v>2168</x:v>
       </x:c>
       <x:c r="H30" s="140"/>
       <x:c r="I30" s="111"/>
@@ -53696,7 +53701,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="61" t="s">
-        <x:v>2168</x:v>
+        <x:v>2169</x:v>
       </x:c>
       <x:c r="H31" s="140"/>
       <x:c r="I31" s="133" t="s">
@@ -53795,7 +53800,7 @@
         <x:v>1309</x:v>
       </x:c>
       <x:c r="D36" s="134" t="s">
-        <x:v>2169</x:v>
+        <x:v>2170</x:v>
       </x:c>
       <x:c r="E36" s="134" t="s">
         <x:v>1311</x:v>
@@ -53807,7 +53812,7 @@
         <x:v>988</x:v>
       </x:c>
       <x:c r="H36" s="297" t="s">
-        <x:v>2170</x:v>
+        <x:v>2171</x:v>
       </x:c>
       <x:c r="I36" s="134" t="s">
         <x:v>1312</x:v>
@@ -53829,7 +53834,7 @@
         <x:v>990</x:v>
       </x:c>
       <x:c r="H37" s="314" t="s">
-        <x:v>2171</x:v>
+        <x:v>2172</x:v>
       </x:c>
       <x:c r="I37" s="134"/>
       <x:c r="J37" s="9"/>
@@ -53865,7 +53870,7 @@
         <x:v>1314</x:v>
       </x:c>
       <x:c r="D39" s="134" t="s">
-        <x:v>2172</x:v>
+        <x:v>2173</x:v>
       </x:c>
       <x:c r="E39" s="134" t="s">
         <x:v>1311</x:v>
@@ -53874,10 +53879,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G39" s="319" t="s">
-        <x:v>2173</x:v>
+        <x:v>2174</x:v>
       </x:c>
       <x:c r="H39" s="297" t="s">
-        <x:v>2174</x:v>
+        <x:v>2175</x:v>
       </x:c>
       <x:c r="I39" s="134" t="s">
         <x:v>1317</x:v>
@@ -53899,7 +53904,7 @@
         <x:v>990</x:v>
       </x:c>
       <x:c r="H40" s="314" t="s">
-        <x:v>2171</x:v>
+        <x:v>2172</x:v>
       </x:c>
       <x:c r="I40" s="134"/>
       <x:c r="J40" s="9"/>
@@ -56835,17 +56840,17 @@
     <x:mergeCell ref="J168:J171"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H22" r:id="rId148"/>
-    <x:hyperlink ref="H28" r:id="rId149"/>
-    <x:hyperlink ref="H11" r:id="rId150"/>
-    <x:hyperlink ref="H16" r:id="rId151"/>
-    <x:hyperlink ref="H37" r:id="rId152"/>
-    <x:hyperlink ref="H40" r:id="rId153"/>
-    <x:hyperlink ref="H130" r:id="rId154"/>
-    <x:hyperlink ref="H136" r:id="rId155"/>
-    <x:hyperlink ref="H142" r:id="rId156"/>
-    <x:hyperlink ref="H148" r:id="rId157"/>
-    <x:hyperlink ref="H154" r:id="rId158"/>
+    <x:hyperlink ref="H22" r:id="rId150"/>
+    <x:hyperlink ref="H28" r:id="rId151"/>
+    <x:hyperlink ref="H11" r:id="rId152"/>
+    <x:hyperlink ref="H16" r:id="rId153"/>
+    <x:hyperlink ref="H37" r:id="rId154"/>
+    <x:hyperlink ref="H40" r:id="rId155"/>
+    <x:hyperlink ref="H130" r:id="rId156"/>
+    <x:hyperlink ref="H136" r:id="rId157"/>
+    <x:hyperlink ref="H142" r:id="rId158"/>
+    <x:hyperlink ref="H148" r:id="rId159"/>
+    <x:hyperlink ref="H154" r:id="rId160"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -56879,40 +56884,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:12">
-      <x:c r="A1" s="396" t="s">
+      <x:c r="A1" s="397" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B1" s="396" t="s">
+      <x:c r="B1" s="397" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="C1" s="396" t="s">
+      <x:c r="C1" s="397" t="s">
         <x:v>403</x:v>
       </x:c>
-      <x:c r="D1" s="396" t="s">
+      <x:c r="D1" s="397" t="s">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="E1" s="396" t="s">
+      <x:c r="E1" s="397" t="s">
         <x:v>405</x:v>
       </x:c>
-      <x:c r="F1" s="397" t="s">
+      <x:c r="F1" s="398" t="s">
         <x:v>406</x:v>
       </x:c>
-      <x:c r="G1" s="396" t="s">
+      <x:c r="G1" s="397" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="H1" s="396" t="s">
+      <x:c r="H1" s="397" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="I1" s="396" t="s">
+      <x:c r="I1" s="397" t="s">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="J1" s="396" t="s">
+      <x:c r="J1" s="397" t="s">
         <x:v>410</x:v>
       </x:c>
-      <x:c r="K1" s="396" t="s">
+      <x:c r="K1" s="397" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="L1" s="396" t="s">
+      <x:c r="L1" s="397" t="s">
         <x:v>2005</x:v>
       </x:c>
     </x:row>
@@ -56930,19 +56935,19 @@
         <x:v>705</x:v>
       </x:c>
       <x:c r="E2" s="116" t="s">
-        <x:v>2175</x:v>
+        <x:v>2176</x:v>
       </x:c>
       <x:c r="F2" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G2" s="327" t="s">
-        <x:v>2176</x:v>
+        <x:v>2177</x:v>
       </x:c>
       <x:c r="H2" s="116" t="s">
-        <x:v>2177</x:v>
+        <x:v>2178</x:v>
       </x:c>
       <x:c r="I2" s="289" t="s">
-        <x:v>2178</x:v>
+        <x:v>2179</x:v>
       </x:c>
       <x:c r="J2" s="1"/>
       <x:c r="K2" s="1"/>
@@ -56958,11 +56963,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G3" s="327" t="s">
-        <x:v>2179</x:v>
+        <x:v>2180</x:v>
       </x:c>
       <x:c r="H3" s="116"/>
       <x:c r="I3" s="289" t="s">
-        <x:v>2180</x:v>
+        <x:v>2181</x:v>
       </x:c>
       <x:c r="J3" s="1"/>
       <x:c r="K3" s="1"/>
@@ -56982,19 +56987,19 @@
         <x:v>707</x:v>
       </x:c>
       <x:c r="E4" s="116" t="s">
-        <x:v>2175</x:v>
+        <x:v>2176</x:v>
       </x:c>
       <x:c r="F4" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="327" t="s">
-        <x:v>2181</x:v>
+        <x:v>2182</x:v>
       </x:c>
       <x:c r="H4" s="116" t="s">
-        <x:v>2182</x:v>
+        <x:v>2183</x:v>
       </x:c>
       <x:c r="I4" s="289" t="s">
-        <x:v>2183</x:v>
+        <x:v>2184</x:v>
       </x:c>
       <x:c r="J4" s="61"/>
       <x:c r="K4" s="1"/>
@@ -57010,11 +57015,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G5" s="327" t="s">
-        <x:v>2184</x:v>
+        <x:v>2185</x:v>
       </x:c>
       <x:c r="H5" s="116"/>
       <x:c r="I5" s="289" t="s">
-        <x:v>2185</x:v>
+        <x:v>2186</x:v>
       </x:c>
       <x:c r="J5" s="61"/>
       <x:c r="K5" s="1"/>
@@ -57030,11 +57035,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G6" s="327" t="s">
-        <x:v>2078</x:v>
+        <x:v>2079</x:v>
       </x:c>
       <x:c r="H6" s="116"/>
       <x:c r="I6" s="289" t="s">
-        <x:v>2186</x:v>
+        <x:v>2187</x:v>
       </x:c>
       <x:c r="J6" s="61"/>
       <x:c r="K6" s="1"/>
@@ -57054,19 +57059,19 @@
         <x:v>709</x:v>
       </x:c>
       <x:c r="E7" s="116" t="s">
-        <x:v>2187</x:v>
+        <x:v>2188</x:v>
       </x:c>
       <x:c r="F7" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="327" t="s">
-        <x:v>2188</x:v>
+        <x:v>2189</x:v>
       </x:c>
       <x:c r="H7" s="116" t="s">
-        <x:v>2189</x:v>
+        <x:v>2190</x:v>
       </x:c>
       <x:c r="I7" s="289" t="s">
-        <x:v>2190</x:v>
+        <x:v>2191</x:v>
       </x:c>
       <x:c r="J7" s="61"/>
       <x:c r="K7" s="1"/>
@@ -57082,11 +57087,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G8" s="327" t="s">
-        <x:v>2078</x:v>
+        <x:v>2079</x:v>
       </x:c>
       <x:c r="H8" s="116"/>
       <x:c r="I8" s="289" t="s">
-        <x:v>2191</x:v>
+        <x:v>2192</x:v>
       </x:c>
       <x:c r="J8" s="61"/>
       <x:c r="K8" s="1"/>
@@ -57102,11 +57107,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G9" s="327" t="s">
-        <x:v>2192</x:v>
+        <x:v>2193</x:v>
       </x:c>
       <x:c r="H9" s="116"/>
       <x:c r="I9" s="289" t="s">
-        <x:v>2193</x:v>
+        <x:v>2194</x:v>
       </x:c>
       <x:c r="J9" s="61"/>
       <x:c r="K9" s="1"/>
@@ -57123,20 +57128,20 @@
         <x:v>717</x:v>
       </x:c>
       <x:c r="D10" s="116" t="s">
-        <x:v>2194</x:v>
+        <x:v>2195</x:v>
       </x:c>
       <x:c r="E10" s="116" t="s">
-        <x:v>2195</x:v>
+        <x:v>2196</x:v>
       </x:c>
       <x:c r="F10" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="327" t="s">
-        <x:v>2099</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="H10" s="116"/>
       <x:c r="I10" s="289" t="s">
-        <x:v>2196</x:v>
+        <x:v>2197</x:v>
       </x:c>
       <x:c r="J10" s="61"/>
       <x:c r="K10" s="1"/>
@@ -57152,11 +57157,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G11" s="327" t="s">
-        <x:v>2197</x:v>
+        <x:v>2198</x:v>
       </x:c>
       <x:c r="H11" s="116"/>
       <x:c r="I11" s="289" t="s">
-        <x:v>2198</x:v>
+        <x:v>2199</x:v>
       </x:c>
       <x:c r="J11" s="61"/>
       <x:c r="K11" s="1"/>
@@ -57172,11 +57177,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G12" s="327" t="s">
-        <x:v>2199</x:v>
+        <x:v>2200</x:v>
       </x:c>
       <x:c r="H12" s="116"/>
       <x:c r="I12" s="289" t="s">
-        <x:v>2200</x:v>
+        <x:v>2201</x:v>
       </x:c>
       <x:c r="J12" s="61"/>
       <x:c r="K12" s="1"/>
@@ -57193,20 +57198,20 @@
         <x:v>722</x:v>
       </x:c>
       <x:c r="D13" s="116" t="s">
-        <x:v>2201</x:v>
+        <x:v>2202</x:v>
       </x:c>
       <x:c r="E13" s="116" t="s">
-        <x:v>2202</x:v>
+        <x:v>2203</x:v>
       </x:c>
       <x:c r="F13" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="327" t="s">
-        <x:v>2078</x:v>
+        <x:v>2079</x:v>
       </x:c>
       <x:c r="H13" s="116"/>
       <x:c r="I13" s="289" t="s">
-        <x:v>2203</x:v>
+        <x:v>2204</x:v>
       </x:c>
       <x:c r="J13" s="61"/>
       <x:c r="K13" s="1"/>
@@ -57222,11 +57227,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="327" t="s">
-        <x:v>2204</x:v>
+        <x:v>2205</x:v>
       </x:c>
       <x:c r="H14" s="116"/>
       <x:c r="I14" s="289" t="s">
-        <x:v>2205</x:v>
+        <x:v>2206</x:v>
       </x:c>
       <x:c r="J14" s="61"/>
       <x:c r="K14" s="1"/>
@@ -57243,22 +57248,22 @@
         <x:v>724</x:v>
       </x:c>
       <x:c r="D15" s="116" t="s">
-        <x:v>2206</x:v>
+        <x:v>2207</x:v>
       </x:c>
       <x:c r="E15" s="116" t="s">
-        <x:v>2207</x:v>
+        <x:v>2208</x:v>
       </x:c>
       <x:c r="F15" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G15" s="327" t="s">
-        <x:v>2208</x:v>
+        <x:v>2209</x:v>
       </x:c>
       <x:c r="H15" s="116" t="s">
-        <x:v>2209</x:v>
+        <x:v>2210</x:v>
       </x:c>
       <x:c r="I15" s="289" t="s">
-        <x:v>2210</x:v>
+        <x:v>2211</x:v>
       </x:c>
       <x:c r="J15" s="61"/>
       <x:c r="K15" s="1"/>
@@ -57274,11 +57279,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G16" s="327" t="s">
-        <x:v>2211</x:v>
+        <x:v>2212</x:v>
       </x:c>
       <x:c r="H16" s="116"/>
       <x:c r="I16" s="289" t="s">
-        <x:v>2212</x:v>
+        <x:v>2213</x:v>
       </x:c>
       <x:c r="J16" s="61"/>
       <x:c r="K16" s="1"/>
@@ -57294,11 +57299,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G17" s="327" t="s">
-        <x:v>2213</x:v>
+        <x:v>2214</x:v>
       </x:c>
       <x:c r="H17" s="116"/>
       <x:c r="I17" s="289" t="s">
-        <x:v>2214</x:v>
+        <x:v>2215</x:v>
       </x:c>
       <x:c r="J17" s="61"/>
       <x:c r="K17" s="1"/>
@@ -57315,20 +57320,20 @@
         <x:v>726</x:v>
       </x:c>
       <x:c r="D18" s="116" t="s">
-        <x:v>2215</x:v>
+        <x:v>2216</x:v>
       </x:c>
       <x:c r="E18" s="116" t="s">
-        <x:v>2216</x:v>
+        <x:v>2217</x:v>
       </x:c>
       <x:c r="F18" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="327" t="s">
-        <x:v>2217</x:v>
+        <x:v>2218</x:v>
       </x:c>
       <x:c r="H18" s="116"/>
       <x:c r="I18" s="289" t="s">
-        <x:v>2218</x:v>
+        <x:v>2219</x:v>
       </x:c>
       <x:c r="J18" s="61"/>
       <x:c r="K18" s="1"/>
@@ -57344,13 +57349,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="327" t="s">
-        <x:v>2219</x:v>
+        <x:v>2220</x:v>
       </x:c>
       <x:c r="H19" s="116" t="s">
-        <x:v>2220</x:v>
+        <x:v>2221</x:v>
       </x:c>
       <x:c r="I19" s="289" t="s">
-        <x:v>2221</x:v>
+        <x:v>2222</x:v>
       </x:c>
       <x:c r="J19" s="61"/>
       <x:c r="K19" s="1"/>
@@ -57366,11 +57371,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="327" t="s">
-        <x:v>2222</x:v>
+        <x:v>2223</x:v>
       </x:c>
       <x:c r="H20" s="116"/>
       <x:c r="I20" s="289" t="s">
-        <x:v>2223</x:v>
+        <x:v>2224</x:v>
       </x:c>
       <x:c r="J20" s="61"/>
       <x:c r="K20" s="1"/>
@@ -57381,7 +57386,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B21" s="116" t="s">
-        <x:v>2224</x:v>
+        <x:v>2225</x:v>
       </x:c>
       <x:c r="C21" s="116" t="s">
         <x:v>732</x:v>
@@ -57390,19 +57395,19 @@
         <x:v>733</x:v>
       </x:c>
       <x:c r="E21" s="116" t="s">
-        <x:v>2225</x:v>
+        <x:v>2226</x:v>
       </x:c>
       <x:c r="F21" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G21" s="327" t="s">
-        <x:v>2226</x:v>
+        <x:v>2227</x:v>
       </x:c>
       <x:c r="H21" s="116" t="s">
         <x:v>741</x:v>
       </x:c>
       <x:c r="I21" s="289" t="s">
-        <x:v>2227</x:v>
+        <x:v>2228</x:v>
       </x:c>
       <x:c r="J21" s="61"/>
       <x:c r="K21" s="1"/>
@@ -57418,11 +57423,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G22" s="327" t="s">
-        <x:v>2228</x:v>
+        <x:v>2229</x:v>
       </x:c>
       <x:c r="H22" s="116"/>
       <x:c r="I22" s="289" t="s">
-        <x:v>2229</x:v>
+        <x:v>2230</x:v>
       </x:c>
       <x:c r="J22" s="61"/>
       <x:c r="K22" s="1"/>
@@ -57438,11 +57443,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G23" s="327" t="s">
-        <x:v>2230</x:v>
+        <x:v>2231</x:v>
       </x:c>
       <x:c r="H23" s="116"/>
       <x:c r="I23" s="289" t="s">
-        <x:v>2231</x:v>
+        <x:v>2232</x:v>
       </x:c>
       <x:c r="J23" s="61"/>
       <x:c r="K23" s="1"/>
@@ -57459,20 +57464,20 @@
         <x:v>737</x:v>
       </x:c>
       <x:c r="D24" s="116" t="s">
-        <x:v>2232</x:v>
+        <x:v>2233</x:v>
       </x:c>
       <x:c r="E24" s="116" t="s">
-        <x:v>2233</x:v>
+        <x:v>2234</x:v>
       </x:c>
       <x:c r="F24" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G24" s="327" t="s">
-        <x:v>2234</x:v>
+        <x:v>2235</x:v>
       </x:c>
       <x:c r="H24" s="116"/>
       <x:c r="I24" s="289" t="s">
-        <x:v>2235</x:v>
+        <x:v>2236</x:v>
       </x:c>
       <x:c r="J24" s="61"/>
       <x:c r="K24" s="35"/>
@@ -57488,11 +57493,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G25" s="327" t="s">
-        <x:v>2236</x:v>
+        <x:v>2237</x:v>
       </x:c>
       <x:c r="H25" s="116"/>
       <x:c r="I25" s="289" t="s">
-        <x:v>2237</x:v>
+        <x:v>2238</x:v>
       </x:c>
       <x:c r="J25" s="61"/>
       <x:c r="K25" s="35"/>
@@ -57508,11 +57513,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G26" s="327" t="s">
-        <x:v>2129</x:v>
+        <x:v>2130</x:v>
       </x:c>
       <x:c r="H26" s="116"/>
       <x:c r="I26" s="289" t="s">
-        <x:v>2238</x:v>
+        <x:v>2239</x:v>
       </x:c>
       <x:c r="J26" s="61"/>
       <x:c r="K26" s="35"/>
@@ -57529,20 +57534,20 @@
         <x:v>751</x:v>
       </x:c>
       <x:c r="D27" s="116" t="s">
-        <x:v>2239</x:v>
+        <x:v>2240</x:v>
       </x:c>
       <x:c r="E27" s="116" t="s">
-        <x:v>2240</x:v>
+        <x:v>2241</x:v>
       </x:c>
       <x:c r="F27" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G27" s="327" t="s">
-        <x:v>2241</x:v>
+        <x:v>2242</x:v>
       </x:c>
       <x:c r="H27" s="116"/>
       <x:c r="I27" s="327" t="s">
-        <x:v>2084</x:v>
+        <x:v>2085</x:v>
       </x:c>
       <x:c r="J27" s="61"/>
       <x:c r="K27" s="35"/>
@@ -57558,11 +57563,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G28" s="327" t="s">
-        <x:v>2242</x:v>
+        <x:v>2243</x:v>
       </x:c>
       <x:c r="H28" s="116"/>
       <x:c r="I28" s="289" t="s">
-        <x:v>2243</x:v>
+        <x:v>2244</x:v>
       </x:c>
       <x:c r="J28" s="61"/>
       <x:c r="K28" s="35"/>
@@ -57579,20 +57584,20 @@
         <x:v>753</x:v>
       </x:c>
       <x:c r="D29" s="116" t="s">
-        <x:v>2244</x:v>
+        <x:v>2245</x:v>
       </x:c>
       <x:c r="E29" s="116" t="s">
-        <x:v>2240</x:v>
+        <x:v>2241</x:v>
       </x:c>
       <x:c r="F29" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G29" s="327" t="s">
-        <x:v>2245</x:v>
+        <x:v>2246</x:v>
       </x:c>
       <x:c r="H29" s="116"/>
       <x:c r="I29" s="327" t="s">
-        <x:v>2084</x:v>
+        <x:v>2085</x:v>
       </x:c>
       <x:c r="J29" s="61"/>
       <x:c r="K29" s="35"/>
@@ -57608,11 +57613,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G30" s="327" t="s">
-        <x:v>2246</x:v>
+        <x:v>2247</x:v>
       </x:c>
       <x:c r="H30" s="116"/>
       <x:c r="I30" s="289" t="s">
-        <x:v>2247</x:v>
+        <x:v>2248</x:v>
       </x:c>
       <x:c r="J30" s="61"/>
       <x:c r="K30" s="35"/>
@@ -57632,19 +57637,19 @@
         <x:v>793</x:v>
       </x:c>
       <x:c r="E31" s="116" t="s">
-        <x:v>2248</x:v>
+        <x:v>2249</x:v>
       </x:c>
       <x:c r="F31" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="327" t="s">
-        <x:v>2249</x:v>
+        <x:v>2250</x:v>
       </x:c>
       <x:c r="H31" s="116" t="s">
-        <x:v>2250</x:v>
+        <x:v>2251</x:v>
       </x:c>
       <x:c r="I31" s="289" t="s">
-        <x:v>2251</x:v>
+        <x:v>2252</x:v>
       </x:c>
       <x:c r="J31" s="61"/>
       <x:c r="K31" s="35"/>
@@ -57660,11 +57665,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G32" s="327" t="s">
-        <x:v>2252</x:v>
+        <x:v>2253</x:v>
       </x:c>
       <x:c r="H32" s="116"/>
       <x:c r="I32" s="289" t="s">
-        <x:v>2253</x:v>
+        <x:v>2254</x:v>
       </x:c>
       <x:c r="J32" s="61"/>
       <x:c r="K32" s="35"/>
@@ -57684,19 +57689,19 @@
         <x:v>798</x:v>
       </x:c>
       <x:c r="E33" s="116" t="s">
-        <x:v>2254</x:v>
+        <x:v>2255</x:v>
       </x:c>
       <x:c r="F33" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G33" s="327" t="s">
-        <x:v>2255</x:v>
+        <x:v>2256</x:v>
       </x:c>
       <x:c r="H33" s="116" t="s">
-        <x:v>2250</x:v>
+        <x:v>2251</x:v>
       </x:c>
       <x:c r="I33" s="327" t="s">
-        <x:v>2084</x:v>
+        <x:v>2085</x:v>
       </x:c>
       <x:c r="J33" s="61"/>
       <x:c r="K33" s="35"/>
@@ -57712,11 +57717,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G34" s="327" t="s">
-        <x:v>2256</x:v>
+        <x:v>2257</x:v>
       </x:c>
       <x:c r="H34" s="116"/>
       <x:c r="I34" s="289" t="s">
-        <x:v>2257</x:v>
+        <x:v>2258</x:v>
       </x:c>
       <x:c r="J34" s="292"/>
       <x:c r="K34" s="35"/>
@@ -57733,20 +57738,20 @@
         <x:v>802</x:v>
       </x:c>
       <x:c r="D35" s="116" t="s">
-        <x:v>2258</x:v>
+        <x:v>2259</x:v>
       </x:c>
       <x:c r="E35" s="116" t="s">
-        <x:v>2259</x:v>
+        <x:v>2260</x:v>
       </x:c>
       <x:c r="F35" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G35" s="327" t="s">
-        <x:v>2260</x:v>
+        <x:v>2261</x:v>
       </x:c>
       <x:c r="H35" s="116"/>
       <x:c r="I35" s="289" t="s">
-        <x:v>2261</x:v>
+        <x:v>2262</x:v>
       </x:c>
       <x:c r="J35" s="61"/>
       <x:c r="K35" s="35"/>
@@ -57762,11 +57767,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G36" s="327" t="s">
-        <x:v>2262</x:v>
+        <x:v>2263</x:v>
       </x:c>
       <x:c r="H36" s="116"/>
       <x:c r="I36" s="289" t="s">
-        <x:v>2263</x:v>
+        <x:v>2264</x:v>
       </x:c>
       <x:c r="J36" s="61"/>
       <x:c r="K36" s="35"/>
@@ -57782,13 +57787,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G37" s="327" t="s">
-        <x:v>2264</x:v>
+        <x:v>2265</x:v>
       </x:c>
       <x:c r="H37" s="116" t="s">
-        <x:v>2265</x:v>
+        <x:v>2266</x:v>
       </x:c>
       <x:c r="I37" s="289" t="s">
-        <x:v>2266</x:v>
+        <x:v>2267</x:v>
       </x:c>
       <x:c r="J37" s="61"/>
       <x:c r="K37" s="35"/>
@@ -57805,20 +57810,20 @@
         <x:v>814</x:v>
       </x:c>
       <x:c r="D38" s="116" t="s">
-        <x:v>2267</x:v>
+        <x:v>2268</x:v>
       </x:c>
       <x:c r="E38" s="116" t="s">
-        <x:v>2268</x:v>
+        <x:v>2269</x:v>
       </x:c>
       <x:c r="F38" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G38" s="327" t="s">
-        <x:v>2269</x:v>
+        <x:v>2270</x:v>
       </x:c>
       <x:c r="H38" s="116"/>
       <x:c r="I38" s="289" t="s">
-        <x:v>2270</x:v>
+        <x:v>2271</x:v>
       </x:c>
       <x:c r="J38" s="61"/>
       <x:c r="K38" s="35"/>
@@ -57834,11 +57839,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G39" s="327" t="s">
-        <x:v>2271</x:v>
+        <x:v>2272</x:v>
       </x:c>
       <x:c r="H39" s="116"/>
       <x:c r="I39" s="289" t="s">
-        <x:v>2272</x:v>
+        <x:v>2273</x:v>
       </x:c>
       <x:c r="J39" s="61"/>
       <x:c r="K39" s="35"/>
@@ -57854,13 +57859,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G40" s="327" t="s">
-        <x:v>2273</x:v>
+        <x:v>2274</x:v>
       </x:c>
       <x:c r="H40" s="116" t="s">
-        <x:v>2265</x:v>
+        <x:v>2266</x:v>
       </x:c>
       <x:c r="I40" s="289" t="s">
-        <x:v>2274</x:v>
+        <x:v>2275</x:v>
       </x:c>
       <x:c r="J40" s="61"/>
       <x:c r="K40" s="35"/>
@@ -57876,11 +57881,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G41" s="327" t="s">
-        <x:v>2275</x:v>
+        <x:v>2276</x:v>
       </x:c>
       <x:c r="H41" s="116"/>
       <x:c r="I41" s="289" t="s">
-        <x:v>2276</x:v>
+        <x:v>2277</x:v>
       </x:c>
       <x:c r="J41" s="61"/>
       <x:c r="K41" s="35"/>
@@ -57897,20 +57902,20 @@
         <x:v>824</x:v>
       </x:c>
       <x:c r="D42" s="116" t="s">
-        <x:v>2277</x:v>
+        <x:v>2278</x:v>
       </x:c>
       <x:c r="E42" s="116" t="s">
-        <x:v>2278</x:v>
+        <x:v>2279</x:v>
       </x:c>
       <x:c r="F42" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G42" s="327" t="s">
-        <x:v>2279</x:v>
+        <x:v>2280</x:v>
       </x:c>
       <x:c r="H42" s="116"/>
       <x:c r="I42" s="289" t="s">
-        <x:v>2280</x:v>
+        <x:v>2281</x:v>
       </x:c>
       <x:c r="J42" s="61"/>
       <x:c r="K42" s="35"/>
@@ -57926,11 +57931,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G43" s="327" t="s">
-        <x:v>2281</x:v>
+        <x:v>2282</x:v>
       </x:c>
       <x:c r="H43" s="116"/>
       <x:c r="I43" s="289" t="s">
-        <x:v>2282</x:v>
+        <x:v>2283</x:v>
       </x:c>
       <x:c r="J43" s="61"/>
       <x:c r="K43" s="35"/>
@@ -57946,11 +57951,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G44" s="327" t="s">
-        <x:v>2283</x:v>
+        <x:v>2284</x:v>
       </x:c>
       <x:c r="H44" s="116"/>
       <x:c r="I44" s="289" t="s">
-        <x:v>2284</x:v>
+        <x:v>2285</x:v>
       </x:c>
       <x:c r="J44" s="61"/>
       <x:c r="K44" s="35"/>
@@ -57966,11 +57971,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G45" s="327" t="s">
-        <x:v>2285</x:v>
+        <x:v>2286</x:v>
       </x:c>
       <x:c r="H45" s="116"/>
       <x:c r="I45" s="289" t="s">
-        <x:v>2286</x:v>
+        <x:v>2287</x:v>
       </x:c>
       <x:c r="J45" s="61"/>
       <x:c r="K45" s="35"/>
@@ -57987,20 +57992,20 @@
         <x:v>835</x:v>
       </x:c>
       <x:c r="D46" s="116" t="s">
-        <x:v>2287</x:v>
+        <x:v>2288</x:v>
       </x:c>
       <x:c r="E46" s="116" t="s">
-        <x:v>2288</x:v>
+        <x:v>2289</x:v>
       </x:c>
       <x:c r="F46" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G46" s="327" t="s">
-        <x:v>2279</x:v>
+        <x:v>2280</x:v>
       </x:c>
       <x:c r="H46" s="116"/>
       <x:c r="I46" s="289" t="s">
-        <x:v>2289</x:v>
+        <x:v>2290</x:v>
       </x:c>
       <x:c r="J46" s="61"/>
       <x:c r="K46" s="35"/>
@@ -58016,13 +58021,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G47" s="327" t="s">
-        <x:v>2290</x:v>
+        <x:v>2291</x:v>
       </x:c>
       <x:c r="H47" s="116" t="s">
-        <x:v>2265</x:v>
+        <x:v>2266</x:v>
       </x:c>
       <x:c r="I47" s="289" t="s">
-        <x:v>2291</x:v>
+        <x:v>2292</x:v>
       </x:c>
       <x:c r="J47" s="61"/>
       <x:c r="K47" s="35"/>
@@ -58038,11 +58043,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G48" s="327" t="s">
-        <x:v>2292</x:v>
+        <x:v>2293</x:v>
       </x:c>
       <x:c r="H48" s="116"/>
       <x:c r="I48" s="289" t="s">
-        <x:v>2293</x:v>
+        <x:v>2294</x:v>
       </x:c>
       <x:c r="J48" s="61"/>
       <x:c r="K48" s="35"/>
@@ -58141,10 +58146,10 @@
         <x:v>999</x:v>
       </x:c>
       <x:c r="H52" s="334" t="s">
-        <x:v>2294</x:v>
+        <x:v>2295</x:v>
       </x:c>
       <x:c r="I52" s="51" t="s">
-        <x:v>2295</x:v>
+        <x:v>2296</x:v>
       </x:c>
       <x:c r="J52" s="51"/>
       <x:c r="K52" s="35"/>
@@ -58163,7 +58168,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H53" s="314" t="s">
-        <x:v>2296</x:v>
+        <x:v>2297</x:v>
       </x:c>
       <x:c r="I53" s="51"/>
       <x:c r="J53" s="51"/>
@@ -58214,7 +58219,7 @@
         <x:v>1000</x:v>
       </x:c>
       <x:c r="I55" s="51" t="s">
-        <x:v>2297</x:v>
+        <x:v>2298</x:v>
       </x:c>
       <x:c r="J55" s="51"/>
       <x:c r="K55" s="35"/>
@@ -58233,7 +58238,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H56" s="314" t="s">
-        <x:v>2298</x:v>
+        <x:v>2299</x:v>
       </x:c>
       <x:c r="I56" s="51"/>
       <x:c r="J56" s="51"/>
@@ -58352,7 +58357,7 @@
         <x:v>422</x:v>
       </x:c>
       <x:c r="I61" s="51" t="s">
-        <x:v>2299</x:v>
+        <x:v>2300</x:v>
       </x:c>
       <x:c r="J61" s="51"/>
       <x:c r="K61" s="35"/>
@@ -58650,7 +58655,7 @@
         <x:v>1037</x:v>
       </x:c>
       <x:c r="I74" s="51" t="s">
-        <x:v>2300</x:v>
+        <x:v>2301</x:v>
       </x:c>
       <x:c r="J74" s="51"/>
       <x:c r="K74" s="35"/>
@@ -59346,19 +59351,19 @@
         <x:v>843</x:v>
       </x:c>
       <x:c r="E106" s="116" t="s">
-        <x:v>2301</x:v>
+        <x:v>2302</x:v>
       </x:c>
       <x:c r="F106" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G106" s="327" t="s">
-        <x:v>2302</x:v>
+        <x:v>2303</x:v>
       </x:c>
       <x:c r="H106" s="116" t="s">
-        <x:v>2303</x:v>
+        <x:v>2304</x:v>
       </x:c>
       <x:c r="I106" s="289" t="s">
-        <x:v>2304</x:v>
+        <x:v>2305</x:v>
       </x:c>
       <x:c r="J106" s="61"/>
       <x:c r="K106" s="140"/>
@@ -59374,11 +59379,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G107" s="327" t="s">
-        <x:v>2305</x:v>
+        <x:v>2306</x:v>
       </x:c>
       <x:c r="H107" s="116"/>
       <x:c r="I107" s="289" t="s">
-        <x:v>2306</x:v>
+        <x:v>2307</x:v>
       </x:c>
       <x:c r="J107" s="61"/>
       <x:c r="K107" s="140"/>
@@ -59394,13 +59399,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G108" s="327" t="s">
-        <x:v>2307</x:v>
+        <x:v>2308</x:v>
       </x:c>
       <x:c r="H108" s="116" t="s">
-        <x:v>2308</x:v>
+        <x:v>2309</x:v>
       </x:c>
       <x:c r="I108" s="289" t="s">
-        <x:v>2309</x:v>
+        <x:v>2310</x:v>
       </x:c>
       <x:c r="J108" s="61"/>
       <x:c r="K108" s="140"/>
@@ -59416,11 +59421,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G109" s="327" t="s">
-        <x:v>2310</x:v>
+        <x:v>2311</x:v>
       </x:c>
       <x:c r="H109" s="116"/>
       <x:c r="I109" s="289" t="s">
-        <x:v>2311</x:v>
+        <x:v>2312</x:v>
       </x:c>
       <x:c r="J109" s="61"/>
       <x:c r="K109" s="140"/>
@@ -59440,19 +59445,19 @@
         <x:v>854</x:v>
       </x:c>
       <x:c r="E110" s="116" t="s">
-        <x:v>2312</x:v>
+        <x:v>2313</x:v>
       </x:c>
       <x:c r="F110" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G110" s="327" t="s">
-        <x:v>2313</x:v>
+        <x:v>2314</x:v>
       </x:c>
       <x:c r="H110" s="116" t="s">
-        <x:v>2314</x:v>
+        <x:v>2315</x:v>
       </x:c>
       <x:c r="I110" s="289" t="s">
-        <x:v>2315</x:v>
+        <x:v>2316</x:v>
       </x:c>
       <x:c r="J110" s="61"/>
       <x:c r="K110" s="140"/>
@@ -59468,11 +59473,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G111" s="327" t="s">
-        <x:v>2305</x:v>
+        <x:v>2306</x:v>
       </x:c>
       <x:c r="H111" s="116"/>
       <x:c r="I111" s="289" t="s">
-        <x:v>2316</x:v>
+        <x:v>2317</x:v>
       </x:c>
       <x:c r="J111" s="61"/>
       <x:c r="K111" s="140"/>
@@ -59488,13 +59493,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G112" s="327" t="s">
-        <x:v>2317</x:v>
+        <x:v>2318</x:v>
       </x:c>
       <x:c r="H112" s="116" t="s">
-        <x:v>2318</x:v>
+        <x:v>2319</x:v>
       </x:c>
       <x:c r="I112" s="289" t="s">
-        <x:v>2319</x:v>
+        <x:v>2320</x:v>
       </x:c>
       <x:c r="J112" s="61"/>
       <x:c r="K112" s="140"/>
@@ -59510,11 +59515,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G113" s="327" t="s">
-        <x:v>2320</x:v>
+        <x:v>2321</x:v>
       </x:c>
       <x:c r="H113" s="116"/>
       <x:c r="I113" s="289" t="s">
-        <x:v>2321</x:v>
+        <x:v>2322</x:v>
       </x:c>
       <x:c r="J113" s="61"/>
       <x:c r="K113" s="140"/>
@@ -59531,7 +59536,7 @@
         <x:v>863</x:v>
       </x:c>
       <x:c r="D114" s="140" t="s">
-        <x:v>2322</x:v>
+        <x:v>2323</x:v>
       </x:c>
       <x:c r="E114" s="140" t="s">
         <x:v>865</x:v>
@@ -59540,7 +59545,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G114" s="61" t="s">
-        <x:v>2323</x:v>
+        <x:v>2324</x:v>
       </x:c>
       <x:c r="H114" s="140"/>
       <x:c r="I114" s="61" t="s">
@@ -59560,7 +59565,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G115" s="61" t="s">
-        <x:v>2324</x:v>
+        <x:v>2325</x:v>
       </x:c>
       <x:c r="H115" s="140"/>
       <x:c r="I115" s="61" t="s">
@@ -59580,10 +59585,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G116" s="61" t="s">
-        <x:v>2325</x:v>
+        <x:v>2326</x:v>
       </x:c>
       <x:c r="H116" s="140" t="s">
-        <x:v>2326</x:v>
+        <x:v>2327</x:v>
       </x:c>
       <x:c r="I116" s="61"/>
       <x:c r="J116" s="140"/>
@@ -59600,10 +59605,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G117" s="61" t="s">
-        <x:v>2327</x:v>
+        <x:v>2328</x:v>
       </x:c>
       <x:c r="H117" s="140" t="s">
-        <x:v>2328</x:v>
+        <x:v>2329</x:v>
       </x:c>
       <x:c r="I117" s="61"/>
       <x:c r="J117" s="140"/>
@@ -59638,7 +59643,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G119" s="61" t="s">
-        <x:v>2329</x:v>
+        <x:v>2330</x:v>
       </x:c>
       <x:c r="H119" s="140" t="s">
         <x:v>877</x:v>
@@ -59658,7 +59663,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G120" s="61" t="s">
-        <x:v>2330</x:v>
+        <x:v>2331</x:v>
       </x:c>
       <x:c r="H120" s="251">
         <x:v>0.375</x:v>
@@ -59678,7 +59683,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G121" s="61" t="s">
-        <x:v>2331</x:v>
+        <x:v>2332</x:v>
       </x:c>
       <x:c r="H121" s="140">
         <x:v>100000</x:v>
@@ -59698,7 +59703,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="G122" s="61" t="s">
-        <x:v>2332</x:v>
+        <x:v>2333</x:v>
       </x:c>
       <x:c r="H122" s="140">
         <x:v>1</x:v>
@@ -59718,7 +59723,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G123" s="61" t="s">
-        <x:v>2333</x:v>
+        <x:v>2334</x:v>
       </x:c>
       <x:c r="H123" s="140"/>
       <x:c r="I123" s="61" t="s">
@@ -59739,7 +59744,7 @@
         <x:v>884</x:v>
       </x:c>
       <x:c r="D124" s="140" t="s">
-        <x:v>2334</x:v>
+        <x:v>2335</x:v>
       </x:c>
       <x:c r="E124" s="140" t="s">
         <x:v>886</x:v>
@@ -59748,7 +59753,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G124" s="61" t="s">
-        <x:v>2335</x:v>
+        <x:v>2336</x:v>
       </x:c>
       <x:c r="H124" s="140"/>
       <x:c r="I124" s="140" t="s">
@@ -59768,7 +59773,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G125" s="61" t="s">
-        <x:v>2336</x:v>
+        <x:v>2337</x:v>
       </x:c>
       <x:c r="H125" s="140"/>
       <x:c r="I125" s="140"/>
@@ -59786,10 +59791,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G126" s="61" t="s">
-        <x:v>2337</x:v>
+        <x:v>2338</x:v>
       </x:c>
       <x:c r="H126" s="140" t="s">
-        <x:v>2338</x:v>
+        <x:v>2339</x:v>
       </x:c>
       <x:c r="I126" s="140"/>
       <x:c r="J126" s="140"/>
@@ -59806,10 +59811,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G127" s="61" t="s">
-        <x:v>2339</x:v>
+        <x:v>2340</x:v>
       </x:c>
       <x:c r="H127" s="140" t="s">
-        <x:v>2340</x:v>
+        <x:v>2341</x:v>
       </x:c>
       <x:c r="I127" s="140"/>
       <x:c r="J127" s="140"/>
@@ -59826,7 +59831,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G128" s="61" t="s">
-        <x:v>2341</x:v>
+        <x:v>2342</x:v>
       </x:c>
       <x:c r="H128" s="140" t="s">
         <x:v>877</x:v>
@@ -59864,7 +59869,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G130" s="61" t="s">
-        <x:v>2342</x:v>
+        <x:v>2343</x:v>
       </x:c>
       <x:c r="H130" s="140">
         <x:v>100000</x:v>
@@ -59884,7 +59889,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="G131" s="61" t="s">
-        <x:v>2343</x:v>
+        <x:v>2344</x:v>
       </x:c>
       <x:c r="H131" s="140">
         <x:v>1</x:v>
@@ -59904,7 +59909,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G132" s="61" t="s">
-        <x:v>2344</x:v>
+        <x:v>2345</x:v>
       </x:c>
       <x:c r="H132" s="140"/>
       <x:c r="I132" s="140"/>
@@ -59923,7 +59928,7 @@
         <x:v>900</x:v>
       </x:c>
       <x:c r="D133" s="140" t="s">
-        <x:v>2345</x:v>
+        <x:v>2346</x:v>
       </x:c>
       <x:c r="E133" s="140" t="s">
         <x:v>886</x:v>
@@ -59932,7 +59937,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G133" s="61" t="s">
-        <x:v>2346</x:v>
+        <x:v>2347</x:v>
       </x:c>
       <x:c r="H133" s="140"/>
       <x:c r="I133" s="140" t="s">
@@ -59952,7 +59957,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G134" s="61" t="s">
-        <x:v>2347</x:v>
+        <x:v>2348</x:v>
       </x:c>
       <x:c r="H134" s="140"/>
       <x:c r="I134" s="140"/>
@@ -59970,7 +59975,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G135" s="61" t="s">
-        <x:v>2348</x:v>
+        <x:v>2349</x:v>
       </x:c>
       <x:c r="H135" s="140" t="s">
         <x:v>891</x:v>
@@ -60048,7 +60053,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G139" s="61" t="s">
-        <x:v>2349</x:v>
+        <x:v>2350</x:v>
       </x:c>
       <x:c r="H139" s="140">
         <x:f>1</x:f>
@@ -60068,7 +60073,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G140" s="61" t="s">
-        <x:v>2350</x:v>
+        <x:v>2351</x:v>
       </x:c>
       <x:c r="H140" s="140"/>
       <x:c r="I140" s="140"/>
@@ -60087,7 +60092,7 @@
         <x:v>911</x:v>
       </x:c>
       <x:c r="D141" s="140" t="s">
-        <x:v>2351</x:v>
+        <x:v>2352</x:v>
       </x:c>
       <x:c r="E141" s="140" t="s">
         <x:v>886</x:v>
@@ -60096,7 +60101,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G141" s="61" t="s">
-        <x:v>2352</x:v>
+        <x:v>2353</x:v>
       </x:c>
       <x:c r="H141" s="140"/>
       <x:c r="I141" s="140" t="s">
@@ -60116,7 +60121,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G142" s="61" t="s">
-        <x:v>2353</x:v>
+        <x:v>2354</x:v>
       </x:c>
       <x:c r="H142" s="140"/>
       <x:c r="I142" s="140"/>
@@ -60134,7 +60139,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G143" s="61" t="s">
-        <x:v>2354</x:v>
+        <x:v>2355</x:v>
       </x:c>
       <x:c r="H143" s="140" t="s">
         <x:v>891</x:v>
@@ -60232,7 +60237,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G148" s="61" t="s">
-        <x:v>2355</x:v>
+        <x:v>2356</x:v>
       </x:c>
       <x:c r="H148" s="140"/>
       <x:c r="I148" s="140"/>
@@ -60251,22 +60256,22 @@
         <x:v>921</x:v>
       </x:c>
       <x:c r="D149" s="116" t="s">
-        <x:v>2356</x:v>
+        <x:v>2357</x:v>
       </x:c>
       <x:c r="E149" s="116" t="s">
-        <x:v>2357</x:v>
+        <x:v>2358</x:v>
       </x:c>
       <x:c r="F149" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G149" s="327" t="s">
-        <x:v>2358</x:v>
+        <x:v>2359</x:v>
       </x:c>
       <x:c r="H149" s="116" t="s">
-        <x:v>2359</x:v>
+        <x:v>2360</x:v>
       </x:c>
       <x:c r="I149" s="289" t="s">
-        <x:v>2360</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="J149" s="61"/>
       <x:c r="K149" s="140"/>
@@ -60282,11 +60287,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G150" s="327" t="s">
-        <x:v>2361</x:v>
+        <x:v>2362</x:v>
       </x:c>
       <x:c r="H150" s="116"/>
       <x:c r="I150" s="289" t="s">
-        <x:v>2362</x:v>
+        <x:v>2363</x:v>
       </x:c>
       <x:c r="J150" s="61"/>
       <x:c r="K150" s="140"/>
@@ -60302,13 +60307,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G151" s="327" t="s">
-        <x:v>2363</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="H151" s="116" t="s">
-        <x:v>2364</x:v>
+        <x:v>2365</x:v>
       </x:c>
       <x:c r="I151" s="289" t="s">
-        <x:v>2365</x:v>
+        <x:v>2366</x:v>
       </x:c>
       <x:c r="J151" s="61"/>
       <x:c r="K151" s="140"/>
@@ -60324,11 +60329,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G152" s="327" t="s">
-        <x:v>2366</x:v>
+        <x:v>2367</x:v>
       </x:c>
       <x:c r="H152" s="116"/>
       <x:c r="I152" s="289" t="s">
-        <x:v>2367</x:v>
+        <x:v>2368</x:v>
       </x:c>
       <x:c r="J152" s="61"/>
       <x:c r="K152" s="140"/>
@@ -60344,11 +60349,11 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G153" s="327" t="s">
-        <x:v>2368</x:v>
+        <x:v>2369</x:v>
       </x:c>
       <x:c r="H153" s="116"/>
       <x:c r="I153" s="289" t="s">
-        <x:v>2369</x:v>
+        <x:v>2370</x:v>
       </x:c>
       <x:c r="J153" s="61"/>
       <x:c r="K153" s="140"/>
@@ -60685,17 +60690,17 @@
     <x:mergeCell ref="L149:L153"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H49" r:id="rId159"/>
-    <x:hyperlink ref="H50" r:id="rId160"/>
-    <x:hyperlink ref="H55" r:id="rId161"/>
-    <x:hyperlink ref="H56" r:id="rId162"/>
-    <x:hyperlink ref="H59" r:id="rId163"/>
-    <x:hyperlink ref="H64" r:id="rId164"/>
-    <x:hyperlink ref="H65" r:id="rId165"/>
-    <x:hyperlink ref="H67" r:id="rId166"/>
-    <x:hyperlink ref="H68" r:id="rId167"/>
-    <x:hyperlink ref="H52" r:id="rId168"/>
-    <x:hyperlink ref="H61" r:id="rId169"/>
+    <x:hyperlink ref="H49" r:id="rId161"/>
+    <x:hyperlink ref="H50" r:id="rId162"/>
+    <x:hyperlink ref="H55" r:id="rId163"/>
+    <x:hyperlink ref="H56" r:id="rId164"/>
+    <x:hyperlink ref="H59" r:id="rId165"/>
+    <x:hyperlink ref="H64" r:id="rId166"/>
+    <x:hyperlink ref="H65" r:id="rId167"/>
+    <x:hyperlink ref="H67" r:id="rId168"/>
+    <x:hyperlink ref="H68" r:id="rId169"/>
+    <x:hyperlink ref="H52" r:id="rId170"/>
+    <x:hyperlink ref="H61" r:id="rId171"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -60729,40 +60734,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:12" ht="27.6" customHeight="1">
-      <x:c r="A1" s="396" t="s">
+      <x:c r="A1" s="397" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B1" s="396" t="s">
+      <x:c r="B1" s="397" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="C1" s="396" t="s">
+      <x:c r="C1" s="397" t="s">
         <x:v>403</x:v>
       </x:c>
-      <x:c r="D1" s="396" t="s">
+      <x:c r="D1" s="397" t="s">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="E1" s="396" t="s">
+      <x:c r="E1" s="397" t="s">
         <x:v>405</x:v>
       </x:c>
-      <x:c r="F1" s="397" t="s">
+      <x:c r="F1" s="398" t="s">
         <x:v>406</x:v>
       </x:c>
-      <x:c r="G1" s="396" t="s">
+      <x:c r="G1" s="397" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="H1" s="396" t="s">
+      <x:c r="H1" s="397" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="I1" s="396" t="s">
+      <x:c r="I1" s="397" t="s">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="J1" s="396" t="s">
+      <x:c r="J1" s="397" t="s">
         <x:v>410</x:v>
       </x:c>
-      <x:c r="K1" s="396" t="s">
+      <x:c r="K1" s="397" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="L1" s="396" t="s">
+      <x:c r="L1" s="397" t="s">
         <x:v>2005</x:v>
       </x:c>
     </x:row>
@@ -60789,7 +60794,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H2" s="340" t="s">
-        <x:v>2370</x:v>
+        <x:v>2371</x:v>
       </x:c>
       <x:c r="I2" s="51" t="s">
         <x:v>1102</x:v>
@@ -61028,7 +61033,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G14" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H14" s="292"/>
       <x:c r="I14" s="51"/>
@@ -61298,7 +61303,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G27" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H27" s="292"/>
       <x:c r="I27" s="51"/>
@@ -61329,7 +61334,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H28" s="340" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="I28" s="51" t="s">
         <x:v>1127</x:v>
@@ -61568,7 +61573,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G40" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H40" s="292"/>
       <x:c r="I40" s="51"/>
@@ -61599,7 +61604,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H41" s="340" t="s">
-        <x:v>2373</x:v>
+        <x:v>2374</x:v>
       </x:c>
       <x:c r="I41" s="51" t="s">
         <x:v>1130</x:v>
@@ -61838,7 +61843,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G53" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H53" s="292"/>
       <x:c r="I53" s="51"/>
@@ -61869,7 +61874,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H54" s="340" t="s">
-        <x:v>2374</x:v>
+        <x:v>2375</x:v>
       </x:c>
       <x:c r="I54" s="51" t="s">
         <x:v>1134</x:v>
@@ -62108,7 +62113,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G66" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H66" s="292"/>
       <x:c r="I66" s="51"/>
@@ -62139,7 +62144,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H67" s="340" t="s">
-        <x:v>2375</x:v>
+        <x:v>2376</x:v>
       </x:c>
       <x:c r="I67" s="51" t="s">
         <x:v>1138</x:v>
@@ -62378,7 +62383,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G79" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H79" s="292"/>
       <x:c r="I79" s="51"/>
@@ -62409,7 +62414,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H80" s="340" t="s">
-        <x:v>2376</x:v>
+        <x:v>2377</x:v>
       </x:c>
       <x:c r="I80" s="51" t="s">
         <x:v>1141</x:v>
@@ -62648,7 +62653,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G92" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H92" s="292"/>
       <x:c r="I92" s="51"/>
@@ -62679,7 +62684,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H93" s="340" t="s">
-        <x:v>2377</x:v>
+        <x:v>2378</x:v>
       </x:c>
       <x:c r="I93" s="51" t="s">
         <x:v>1145</x:v>
@@ -62918,7 +62923,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G105" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H105" s="292"/>
       <x:c r="I105" s="51"/>
@@ -62949,7 +62954,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H106" s="340" t="s">
-        <x:v>2377</x:v>
+        <x:v>2378</x:v>
       </x:c>
       <x:c r="I106" s="51" t="s">
         <x:v>1149</x:v>
@@ -63188,7 +63193,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G118" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H118" s="292"/>
       <x:c r="I118" s="51"/>
@@ -63219,7 +63224,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H119" s="340" t="s">
-        <x:v>2378</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="I119" s="51" t="s">
         <x:v>1149</x:v>
@@ -63458,7 +63463,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G131" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H131" s="292"/>
       <x:c r="I131" s="51"/>
@@ -63489,7 +63494,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H132" s="340" t="s">
-        <x:v>2379</x:v>
+        <x:v>2380</x:v>
       </x:c>
       <x:c r="I132" s="51" t="s">
         <x:v>1160</x:v>
@@ -63728,7 +63733,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G144" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H144" s="292"/>
       <x:c r="I144" s="51"/>
@@ -63759,7 +63764,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H145" s="340" t="s">
-        <x:v>2380</x:v>
+        <x:v>2381</x:v>
       </x:c>
       <x:c r="I145" s="51" t="s">
         <x:v>1160</x:v>
@@ -63998,7 +64003,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G157" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H157" s="292"/>
       <x:c r="I157" s="51"/>
@@ -64029,7 +64034,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H158" s="340" t="s">
-        <x:v>2381</x:v>
+        <x:v>2382</x:v>
       </x:c>
       <x:c r="I158" s="51" t="s">
         <x:v>1160</x:v>
@@ -64268,7 +64273,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G170" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H170" s="292"/>
       <x:c r="I170" s="51"/>
@@ -64299,7 +64304,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H171" s="340" t="s">
-        <x:v>2382</x:v>
+        <x:v>2383</x:v>
       </x:c>
       <x:c r="I171" s="51" t="s">
         <x:v>1160</x:v>
@@ -64538,7 +64543,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G183" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H183" s="292"/>
       <x:c r="I183" s="51"/>
@@ -64808,7 +64813,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G196" s="292" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="H196" s="340"/>
       <x:c r="I196" s="51"/>
@@ -64839,7 +64844,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H197" s="340" t="s">
-        <x:v>2383</x:v>
+        <x:v>2384</x:v>
       </x:c>
       <x:c r="I197" s="134" t="s">
         <x:v>1178</x:v>
@@ -65109,7 +65114,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H210" s="340" t="s">
-        <x:v>2384</x:v>
+        <x:v>2385</x:v>
       </x:c>
       <x:c r="I210" s="134" t="s">
         <x:v>1187</x:v>
@@ -65367,7 +65372,7 @@
         <x:v>1189</x:v>
       </x:c>
       <x:c r="D223" s="134" t="s">
-        <x:v>2385</x:v>
+        <x:v>2386</x:v>
       </x:c>
       <x:c r="E223" s="35" t="s">
         <x:v>1176</x:v>
@@ -65379,7 +65384,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H223" s="340" t="s">
-        <x:v>2386</x:v>
+        <x:v>2387</x:v>
       </x:c>
       <x:c r="I223" s="10" t="s">
         <x:v>1192</x:v>
@@ -65649,7 +65654,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H236" s="340" t="s">
-        <x:v>2387</x:v>
+        <x:v>2388</x:v>
       </x:c>
       <x:c r="I236" s="10" t="s">
         <x:v>1197</x:v>
@@ -65919,7 +65924,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H249" s="340" t="s">
-        <x:v>2388</x:v>
+        <x:v>2389</x:v>
       </x:c>
       <x:c r="I249" s="10" t="s">
         <x:v>1203</x:v>
@@ -66101,7 +66106,7 @@
         <x:v>1115</x:v>
       </x:c>
       <x:c r="H258" s="292" t="s">
-        <x:v>2389</x:v>
+        <x:v>2390</x:v>
       </x:c>
       <x:c r="I258" s="9"/>
       <x:c r="J258" s="9"/>
@@ -66447,7 +66452,7 @@
         <x:v>1212</x:v>
       </x:c>
       <x:c r="D275" s="35" t="s">
-        <x:v>2390</x:v>
+        <x:v>2391</x:v>
       </x:c>
       <x:c r="E275" s="35" t="s">
         <x:v>1214</x:v>
@@ -66456,10 +66461,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G275" s="297" t="s">
-        <x:v>2391</x:v>
+        <x:v>2392</x:v>
       </x:c>
       <x:c r="I275" s="10" t="s">
-        <x:v>2392</x:v>
+        <x:v>2393</x:v>
       </x:c>
       <x:c r="J275" s="10"/>
       <x:c r="K275" s="35"/>
@@ -66475,7 +66480,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G276" s="297" t="s">
-        <x:v>2393</x:v>
+        <x:v>2394</x:v>
       </x:c>
       <x:c r="I276" s="9"/>
       <x:c r="J276" s="9"/>
@@ -66492,10 +66497,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G277" s="297" t="s">
-        <x:v>2394</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H277" s="297" t="s">
-        <x:v>2395</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="I277" s="9"/>
       <x:c r="J277" s="9"/>
@@ -66534,13 +66539,13 @@
         <x:v>1220</x:v>
       </x:c>
       <x:c r="E279" s="35" t="s">
-        <x:v>2396</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="F279" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G279" s="297" t="s">
-        <x:v>2391</x:v>
+        <x:v>2392</x:v>
       </x:c>
       <x:c r="I279" s="10" t="s">
         <x:v>1223</x:v>
@@ -66559,7 +66564,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G280" s="297" t="s">
-        <x:v>2397</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="H280" s="297" t="s">
         <x:v>1117</x:v>
@@ -66601,17 +66606,17 @@
         <x:v>1226</x:v>
       </x:c>
       <x:c r="E282" s="35" t="s">
-        <x:v>2398</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="F282" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G282" s="297" t="s">
-        <x:v>2391</x:v>
+        <x:v>2392</x:v>
       </x:c>
       <x:c r="H282" s="297"/>
       <x:c r="I282" s="10" t="s">
-        <x:v>2399</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="J282" s="10"/>
       <x:c r="K282" s="35"/>
@@ -66627,7 +66632,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G283" s="297" t="s">
-        <x:v>2393</x:v>
+        <x:v>2394</x:v>
       </x:c>
       <x:c r="H283" s="297"/>
       <x:c r="I283" s="9"/>
@@ -66645,10 +66650,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G284" s="297" t="s">
-        <x:v>2400</x:v>
+        <x:v>2401</x:v>
       </x:c>
       <x:c r="H284" s="323" t="s">
-        <x:v>2401</x:v>
+        <x:v>2402</x:v>
       </x:c>
       <x:c r="I284" s="9"/>
       <x:c r="J284" s="9"/>
@@ -66687,17 +66692,17 @@
         <x:v>1233</x:v>
       </x:c>
       <x:c r="E286" s="35" t="s">
-        <x:v>2398</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="F286" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G286" s="297" t="s">
-        <x:v>2391</x:v>
+        <x:v>2392</x:v>
       </x:c>
       <x:c r="H286" s="297"/>
       <x:c r="I286" s="10" t="s">
-        <x:v>2399</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="J286" s="10"/>
       <x:c r="K286" s="35"/>
@@ -66713,7 +66718,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G287" s="297" t="s">
-        <x:v>2393</x:v>
+        <x:v>2394</x:v>
       </x:c>
       <x:c r="H287" s="297"/>
       <x:c r="I287" s="9"/>
@@ -66731,10 +66736,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G288" s="297" t="s">
-        <x:v>2402</x:v>
+        <x:v>2403</x:v>
       </x:c>
       <x:c r="H288" s="297" t="s">
-        <x:v>2403</x:v>
+        <x:v>2404</x:v>
       </x:c>
       <x:c r="I288" s="9"/>
       <x:c r="J288" s="9"/>
@@ -66782,7 +66787,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H290" s="340" t="s">
-        <x:v>2404</x:v>
+        <x:v>2405</x:v>
       </x:c>
       <x:c r="I290" s="51" t="s">
         <x:v>1102</x:v>
@@ -66861,7 +66866,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G294" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H294" s="312" t="s">
         <x:v>1117</x:v>
@@ -66881,7 +66886,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G295" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H295" s="312">
         <x:v>45758</x:v>
@@ -67001,7 +67006,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G301" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H301" s="297"/>
       <x:c r="I301" s="51"/>
@@ -67111,7 +67116,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G306" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H306" s="312" t="s">
         <x:v>1117</x:v>
@@ -67131,7 +67136,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G307" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H307" s="312">
         <x:v>45758</x:v>
@@ -67251,7 +67256,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G313" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I313" s="51"/>
       <x:c r="J313" s="48"/>
@@ -67281,7 +67286,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H314" s="340" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I314" s="51" t="s">
         <x:v>1127</x:v>
@@ -67358,7 +67363,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G318" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H318" s="312" t="s">
         <x:v>1117</x:v>
@@ -67378,7 +67383,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G319" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H319" s="312">
         <x:v>45758</x:v>
@@ -67498,7 +67503,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G325" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I325" s="51"/>
       <x:c r="J325" s="48"/>
@@ -67528,7 +67533,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H326" s="340" t="s">
-        <x:v>2409</x:v>
+        <x:v>2410</x:v>
       </x:c>
       <x:c r="I326" s="51" t="s">
         <x:v>1130</x:v>
@@ -67605,7 +67610,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G330" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H330" s="312" t="s">
         <x:v>1117</x:v>
@@ -67625,7 +67630,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G331" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H331" s="312">
         <x:v>45758</x:v>
@@ -67745,7 +67750,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G337" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I337" s="51"/>
       <x:c r="J337" s="48"/>
@@ -67775,7 +67780,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H338" s="340" t="s">
-        <x:v>2410</x:v>
+        <x:v>2411</x:v>
       </x:c>
       <x:c r="I338" s="51" t="s">
         <x:v>1134</x:v>
@@ -67854,7 +67859,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G342" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H342" s="312"/>
       <x:c r="I342" s="51"/>
@@ -67872,7 +67877,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G343" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H343" s="312">
         <x:v>45758</x:v>
@@ -67992,7 +67997,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G349" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I349" s="51"/>
       <x:c r="J349" s="48"/>
@@ -68022,7 +68027,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H350" s="340" t="s">
-        <x:v>2410</x:v>
+        <x:v>2411</x:v>
       </x:c>
       <x:c r="I350" s="51" t="s">
         <x:v>1138</x:v>
@@ -68101,7 +68106,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G354" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H354" s="312" t="s">
         <x:v>1117</x:v>
@@ -68121,7 +68126,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G355" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H355" s="312"/>
       <x:c r="I355" s="51"/>
@@ -68239,7 +68244,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G361" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I361" s="51"/>
       <x:c r="J361" s="48"/>
@@ -68257,7 +68262,7 @@
         <x:v>1254</x:v>
       </x:c>
       <x:c r="D362" s="51" t="s">
-        <x:v>2411</x:v>
+        <x:v>2412</x:v>
       </x:c>
       <x:c r="E362" s="51" t="s">
         <x:v>1099</x:v>
@@ -68269,10 +68274,10 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H362" s="340" t="s">
-        <x:v>2412</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="I362" s="51" t="s">
-        <x:v>2413</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="J362" s="50"/>
       <x:c r="K362" s="51"/>
@@ -68346,7 +68351,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G366" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H366" s="312" t="s">
         <x:v>1117</x:v>
@@ -68366,7 +68371,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G367" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H367" s="312">
         <x:v>49410</x:v>
@@ -68484,7 +68489,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G373" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H373" s="292"/>
       <x:c r="I373" s="51"/>
@@ -68515,7 +68520,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H374" s="340" t="s">
-        <x:v>2414</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I374" s="51" t="s">
         <x:v>1145</x:v>
@@ -68594,7 +68599,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G378" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H378" s="312" t="s">
         <x:v>1117</x:v>
@@ -68614,7 +68619,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G379" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H379" s="312">
         <x:v>45758</x:v>
@@ -68732,7 +68737,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G385" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I385" s="51"/>
       <x:c r="J385" s="48"/>
@@ -68762,7 +68767,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H386" s="340" t="s">
-        <x:v>2415</x:v>
+        <x:v>2416</x:v>
       </x:c>
       <x:c r="I386" s="51" t="s">
         <x:v>1149</x:v>
@@ -68841,7 +68846,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G390" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H390" s="312" t="s">
         <x:v>1117</x:v>
@@ -68861,7 +68866,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G391" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H391" s="312">
         <x:v>45758</x:v>
@@ -68979,7 +68984,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G397" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I397" s="51"/>
       <x:c r="J397" s="48"/>
@@ -69009,7 +69014,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H398" s="340" t="s">
-        <x:v>2416</x:v>
+        <x:v>2417</x:v>
       </x:c>
       <x:c r="I398" s="51" t="s">
         <x:v>1149</x:v>
@@ -69086,7 +69091,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G402" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H402" s="312" t="s">
         <x:v>1117</x:v>
@@ -69106,7 +69111,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G403" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H403" s="312">
         <x:v>45758</x:v>
@@ -69226,7 +69231,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G409" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I409" s="51"/>
       <x:c r="J409" s="48"/>
@@ -69256,7 +69261,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H410" s="340" t="s">
-        <x:v>2417</x:v>
+        <x:v>2418</x:v>
       </x:c>
       <x:c r="I410" s="51" t="s">
         <x:v>1160</x:v>
@@ -69335,7 +69340,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G414" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H414" s="312" t="s">
         <x:v>1117</x:v>
@@ -69355,7 +69360,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G415" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H415" s="312">
         <x:v>45758</x:v>
@@ -69473,7 +69478,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G421" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I421" s="51"/>
       <x:c r="J421" s="48"/>
@@ -69491,7 +69496,7 @@
         <x:v>1260</x:v>
       </x:c>
       <x:c r="D422" s="51" t="s">
-        <x:v>2418</x:v>
+        <x:v>2419</x:v>
       </x:c>
       <x:c r="E422" s="51" t="s">
         <x:v>1099</x:v>
@@ -69503,10 +69508,10 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H422" s="340" t="s">
-        <x:v>2419</x:v>
+        <x:v>2420</x:v>
       </x:c>
       <x:c r="I422" s="51" t="s">
-        <x:v>2420</x:v>
+        <x:v>2421</x:v>
       </x:c>
       <x:c r="J422" s="50"/>
       <x:c r="K422" s="51"/>
@@ -69582,7 +69587,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G426" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H426" s="312" t="s">
         <x:v>1117</x:v>
@@ -69602,7 +69607,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G427" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H427" s="312">
         <x:v>45758</x:v>
@@ -69722,7 +69727,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G433" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I433" s="51"/>
       <x:c r="J433" s="48"/>
@@ -69752,7 +69757,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H434" s="340" t="s">
-        <x:v>2421</x:v>
+        <x:v>2422</x:v>
       </x:c>
       <x:c r="I434" s="51" t="s">
         <x:v>1160</x:v>
@@ -69831,7 +69836,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G438" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H438" s="312" t="s">
         <x:v>1117</x:v>
@@ -69851,7 +69856,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G439" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H439" s="312">
         <x:v>45758</x:v>
@@ -69969,7 +69974,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G445" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I445" s="51"/>
       <x:c r="J445" s="48"/>
@@ -69999,7 +70004,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H446" s="340" t="s">
-        <x:v>2422</x:v>
+        <x:v>2423</x:v>
       </x:c>
       <x:c r="I446" s="51" t="s">
         <x:v>1160</x:v>
@@ -70078,7 +70083,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G450" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H450" s="312" t="s">
         <x:v>1117</x:v>
@@ -70098,7 +70103,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G451" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H451" s="312">
         <x:v>45758</x:v>
@@ -70216,7 +70221,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G457" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="I457" s="51"/>
       <x:c r="J457" s="48"/>
@@ -70325,7 +70330,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G462" s="292" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="H462" s="340" t="s">
         <x:v>437</x:v>
@@ -70345,7 +70350,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G463" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H463" s="340" t="s">
         <x:v>437</x:v>
@@ -70465,7 +70470,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G469" s="288" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H469" s="340" t="s">
         <x:v>437</x:v>
@@ -70799,7 +70804,7 @@
     <x:mergeCell ref="K458:K469"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H284" r:id="rId170"/>
+    <x:hyperlink ref="H284" r:id="rId172"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -70823,13 +70828,13 @@
   <x:sheetData>
     <x:row r="2" spans="1:7">
       <x:c r="A2" s="196" t="s">
-        <x:v>2423</x:v>
+        <x:v>2424</x:v>
       </x:c>
       <x:c r="D2" s="196" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="G2" s="196" t="s">
-        <x:v>2424</x:v>
+        <x:v>2425</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
@@ -70837,7 +70842,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>2425</x:v>
+        <x:v>2426</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
         <x:v>244</x:v>
@@ -70848,7 +70853,7 @@
         <x:v>245</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>2426</x:v>
+        <x:v>2427</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
         <x:v>234</x:v>
@@ -70856,10 +70861,10 @@
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="A5" s="0" t="s">
-        <x:v>2427</x:v>
+        <x:v>2428</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>2428</x:v>
+        <x:v>2429</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
         <x:v>239</x:v>

</xml_diff>

<commit_message>
Test: Using JS click fix for admin search timeout error, password TC_REG_01 to 07 works smoothly.
</commit_message>
<xml_diff>
--- a/sqa-testing-report/Data/DataTest.xlsx
+++ b/sqa-testing-report/Data/DataTest.xlsx
@@ -7716,8 +7716,10 @@
     <x:t>Hệ thống báo lỗi mật khẩu không đúng định dạng thành công.</x:t>
   </x:si>
   <x:si>
-    <x:t>Lỗi: invalid argument: No dialog is showing
-  (Session info: chrome=146.0.7680.165)</x:t>
+    <x:t xml:space="preserve">Lỗi:   Lỗi thực tế: Đăng ký thành công!
+  Expected: True
+  But was:  False
+</x:t>
   </x:si>
   <x:si>
     <x:t>Fail</x:t>
@@ -7727,6 +7729,9 @@
   </x:si>
   <x:si>
     <x:t>Kho@090xxxx</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hệ thống chặn đăng ký và báo lỗi đã tồn tại thành công.</x:t>
   </x:si>
   <x:si>
     <x:t>Kiểm tra đăng ký với mật khẩu chứa ký tự đặc biệt gây lỗi (SQL Injection).</x:t>
@@ -48208,41 +48213,41 @@
   </x:mergeCells>
   <x:phoneticPr fontId="16" type="noConversion"/>
   <x:hyperlinks>
-    <x:hyperlink ref="H382" r:id="rId105"/>
-    <x:hyperlink ref="H388" r:id="rId106"/>
-    <x:hyperlink ref="H396" r:id="rId107"/>
-    <x:hyperlink ref="H397" r:id="rId108"/>
-    <x:hyperlink ref="H415" r:id="rId109"/>
-    <x:hyperlink ref="H418" r:id="rId110"/>
-    <x:hyperlink ref="H420" r:id="rId111"/>
-    <x:hyperlink ref="H421" r:id="rId112"/>
-    <x:hyperlink ref="H423" r:id="rId113"/>
-    <x:hyperlink ref="H424" r:id="rId114"/>
-    <x:hyperlink ref="H53" r:id="rId115"/>
-    <x:hyperlink ref="H61" r:id="rId116"/>
-    <x:hyperlink ref="H65" r:id="rId117"/>
-    <x:hyperlink ref="H69" r:id="rId118"/>
-    <x:hyperlink ref="H73" r:id="rId119"/>
-    <x:hyperlink ref="H77" r:id="rId120"/>
-    <x:hyperlink ref="H81" r:id="rId121"/>
-    <x:hyperlink ref="H112" r:id="rId122"/>
-    <x:hyperlink ref="H115" r:id="rId123"/>
-    <x:hyperlink ref="H118" r:id="rId124"/>
-    <x:hyperlink ref="H399" r:id="rId125"/>
-    <x:hyperlink ref="H402" r:id="rId126"/>
-    <x:hyperlink ref="H405" r:id="rId127"/>
-    <x:hyperlink ref="H408" r:id="rId128"/>
-    <x:hyperlink ref="H411" r:id="rId129"/>
-    <x:hyperlink ref="H400" r:id="rId130"/>
-    <x:hyperlink ref="H403" r:id="rId131"/>
-    <x:hyperlink ref="H406" r:id="rId132"/>
-    <x:hyperlink ref="H409" r:id="rId133"/>
-    <x:hyperlink ref="H412" r:id="rId134"/>
-    <x:hyperlink ref="H1075" r:id="rId135"/>
-    <x:hyperlink ref="H1081" r:id="rId136"/>
-    <x:hyperlink ref="H1087" r:id="rId137"/>
-    <x:hyperlink ref="H1093" r:id="rId138"/>
-    <x:hyperlink ref="H1099" r:id="rId139"/>
+    <x:hyperlink ref="H382" r:id="rId82"/>
+    <x:hyperlink ref="H388" r:id="rId83"/>
+    <x:hyperlink ref="H396" r:id="rId84"/>
+    <x:hyperlink ref="H397" r:id="rId85"/>
+    <x:hyperlink ref="H415" r:id="rId86"/>
+    <x:hyperlink ref="H418" r:id="rId87"/>
+    <x:hyperlink ref="H420" r:id="rId88"/>
+    <x:hyperlink ref="H421" r:id="rId89"/>
+    <x:hyperlink ref="H423" r:id="rId90"/>
+    <x:hyperlink ref="H424" r:id="rId91"/>
+    <x:hyperlink ref="H53" r:id="rId92"/>
+    <x:hyperlink ref="H61" r:id="rId93"/>
+    <x:hyperlink ref="H65" r:id="rId94"/>
+    <x:hyperlink ref="H69" r:id="rId95"/>
+    <x:hyperlink ref="H73" r:id="rId96"/>
+    <x:hyperlink ref="H77" r:id="rId97"/>
+    <x:hyperlink ref="H81" r:id="rId98"/>
+    <x:hyperlink ref="H112" r:id="rId99"/>
+    <x:hyperlink ref="H115" r:id="rId100"/>
+    <x:hyperlink ref="H118" r:id="rId101"/>
+    <x:hyperlink ref="H399" r:id="rId102"/>
+    <x:hyperlink ref="H402" r:id="rId103"/>
+    <x:hyperlink ref="H405" r:id="rId104"/>
+    <x:hyperlink ref="H408" r:id="rId173"/>
+    <x:hyperlink ref="H411" r:id="rId174"/>
+    <x:hyperlink ref="H400" r:id="rId175"/>
+    <x:hyperlink ref="H403" r:id="rId176"/>
+    <x:hyperlink ref="H406" r:id="rId177"/>
+    <x:hyperlink ref="H409" r:id="rId178"/>
+    <x:hyperlink ref="H412" r:id="rId179"/>
+    <x:hyperlink ref="H1075" r:id="rId180"/>
+    <x:hyperlink ref="H1081" r:id="rId181"/>
+    <x:hyperlink ref="H1087" r:id="rId182"/>
+    <x:hyperlink ref="H1093" r:id="rId183"/>
+    <x:hyperlink ref="H1099" r:id="rId184"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -49491,9 +49496,13 @@
       <x:c r="I56" s="138" t="s">
         <x:v>447</x:v>
       </x:c>
-      <x:c r="J56" s="137"/>
-      <x:c r="K56" s="137"/>
-      <x:c r="L56" s="137"/>
+      <x:c r="J56" s="137" t="s">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="K56" s="137" t="s">
+        <x:v>2008</x:v>
+      </x:c>
+      <x:c r="L56" s="137" t="s"/>
     </x:row>
     <x:row r="57" spans="1:12">
       <x:c r="A57" s="140"/>
@@ -50040,7 +50049,7 @@
         <x:v>468</x:v>
       </x:c>
       <x:c r="D83" s="140" t="s">
-        <x:v>2018</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="E83" s="140" t="s">
         <x:v>434</x:v>
@@ -50172,7 +50181,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H89" s="25" t="s">
-        <x:v>2019</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="I89" s="138"/>
       <x:c r="J89" s="136"/>
@@ -50192,7 +50201,7 @@
         <x:v>445</x:v>
       </x:c>
       <x:c r="H90" s="25" t="s">
-        <x:v>2019</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="I90" s="138"/>
       <x:c r="J90" s="136"/>
@@ -50260,7 +50269,7 @@
         <x:v>419</x:v>
       </x:c>
       <x:c r="H93" s="140" t="s">
-        <x:v>2020</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="I93" s="138"/>
       <x:c r="J93" s="136"/>
@@ -50488,7 +50497,7 @@
         <x:v>439</x:v>
       </x:c>
       <x:c r="H104" s="139" t="s">
-        <x:v>2021</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="I104" s="138"/>
       <x:c r="J104" s="134"/>
@@ -51053,7 +51062,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I129" s="138" t="s">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="J129" s="134"/>
       <x:c r="K129" s="134"/>
@@ -51123,7 +51132,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I132" s="123" t="s">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="J132" s="134"/>
       <x:c r="K132" s="134"/>
@@ -51193,7 +51202,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I135" s="138" t="s">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="J135" s="134"/>
       <x:c r="K135" s="134"/>
@@ -51260,10 +51269,10 @@
         <x:v>480</x:v>
       </x:c>
       <x:c r="H138" s="316" t="s">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="I138" s="120" t="s">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="J138" s="134"/>
       <x:c r="K138" s="134"/>
@@ -51333,7 +51342,7 @@
         <x:v>2009</x:v>
       </x:c>
       <x:c r="I141" s="138" t="s">
-        <x:v>2027</x:v>
+        <x:v>2028</x:v>
       </x:c>
       <x:c r="J141" s="118"/>
       <x:c r="K141" s="134"/>
@@ -51397,11 +51406,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G144" s="138" t="s">
-        <x:v>2028</x:v>
+        <x:v>2029</x:v>
       </x:c>
       <x:c r="H144" s="140"/>
       <x:c r="I144" s="138" t="s">
-        <x:v>2029</x:v>
+        <x:v>2030</x:v>
       </x:c>
       <x:c r="J144" s="134"/>
       <x:c r="K144" s="134"/>
@@ -51417,10 +51426,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G145" s="319" t="s">
-        <x:v>2030</x:v>
+        <x:v>2031</x:v>
       </x:c>
       <x:c r="H145" s="134" t="s">
-        <x:v>2031</x:v>
+        <x:v>2032</x:v>
       </x:c>
       <x:c r="I145" s="138"/>
       <x:c r="J145" s="134"/>
@@ -51437,10 +51446,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G146" s="138" t="s">
-        <x:v>2032</x:v>
+        <x:v>2033</x:v>
       </x:c>
       <x:c r="H146" s="317" t="s">
-        <x:v>2033</x:v>
+        <x:v>2034</x:v>
       </x:c>
       <x:c r="I146" s="138"/>
       <x:c r="J146" s="134"/>
@@ -51457,10 +51466,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G147" s="138" t="s">
+        <x:v>2035</x:v>
+      </x:c>
+      <x:c r="H147" s="134" t="s">
         <x:v>2034</x:v>
-      </x:c>
-      <x:c r="H147" s="134" t="s">
-        <x:v>2033</x:v>
       </x:c>
       <x:c r="I147" s="138"/>
       <x:c r="J147" s="134"/>
@@ -51477,7 +51486,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G148" s="138" t="s">
-        <x:v>2035</x:v>
+        <x:v>2036</x:v>
       </x:c>
       <x:c r="H148" s="134"/>
       <x:c r="I148" s="138"/>
@@ -51511,7 +51520,7 @@
         <x:v>590</x:v>
       </x:c>
       <x:c r="I149" s="138" t="s">
-        <x:v>2036</x:v>
+        <x:v>2037</x:v>
       </x:c>
       <x:c r="J149" s="298"/>
       <x:c r="K149" s="134"/>
@@ -51531,7 +51540,7 @@
       </x:c>
       <x:c r="H150" s="140"/>
       <x:c r="I150" s="138" t="s">
-        <x:v>2037</x:v>
+        <x:v>2038</x:v>
       </x:c>
       <x:c r="J150" s="298"/>
       <x:c r="K150" s="134"/>
@@ -51551,7 +51560,7 @@
       </x:c>
       <x:c r="H151" s="140"/>
       <x:c r="I151" s="138" t="s">
-        <x:v>2038</x:v>
+        <x:v>2039</x:v>
       </x:c>
       <x:c r="J151" s="298"/>
       <x:c r="K151" s="134"/>
@@ -51627,10 +51636,10 @@
       </x:c>
       <x:c r="H154" s="140"/>
       <x:c r="I154" s="138" t="s">
-        <x:v>2039</x:v>
+        <x:v>2040</x:v>
       </x:c>
       <x:c r="J154" s="134" t="s">
-        <x:v>2040</x:v>
+        <x:v>2041</x:v>
       </x:c>
       <x:c r="K154" s="134" t="s">
         <x:v>2008</x:v>
@@ -51647,16 +51656,16 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G155" s="138" t="s">
-        <x:v>2041</x:v>
+        <x:v>2042</x:v>
       </x:c>
       <x:c r="H155" s="140" t="s">
-        <x:v>2042</x:v>
+        <x:v>2043</x:v>
       </x:c>
       <x:c r="I155" s="138" t="s">
-        <x:v>2043</x:v>
+        <x:v>2044</x:v>
       </x:c>
       <x:c r="J155" s="134" t="s">
-        <x:v>2044</x:v>
+        <x:v>2045</x:v>
       </x:c>
       <x:c r="K155" s="134"/>
       <x:c r="L155" s="134"/>
@@ -51672,7 +51681,7 @@
         <x:v>626</x:v>
       </x:c>
       <x:c r="D156" s="140" t="s">
-        <x:v>2045</x:v>
+        <x:v>2046</x:v>
       </x:c>
       <x:c r="E156" s="140" t="s">
         <x:v>616</x:v>
@@ -51681,13 +51690,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G156" s="138" t="s">
-        <x:v>2046</x:v>
+        <x:v>2047</x:v>
       </x:c>
       <x:c r="H156" s="140" t="s">
-        <x:v>2047</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="I156" s="138" t="s">
-        <x:v>2048</x:v>
+        <x:v>2049</x:v>
       </x:c>
       <x:c r="J156" s="134"/>
       <x:c r="K156" s="134"/>
@@ -51713,16 +51722,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G157" s="138" t="s">
-        <x:v>2049</x:v>
+        <x:v>2050</x:v>
       </x:c>
       <x:c r="H157" s="140" t="s">
-        <x:v>2050</x:v>
+        <x:v>2051</x:v>
       </x:c>
       <x:c r="I157" s="138" t="s">
-        <x:v>2051</x:v>
+        <x:v>2052</x:v>
       </x:c>
       <x:c r="J157" s="134" t="s">
-        <x:v>2052</x:v>
+        <x:v>2053</x:v>
       </x:c>
       <x:c r="K157" s="134" t="s">
         <x:v>2008</x:v>
@@ -51739,14 +51748,14 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G158" s="138" t="s">
-        <x:v>2053</x:v>
+        <x:v>2054</x:v>
       </x:c>
       <x:c r="H158" s="140"/>
       <x:c r="I158" s="138" t="s">
-        <x:v>2054</x:v>
+        <x:v>2055</x:v>
       </x:c>
       <x:c r="J158" s="134" t="s">
-        <x:v>2055</x:v>
+        <x:v>2056</x:v>
       </x:c>
       <x:c r="K158" s="134"/>
       <x:c r="L158" s="134"/>
@@ -51761,14 +51770,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G159" s="138" t="s">
-        <x:v>2056</x:v>
+        <x:v>2057</x:v>
       </x:c>
       <x:c r="H159" s="140"/>
       <x:c r="I159" s="138" t="s">
-        <x:v>2057</x:v>
+        <x:v>2058</x:v>
       </x:c>
       <x:c r="J159" s="134" t="s">
-        <x:v>2058</x:v>
+        <x:v>2059</x:v>
       </x:c>
       <x:c r="K159" s="134"/>
       <x:c r="L159" s="134"/>
@@ -51793,13 +51802,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G160" s="138" t="s">
-        <x:v>2049</x:v>
+        <x:v>2050</x:v>
       </x:c>
       <x:c r="H160" s="140" t="s">
-        <x:v>2050</x:v>
+        <x:v>2051</x:v>
       </x:c>
       <x:c r="I160" s="138" t="s">
-        <x:v>2059</x:v>
+        <x:v>2060</x:v>
       </x:c>
       <x:c r="J160" s="134"/>
       <x:c r="K160" s="134"/>
@@ -51815,7 +51824,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G161" s="138" t="s">
-        <x:v>2060</x:v>
+        <x:v>2061</x:v>
       </x:c>
       <x:c r="H161" s="313">
         <x:v>46109</x:v>
@@ -51836,25 +51845,25 @@
         <x:v>644</x:v>
       </x:c>
       <x:c r="D162" s="116" t="s">
-        <x:v>2061</x:v>
+        <x:v>2062</x:v>
       </x:c>
       <x:c r="E162" s="116" t="s">
-        <x:v>2062</x:v>
+        <x:v>2063</x:v>
       </x:c>
       <x:c r="F162" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G162" s="320" t="s">
-        <x:v>2063</x:v>
+        <x:v>2064</x:v>
       </x:c>
       <x:c r="H162" s="116" t="s">
-        <x:v>2050</x:v>
+        <x:v>2051</x:v>
       </x:c>
       <x:c r="I162" s="320" t="s">
-        <x:v>2051</x:v>
+        <x:v>2052</x:v>
       </x:c>
       <x:c r="J162" s="134" t="s">
-        <x:v>2064</x:v>
+        <x:v>2065</x:v>
       </x:c>
       <x:c r="K162" s="134" t="s">
         <x:v>2008</x:v>
@@ -51871,14 +51880,14 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G163" s="320" t="s">
-        <x:v>2065</x:v>
+        <x:v>2066</x:v>
       </x:c>
       <x:c r="H163" s="116"/>
       <x:c r="I163" s="320" t="s">
-        <x:v>2066</x:v>
+        <x:v>2067</x:v>
       </x:c>
       <x:c r="J163" s="134" t="s">
-        <x:v>2067</x:v>
+        <x:v>2068</x:v>
       </x:c>
       <x:c r="K163" s="134"/>
       <x:c r="L163" s="134"/>
@@ -51893,14 +51902,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G164" s="320" t="s">
-        <x:v>2068</x:v>
+        <x:v>2069</x:v>
       </x:c>
       <x:c r="H164" s="116"/>
       <x:c r="I164" s="320" t="s">
-        <x:v>2069</x:v>
+        <x:v>2070</x:v>
       </x:c>
       <x:c r="J164" s="134" t="s">
-        <x:v>2070</x:v>
+        <x:v>2071</x:v>
       </x:c>
       <x:c r="K164" s="134"/>
       <x:c r="L164" s="134"/>
@@ -51925,13 +51934,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G165" s="320" t="s">
-        <x:v>2071</x:v>
+        <x:v>2072</x:v>
       </x:c>
       <x:c r="H165" s="318">
         <x:v>0.333333333333333</x:v>
       </x:c>
       <x:c r="I165" s="320" t="s">
-        <x:v>2072</x:v>
+        <x:v>2073</x:v>
       </x:c>
       <x:c r="J165" s="134"/>
       <x:c r="K165" s="134"/>
@@ -51947,13 +51956,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G166" s="320" t="s">
-        <x:v>2073</x:v>
+        <x:v>2074</x:v>
       </x:c>
       <x:c r="H166" s="116" t="s">
-        <x:v>2074</x:v>
+        <x:v>2075</x:v>
       </x:c>
       <x:c r="I166" s="320" t="s">
-        <x:v>2075</x:v>
+        <x:v>2076</x:v>
       </x:c>
       <x:c r="J166" s="134"/>
       <x:c r="K166" s="134"/>
@@ -51969,13 +51978,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G167" s="320" t="s">
-        <x:v>2076</x:v>
+        <x:v>2077</x:v>
       </x:c>
       <x:c r="H167" s="116" t="s">
-        <x:v>2077</x:v>
+        <x:v>2078</x:v>
       </x:c>
       <x:c r="I167" s="320" t="s">
-        <x:v>2078</x:v>
+        <x:v>2079</x:v>
       </x:c>
       <x:c r="J167" s="134"/>
       <x:c r="K167" s="134"/>
@@ -51991,11 +52000,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G168" s="320" t="s">
-        <x:v>2079</x:v>
+        <x:v>2080</x:v>
       </x:c>
       <x:c r="H168" s="116"/>
       <x:c r="I168" s="320" t="s">
-        <x:v>2080</x:v>
+        <x:v>2081</x:v>
       </x:c>
       <x:c r="J168" s="134"/>
       <x:c r="K168" s="134"/>
@@ -52012,22 +52021,22 @@
         <x:v>658</x:v>
       </x:c>
       <x:c r="D169" s="116" t="s">
-        <x:v>2081</x:v>
+        <x:v>2082</x:v>
       </x:c>
       <x:c r="E169" s="116" t="s">
-        <x:v>2082</x:v>
+        <x:v>2083</x:v>
       </x:c>
       <x:c r="F169" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G169" s="320" t="s">
-        <x:v>2083</x:v>
+        <x:v>2084</x:v>
       </x:c>
       <x:c r="H169" s="116" t="s">
-        <x:v>2084</x:v>
+        <x:v>2085</x:v>
       </x:c>
       <x:c r="I169" s="320" t="s">
-        <x:v>2085</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="J169" s="134"/>
       <x:c r="K169" s="134"/>
@@ -52043,11 +52052,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G170" s="320" t="s">
-        <x:v>2086</x:v>
+        <x:v>2087</x:v>
       </x:c>
       <x:c r="H170" s="116"/>
       <x:c r="I170" s="320" t="s">
-        <x:v>2087</x:v>
+        <x:v>2088</x:v>
       </x:c>
       <x:c r="J170" s="134"/>
       <x:c r="K170" s="134"/>
@@ -52063,11 +52072,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G171" s="320" t="s">
-        <x:v>2088</x:v>
+        <x:v>2089</x:v>
       </x:c>
       <x:c r="H171" s="116"/>
       <x:c r="I171" s="320" t="s">
-        <x:v>2089</x:v>
+        <x:v>2090</x:v>
       </x:c>
       <x:c r="J171" s="134"/>
       <x:c r="K171" s="134"/>
@@ -52093,13 +52102,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G172" s="320" t="s">
-        <x:v>2090</x:v>
+        <x:v>2091</x:v>
       </x:c>
       <x:c r="H172" s="116" t="s">
-        <x:v>2084</x:v>
+        <x:v>2085</x:v>
       </x:c>
       <x:c r="I172" s="320" t="s">
-        <x:v>2085</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="J172" s="134"/>
       <x:c r="K172" s="134"/>
@@ -52115,11 +52124,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G173" s="320" t="s">
-        <x:v>2091</x:v>
+        <x:v>2092</x:v>
       </x:c>
       <x:c r="H173" s="116"/>
       <x:c r="I173" s="320" t="s">
-        <x:v>2092</x:v>
+        <x:v>2093</x:v>
       </x:c>
       <x:c r="J173" s="134"/>
       <x:c r="K173" s="134"/>
@@ -52145,13 +52154,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G174" s="320" t="s">
-        <x:v>2093</x:v>
+        <x:v>2094</x:v>
       </x:c>
       <x:c r="H174" s="116" t="s">
-        <x:v>2084</x:v>
+        <x:v>2085</x:v>
       </x:c>
       <x:c r="I174" s="320" t="s">
-        <x:v>2094</x:v>
+        <x:v>2095</x:v>
       </x:c>
       <x:c r="J174" s="134"/>
       <x:c r="K174" s="134"/>
@@ -52167,11 +52176,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G175" s="320" t="s">
-        <x:v>2095</x:v>
+        <x:v>2096</x:v>
       </x:c>
       <x:c r="H175" s="116"/>
       <x:c r="I175" s="320" t="s">
-        <x:v>2085</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="J175" s="134"/>
       <x:c r="K175" s="134"/>
@@ -52187,11 +52196,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G176" s="320" t="s">
-        <x:v>2096</x:v>
+        <x:v>2097</x:v>
       </x:c>
       <x:c r="H176" s="116"/>
       <x:c r="I176" s="320" t="s">
-        <x:v>2097</x:v>
+        <x:v>2098</x:v>
       </x:c>
       <x:c r="J176" s="134"/>
       <x:c r="K176" s="134"/>
@@ -52208,20 +52217,20 @@
         <x:v>674</x:v>
       </x:c>
       <x:c r="D177" s="116" t="s">
-        <x:v>2098</x:v>
+        <x:v>2099</x:v>
       </x:c>
       <x:c r="E177" s="116" t="s">
-        <x:v>2099</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="F177" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G177" s="320" t="s">
-        <x:v>2100</x:v>
+        <x:v>2101</x:v>
       </x:c>
       <x:c r="H177" s="116"/>
       <x:c r="I177" s="320" t="s">
-        <x:v>2101</x:v>
+        <x:v>2102</x:v>
       </x:c>
       <x:c r="J177" s="134"/>
       <x:c r="K177" s="134"/>
@@ -52237,11 +52246,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G178" s="320" t="s">
-        <x:v>2102</x:v>
+        <x:v>2103</x:v>
       </x:c>
       <x:c r="H178" s="116"/>
       <x:c r="I178" s="320" t="s">
-        <x:v>2103</x:v>
+        <x:v>2104</x:v>
       </x:c>
       <x:c r="J178" s="134"/>
       <x:c r="K178" s="134"/>
@@ -52258,22 +52267,22 @@
         <x:v>677</x:v>
       </x:c>
       <x:c r="D179" s="116" t="s">
-        <x:v>2104</x:v>
+        <x:v>2105</x:v>
       </x:c>
       <x:c r="E179" s="116" t="s">
-        <x:v>2105</x:v>
+        <x:v>2106</x:v>
       </x:c>
       <x:c r="F179" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G179" s="320" t="s">
-        <x:v>2106</x:v>
+        <x:v>2107</x:v>
       </x:c>
       <x:c r="H179" s="116" t="s">
         <x:v>681</x:v>
       </x:c>
       <x:c r="I179" s="320" t="s">
-        <x:v>2107</x:v>
+        <x:v>2108</x:v>
       </x:c>
       <x:c r="J179" s="116"/>
       <x:c r="K179" s="134"/>
@@ -52289,13 +52298,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G180" s="321" t="s">
-        <x:v>2108</x:v>
+        <x:v>2109</x:v>
       </x:c>
       <x:c r="H180" s="115" t="s">
-        <x:v>2109</x:v>
+        <x:v>2110</x:v>
       </x:c>
       <x:c r="I180" s="321" t="s">
-        <x:v>2110</x:v>
+        <x:v>2111</x:v>
       </x:c>
       <x:c r="J180" s="115"/>
       <x:c r="K180" s="137"/>
@@ -52312,22 +52321,22 @@
         <x:v>686</x:v>
       </x:c>
       <x:c r="D181" s="116" t="s">
-        <x:v>2111</x:v>
+        <x:v>2112</x:v>
       </x:c>
       <x:c r="E181" s="116" t="s">
-        <x:v>2112</x:v>
+        <x:v>2113</x:v>
       </x:c>
       <x:c r="F181" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G181" s="320" t="s">
-        <x:v>2113</x:v>
+        <x:v>2114</x:v>
       </x:c>
       <x:c r="H181" s="116" t="s">
-        <x:v>2114</x:v>
+        <x:v>2115</x:v>
       </x:c>
       <x:c r="I181" s="320" t="s">
-        <x:v>2115</x:v>
+        <x:v>2116</x:v>
       </x:c>
       <x:c r="J181" s="134"/>
       <x:c r="K181" s="134"/>
@@ -52343,13 +52352,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G182" s="320" t="s">
-        <x:v>2116</x:v>
+        <x:v>2117</x:v>
       </x:c>
       <x:c r="H182" s="116" t="s">
-        <x:v>2117</x:v>
+        <x:v>2118</x:v>
       </x:c>
       <x:c r="I182" s="320" t="s">
-        <x:v>2118</x:v>
+        <x:v>2119</x:v>
       </x:c>
       <x:c r="J182" s="134"/>
       <x:c r="K182" s="134"/>
@@ -52365,11 +52374,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G183" s="320" t="s">
-        <x:v>2119</x:v>
+        <x:v>2120</x:v>
       </x:c>
       <x:c r="H183" s="116"/>
       <x:c r="I183" s="320" t="s">
-        <x:v>2120</x:v>
+        <x:v>2121</x:v>
       </x:c>
       <x:c r="J183" s="134"/>
       <x:c r="K183" s="134"/>
@@ -52386,20 +52395,20 @@
         <x:v>696</x:v>
       </x:c>
       <x:c r="D184" s="116" t="s">
-        <x:v>2121</x:v>
+        <x:v>2122</x:v>
       </x:c>
       <x:c r="E184" s="116" t="s">
-        <x:v>2122</x:v>
+        <x:v>2123</x:v>
       </x:c>
       <x:c r="F184" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G184" s="320" t="s">
-        <x:v>2123</x:v>
+        <x:v>2124</x:v>
       </x:c>
       <x:c r="H184" s="116"/>
       <x:c r="I184" s="320" t="s">
-        <x:v>2124</x:v>
+        <x:v>2125</x:v>
       </x:c>
       <x:c r="J184" s="134"/>
       <x:c r="K184" s="134"/>
@@ -52415,13 +52424,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G185" s="320" t="s">
-        <x:v>2125</x:v>
+        <x:v>2126</x:v>
       </x:c>
       <x:c r="H185" s="116" t="s">
-        <x:v>2126</x:v>
+        <x:v>2127</x:v>
       </x:c>
       <x:c r="I185" s="320" t="s">
-        <x:v>2127</x:v>
+        <x:v>2128</x:v>
       </x:c>
       <x:c r="J185" s="134"/>
       <x:c r="K185" s="134"/>
@@ -52437,11 +52446,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G186" s="320" t="s">
-        <x:v>2128</x:v>
+        <x:v>2129</x:v>
       </x:c>
       <x:c r="H186" s="116"/>
       <x:c r="I186" s="320" t="s">
-        <x:v>2129</x:v>
+        <x:v>2130</x:v>
       </x:c>
       <x:c r="J186" s="134"/>
       <x:c r="K186" s="134"/>
@@ -52457,11 +52466,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G187" s="320" t="s">
-        <x:v>2130</x:v>
+        <x:v>2131</x:v>
       </x:c>
       <x:c r="H187" s="116"/>
       <x:c r="I187" s="320" t="s">
-        <x:v>2131</x:v>
+        <x:v>2132</x:v>
       </x:c>
       <x:c r="J187" s="134"/>
       <x:c r="K187" s="134"/>
@@ -52478,22 +52487,22 @@
         <x:v>932</x:v>
       </x:c>
       <x:c r="D188" s="114" t="s">
-        <x:v>2132</x:v>
+        <x:v>2133</x:v>
       </x:c>
       <x:c r="E188" s="114" t="s">
-        <x:v>2133</x:v>
+        <x:v>2134</x:v>
       </x:c>
       <x:c r="F188" s="329">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G188" s="324" t="s">
-        <x:v>2134</x:v>
+        <x:v>2135</x:v>
       </x:c>
       <x:c r="H188" s="324" t="s">
-        <x:v>2135</x:v>
+        <x:v>2136</x:v>
       </x:c>
       <x:c r="I188" s="325" t="s">
-        <x:v>2136</x:v>
+        <x:v>2137</x:v>
       </x:c>
       <x:c r="J188" s="61"/>
       <x:c r="K188" s="133"/>
@@ -52509,13 +52518,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G189" s="324" t="s">
-        <x:v>2137</x:v>
+        <x:v>2138</x:v>
       </x:c>
       <x:c r="H189" s="324" t="s">
-        <x:v>2138</x:v>
+        <x:v>2139</x:v>
       </x:c>
       <x:c r="I189" s="325" t="s">
-        <x:v>2139</x:v>
+        <x:v>2140</x:v>
       </x:c>
       <x:c r="J189" s="61"/>
       <x:c r="K189" s="124"/>
@@ -52531,11 +52540,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G190" s="324" t="s">
-        <x:v>2140</x:v>
+        <x:v>2141</x:v>
       </x:c>
       <x:c r="H190" s="324"/>
       <x:c r="I190" s="325" t="s">
-        <x:v>2141</x:v>
+        <x:v>2142</x:v>
       </x:c>
       <x:c r="J190" s="61"/>
       <x:c r="K190" s="111"/>
@@ -52552,20 +52561,20 @@
         <x:v>947</x:v>
       </x:c>
       <x:c r="D191" s="114" t="s">
-        <x:v>2142</x:v>
+        <x:v>2143</x:v>
       </x:c>
       <x:c r="E191" s="114" t="s">
-        <x:v>2143</x:v>
+        <x:v>2144</x:v>
       </x:c>
       <x:c r="F191" s="329">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G191" s="324" t="s">
-        <x:v>2144</x:v>
+        <x:v>2145</x:v>
       </x:c>
       <x:c r="H191" s="324"/>
       <x:c r="I191" s="325" t="s">
-        <x:v>2145</x:v>
+        <x:v>2146</x:v>
       </x:c>
       <x:c r="J191" s="61"/>
       <x:c r="K191" s="133"/>
@@ -52581,11 +52590,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G192" s="324" t="s">
-        <x:v>2146</x:v>
+        <x:v>2147</x:v>
       </x:c>
       <x:c r="H192" s="324"/>
       <x:c r="I192" s="325" t="s">
-        <x:v>2147</x:v>
+        <x:v>2148</x:v>
       </x:c>
       <x:c r="J192" s="61"/>
       <x:c r="K192" s="124"/>
@@ -52601,13 +52610,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G193" s="324" t="s">
-        <x:v>2148</x:v>
+        <x:v>2149</x:v>
       </x:c>
       <x:c r="H193" s="324" t="s">
-        <x:v>2149</x:v>
+        <x:v>2150</x:v>
       </x:c>
       <x:c r="I193" s="325" t="s">
-        <x:v>2150</x:v>
+        <x:v>2151</x:v>
       </x:c>
       <x:c r="J193" s="61"/>
       <x:c r="K193" s="111"/>
@@ -52952,16 +52961,16 @@
     <x:mergeCell ref="L191:L193"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H49" r:id="rId140"/>
-    <x:hyperlink ref="H67" r:id="rId141"/>
-    <x:hyperlink ref="H76" r:id="rId142"/>
-    <x:hyperlink ref="H85" r:id="rId143"/>
-    <x:hyperlink ref="H94" r:id="rId144"/>
-    <x:hyperlink ref="H103" r:id="rId145"/>
-    <x:hyperlink ref="H112" r:id="rId146"/>
-    <x:hyperlink ref="H4" r:id="rId147"/>
-    <x:hyperlink ref="H54" r:id="rId148"/>
-    <x:hyperlink ref="H58" r:id="rId149"/>
+    <x:hyperlink ref="H49" r:id="rId185"/>
+    <x:hyperlink ref="H67" r:id="rId186"/>
+    <x:hyperlink ref="H76" r:id="rId187"/>
+    <x:hyperlink ref="H85" r:id="rId188"/>
+    <x:hyperlink ref="H94" r:id="rId189"/>
+    <x:hyperlink ref="H103" r:id="rId190"/>
+    <x:hyperlink ref="H112" r:id="rId191"/>
+    <x:hyperlink ref="H4" r:id="rId192"/>
+    <x:hyperlink ref="H54" r:id="rId193"/>
+    <x:hyperlink ref="H58" r:id="rId194"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -53054,7 +53063,7 @@
         <x:v>1270</x:v>
       </x:c>
       <x:c r="H2" s="288" t="s">
-        <x:v>2151</x:v>
+        <x:v>2152</x:v>
       </x:c>
       <x:c r="I2" s="134" t="s">
         <x:v>1272</x:v>
@@ -53101,7 +53110,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="297" t="s">
-        <x:v>2152</x:v>
+        <x:v>2153</x:v>
       </x:c>
       <x:c r="H4" s="297" t="s">
         <x:v>1277</x:v>
@@ -53181,7 +53190,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="297" t="s">
-        <x:v>2153</x:v>
+        <x:v>2154</x:v>
       </x:c>
       <x:c r="H7" s="297"/>
       <x:c r="I7" s="298" t="s">
@@ -53214,7 +53223,7 @@
         <x:v>1297</x:v>
       </x:c>
       <x:c r="H8" s="297" t="s">
-        <x:v>2154</x:v>
+        <x:v>2155</x:v>
       </x:c>
       <x:c r="I8" s="134" t="s">
         <x:v>1299</x:v>
@@ -53233,7 +53242,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G9" s="319" t="s">
-        <x:v>2155</x:v>
+        <x:v>2156</x:v>
       </x:c>
       <x:c r="H9" s="297"/>
       <x:c r="I9" s="134"/>
@@ -53322,7 +53331,7 @@
         <x:v>1297</x:v>
       </x:c>
       <x:c r="H13" s="297" t="s">
-        <x:v>2156</x:v>
+        <x:v>2157</x:v>
       </x:c>
       <x:c r="I13" s="134" t="s">
         <x:v>1307</x:v>
@@ -53341,7 +53350,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="319" t="s">
-        <x:v>2155</x:v>
+        <x:v>2156</x:v>
       </x:c>
       <x:c r="H14" s="297"/>
       <x:c r="I14" s="134"/>
@@ -53427,7 +53436,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="61" t="s">
-        <x:v>2157</x:v>
+        <x:v>2158</x:v>
       </x:c>
       <x:c r="H18" s="140"/>
       <x:c r="I18" s="140" t="s">
@@ -53447,7 +53456,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="61" t="s">
-        <x:v>2158</x:v>
+        <x:v>2159</x:v>
       </x:c>
       <x:c r="H19" s="140" t="s">
         <x:v>965</x:v>
@@ -53467,7 +53476,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="61" t="s">
-        <x:v>2159</x:v>
+        <x:v>2160</x:v>
       </x:c>
       <x:c r="H20" s="140"/>
       <x:c r="I20" s="140"/>
@@ -53485,7 +53494,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G21" s="61" t="s">
-        <x:v>2160</x:v>
+        <x:v>2161</x:v>
       </x:c>
       <x:c r="H21" s="140" t="s">
         <x:v>968</x:v>
@@ -53505,7 +53514,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G22" s="61" t="s">
-        <x:v>2161</x:v>
+        <x:v>2162</x:v>
       </x:c>
       <x:c r="H22" s="314" t="s">
         <x:v>970</x:v>
@@ -53525,7 +53534,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G23" s="61" t="s">
-        <x:v>2162</x:v>
+        <x:v>2163</x:v>
       </x:c>
       <x:c r="H23" s="140">
         <x:v>1</x:v>
@@ -53545,7 +53554,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G24" s="61" t="s">
-        <x:v>2163</x:v>
+        <x:v>2164</x:v>
       </x:c>
       <x:c r="H24" s="140" t="s">
         <x:v>973</x:v>
@@ -53565,7 +53574,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G25" s="61" t="s">
-        <x:v>2164</x:v>
+        <x:v>2165</x:v>
       </x:c>
       <x:c r="H25" s="140"/>
       <x:c r="I25" s="140"/>
@@ -53593,7 +53602,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G26" s="61" t="s">
-        <x:v>2165</x:v>
+        <x:v>2166</x:v>
       </x:c>
       <x:c r="H26" s="140"/>
       <x:c r="I26" s="133" t="s">
@@ -53633,7 +53642,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G28" s="61" t="s">
-        <x:v>2166</x:v>
+        <x:v>2167</x:v>
       </x:c>
       <x:c r="H28" s="239" t="s">
         <x:v>970</x:v>
@@ -53653,7 +53662,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G29" s="61" t="s">
-        <x:v>2167</x:v>
+        <x:v>2168</x:v>
       </x:c>
       <x:c r="H29" s="140">
         <x:v>1</x:v>
@@ -53673,7 +53682,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G30" s="61" t="s">
-        <x:v>2168</x:v>
+        <x:v>2169</x:v>
       </x:c>
       <x:c r="H30" s="140"/>
       <x:c r="I30" s="111"/>
@@ -53701,7 +53710,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="61" t="s">
-        <x:v>2169</x:v>
+        <x:v>2170</x:v>
       </x:c>
       <x:c r="H31" s="140"/>
       <x:c r="I31" s="133" t="s">
@@ -53800,7 +53809,7 @@
         <x:v>1309</x:v>
       </x:c>
       <x:c r="D36" s="134" t="s">
-        <x:v>2170</x:v>
+        <x:v>2171</x:v>
       </x:c>
       <x:c r="E36" s="134" t="s">
         <x:v>1311</x:v>
@@ -53812,7 +53821,7 @@
         <x:v>988</x:v>
       </x:c>
       <x:c r="H36" s="297" t="s">
-        <x:v>2171</x:v>
+        <x:v>2172</x:v>
       </x:c>
       <x:c r="I36" s="134" t="s">
         <x:v>1312</x:v>
@@ -53834,7 +53843,7 @@
         <x:v>990</x:v>
       </x:c>
       <x:c r="H37" s="314" t="s">
-        <x:v>2172</x:v>
+        <x:v>2173</x:v>
       </x:c>
       <x:c r="I37" s="134"/>
       <x:c r="J37" s="9"/>
@@ -53870,7 +53879,7 @@
         <x:v>1314</x:v>
       </x:c>
       <x:c r="D39" s="134" t="s">
-        <x:v>2173</x:v>
+        <x:v>2174</x:v>
       </x:c>
       <x:c r="E39" s="134" t="s">
         <x:v>1311</x:v>
@@ -53879,10 +53888,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G39" s="319" t="s">
-        <x:v>2174</x:v>
+        <x:v>2175</x:v>
       </x:c>
       <x:c r="H39" s="297" t="s">
-        <x:v>2175</x:v>
+        <x:v>2176</x:v>
       </x:c>
       <x:c r="I39" s="134" t="s">
         <x:v>1317</x:v>
@@ -53904,7 +53913,7 @@
         <x:v>990</x:v>
       </x:c>
       <x:c r="H40" s="314" t="s">
-        <x:v>2172</x:v>
+        <x:v>2173</x:v>
       </x:c>
       <x:c r="I40" s="134"/>
       <x:c r="J40" s="9"/>
@@ -56840,17 +56849,17 @@
     <x:mergeCell ref="J168:J171"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H22" r:id="rId150"/>
-    <x:hyperlink ref="H28" r:id="rId151"/>
-    <x:hyperlink ref="H11" r:id="rId152"/>
-    <x:hyperlink ref="H16" r:id="rId153"/>
-    <x:hyperlink ref="H37" r:id="rId154"/>
-    <x:hyperlink ref="H40" r:id="rId155"/>
-    <x:hyperlink ref="H130" r:id="rId156"/>
-    <x:hyperlink ref="H136" r:id="rId157"/>
-    <x:hyperlink ref="H142" r:id="rId158"/>
-    <x:hyperlink ref="H148" r:id="rId159"/>
-    <x:hyperlink ref="H154" r:id="rId160"/>
+    <x:hyperlink ref="H22" r:id="rId195"/>
+    <x:hyperlink ref="H28" r:id="rId196"/>
+    <x:hyperlink ref="H11" r:id="rId197"/>
+    <x:hyperlink ref="H16" r:id="rId198"/>
+    <x:hyperlink ref="H37" r:id="rId199"/>
+    <x:hyperlink ref="H40" r:id="rId200"/>
+    <x:hyperlink ref="H130" r:id="rId201"/>
+    <x:hyperlink ref="H136" r:id="rId202"/>
+    <x:hyperlink ref="H142" r:id="rId203"/>
+    <x:hyperlink ref="H148" r:id="rId204"/>
+    <x:hyperlink ref="H154" r:id="rId205"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -56935,19 +56944,19 @@
         <x:v>705</x:v>
       </x:c>
       <x:c r="E2" s="116" t="s">
-        <x:v>2176</x:v>
+        <x:v>2177</x:v>
       </x:c>
       <x:c r="F2" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G2" s="327" t="s">
-        <x:v>2177</x:v>
+        <x:v>2178</x:v>
       </x:c>
       <x:c r="H2" s="116" t="s">
-        <x:v>2178</x:v>
+        <x:v>2179</x:v>
       </x:c>
       <x:c r="I2" s="289" t="s">
-        <x:v>2179</x:v>
+        <x:v>2180</x:v>
       </x:c>
       <x:c r="J2" s="1"/>
       <x:c r="K2" s="1"/>
@@ -56963,11 +56972,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G3" s="327" t="s">
-        <x:v>2180</x:v>
+        <x:v>2181</x:v>
       </x:c>
       <x:c r="H3" s="116"/>
       <x:c r="I3" s="289" t="s">
-        <x:v>2181</x:v>
+        <x:v>2182</x:v>
       </x:c>
       <x:c r="J3" s="1"/>
       <x:c r="K3" s="1"/>
@@ -56987,19 +56996,19 @@
         <x:v>707</x:v>
       </x:c>
       <x:c r="E4" s="116" t="s">
-        <x:v>2176</x:v>
+        <x:v>2177</x:v>
       </x:c>
       <x:c r="F4" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="327" t="s">
-        <x:v>2182</x:v>
+        <x:v>2183</x:v>
       </x:c>
       <x:c r="H4" s="116" t="s">
-        <x:v>2183</x:v>
+        <x:v>2184</x:v>
       </x:c>
       <x:c r="I4" s="289" t="s">
-        <x:v>2184</x:v>
+        <x:v>2185</x:v>
       </x:c>
       <x:c r="J4" s="61"/>
       <x:c r="K4" s="1"/>
@@ -57015,11 +57024,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G5" s="327" t="s">
-        <x:v>2185</x:v>
+        <x:v>2186</x:v>
       </x:c>
       <x:c r="H5" s="116"/>
       <x:c r="I5" s="289" t="s">
-        <x:v>2186</x:v>
+        <x:v>2187</x:v>
       </x:c>
       <x:c r="J5" s="61"/>
       <x:c r="K5" s="1"/>
@@ -57035,11 +57044,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G6" s="327" t="s">
-        <x:v>2079</x:v>
+        <x:v>2080</x:v>
       </x:c>
       <x:c r="H6" s="116"/>
       <x:c r="I6" s="289" t="s">
-        <x:v>2187</x:v>
+        <x:v>2188</x:v>
       </x:c>
       <x:c r="J6" s="61"/>
       <x:c r="K6" s="1"/>
@@ -57059,19 +57068,19 @@
         <x:v>709</x:v>
       </x:c>
       <x:c r="E7" s="116" t="s">
-        <x:v>2188</x:v>
+        <x:v>2189</x:v>
       </x:c>
       <x:c r="F7" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="327" t="s">
-        <x:v>2189</x:v>
+        <x:v>2190</x:v>
       </x:c>
       <x:c r="H7" s="116" t="s">
-        <x:v>2190</x:v>
+        <x:v>2191</x:v>
       </x:c>
       <x:c r="I7" s="289" t="s">
-        <x:v>2191</x:v>
+        <x:v>2192</x:v>
       </x:c>
       <x:c r="J7" s="61"/>
       <x:c r="K7" s="1"/>
@@ -57087,11 +57096,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G8" s="327" t="s">
-        <x:v>2079</x:v>
+        <x:v>2080</x:v>
       </x:c>
       <x:c r="H8" s="116"/>
       <x:c r="I8" s="289" t="s">
-        <x:v>2192</x:v>
+        <x:v>2193</x:v>
       </x:c>
       <x:c r="J8" s="61"/>
       <x:c r="K8" s="1"/>
@@ -57107,11 +57116,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G9" s="327" t="s">
-        <x:v>2193</x:v>
+        <x:v>2194</x:v>
       </x:c>
       <x:c r="H9" s="116"/>
       <x:c r="I9" s="289" t="s">
-        <x:v>2194</x:v>
+        <x:v>2195</x:v>
       </x:c>
       <x:c r="J9" s="61"/>
       <x:c r="K9" s="1"/>
@@ -57128,20 +57137,20 @@
         <x:v>717</x:v>
       </x:c>
       <x:c r="D10" s="116" t="s">
-        <x:v>2195</x:v>
+        <x:v>2196</x:v>
       </x:c>
       <x:c r="E10" s="116" t="s">
-        <x:v>2196</x:v>
+        <x:v>2197</x:v>
       </x:c>
       <x:c r="F10" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="327" t="s">
-        <x:v>2100</x:v>
+        <x:v>2101</x:v>
       </x:c>
       <x:c r="H10" s="116"/>
       <x:c r="I10" s="289" t="s">
-        <x:v>2197</x:v>
+        <x:v>2198</x:v>
       </x:c>
       <x:c r="J10" s="61"/>
       <x:c r="K10" s="1"/>
@@ -57157,11 +57166,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G11" s="327" t="s">
-        <x:v>2198</x:v>
+        <x:v>2199</x:v>
       </x:c>
       <x:c r="H11" s="116"/>
       <x:c r="I11" s="289" t="s">
-        <x:v>2199</x:v>
+        <x:v>2200</x:v>
       </x:c>
       <x:c r="J11" s="61"/>
       <x:c r="K11" s="1"/>
@@ -57177,11 +57186,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G12" s="327" t="s">
-        <x:v>2200</x:v>
+        <x:v>2201</x:v>
       </x:c>
       <x:c r="H12" s="116"/>
       <x:c r="I12" s="289" t="s">
-        <x:v>2201</x:v>
+        <x:v>2202</x:v>
       </x:c>
       <x:c r="J12" s="61"/>
       <x:c r="K12" s="1"/>
@@ -57198,20 +57207,20 @@
         <x:v>722</x:v>
       </x:c>
       <x:c r="D13" s="116" t="s">
-        <x:v>2202</x:v>
+        <x:v>2203</x:v>
       </x:c>
       <x:c r="E13" s="116" t="s">
-        <x:v>2203</x:v>
+        <x:v>2204</x:v>
       </x:c>
       <x:c r="F13" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="327" t="s">
-        <x:v>2079</x:v>
+        <x:v>2080</x:v>
       </x:c>
       <x:c r="H13" s="116"/>
       <x:c r="I13" s="289" t="s">
-        <x:v>2204</x:v>
+        <x:v>2205</x:v>
       </x:c>
       <x:c r="J13" s="61"/>
       <x:c r="K13" s="1"/>
@@ -57227,11 +57236,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="327" t="s">
-        <x:v>2205</x:v>
+        <x:v>2206</x:v>
       </x:c>
       <x:c r="H14" s="116"/>
       <x:c r="I14" s="289" t="s">
-        <x:v>2206</x:v>
+        <x:v>2207</x:v>
       </x:c>
       <x:c r="J14" s="61"/>
       <x:c r="K14" s="1"/>
@@ -57248,22 +57257,22 @@
         <x:v>724</x:v>
       </x:c>
       <x:c r="D15" s="116" t="s">
-        <x:v>2207</x:v>
+        <x:v>2208</x:v>
       </x:c>
       <x:c r="E15" s="116" t="s">
-        <x:v>2208</x:v>
+        <x:v>2209</x:v>
       </x:c>
       <x:c r="F15" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G15" s="327" t="s">
-        <x:v>2209</x:v>
+        <x:v>2210</x:v>
       </x:c>
       <x:c r="H15" s="116" t="s">
-        <x:v>2210</x:v>
+        <x:v>2211</x:v>
       </x:c>
       <x:c r="I15" s="289" t="s">
-        <x:v>2211</x:v>
+        <x:v>2212</x:v>
       </x:c>
       <x:c r="J15" s="61"/>
       <x:c r="K15" s="1"/>
@@ -57279,11 +57288,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G16" s="327" t="s">
-        <x:v>2212</x:v>
+        <x:v>2213</x:v>
       </x:c>
       <x:c r="H16" s="116"/>
       <x:c r="I16" s="289" t="s">
-        <x:v>2213</x:v>
+        <x:v>2214</x:v>
       </x:c>
       <x:c r="J16" s="61"/>
       <x:c r="K16" s="1"/>
@@ -57299,11 +57308,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G17" s="327" t="s">
-        <x:v>2214</x:v>
+        <x:v>2215</x:v>
       </x:c>
       <x:c r="H17" s="116"/>
       <x:c r="I17" s="289" t="s">
-        <x:v>2215</x:v>
+        <x:v>2216</x:v>
       </x:c>
       <x:c r="J17" s="61"/>
       <x:c r="K17" s="1"/>
@@ -57320,20 +57329,20 @@
         <x:v>726</x:v>
       </x:c>
       <x:c r="D18" s="116" t="s">
-        <x:v>2216</x:v>
+        <x:v>2217</x:v>
       </x:c>
       <x:c r="E18" s="116" t="s">
-        <x:v>2217</x:v>
+        <x:v>2218</x:v>
       </x:c>
       <x:c r="F18" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="327" t="s">
-        <x:v>2218</x:v>
+        <x:v>2219</x:v>
       </x:c>
       <x:c r="H18" s="116"/>
       <x:c r="I18" s="289" t="s">
-        <x:v>2219</x:v>
+        <x:v>2220</x:v>
       </x:c>
       <x:c r="J18" s="61"/>
       <x:c r="K18" s="1"/>
@@ -57349,13 +57358,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="327" t="s">
-        <x:v>2220</x:v>
+        <x:v>2221</x:v>
       </x:c>
       <x:c r="H19" s="116" t="s">
-        <x:v>2221</x:v>
+        <x:v>2222</x:v>
       </x:c>
       <x:c r="I19" s="289" t="s">
-        <x:v>2222</x:v>
+        <x:v>2223</x:v>
       </x:c>
       <x:c r="J19" s="61"/>
       <x:c r="K19" s="1"/>
@@ -57371,11 +57380,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="327" t="s">
-        <x:v>2223</x:v>
+        <x:v>2224</x:v>
       </x:c>
       <x:c r="H20" s="116"/>
       <x:c r="I20" s="289" t="s">
-        <x:v>2224</x:v>
+        <x:v>2225</x:v>
       </x:c>
       <x:c r="J20" s="61"/>
       <x:c r="K20" s="1"/>
@@ -57386,7 +57395,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B21" s="116" t="s">
-        <x:v>2225</x:v>
+        <x:v>2226</x:v>
       </x:c>
       <x:c r="C21" s="116" t="s">
         <x:v>732</x:v>
@@ -57395,19 +57404,19 @@
         <x:v>733</x:v>
       </x:c>
       <x:c r="E21" s="116" t="s">
-        <x:v>2226</x:v>
+        <x:v>2227</x:v>
       </x:c>
       <x:c r="F21" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G21" s="327" t="s">
-        <x:v>2227</x:v>
+        <x:v>2228</x:v>
       </x:c>
       <x:c r="H21" s="116" t="s">
         <x:v>741</x:v>
       </x:c>
       <x:c r="I21" s="289" t="s">
-        <x:v>2228</x:v>
+        <x:v>2229</x:v>
       </x:c>
       <x:c r="J21" s="61"/>
       <x:c r="K21" s="1"/>
@@ -57423,11 +57432,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G22" s="327" t="s">
-        <x:v>2229</x:v>
+        <x:v>2230</x:v>
       </x:c>
       <x:c r="H22" s="116"/>
       <x:c r="I22" s="289" t="s">
-        <x:v>2230</x:v>
+        <x:v>2231</x:v>
       </x:c>
       <x:c r="J22" s="61"/>
       <x:c r="K22" s="1"/>
@@ -57443,11 +57452,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G23" s="327" t="s">
-        <x:v>2231</x:v>
+        <x:v>2232</x:v>
       </x:c>
       <x:c r="H23" s="116"/>
       <x:c r="I23" s="289" t="s">
-        <x:v>2232</x:v>
+        <x:v>2233</x:v>
       </x:c>
       <x:c r="J23" s="61"/>
       <x:c r="K23" s="1"/>
@@ -57464,20 +57473,20 @@
         <x:v>737</x:v>
       </x:c>
       <x:c r="D24" s="116" t="s">
-        <x:v>2233</x:v>
+        <x:v>2234</x:v>
       </x:c>
       <x:c r="E24" s="116" t="s">
-        <x:v>2234</x:v>
+        <x:v>2235</x:v>
       </x:c>
       <x:c r="F24" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G24" s="327" t="s">
-        <x:v>2235</x:v>
+        <x:v>2236</x:v>
       </x:c>
       <x:c r="H24" s="116"/>
       <x:c r="I24" s="289" t="s">
-        <x:v>2236</x:v>
+        <x:v>2237</x:v>
       </x:c>
       <x:c r="J24" s="61"/>
       <x:c r="K24" s="35"/>
@@ -57493,11 +57502,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G25" s="327" t="s">
-        <x:v>2237</x:v>
+        <x:v>2238</x:v>
       </x:c>
       <x:c r="H25" s="116"/>
       <x:c r="I25" s="289" t="s">
-        <x:v>2238</x:v>
+        <x:v>2239</x:v>
       </x:c>
       <x:c r="J25" s="61"/>
       <x:c r="K25" s="35"/>
@@ -57513,11 +57522,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G26" s="327" t="s">
-        <x:v>2130</x:v>
+        <x:v>2131</x:v>
       </x:c>
       <x:c r="H26" s="116"/>
       <x:c r="I26" s="289" t="s">
-        <x:v>2239</x:v>
+        <x:v>2240</x:v>
       </x:c>
       <x:c r="J26" s="61"/>
       <x:c r="K26" s="35"/>
@@ -57534,20 +57543,20 @@
         <x:v>751</x:v>
       </x:c>
       <x:c r="D27" s="116" t="s">
-        <x:v>2240</x:v>
+        <x:v>2241</x:v>
       </x:c>
       <x:c r="E27" s="116" t="s">
-        <x:v>2241</x:v>
+        <x:v>2242</x:v>
       </x:c>
       <x:c r="F27" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G27" s="327" t="s">
-        <x:v>2242</x:v>
+        <x:v>2243</x:v>
       </x:c>
       <x:c r="H27" s="116"/>
       <x:c r="I27" s="327" t="s">
-        <x:v>2085</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="J27" s="61"/>
       <x:c r="K27" s="35"/>
@@ -57563,11 +57572,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G28" s="327" t="s">
-        <x:v>2243</x:v>
+        <x:v>2244</x:v>
       </x:c>
       <x:c r="H28" s="116"/>
       <x:c r="I28" s="289" t="s">
-        <x:v>2244</x:v>
+        <x:v>2245</x:v>
       </x:c>
       <x:c r="J28" s="61"/>
       <x:c r="K28" s="35"/>
@@ -57584,20 +57593,20 @@
         <x:v>753</x:v>
       </x:c>
       <x:c r="D29" s="116" t="s">
-        <x:v>2245</x:v>
+        <x:v>2246</x:v>
       </x:c>
       <x:c r="E29" s="116" t="s">
-        <x:v>2241</x:v>
+        <x:v>2242</x:v>
       </x:c>
       <x:c r="F29" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G29" s="327" t="s">
-        <x:v>2246</x:v>
+        <x:v>2247</x:v>
       </x:c>
       <x:c r="H29" s="116"/>
       <x:c r="I29" s="327" t="s">
-        <x:v>2085</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="J29" s="61"/>
       <x:c r="K29" s="35"/>
@@ -57613,11 +57622,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G30" s="327" t="s">
-        <x:v>2247</x:v>
+        <x:v>2248</x:v>
       </x:c>
       <x:c r="H30" s="116"/>
       <x:c r="I30" s="289" t="s">
-        <x:v>2248</x:v>
+        <x:v>2249</x:v>
       </x:c>
       <x:c r="J30" s="61"/>
       <x:c r="K30" s="35"/>
@@ -57637,19 +57646,19 @@
         <x:v>793</x:v>
       </x:c>
       <x:c r="E31" s="116" t="s">
-        <x:v>2249</x:v>
+        <x:v>2250</x:v>
       </x:c>
       <x:c r="F31" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="327" t="s">
-        <x:v>2250</x:v>
+        <x:v>2251</x:v>
       </x:c>
       <x:c r="H31" s="116" t="s">
-        <x:v>2251</x:v>
+        <x:v>2252</x:v>
       </x:c>
       <x:c r="I31" s="289" t="s">
-        <x:v>2252</x:v>
+        <x:v>2253</x:v>
       </x:c>
       <x:c r="J31" s="61"/>
       <x:c r="K31" s="35"/>
@@ -57665,11 +57674,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G32" s="327" t="s">
-        <x:v>2253</x:v>
+        <x:v>2254</x:v>
       </x:c>
       <x:c r="H32" s="116"/>
       <x:c r="I32" s="289" t="s">
-        <x:v>2254</x:v>
+        <x:v>2255</x:v>
       </x:c>
       <x:c r="J32" s="61"/>
       <x:c r="K32" s="35"/>
@@ -57689,19 +57698,19 @@
         <x:v>798</x:v>
       </x:c>
       <x:c r="E33" s="116" t="s">
-        <x:v>2255</x:v>
+        <x:v>2256</x:v>
       </x:c>
       <x:c r="F33" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G33" s="327" t="s">
-        <x:v>2256</x:v>
+        <x:v>2257</x:v>
       </x:c>
       <x:c r="H33" s="116" t="s">
-        <x:v>2251</x:v>
+        <x:v>2252</x:v>
       </x:c>
       <x:c r="I33" s="327" t="s">
-        <x:v>2085</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="J33" s="61"/>
       <x:c r="K33" s="35"/>
@@ -57717,11 +57726,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G34" s="327" t="s">
-        <x:v>2257</x:v>
+        <x:v>2258</x:v>
       </x:c>
       <x:c r="H34" s="116"/>
       <x:c r="I34" s="289" t="s">
-        <x:v>2258</x:v>
+        <x:v>2259</x:v>
       </x:c>
       <x:c r="J34" s="292"/>
       <x:c r="K34" s="35"/>
@@ -57738,20 +57747,20 @@
         <x:v>802</x:v>
       </x:c>
       <x:c r="D35" s="116" t="s">
-        <x:v>2259</x:v>
+        <x:v>2260</x:v>
       </x:c>
       <x:c r="E35" s="116" t="s">
-        <x:v>2260</x:v>
+        <x:v>2261</x:v>
       </x:c>
       <x:c r="F35" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G35" s="327" t="s">
-        <x:v>2261</x:v>
+        <x:v>2262</x:v>
       </x:c>
       <x:c r="H35" s="116"/>
       <x:c r="I35" s="289" t="s">
-        <x:v>2262</x:v>
+        <x:v>2263</x:v>
       </x:c>
       <x:c r="J35" s="61"/>
       <x:c r="K35" s="35"/>
@@ -57767,11 +57776,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G36" s="327" t="s">
-        <x:v>2263</x:v>
+        <x:v>2264</x:v>
       </x:c>
       <x:c r="H36" s="116"/>
       <x:c r="I36" s="289" t="s">
-        <x:v>2264</x:v>
+        <x:v>2265</x:v>
       </x:c>
       <x:c r="J36" s="61"/>
       <x:c r="K36" s="35"/>
@@ -57787,13 +57796,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G37" s="327" t="s">
-        <x:v>2265</x:v>
+        <x:v>2266</x:v>
       </x:c>
       <x:c r="H37" s="116" t="s">
-        <x:v>2266</x:v>
+        <x:v>2267</x:v>
       </x:c>
       <x:c r="I37" s="289" t="s">
-        <x:v>2267</x:v>
+        <x:v>2268</x:v>
       </x:c>
       <x:c r="J37" s="61"/>
       <x:c r="K37" s="35"/>
@@ -57810,20 +57819,20 @@
         <x:v>814</x:v>
       </x:c>
       <x:c r="D38" s="116" t="s">
-        <x:v>2268</x:v>
+        <x:v>2269</x:v>
       </x:c>
       <x:c r="E38" s="116" t="s">
-        <x:v>2269</x:v>
+        <x:v>2270</x:v>
       </x:c>
       <x:c r="F38" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G38" s="327" t="s">
-        <x:v>2270</x:v>
+        <x:v>2271</x:v>
       </x:c>
       <x:c r="H38" s="116"/>
       <x:c r="I38" s="289" t="s">
-        <x:v>2271</x:v>
+        <x:v>2272</x:v>
       </x:c>
       <x:c r="J38" s="61"/>
       <x:c r="K38" s="35"/>
@@ -57839,11 +57848,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G39" s="327" t="s">
-        <x:v>2272</x:v>
+        <x:v>2273</x:v>
       </x:c>
       <x:c r="H39" s="116"/>
       <x:c r="I39" s="289" t="s">
-        <x:v>2273</x:v>
+        <x:v>2274</x:v>
       </x:c>
       <x:c r="J39" s="61"/>
       <x:c r="K39" s="35"/>
@@ -57859,13 +57868,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G40" s="327" t="s">
-        <x:v>2274</x:v>
+        <x:v>2275</x:v>
       </x:c>
       <x:c r="H40" s="116" t="s">
-        <x:v>2266</x:v>
+        <x:v>2267</x:v>
       </x:c>
       <x:c r="I40" s="289" t="s">
-        <x:v>2275</x:v>
+        <x:v>2276</x:v>
       </x:c>
       <x:c r="J40" s="61"/>
       <x:c r="K40" s="35"/>
@@ -57881,11 +57890,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G41" s="327" t="s">
-        <x:v>2276</x:v>
+        <x:v>2277</x:v>
       </x:c>
       <x:c r="H41" s="116"/>
       <x:c r="I41" s="289" t="s">
-        <x:v>2277</x:v>
+        <x:v>2278</x:v>
       </x:c>
       <x:c r="J41" s="61"/>
       <x:c r="K41" s="35"/>
@@ -57902,20 +57911,20 @@
         <x:v>824</x:v>
       </x:c>
       <x:c r="D42" s="116" t="s">
-        <x:v>2278</x:v>
+        <x:v>2279</x:v>
       </x:c>
       <x:c r="E42" s="116" t="s">
-        <x:v>2279</x:v>
+        <x:v>2280</x:v>
       </x:c>
       <x:c r="F42" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G42" s="327" t="s">
-        <x:v>2280</x:v>
+        <x:v>2281</x:v>
       </x:c>
       <x:c r="H42" s="116"/>
       <x:c r="I42" s="289" t="s">
-        <x:v>2281</x:v>
+        <x:v>2282</x:v>
       </x:c>
       <x:c r="J42" s="61"/>
       <x:c r="K42" s="35"/>
@@ -57931,11 +57940,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G43" s="327" t="s">
-        <x:v>2282</x:v>
+        <x:v>2283</x:v>
       </x:c>
       <x:c r="H43" s="116"/>
       <x:c r="I43" s="289" t="s">
-        <x:v>2283</x:v>
+        <x:v>2284</x:v>
       </x:c>
       <x:c r="J43" s="61"/>
       <x:c r="K43" s="35"/>
@@ -57951,11 +57960,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G44" s="327" t="s">
-        <x:v>2284</x:v>
+        <x:v>2285</x:v>
       </x:c>
       <x:c r="H44" s="116"/>
       <x:c r="I44" s="289" t="s">
-        <x:v>2285</x:v>
+        <x:v>2286</x:v>
       </x:c>
       <x:c r="J44" s="61"/>
       <x:c r="K44" s="35"/>
@@ -57971,11 +57980,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G45" s="327" t="s">
-        <x:v>2286</x:v>
+        <x:v>2287</x:v>
       </x:c>
       <x:c r="H45" s="116"/>
       <x:c r="I45" s="289" t="s">
-        <x:v>2287</x:v>
+        <x:v>2288</x:v>
       </x:c>
       <x:c r="J45" s="61"/>
       <x:c r="K45" s="35"/>
@@ -57992,20 +58001,20 @@
         <x:v>835</x:v>
       </x:c>
       <x:c r="D46" s="116" t="s">
-        <x:v>2288</x:v>
+        <x:v>2289</x:v>
       </x:c>
       <x:c r="E46" s="116" t="s">
-        <x:v>2289</x:v>
+        <x:v>2290</x:v>
       </x:c>
       <x:c r="F46" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G46" s="327" t="s">
-        <x:v>2280</x:v>
+        <x:v>2281</x:v>
       </x:c>
       <x:c r="H46" s="116"/>
       <x:c r="I46" s="289" t="s">
-        <x:v>2290</x:v>
+        <x:v>2291</x:v>
       </x:c>
       <x:c r="J46" s="61"/>
       <x:c r="K46" s="35"/>
@@ -58021,13 +58030,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G47" s="327" t="s">
-        <x:v>2291</x:v>
+        <x:v>2292</x:v>
       </x:c>
       <x:c r="H47" s="116" t="s">
-        <x:v>2266</x:v>
+        <x:v>2267</x:v>
       </x:c>
       <x:c r="I47" s="289" t="s">
-        <x:v>2292</x:v>
+        <x:v>2293</x:v>
       </x:c>
       <x:c r="J47" s="61"/>
       <x:c r="K47" s="35"/>
@@ -58043,11 +58052,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G48" s="327" t="s">
-        <x:v>2293</x:v>
+        <x:v>2294</x:v>
       </x:c>
       <x:c r="H48" s="116"/>
       <x:c r="I48" s="289" t="s">
-        <x:v>2294</x:v>
+        <x:v>2295</x:v>
       </x:c>
       <x:c r="J48" s="61"/>
       <x:c r="K48" s="35"/>
@@ -58146,10 +58155,10 @@
         <x:v>999</x:v>
       </x:c>
       <x:c r="H52" s="334" t="s">
-        <x:v>2295</x:v>
+        <x:v>2296</x:v>
       </x:c>
       <x:c r="I52" s="51" t="s">
-        <x:v>2296</x:v>
+        <x:v>2297</x:v>
       </x:c>
       <x:c r="J52" s="51"/>
       <x:c r="K52" s="35"/>
@@ -58168,7 +58177,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H53" s="314" t="s">
-        <x:v>2297</x:v>
+        <x:v>2298</x:v>
       </x:c>
       <x:c r="I53" s="51"/>
       <x:c r="J53" s="51"/>
@@ -58219,7 +58228,7 @@
         <x:v>1000</x:v>
       </x:c>
       <x:c r="I55" s="51" t="s">
-        <x:v>2298</x:v>
+        <x:v>2299</x:v>
       </x:c>
       <x:c r="J55" s="51"/>
       <x:c r="K55" s="35"/>
@@ -58238,7 +58247,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H56" s="314" t="s">
-        <x:v>2299</x:v>
+        <x:v>2300</x:v>
       </x:c>
       <x:c r="I56" s="51"/>
       <x:c r="J56" s="51"/>
@@ -58357,7 +58366,7 @@
         <x:v>422</x:v>
       </x:c>
       <x:c r="I61" s="51" t="s">
-        <x:v>2300</x:v>
+        <x:v>2301</x:v>
       </x:c>
       <x:c r="J61" s="51"/>
       <x:c r="K61" s="35"/>
@@ -58655,7 +58664,7 @@
         <x:v>1037</x:v>
       </x:c>
       <x:c r="I74" s="51" t="s">
-        <x:v>2301</x:v>
+        <x:v>2302</x:v>
       </x:c>
       <x:c r="J74" s="51"/>
       <x:c r="K74" s="35"/>
@@ -59351,19 +59360,19 @@
         <x:v>843</x:v>
       </x:c>
       <x:c r="E106" s="116" t="s">
-        <x:v>2302</x:v>
+        <x:v>2303</x:v>
       </x:c>
       <x:c r="F106" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G106" s="327" t="s">
-        <x:v>2303</x:v>
+        <x:v>2304</x:v>
       </x:c>
       <x:c r="H106" s="116" t="s">
-        <x:v>2304</x:v>
+        <x:v>2305</x:v>
       </x:c>
       <x:c r="I106" s="289" t="s">
-        <x:v>2305</x:v>
+        <x:v>2306</x:v>
       </x:c>
       <x:c r="J106" s="61"/>
       <x:c r="K106" s="140"/>
@@ -59379,11 +59388,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G107" s="327" t="s">
-        <x:v>2306</x:v>
+        <x:v>2307</x:v>
       </x:c>
       <x:c r="H107" s="116"/>
       <x:c r="I107" s="289" t="s">
-        <x:v>2307</x:v>
+        <x:v>2308</x:v>
       </x:c>
       <x:c r="J107" s="61"/>
       <x:c r="K107" s="140"/>
@@ -59399,13 +59408,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G108" s="327" t="s">
-        <x:v>2308</x:v>
+        <x:v>2309</x:v>
       </x:c>
       <x:c r="H108" s="116" t="s">
-        <x:v>2309</x:v>
+        <x:v>2310</x:v>
       </x:c>
       <x:c r="I108" s="289" t="s">
-        <x:v>2310</x:v>
+        <x:v>2311</x:v>
       </x:c>
       <x:c r="J108" s="61"/>
       <x:c r="K108" s="140"/>
@@ -59421,11 +59430,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G109" s="327" t="s">
-        <x:v>2311</x:v>
+        <x:v>2312</x:v>
       </x:c>
       <x:c r="H109" s="116"/>
       <x:c r="I109" s="289" t="s">
-        <x:v>2312</x:v>
+        <x:v>2313</x:v>
       </x:c>
       <x:c r="J109" s="61"/>
       <x:c r="K109" s="140"/>
@@ -59445,19 +59454,19 @@
         <x:v>854</x:v>
       </x:c>
       <x:c r="E110" s="116" t="s">
-        <x:v>2313</x:v>
+        <x:v>2314</x:v>
       </x:c>
       <x:c r="F110" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G110" s="327" t="s">
-        <x:v>2314</x:v>
+        <x:v>2315</x:v>
       </x:c>
       <x:c r="H110" s="116" t="s">
-        <x:v>2315</x:v>
+        <x:v>2316</x:v>
       </x:c>
       <x:c r="I110" s="289" t="s">
-        <x:v>2316</x:v>
+        <x:v>2317</x:v>
       </x:c>
       <x:c r="J110" s="61"/>
       <x:c r="K110" s="140"/>
@@ -59473,11 +59482,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G111" s="327" t="s">
-        <x:v>2306</x:v>
+        <x:v>2307</x:v>
       </x:c>
       <x:c r="H111" s="116"/>
       <x:c r="I111" s="289" t="s">
-        <x:v>2317</x:v>
+        <x:v>2318</x:v>
       </x:c>
       <x:c r="J111" s="61"/>
       <x:c r="K111" s="140"/>
@@ -59493,13 +59502,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G112" s="327" t="s">
-        <x:v>2318</x:v>
+        <x:v>2319</x:v>
       </x:c>
       <x:c r="H112" s="116" t="s">
-        <x:v>2319</x:v>
+        <x:v>2320</x:v>
       </x:c>
       <x:c r="I112" s="289" t="s">
-        <x:v>2320</x:v>
+        <x:v>2321</x:v>
       </x:c>
       <x:c r="J112" s="61"/>
       <x:c r="K112" s="140"/>
@@ -59515,11 +59524,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G113" s="327" t="s">
-        <x:v>2321</x:v>
+        <x:v>2322</x:v>
       </x:c>
       <x:c r="H113" s="116"/>
       <x:c r="I113" s="289" t="s">
-        <x:v>2322</x:v>
+        <x:v>2323</x:v>
       </x:c>
       <x:c r="J113" s="61"/>
       <x:c r="K113" s="140"/>
@@ -59536,7 +59545,7 @@
         <x:v>863</x:v>
       </x:c>
       <x:c r="D114" s="140" t="s">
-        <x:v>2323</x:v>
+        <x:v>2324</x:v>
       </x:c>
       <x:c r="E114" s="140" t="s">
         <x:v>865</x:v>
@@ -59545,7 +59554,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G114" s="61" t="s">
-        <x:v>2324</x:v>
+        <x:v>2325</x:v>
       </x:c>
       <x:c r="H114" s="140"/>
       <x:c r="I114" s="61" t="s">
@@ -59565,7 +59574,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G115" s="61" t="s">
-        <x:v>2325</x:v>
+        <x:v>2326</x:v>
       </x:c>
       <x:c r="H115" s="140"/>
       <x:c r="I115" s="61" t="s">
@@ -59585,10 +59594,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G116" s="61" t="s">
-        <x:v>2326</x:v>
+        <x:v>2327</x:v>
       </x:c>
       <x:c r="H116" s="140" t="s">
-        <x:v>2327</x:v>
+        <x:v>2328</x:v>
       </x:c>
       <x:c r="I116" s="61"/>
       <x:c r="J116" s="140"/>
@@ -59605,10 +59614,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G117" s="61" t="s">
-        <x:v>2328</x:v>
+        <x:v>2329</x:v>
       </x:c>
       <x:c r="H117" s="140" t="s">
-        <x:v>2329</x:v>
+        <x:v>2330</x:v>
       </x:c>
       <x:c r="I117" s="61"/>
       <x:c r="J117" s="140"/>
@@ -59643,7 +59652,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G119" s="61" t="s">
-        <x:v>2330</x:v>
+        <x:v>2331</x:v>
       </x:c>
       <x:c r="H119" s="140" t="s">
         <x:v>877</x:v>
@@ -59663,7 +59672,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G120" s="61" t="s">
-        <x:v>2331</x:v>
+        <x:v>2332</x:v>
       </x:c>
       <x:c r="H120" s="251">
         <x:v>0.375</x:v>
@@ -59683,7 +59692,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G121" s="61" t="s">
-        <x:v>2332</x:v>
+        <x:v>2333</x:v>
       </x:c>
       <x:c r="H121" s="140">
         <x:v>100000</x:v>
@@ -59703,7 +59712,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="G122" s="61" t="s">
-        <x:v>2333</x:v>
+        <x:v>2334</x:v>
       </x:c>
       <x:c r="H122" s="140">
         <x:v>1</x:v>
@@ -59723,7 +59732,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G123" s="61" t="s">
-        <x:v>2334</x:v>
+        <x:v>2335</x:v>
       </x:c>
       <x:c r="H123" s="140"/>
       <x:c r="I123" s="61" t="s">
@@ -59744,7 +59753,7 @@
         <x:v>884</x:v>
       </x:c>
       <x:c r="D124" s="140" t="s">
-        <x:v>2335</x:v>
+        <x:v>2336</x:v>
       </x:c>
       <x:c r="E124" s="140" t="s">
         <x:v>886</x:v>
@@ -59753,7 +59762,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G124" s="61" t="s">
-        <x:v>2336</x:v>
+        <x:v>2337</x:v>
       </x:c>
       <x:c r="H124" s="140"/>
       <x:c r="I124" s="140" t="s">
@@ -59773,7 +59782,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G125" s="61" t="s">
-        <x:v>2337</x:v>
+        <x:v>2338</x:v>
       </x:c>
       <x:c r="H125" s="140"/>
       <x:c r="I125" s="140"/>
@@ -59791,10 +59800,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G126" s="61" t="s">
-        <x:v>2338</x:v>
+        <x:v>2339</x:v>
       </x:c>
       <x:c r="H126" s="140" t="s">
-        <x:v>2339</x:v>
+        <x:v>2340</x:v>
       </x:c>
       <x:c r="I126" s="140"/>
       <x:c r="J126" s="140"/>
@@ -59811,10 +59820,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G127" s="61" t="s">
-        <x:v>2340</x:v>
+        <x:v>2341</x:v>
       </x:c>
       <x:c r="H127" s="140" t="s">
-        <x:v>2341</x:v>
+        <x:v>2342</x:v>
       </x:c>
       <x:c r="I127" s="140"/>
       <x:c r="J127" s="140"/>
@@ -59831,7 +59840,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G128" s="61" t="s">
-        <x:v>2342</x:v>
+        <x:v>2343</x:v>
       </x:c>
       <x:c r="H128" s="140" t="s">
         <x:v>877</x:v>
@@ -59869,7 +59878,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G130" s="61" t="s">
-        <x:v>2343</x:v>
+        <x:v>2344</x:v>
       </x:c>
       <x:c r="H130" s="140">
         <x:v>100000</x:v>
@@ -59889,7 +59898,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="G131" s="61" t="s">
-        <x:v>2344</x:v>
+        <x:v>2345</x:v>
       </x:c>
       <x:c r="H131" s="140">
         <x:v>1</x:v>
@@ -59909,7 +59918,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G132" s="61" t="s">
-        <x:v>2345</x:v>
+        <x:v>2346</x:v>
       </x:c>
       <x:c r="H132" s="140"/>
       <x:c r="I132" s="140"/>
@@ -59928,7 +59937,7 @@
         <x:v>900</x:v>
       </x:c>
       <x:c r="D133" s="140" t="s">
-        <x:v>2346</x:v>
+        <x:v>2347</x:v>
       </x:c>
       <x:c r="E133" s="140" t="s">
         <x:v>886</x:v>
@@ -59937,7 +59946,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G133" s="61" t="s">
-        <x:v>2347</x:v>
+        <x:v>2348</x:v>
       </x:c>
       <x:c r="H133" s="140"/>
       <x:c r="I133" s="140" t="s">
@@ -59957,7 +59966,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G134" s="61" t="s">
-        <x:v>2348</x:v>
+        <x:v>2349</x:v>
       </x:c>
       <x:c r="H134" s="140"/>
       <x:c r="I134" s="140"/>
@@ -59975,7 +59984,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G135" s="61" t="s">
-        <x:v>2349</x:v>
+        <x:v>2350</x:v>
       </x:c>
       <x:c r="H135" s="140" t="s">
         <x:v>891</x:v>
@@ -60053,7 +60062,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G139" s="61" t="s">
-        <x:v>2350</x:v>
+        <x:v>2351</x:v>
       </x:c>
       <x:c r="H139" s="140">
         <x:f>1</x:f>
@@ -60073,7 +60082,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G140" s="61" t="s">
-        <x:v>2351</x:v>
+        <x:v>2352</x:v>
       </x:c>
       <x:c r="H140" s="140"/>
       <x:c r="I140" s="140"/>
@@ -60092,7 +60101,7 @@
         <x:v>911</x:v>
       </x:c>
       <x:c r="D141" s="140" t="s">
-        <x:v>2352</x:v>
+        <x:v>2353</x:v>
       </x:c>
       <x:c r="E141" s="140" t="s">
         <x:v>886</x:v>
@@ -60101,7 +60110,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G141" s="61" t="s">
-        <x:v>2353</x:v>
+        <x:v>2354</x:v>
       </x:c>
       <x:c r="H141" s="140"/>
       <x:c r="I141" s="140" t="s">
@@ -60121,7 +60130,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G142" s="61" t="s">
-        <x:v>2354</x:v>
+        <x:v>2355</x:v>
       </x:c>
       <x:c r="H142" s="140"/>
       <x:c r="I142" s="140"/>
@@ -60139,7 +60148,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G143" s="61" t="s">
-        <x:v>2355</x:v>
+        <x:v>2356</x:v>
       </x:c>
       <x:c r="H143" s="140" t="s">
         <x:v>891</x:v>
@@ -60237,7 +60246,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G148" s="61" t="s">
-        <x:v>2356</x:v>
+        <x:v>2357</x:v>
       </x:c>
       <x:c r="H148" s="140"/>
       <x:c r="I148" s="140"/>
@@ -60256,22 +60265,22 @@
         <x:v>921</x:v>
       </x:c>
       <x:c r="D149" s="116" t="s">
-        <x:v>2357</x:v>
+        <x:v>2358</x:v>
       </x:c>
       <x:c r="E149" s="116" t="s">
-        <x:v>2358</x:v>
+        <x:v>2359</x:v>
       </x:c>
       <x:c r="F149" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G149" s="327" t="s">
-        <x:v>2359</x:v>
+        <x:v>2360</x:v>
       </x:c>
       <x:c r="H149" s="116" t="s">
-        <x:v>2360</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="I149" s="289" t="s">
-        <x:v>2361</x:v>
+        <x:v>2362</x:v>
       </x:c>
       <x:c r="J149" s="61"/>
       <x:c r="K149" s="140"/>
@@ -60287,11 +60296,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G150" s="327" t="s">
-        <x:v>2362</x:v>
+        <x:v>2363</x:v>
       </x:c>
       <x:c r="H150" s="116"/>
       <x:c r="I150" s="289" t="s">
-        <x:v>2363</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="J150" s="61"/>
       <x:c r="K150" s="140"/>
@@ -60307,13 +60316,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G151" s="327" t="s">
-        <x:v>2364</x:v>
+        <x:v>2365</x:v>
       </x:c>
       <x:c r="H151" s="116" t="s">
-        <x:v>2365</x:v>
+        <x:v>2366</x:v>
       </x:c>
       <x:c r="I151" s="289" t="s">
-        <x:v>2366</x:v>
+        <x:v>2367</x:v>
       </x:c>
       <x:c r="J151" s="61"/>
       <x:c r="K151" s="140"/>
@@ -60329,11 +60338,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G152" s="327" t="s">
-        <x:v>2367</x:v>
+        <x:v>2368</x:v>
       </x:c>
       <x:c r="H152" s="116"/>
       <x:c r="I152" s="289" t="s">
-        <x:v>2368</x:v>
+        <x:v>2369</x:v>
       </x:c>
       <x:c r="J152" s="61"/>
       <x:c r="K152" s="140"/>
@@ -60349,11 +60358,11 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G153" s="327" t="s">
-        <x:v>2369</x:v>
+        <x:v>2370</x:v>
       </x:c>
       <x:c r="H153" s="116"/>
       <x:c r="I153" s="289" t="s">
-        <x:v>2370</x:v>
+        <x:v>2371</x:v>
       </x:c>
       <x:c r="J153" s="61"/>
       <x:c r="K153" s="140"/>
@@ -60690,17 +60699,17 @@
     <x:mergeCell ref="L149:L153"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H49" r:id="rId161"/>
-    <x:hyperlink ref="H50" r:id="rId162"/>
-    <x:hyperlink ref="H55" r:id="rId163"/>
-    <x:hyperlink ref="H56" r:id="rId164"/>
-    <x:hyperlink ref="H59" r:id="rId165"/>
-    <x:hyperlink ref="H64" r:id="rId166"/>
-    <x:hyperlink ref="H65" r:id="rId167"/>
-    <x:hyperlink ref="H67" r:id="rId168"/>
-    <x:hyperlink ref="H68" r:id="rId169"/>
-    <x:hyperlink ref="H52" r:id="rId170"/>
-    <x:hyperlink ref="H61" r:id="rId171"/>
+    <x:hyperlink ref="H49" r:id="rId206"/>
+    <x:hyperlink ref="H50" r:id="rId207"/>
+    <x:hyperlink ref="H55" r:id="rId208"/>
+    <x:hyperlink ref="H56" r:id="rId209"/>
+    <x:hyperlink ref="H59" r:id="rId210"/>
+    <x:hyperlink ref="H64" r:id="rId211"/>
+    <x:hyperlink ref="H65" r:id="rId212"/>
+    <x:hyperlink ref="H67" r:id="rId213"/>
+    <x:hyperlink ref="H68" r:id="rId214"/>
+    <x:hyperlink ref="H52" r:id="rId215"/>
+    <x:hyperlink ref="H61" r:id="rId216"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -60794,7 +60803,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H2" s="340" t="s">
-        <x:v>2371</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="I2" s="51" t="s">
         <x:v>1102</x:v>
@@ -61033,7 +61042,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G14" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H14" s="292"/>
       <x:c r="I14" s="51"/>
@@ -61303,7 +61312,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G27" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H27" s="292"/>
       <x:c r="I27" s="51"/>
@@ -61334,7 +61343,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H28" s="340" t="s">
-        <x:v>2373</x:v>
+        <x:v>2374</x:v>
       </x:c>
       <x:c r="I28" s="51" t="s">
         <x:v>1127</x:v>
@@ -61573,7 +61582,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G40" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H40" s="292"/>
       <x:c r="I40" s="51"/>
@@ -61604,7 +61613,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H41" s="340" t="s">
-        <x:v>2374</x:v>
+        <x:v>2375</x:v>
       </x:c>
       <x:c r="I41" s="51" t="s">
         <x:v>1130</x:v>
@@ -61843,7 +61852,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G53" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H53" s="292"/>
       <x:c r="I53" s="51"/>
@@ -61874,7 +61883,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H54" s="340" t="s">
-        <x:v>2375</x:v>
+        <x:v>2376</x:v>
       </x:c>
       <x:c r="I54" s="51" t="s">
         <x:v>1134</x:v>
@@ -62113,7 +62122,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G66" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H66" s="292"/>
       <x:c r="I66" s="51"/>
@@ -62144,7 +62153,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H67" s="340" t="s">
-        <x:v>2376</x:v>
+        <x:v>2377</x:v>
       </x:c>
       <x:c r="I67" s="51" t="s">
         <x:v>1138</x:v>
@@ -62383,7 +62392,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G79" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H79" s="292"/>
       <x:c r="I79" s="51"/>
@@ -62414,7 +62423,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H80" s="340" t="s">
-        <x:v>2377</x:v>
+        <x:v>2378</x:v>
       </x:c>
       <x:c r="I80" s="51" t="s">
         <x:v>1141</x:v>
@@ -62653,7 +62662,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G92" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H92" s="292"/>
       <x:c r="I92" s="51"/>
@@ -62684,7 +62693,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H93" s="340" t="s">
-        <x:v>2378</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="I93" s="51" t="s">
         <x:v>1145</x:v>
@@ -62923,7 +62932,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G105" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H105" s="292"/>
       <x:c r="I105" s="51"/>
@@ -62954,7 +62963,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H106" s="340" t="s">
-        <x:v>2378</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="I106" s="51" t="s">
         <x:v>1149</x:v>
@@ -63193,7 +63202,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G118" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H118" s="292"/>
       <x:c r="I118" s="51"/>
@@ -63224,7 +63233,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H119" s="340" t="s">
-        <x:v>2379</x:v>
+        <x:v>2380</x:v>
       </x:c>
       <x:c r="I119" s="51" t="s">
         <x:v>1149</x:v>
@@ -63463,7 +63472,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G131" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H131" s="292"/>
       <x:c r="I131" s="51"/>
@@ -63494,7 +63503,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H132" s="340" t="s">
-        <x:v>2380</x:v>
+        <x:v>2381</x:v>
       </x:c>
       <x:c r="I132" s="51" t="s">
         <x:v>1160</x:v>
@@ -63733,7 +63742,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G144" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H144" s="292"/>
       <x:c r="I144" s="51"/>
@@ -63764,7 +63773,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H145" s="340" t="s">
-        <x:v>2381</x:v>
+        <x:v>2382</x:v>
       </x:c>
       <x:c r="I145" s="51" t="s">
         <x:v>1160</x:v>
@@ -64003,7 +64012,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G157" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H157" s="292"/>
       <x:c r="I157" s="51"/>
@@ -64034,7 +64043,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H158" s="340" t="s">
-        <x:v>2382</x:v>
+        <x:v>2383</x:v>
       </x:c>
       <x:c r="I158" s="51" t="s">
         <x:v>1160</x:v>
@@ -64273,7 +64282,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G170" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H170" s="292"/>
       <x:c r="I170" s="51"/>
@@ -64304,7 +64313,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H171" s="340" t="s">
-        <x:v>2383</x:v>
+        <x:v>2384</x:v>
       </x:c>
       <x:c r="I171" s="51" t="s">
         <x:v>1160</x:v>
@@ -64543,7 +64552,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G183" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H183" s="292"/>
       <x:c r="I183" s="51"/>
@@ -64813,7 +64822,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G196" s="292" t="s">
-        <x:v>2372</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="H196" s="340"/>
       <x:c r="I196" s="51"/>
@@ -64844,7 +64853,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H197" s="340" t="s">
-        <x:v>2384</x:v>
+        <x:v>2385</x:v>
       </x:c>
       <x:c r="I197" s="134" t="s">
         <x:v>1178</x:v>
@@ -65114,7 +65123,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H210" s="340" t="s">
-        <x:v>2385</x:v>
+        <x:v>2386</x:v>
       </x:c>
       <x:c r="I210" s="134" t="s">
         <x:v>1187</x:v>
@@ -65372,7 +65381,7 @@
         <x:v>1189</x:v>
       </x:c>
       <x:c r="D223" s="134" t="s">
-        <x:v>2386</x:v>
+        <x:v>2387</x:v>
       </x:c>
       <x:c r="E223" s="35" t="s">
         <x:v>1176</x:v>
@@ -65384,7 +65393,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H223" s="340" t="s">
-        <x:v>2387</x:v>
+        <x:v>2388</x:v>
       </x:c>
       <x:c r="I223" s="10" t="s">
         <x:v>1192</x:v>
@@ -65654,7 +65663,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H236" s="340" t="s">
-        <x:v>2388</x:v>
+        <x:v>2389</x:v>
       </x:c>
       <x:c r="I236" s="10" t="s">
         <x:v>1197</x:v>
@@ -65924,7 +65933,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H249" s="340" t="s">
-        <x:v>2389</x:v>
+        <x:v>2390</x:v>
       </x:c>
       <x:c r="I249" s="10" t="s">
         <x:v>1203</x:v>
@@ -66106,7 +66115,7 @@
         <x:v>1115</x:v>
       </x:c>
       <x:c r="H258" s="292" t="s">
-        <x:v>2390</x:v>
+        <x:v>2391</x:v>
       </x:c>
       <x:c r="I258" s="9"/>
       <x:c r="J258" s="9"/>
@@ -66452,7 +66461,7 @@
         <x:v>1212</x:v>
       </x:c>
       <x:c r="D275" s="35" t="s">
-        <x:v>2391</x:v>
+        <x:v>2392</x:v>
       </x:c>
       <x:c r="E275" s="35" t="s">
         <x:v>1214</x:v>
@@ -66461,10 +66470,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G275" s="297" t="s">
-        <x:v>2392</x:v>
+        <x:v>2393</x:v>
       </x:c>
       <x:c r="I275" s="10" t="s">
-        <x:v>2393</x:v>
+        <x:v>2394</x:v>
       </x:c>
       <x:c r="J275" s="10"/>
       <x:c r="K275" s="35"/>
@@ -66480,7 +66489,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G276" s="297" t="s">
-        <x:v>2394</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="I276" s="9"/>
       <x:c r="J276" s="9"/>
@@ -66497,10 +66506,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G277" s="297" t="s">
-        <x:v>2395</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="H277" s="297" t="s">
-        <x:v>2396</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I277" s="9"/>
       <x:c r="J277" s="9"/>
@@ -66539,13 +66548,13 @@
         <x:v>1220</x:v>
       </x:c>
       <x:c r="E279" s="35" t="s">
-        <x:v>2397</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="F279" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G279" s="297" t="s">
-        <x:v>2392</x:v>
+        <x:v>2393</x:v>
       </x:c>
       <x:c r="I279" s="10" t="s">
         <x:v>1223</x:v>
@@ -66564,7 +66573,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G280" s="297" t="s">
-        <x:v>2398</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H280" s="297" t="s">
         <x:v>1117</x:v>
@@ -66606,17 +66615,17 @@
         <x:v>1226</x:v>
       </x:c>
       <x:c r="E282" s="35" t="s">
-        <x:v>2399</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="F282" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G282" s="297" t="s">
-        <x:v>2392</x:v>
+        <x:v>2393</x:v>
       </x:c>
       <x:c r="H282" s="297"/>
       <x:c r="I282" s="10" t="s">
-        <x:v>2400</x:v>
+        <x:v>2401</x:v>
       </x:c>
       <x:c r="J282" s="10"/>
       <x:c r="K282" s="35"/>
@@ -66632,7 +66641,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G283" s="297" t="s">
-        <x:v>2394</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H283" s="297"/>
       <x:c r="I283" s="9"/>
@@ -66650,10 +66659,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G284" s="297" t="s">
-        <x:v>2401</x:v>
+        <x:v>2402</x:v>
       </x:c>
       <x:c r="H284" s="323" t="s">
-        <x:v>2402</x:v>
+        <x:v>2403</x:v>
       </x:c>
       <x:c r="I284" s="9"/>
       <x:c r="J284" s="9"/>
@@ -66692,17 +66701,17 @@
         <x:v>1233</x:v>
       </x:c>
       <x:c r="E286" s="35" t="s">
-        <x:v>2399</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="F286" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G286" s="297" t="s">
-        <x:v>2392</x:v>
+        <x:v>2393</x:v>
       </x:c>
       <x:c r="H286" s="297"/>
       <x:c r="I286" s="10" t="s">
-        <x:v>2400</x:v>
+        <x:v>2401</x:v>
       </x:c>
       <x:c r="J286" s="10"/>
       <x:c r="K286" s="35"/>
@@ -66718,7 +66727,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G287" s="297" t="s">
-        <x:v>2394</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="H287" s="297"/>
       <x:c r="I287" s="9"/>
@@ -66736,10 +66745,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G288" s="297" t="s">
-        <x:v>2403</x:v>
+        <x:v>2404</x:v>
       </x:c>
       <x:c r="H288" s="297" t="s">
-        <x:v>2404</x:v>
+        <x:v>2405</x:v>
       </x:c>
       <x:c r="I288" s="9"/>
       <x:c r="J288" s="9"/>
@@ -66787,7 +66796,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H290" s="340" t="s">
-        <x:v>2405</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="I290" s="51" t="s">
         <x:v>1102</x:v>
@@ -66866,7 +66875,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G294" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H294" s="312" t="s">
         <x:v>1117</x:v>
@@ -66886,7 +66895,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G295" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H295" s="312">
         <x:v>45758</x:v>
@@ -67006,7 +67015,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G301" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="H301" s="297"/>
       <x:c r="I301" s="51"/>
@@ -67116,7 +67125,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G306" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H306" s="312" t="s">
         <x:v>1117</x:v>
@@ -67136,7 +67145,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G307" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H307" s="312">
         <x:v>45758</x:v>
@@ -67256,7 +67265,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G313" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I313" s="51"/>
       <x:c r="J313" s="48"/>
@@ -67286,7 +67295,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H314" s="340" t="s">
-        <x:v>2409</x:v>
+        <x:v>2410</x:v>
       </x:c>
       <x:c r="I314" s="51" t="s">
         <x:v>1127</x:v>
@@ -67363,7 +67372,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G318" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H318" s="312" t="s">
         <x:v>1117</x:v>
@@ -67383,7 +67392,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G319" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H319" s="312">
         <x:v>45758</x:v>
@@ -67503,7 +67512,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G325" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I325" s="51"/>
       <x:c r="J325" s="48"/>
@@ -67533,7 +67542,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H326" s="340" t="s">
-        <x:v>2410</x:v>
+        <x:v>2411</x:v>
       </x:c>
       <x:c r="I326" s="51" t="s">
         <x:v>1130</x:v>
@@ -67610,7 +67619,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G330" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H330" s="312" t="s">
         <x:v>1117</x:v>
@@ -67630,7 +67639,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G331" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H331" s="312">
         <x:v>45758</x:v>
@@ -67750,7 +67759,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G337" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I337" s="51"/>
       <x:c r="J337" s="48"/>
@@ -67780,7 +67789,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H338" s="340" t="s">
-        <x:v>2411</x:v>
+        <x:v>2412</x:v>
       </x:c>
       <x:c r="I338" s="51" t="s">
         <x:v>1134</x:v>
@@ -67859,7 +67868,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G342" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H342" s="312"/>
       <x:c r="I342" s="51"/>
@@ -67877,7 +67886,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G343" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H343" s="312">
         <x:v>45758</x:v>
@@ -67997,7 +68006,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G349" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I349" s="51"/>
       <x:c r="J349" s="48"/>
@@ -68027,7 +68036,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H350" s="340" t="s">
-        <x:v>2411</x:v>
+        <x:v>2412</x:v>
       </x:c>
       <x:c r="I350" s="51" t="s">
         <x:v>1138</x:v>
@@ -68106,7 +68115,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G354" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H354" s="312" t="s">
         <x:v>1117</x:v>
@@ -68126,7 +68135,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G355" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H355" s="312"/>
       <x:c r="I355" s="51"/>
@@ -68244,7 +68253,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G361" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I361" s="51"/>
       <x:c r="J361" s="48"/>
@@ -68262,7 +68271,7 @@
         <x:v>1254</x:v>
       </x:c>
       <x:c r="D362" s="51" t="s">
-        <x:v>2412</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="E362" s="51" t="s">
         <x:v>1099</x:v>
@@ -68274,10 +68283,10 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H362" s="340" t="s">
-        <x:v>2413</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="I362" s="51" t="s">
-        <x:v>2414</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="J362" s="50"/>
       <x:c r="K362" s="51"/>
@@ -68351,7 +68360,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G366" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H366" s="312" t="s">
         <x:v>1117</x:v>
@@ -68371,7 +68380,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G367" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H367" s="312">
         <x:v>49410</x:v>
@@ -68489,7 +68498,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G373" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="H373" s="292"/>
       <x:c r="I373" s="51"/>
@@ -68520,7 +68529,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H374" s="340" t="s">
-        <x:v>2415</x:v>
+        <x:v>2416</x:v>
       </x:c>
       <x:c r="I374" s="51" t="s">
         <x:v>1145</x:v>
@@ -68599,7 +68608,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G378" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H378" s="312" t="s">
         <x:v>1117</x:v>
@@ -68619,7 +68628,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G379" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H379" s="312">
         <x:v>45758</x:v>
@@ -68737,7 +68746,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G385" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I385" s="51"/>
       <x:c r="J385" s="48"/>
@@ -68767,7 +68776,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H386" s="340" t="s">
-        <x:v>2416</x:v>
+        <x:v>2417</x:v>
       </x:c>
       <x:c r="I386" s="51" t="s">
         <x:v>1149</x:v>
@@ -68846,7 +68855,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G390" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H390" s="312" t="s">
         <x:v>1117</x:v>
@@ -68866,7 +68875,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G391" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H391" s="312">
         <x:v>45758</x:v>
@@ -68984,7 +68993,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G397" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I397" s="51"/>
       <x:c r="J397" s="48"/>
@@ -69014,7 +69023,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H398" s="340" t="s">
-        <x:v>2417</x:v>
+        <x:v>2418</x:v>
       </x:c>
       <x:c r="I398" s="51" t="s">
         <x:v>1149</x:v>
@@ -69091,7 +69100,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G402" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H402" s="312" t="s">
         <x:v>1117</x:v>
@@ -69111,7 +69120,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G403" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H403" s="312">
         <x:v>45758</x:v>
@@ -69231,7 +69240,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G409" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I409" s="51"/>
       <x:c r="J409" s="48"/>
@@ -69261,7 +69270,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H410" s="340" t="s">
-        <x:v>2418</x:v>
+        <x:v>2419</x:v>
       </x:c>
       <x:c r="I410" s="51" t="s">
         <x:v>1160</x:v>
@@ -69340,7 +69349,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G414" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H414" s="312" t="s">
         <x:v>1117</x:v>
@@ -69360,7 +69369,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G415" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H415" s="312">
         <x:v>45758</x:v>
@@ -69478,7 +69487,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G421" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I421" s="51"/>
       <x:c r="J421" s="48"/>
@@ -69496,7 +69505,7 @@
         <x:v>1260</x:v>
       </x:c>
       <x:c r="D422" s="51" t="s">
-        <x:v>2419</x:v>
+        <x:v>2420</x:v>
       </x:c>
       <x:c r="E422" s="51" t="s">
         <x:v>1099</x:v>
@@ -69508,10 +69517,10 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H422" s="340" t="s">
-        <x:v>2420</x:v>
+        <x:v>2421</x:v>
       </x:c>
       <x:c r="I422" s="51" t="s">
-        <x:v>2421</x:v>
+        <x:v>2422</x:v>
       </x:c>
       <x:c r="J422" s="50"/>
       <x:c r="K422" s="51"/>
@@ -69587,7 +69596,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G426" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H426" s="312" t="s">
         <x:v>1117</x:v>
@@ -69607,7 +69616,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G427" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H427" s="312">
         <x:v>45758</x:v>
@@ -69727,7 +69736,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G433" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I433" s="51"/>
       <x:c r="J433" s="48"/>
@@ -69757,7 +69766,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H434" s="340" t="s">
-        <x:v>2422</x:v>
+        <x:v>2423</x:v>
       </x:c>
       <x:c r="I434" s="51" t="s">
         <x:v>1160</x:v>
@@ -69836,7 +69845,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G438" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H438" s="312" t="s">
         <x:v>1117</x:v>
@@ -69856,7 +69865,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G439" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H439" s="312">
         <x:v>45758</x:v>
@@ -69974,7 +69983,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G445" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I445" s="51"/>
       <x:c r="J445" s="48"/>
@@ -70004,7 +70013,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H446" s="340" t="s">
-        <x:v>2423</x:v>
+        <x:v>2424</x:v>
       </x:c>
       <x:c r="I446" s="51" t="s">
         <x:v>1160</x:v>
@@ -70083,7 +70092,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G450" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H450" s="312" t="s">
         <x:v>1117</x:v>
@@ -70103,7 +70112,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G451" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H451" s="312">
         <x:v>45758</x:v>
@@ -70221,7 +70230,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G457" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I457" s="51"/>
       <x:c r="J457" s="48"/>
@@ -70330,7 +70339,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G462" s="292" t="s">
-        <x:v>2406</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="H462" s="340" t="s">
         <x:v>437</x:v>
@@ -70350,7 +70359,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G463" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H463" s="340" t="s">
         <x:v>437</x:v>
@@ -70470,7 +70479,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G469" s="288" t="s">
-        <x:v>2408</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="H469" s="340" t="s">
         <x:v>437</x:v>
@@ -70804,7 +70813,7 @@
     <x:mergeCell ref="K458:K469"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H284" r:id="rId172"/>
+    <x:hyperlink ref="H284" r:id="rId217"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -70828,13 +70837,13 @@
   <x:sheetData>
     <x:row r="2" spans="1:7">
       <x:c r="A2" s="196" t="s">
-        <x:v>2424</x:v>
+        <x:v>2425</x:v>
       </x:c>
       <x:c r="D2" s="196" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="G2" s="196" t="s">
-        <x:v>2425</x:v>
+        <x:v>2426</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
@@ -70842,7 +70851,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>2426</x:v>
+        <x:v>2427</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
         <x:v>244</x:v>
@@ -70853,7 +70862,7 @@
         <x:v>245</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>2427</x:v>
+        <x:v>2428</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
         <x:v>234</x:v>
@@ -70861,10 +70870,10 @@
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="A5" s="0" t="s">
-        <x:v>2428</x:v>
+        <x:v>2429</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>2429</x:v>
+        <x:v>2430</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
         <x:v>239</x:v>

</xml_diff>

<commit_message>
Test: Successfully verified that it blocks spaces (TC_REG_08) and future birth dates (TC_REG_09).
</commit_message>
<xml_diff>
--- a/sqa-testing-report/Data/DataTest.xlsx
+++ b/sqa-testing-report/Data/DataTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\sqa-testing-report\sqa-testing-report\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B3991C-E6A1-4458-8027-922AF348F1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E77FC6-C949-4300-9758-727AE95EC3A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
     <x:workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="664" firstSheet="0" activeTab="3" xr2:uid="{DC4DB269-603C-4B5B-A498-B166C8A18B92}"/>
   </x:bookViews>
@@ -7734,13 +7734,31 @@
     <x:t>Hệ thống chặn đăng ký và báo lỗi đã tồn tại thành công.</x:t>
   </x:si>
   <x:si>
+    <x:t>Hệ thống chặn và hiển thị Alert: Lỗi BadRequest: Số điện thoại không hợp lệ.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hệ thống chặn và hiển thị Alert: Lỗi BadRequest: Bạn chưa đủ 12 tuổi để đăng ký.</x:t>
+  </x:si>
+  <x:si>
     <x:t>Kiểm tra đăng ký với mật khẩu chứa ký tự đặc biệt gây lỗi (SQL Injection).</x:t>
   </x:si>
   <x:si>
+    <x:t>Đánh giá Fail do bước trước đó đã thất bại.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Data/Screenshots/TC_REG_10.png</x:t>
+  </x:si>
+  <x:si>
     <x:t>' OR 1=1 --</x:t>
   </x:si>
   <x:si>
+    <x:t>Data/Screenshots/TC_REG_11.png</x:t>
+  </x:si>
+  <x:si>
     <x:t>chuỗi &gt; 255 kí tự</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Data/Screenshots/TC_REG_12.png</x:t>
   </x:si>
   <x:si>
     <x:t>0376808424B</x:t>
@@ -48213,41 +48231,41 @@
   </x:mergeCells>
   <x:phoneticPr fontId="16" type="noConversion"/>
   <x:hyperlinks>
-    <x:hyperlink ref="H382" r:id="rId82"/>
-    <x:hyperlink ref="H388" r:id="rId83"/>
-    <x:hyperlink ref="H396" r:id="rId84"/>
-    <x:hyperlink ref="H397" r:id="rId85"/>
-    <x:hyperlink ref="H415" r:id="rId86"/>
-    <x:hyperlink ref="H418" r:id="rId87"/>
-    <x:hyperlink ref="H420" r:id="rId88"/>
-    <x:hyperlink ref="H421" r:id="rId89"/>
-    <x:hyperlink ref="H423" r:id="rId90"/>
-    <x:hyperlink ref="H424" r:id="rId91"/>
-    <x:hyperlink ref="H53" r:id="rId92"/>
-    <x:hyperlink ref="H61" r:id="rId93"/>
-    <x:hyperlink ref="H65" r:id="rId94"/>
-    <x:hyperlink ref="H69" r:id="rId95"/>
-    <x:hyperlink ref="H73" r:id="rId96"/>
-    <x:hyperlink ref="H77" r:id="rId97"/>
-    <x:hyperlink ref="H81" r:id="rId98"/>
-    <x:hyperlink ref="H112" r:id="rId99"/>
-    <x:hyperlink ref="H115" r:id="rId100"/>
-    <x:hyperlink ref="H118" r:id="rId101"/>
-    <x:hyperlink ref="H399" r:id="rId102"/>
-    <x:hyperlink ref="H402" r:id="rId103"/>
-    <x:hyperlink ref="H405" r:id="rId104"/>
-    <x:hyperlink ref="H408" r:id="rId173"/>
-    <x:hyperlink ref="H411" r:id="rId174"/>
-    <x:hyperlink ref="H400" r:id="rId175"/>
-    <x:hyperlink ref="H403" r:id="rId176"/>
-    <x:hyperlink ref="H406" r:id="rId177"/>
-    <x:hyperlink ref="H409" r:id="rId178"/>
-    <x:hyperlink ref="H412" r:id="rId179"/>
-    <x:hyperlink ref="H1075" r:id="rId180"/>
-    <x:hyperlink ref="H1081" r:id="rId181"/>
-    <x:hyperlink ref="H1087" r:id="rId182"/>
-    <x:hyperlink ref="H1093" r:id="rId183"/>
-    <x:hyperlink ref="H1099" r:id="rId184"/>
+    <x:hyperlink ref="H382" r:id="rId105"/>
+    <x:hyperlink ref="H388" r:id="rId106"/>
+    <x:hyperlink ref="H396" r:id="rId107"/>
+    <x:hyperlink ref="H397" r:id="rId108"/>
+    <x:hyperlink ref="H415" r:id="rId109"/>
+    <x:hyperlink ref="H418" r:id="rId110"/>
+    <x:hyperlink ref="H420" r:id="rId111"/>
+    <x:hyperlink ref="H421" r:id="rId112"/>
+    <x:hyperlink ref="H423" r:id="rId113"/>
+    <x:hyperlink ref="H424" r:id="rId114"/>
+    <x:hyperlink ref="H53" r:id="rId115"/>
+    <x:hyperlink ref="H61" r:id="rId116"/>
+    <x:hyperlink ref="H65" r:id="rId117"/>
+    <x:hyperlink ref="H69" r:id="rId118"/>
+    <x:hyperlink ref="H73" r:id="rId119"/>
+    <x:hyperlink ref="H77" r:id="rId120"/>
+    <x:hyperlink ref="H81" r:id="rId121"/>
+    <x:hyperlink ref="H112" r:id="rId122"/>
+    <x:hyperlink ref="H115" r:id="rId123"/>
+    <x:hyperlink ref="H118" r:id="rId124"/>
+    <x:hyperlink ref="H399" r:id="rId125"/>
+    <x:hyperlink ref="H402" r:id="rId126"/>
+    <x:hyperlink ref="H405" r:id="rId127"/>
+    <x:hyperlink ref="H408" r:id="rId128"/>
+    <x:hyperlink ref="H411" r:id="rId129"/>
+    <x:hyperlink ref="H400" r:id="rId130"/>
+    <x:hyperlink ref="H403" r:id="rId131"/>
+    <x:hyperlink ref="H406" r:id="rId132"/>
+    <x:hyperlink ref="H409" r:id="rId133"/>
+    <x:hyperlink ref="H412" r:id="rId134"/>
+    <x:hyperlink ref="H1075" r:id="rId135"/>
+    <x:hyperlink ref="H1081" r:id="rId136"/>
+    <x:hyperlink ref="H1087" r:id="rId137"/>
+    <x:hyperlink ref="H1093" r:id="rId138"/>
+    <x:hyperlink ref="H1099" r:id="rId139"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -49688,9 +49706,13 @@
       <x:c r="I65" s="138" t="s">
         <x:v>447</x:v>
       </x:c>
-      <x:c r="J65" s="137"/>
-      <x:c r="K65" s="137"/>
-      <x:c r="L65" s="137"/>
+      <x:c r="J65" s="137" t="s">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="K65" s="137" t="s">
+        <x:v>2008</x:v>
+      </x:c>
+      <x:c r="L65" s="137" t="s"/>
     </x:row>
     <x:row r="66" spans="1:12">
       <x:c r="A66" s="140"/>
@@ -49876,9 +49898,13 @@
       <x:c r="I74" s="138" t="s">
         <x:v>447</x:v>
       </x:c>
-      <x:c r="J74" s="137"/>
-      <x:c r="K74" s="137"/>
-      <x:c r="L74" s="137"/>
+      <x:c r="J74" s="137" t="s">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="K74" s="137" t="s">
+        <x:v>2008</x:v>
+      </x:c>
+      <x:c r="L74" s="137" t="s"/>
     </x:row>
     <x:row r="75" spans="1:12">
       <x:c r="A75" s="140"/>
@@ -49973,7 +49999,7 @@
         <x:v>443</x:v>
       </x:c>
       <x:c r="H79" s="235">
-        <x:v>46507</x:v>
+        <x:v>46172</x:v>
       </x:c>
       <x:c r="I79" s="138"/>
       <x:c r="J79" s="136"/>
@@ -50049,7 +50075,7 @@
         <x:v>468</x:v>
       </x:c>
       <x:c r="D83" s="140" t="s">
-        <x:v>2019</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="E83" s="140" t="s">
         <x:v>434</x:v>
@@ -50064,9 +50090,15 @@
       <x:c r="I83" s="138" t="s">
         <x:v>447</x:v>
       </x:c>
-      <x:c r="J83" s="137"/>
-      <x:c r="K83" s="137"/>
-      <x:c r="L83" s="137"/>
+      <x:c r="J83" s="137" t="s">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="K83" s="137" t="s">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="L83" s="137" t="s">
+        <x:v>2023</x:v>
+      </x:c>
     </x:row>
     <x:row r="84" spans="1:12">
       <x:c r="A84" s="140"/>
@@ -50181,7 +50213,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H89" s="25" t="s">
-        <x:v>2020</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="I89" s="138"/>
       <x:c r="J89" s="136"/>
@@ -50201,7 +50233,7 @@
         <x:v>445</x:v>
       </x:c>
       <x:c r="H90" s="25" t="s">
-        <x:v>2020</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="I90" s="138"/>
       <x:c r="J90" s="136"/>
@@ -50252,9 +50284,15 @@
       <x:c r="I92" s="138" t="s">
         <x:v>447</x:v>
       </x:c>
-      <x:c r="J92" s="137"/>
-      <x:c r="K92" s="137"/>
-      <x:c r="L92" s="137"/>
+      <x:c r="J92" s="137" t="s">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="K92" s="137" t="s">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="L92" s="137" t="s">
+        <x:v>2025</x:v>
+      </x:c>
     </x:row>
     <x:row r="93" spans="1:12">
       <x:c r="A93" s="140"/>
@@ -50269,7 +50307,7 @@
         <x:v>419</x:v>
       </x:c>
       <x:c r="H93" s="140" t="s">
-        <x:v>2021</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="I93" s="138"/>
       <x:c r="J93" s="136"/>
@@ -50440,9 +50478,15 @@
       <x:c r="I101" s="138" t="s">
         <x:v>447</x:v>
       </x:c>
-      <x:c r="J101" s="134"/>
-      <x:c r="K101" s="134"/>
-      <x:c r="L101" s="134"/>
+      <x:c r="J101" s="134" t="s">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="K101" s="134" t="s">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="L101" s="134" t="s">
+        <x:v>2027</x:v>
+      </x:c>
     </x:row>
     <x:row r="102" spans="1:12">
       <x:c r="A102" s="140"/>
@@ -50497,7 +50541,7 @@
         <x:v>439</x:v>
       </x:c>
       <x:c r="H104" s="139" t="s">
-        <x:v>2022</x:v>
+        <x:v>2028</x:v>
       </x:c>
       <x:c r="I104" s="138"/>
       <x:c r="J104" s="134"/>
@@ -51062,7 +51106,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I129" s="138" t="s">
-        <x:v>2023</x:v>
+        <x:v>2029</x:v>
       </x:c>
       <x:c r="J129" s="134"/>
       <x:c r="K129" s="134"/>
@@ -51132,7 +51176,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I132" s="123" t="s">
-        <x:v>2024</x:v>
+        <x:v>2030</x:v>
       </x:c>
       <x:c r="J132" s="134"/>
       <x:c r="K132" s="134"/>
@@ -51202,7 +51246,7 @@
         <x:v>504</x:v>
       </x:c>
       <x:c r="I135" s="138" t="s">
-        <x:v>2025</x:v>
+        <x:v>2031</x:v>
       </x:c>
       <x:c r="J135" s="134"/>
       <x:c r="K135" s="134"/>
@@ -51269,10 +51313,10 @@
         <x:v>480</x:v>
       </x:c>
       <x:c r="H138" s="316" t="s">
-        <x:v>2026</x:v>
+        <x:v>2032</x:v>
       </x:c>
       <x:c r="I138" s="120" t="s">
-        <x:v>2027</x:v>
+        <x:v>2033</x:v>
       </x:c>
       <x:c r="J138" s="134"/>
       <x:c r="K138" s="134"/>
@@ -51342,7 +51386,7 @@
         <x:v>2009</x:v>
       </x:c>
       <x:c r="I141" s="138" t="s">
-        <x:v>2028</x:v>
+        <x:v>2034</x:v>
       </x:c>
       <x:c r="J141" s="118"/>
       <x:c r="K141" s="134"/>
@@ -51406,11 +51450,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G144" s="138" t="s">
-        <x:v>2029</x:v>
+        <x:v>2035</x:v>
       </x:c>
       <x:c r="H144" s="140"/>
       <x:c r="I144" s="138" t="s">
-        <x:v>2030</x:v>
+        <x:v>2036</x:v>
       </x:c>
       <x:c r="J144" s="134"/>
       <x:c r="K144" s="134"/>
@@ -51426,10 +51470,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G145" s="319" t="s">
-        <x:v>2031</x:v>
+        <x:v>2037</x:v>
       </x:c>
       <x:c r="H145" s="134" t="s">
-        <x:v>2032</x:v>
+        <x:v>2038</x:v>
       </x:c>
       <x:c r="I145" s="138"/>
       <x:c r="J145" s="134"/>
@@ -51446,10 +51490,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G146" s="138" t="s">
-        <x:v>2033</x:v>
+        <x:v>2039</x:v>
       </x:c>
       <x:c r="H146" s="317" t="s">
-        <x:v>2034</x:v>
+        <x:v>2040</x:v>
       </x:c>
       <x:c r="I146" s="138"/>
       <x:c r="J146" s="134"/>
@@ -51466,10 +51510,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G147" s="138" t="s">
-        <x:v>2035</x:v>
+        <x:v>2041</x:v>
       </x:c>
       <x:c r="H147" s="134" t="s">
-        <x:v>2034</x:v>
+        <x:v>2040</x:v>
       </x:c>
       <x:c r="I147" s="138"/>
       <x:c r="J147" s="134"/>
@@ -51486,7 +51530,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G148" s="138" t="s">
-        <x:v>2036</x:v>
+        <x:v>2042</x:v>
       </x:c>
       <x:c r="H148" s="134"/>
       <x:c r="I148" s="138"/>
@@ -51520,7 +51564,7 @@
         <x:v>590</x:v>
       </x:c>
       <x:c r="I149" s="138" t="s">
-        <x:v>2037</x:v>
+        <x:v>2043</x:v>
       </x:c>
       <x:c r="J149" s="298"/>
       <x:c r="K149" s="134"/>
@@ -51540,7 +51584,7 @@
       </x:c>
       <x:c r="H150" s="140"/>
       <x:c r="I150" s="138" t="s">
-        <x:v>2038</x:v>
+        <x:v>2044</x:v>
       </x:c>
       <x:c r="J150" s="298"/>
       <x:c r="K150" s="134"/>
@@ -51560,7 +51604,7 @@
       </x:c>
       <x:c r="H151" s="140"/>
       <x:c r="I151" s="138" t="s">
-        <x:v>2039</x:v>
+        <x:v>2045</x:v>
       </x:c>
       <x:c r="J151" s="298"/>
       <x:c r="K151" s="134"/>
@@ -51636,10 +51680,10 @@
       </x:c>
       <x:c r="H154" s="140"/>
       <x:c r="I154" s="138" t="s">
-        <x:v>2040</x:v>
+        <x:v>2046</x:v>
       </x:c>
       <x:c r="J154" s="134" t="s">
-        <x:v>2041</x:v>
+        <x:v>2047</x:v>
       </x:c>
       <x:c r="K154" s="134" t="s">
         <x:v>2008</x:v>
@@ -51656,16 +51700,16 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G155" s="138" t="s">
-        <x:v>2042</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="H155" s="140" t="s">
-        <x:v>2043</x:v>
+        <x:v>2049</x:v>
       </x:c>
       <x:c r="I155" s="138" t="s">
-        <x:v>2044</x:v>
+        <x:v>2050</x:v>
       </x:c>
       <x:c r="J155" s="134" t="s">
-        <x:v>2045</x:v>
+        <x:v>2051</x:v>
       </x:c>
       <x:c r="K155" s="134"/>
       <x:c r="L155" s="134"/>
@@ -51681,7 +51725,7 @@
         <x:v>626</x:v>
       </x:c>
       <x:c r="D156" s="140" t="s">
-        <x:v>2046</x:v>
+        <x:v>2052</x:v>
       </x:c>
       <x:c r="E156" s="140" t="s">
         <x:v>616</x:v>
@@ -51690,13 +51734,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G156" s="138" t="s">
-        <x:v>2047</x:v>
+        <x:v>2053</x:v>
       </x:c>
       <x:c r="H156" s="140" t="s">
-        <x:v>2048</x:v>
+        <x:v>2054</x:v>
       </x:c>
       <x:c r="I156" s="138" t="s">
-        <x:v>2049</x:v>
+        <x:v>2055</x:v>
       </x:c>
       <x:c r="J156" s="134"/>
       <x:c r="K156" s="134"/>
@@ -51722,16 +51766,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G157" s="138" t="s">
-        <x:v>2050</x:v>
+        <x:v>2056</x:v>
       </x:c>
       <x:c r="H157" s="140" t="s">
-        <x:v>2051</x:v>
+        <x:v>2057</x:v>
       </x:c>
       <x:c r="I157" s="138" t="s">
-        <x:v>2052</x:v>
+        <x:v>2058</x:v>
       </x:c>
       <x:c r="J157" s="134" t="s">
-        <x:v>2053</x:v>
+        <x:v>2059</x:v>
       </x:c>
       <x:c r="K157" s="134" t="s">
         <x:v>2008</x:v>
@@ -51748,14 +51792,14 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G158" s="138" t="s">
-        <x:v>2054</x:v>
+        <x:v>2060</x:v>
       </x:c>
       <x:c r="H158" s="140"/>
       <x:c r="I158" s="138" t="s">
-        <x:v>2055</x:v>
+        <x:v>2061</x:v>
       </x:c>
       <x:c r="J158" s="134" t="s">
-        <x:v>2056</x:v>
+        <x:v>2062</x:v>
       </x:c>
       <x:c r="K158" s="134"/>
       <x:c r="L158" s="134"/>
@@ -51770,14 +51814,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G159" s="138" t="s">
-        <x:v>2057</x:v>
+        <x:v>2063</x:v>
       </x:c>
       <x:c r="H159" s="140"/>
       <x:c r="I159" s="138" t="s">
-        <x:v>2058</x:v>
+        <x:v>2064</x:v>
       </x:c>
       <x:c r="J159" s="134" t="s">
-        <x:v>2059</x:v>
+        <x:v>2065</x:v>
       </x:c>
       <x:c r="K159" s="134"/>
       <x:c r="L159" s="134"/>
@@ -51802,13 +51846,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G160" s="138" t="s">
-        <x:v>2050</x:v>
+        <x:v>2056</x:v>
       </x:c>
       <x:c r="H160" s="140" t="s">
-        <x:v>2051</x:v>
+        <x:v>2057</x:v>
       </x:c>
       <x:c r="I160" s="138" t="s">
-        <x:v>2060</x:v>
+        <x:v>2066</x:v>
       </x:c>
       <x:c r="J160" s="134"/>
       <x:c r="K160" s="134"/>
@@ -51824,7 +51868,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G161" s="138" t="s">
-        <x:v>2061</x:v>
+        <x:v>2067</x:v>
       </x:c>
       <x:c r="H161" s="313">
         <x:v>46109</x:v>
@@ -51845,25 +51889,25 @@
         <x:v>644</x:v>
       </x:c>
       <x:c r="D162" s="116" t="s">
-        <x:v>2062</x:v>
+        <x:v>2068</x:v>
       </x:c>
       <x:c r="E162" s="116" t="s">
-        <x:v>2063</x:v>
+        <x:v>2069</x:v>
       </x:c>
       <x:c r="F162" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G162" s="320" t="s">
-        <x:v>2064</x:v>
+        <x:v>2070</x:v>
       </x:c>
       <x:c r="H162" s="116" t="s">
-        <x:v>2051</x:v>
+        <x:v>2057</x:v>
       </x:c>
       <x:c r="I162" s="320" t="s">
-        <x:v>2052</x:v>
+        <x:v>2058</x:v>
       </x:c>
       <x:c r="J162" s="134" t="s">
-        <x:v>2065</x:v>
+        <x:v>2071</x:v>
       </x:c>
       <x:c r="K162" s="134" t="s">
         <x:v>2008</x:v>
@@ -51880,14 +51924,14 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G163" s="320" t="s">
-        <x:v>2066</x:v>
+        <x:v>2072</x:v>
       </x:c>
       <x:c r="H163" s="116"/>
       <x:c r="I163" s="320" t="s">
-        <x:v>2067</x:v>
+        <x:v>2073</x:v>
       </x:c>
       <x:c r="J163" s="134" t="s">
-        <x:v>2068</x:v>
+        <x:v>2074</x:v>
       </x:c>
       <x:c r="K163" s="134"/>
       <x:c r="L163" s="134"/>
@@ -51902,14 +51946,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G164" s="320" t="s">
-        <x:v>2069</x:v>
+        <x:v>2075</x:v>
       </x:c>
       <x:c r="H164" s="116"/>
       <x:c r="I164" s="320" t="s">
-        <x:v>2070</x:v>
+        <x:v>2076</x:v>
       </x:c>
       <x:c r="J164" s="134" t="s">
-        <x:v>2071</x:v>
+        <x:v>2077</x:v>
       </x:c>
       <x:c r="K164" s="134"/>
       <x:c r="L164" s="134"/>
@@ -51934,13 +51978,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G165" s="320" t="s">
-        <x:v>2072</x:v>
+        <x:v>2078</x:v>
       </x:c>
       <x:c r="H165" s="318">
         <x:v>0.333333333333333</x:v>
       </x:c>
       <x:c r="I165" s="320" t="s">
-        <x:v>2073</x:v>
+        <x:v>2079</x:v>
       </x:c>
       <x:c r="J165" s="134"/>
       <x:c r="K165" s="134"/>
@@ -51956,13 +52000,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G166" s="320" t="s">
-        <x:v>2074</x:v>
+        <x:v>2080</x:v>
       </x:c>
       <x:c r="H166" s="116" t="s">
-        <x:v>2075</x:v>
+        <x:v>2081</x:v>
       </x:c>
       <x:c r="I166" s="320" t="s">
-        <x:v>2076</x:v>
+        <x:v>2082</x:v>
       </x:c>
       <x:c r="J166" s="134"/>
       <x:c r="K166" s="134"/>
@@ -51978,13 +52022,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G167" s="320" t="s">
-        <x:v>2077</x:v>
+        <x:v>2083</x:v>
       </x:c>
       <x:c r="H167" s="116" t="s">
-        <x:v>2078</x:v>
+        <x:v>2084</x:v>
       </x:c>
       <x:c r="I167" s="320" t="s">
-        <x:v>2079</x:v>
+        <x:v>2085</x:v>
       </x:c>
       <x:c r="J167" s="134"/>
       <x:c r="K167" s="134"/>
@@ -52000,11 +52044,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G168" s="320" t="s">
-        <x:v>2080</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="H168" s="116"/>
       <x:c r="I168" s="320" t="s">
-        <x:v>2081</x:v>
+        <x:v>2087</x:v>
       </x:c>
       <x:c r="J168" s="134"/>
       <x:c r="K168" s="134"/>
@@ -52021,22 +52065,22 @@
         <x:v>658</x:v>
       </x:c>
       <x:c r="D169" s="116" t="s">
-        <x:v>2082</x:v>
+        <x:v>2088</x:v>
       </x:c>
       <x:c r="E169" s="116" t="s">
-        <x:v>2083</x:v>
+        <x:v>2089</x:v>
       </x:c>
       <x:c r="F169" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G169" s="320" t="s">
-        <x:v>2084</x:v>
+        <x:v>2090</x:v>
       </x:c>
       <x:c r="H169" s="116" t="s">
-        <x:v>2085</x:v>
+        <x:v>2091</x:v>
       </x:c>
       <x:c r="I169" s="320" t="s">
-        <x:v>2086</x:v>
+        <x:v>2092</x:v>
       </x:c>
       <x:c r="J169" s="134"/>
       <x:c r="K169" s="134"/>
@@ -52052,11 +52096,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G170" s="320" t="s">
-        <x:v>2087</x:v>
+        <x:v>2093</x:v>
       </x:c>
       <x:c r="H170" s="116"/>
       <x:c r="I170" s="320" t="s">
-        <x:v>2088</x:v>
+        <x:v>2094</x:v>
       </x:c>
       <x:c r="J170" s="134"/>
       <x:c r="K170" s="134"/>
@@ -52072,11 +52116,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G171" s="320" t="s">
-        <x:v>2089</x:v>
+        <x:v>2095</x:v>
       </x:c>
       <x:c r="H171" s="116"/>
       <x:c r="I171" s="320" t="s">
-        <x:v>2090</x:v>
+        <x:v>2096</x:v>
       </x:c>
       <x:c r="J171" s="134"/>
       <x:c r="K171" s="134"/>
@@ -52102,13 +52146,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G172" s="320" t="s">
+        <x:v>2097</x:v>
+      </x:c>
+      <x:c r="H172" s="116" t="s">
         <x:v>2091</x:v>
       </x:c>
-      <x:c r="H172" s="116" t="s">
-        <x:v>2085</x:v>
-      </x:c>
       <x:c r="I172" s="320" t="s">
-        <x:v>2086</x:v>
+        <x:v>2092</x:v>
       </x:c>
       <x:c r="J172" s="134"/>
       <x:c r="K172" s="134"/>
@@ -52124,11 +52168,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G173" s="320" t="s">
-        <x:v>2092</x:v>
+        <x:v>2098</x:v>
       </x:c>
       <x:c r="H173" s="116"/>
       <x:c r="I173" s="320" t="s">
-        <x:v>2093</x:v>
+        <x:v>2099</x:v>
       </x:c>
       <x:c r="J173" s="134"/>
       <x:c r="K173" s="134"/>
@@ -52154,13 +52198,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G174" s="320" t="s">
-        <x:v>2094</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="H174" s="116" t="s">
-        <x:v>2085</x:v>
+        <x:v>2091</x:v>
       </x:c>
       <x:c r="I174" s="320" t="s">
-        <x:v>2095</x:v>
+        <x:v>2101</x:v>
       </x:c>
       <x:c r="J174" s="134"/>
       <x:c r="K174" s="134"/>
@@ -52176,11 +52220,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G175" s="320" t="s">
-        <x:v>2096</x:v>
+        <x:v>2102</x:v>
       </x:c>
       <x:c r="H175" s="116"/>
       <x:c r="I175" s="320" t="s">
-        <x:v>2086</x:v>
+        <x:v>2092</x:v>
       </x:c>
       <x:c r="J175" s="134"/>
       <x:c r="K175" s="134"/>
@@ -52196,11 +52240,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G176" s="320" t="s">
-        <x:v>2097</x:v>
+        <x:v>2103</x:v>
       </x:c>
       <x:c r="H176" s="116"/>
       <x:c r="I176" s="320" t="s">
-        <x:v>2098</x:v>
+        <x:v>2104</x:v>
       </x:c>
       <x:c r="J176" s="134"/>
       <x:c r="K176" s="134"/>
@@ -52217,20 +52261,20 @@
         <x:v>674</x:v>
       </x:c>
       <x:c r="D177" s="116" t="s">
-        <x:v>2099</x:v>
+        <x:v>2105</x:v>
       </x:c>
       <x:c r="E177" s="116" t="s">
-        <x:v>2100</x:v>
+        <x:v>2106</x:v>
       </x:c>
       <x:c r="F177" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G177" s="320" t="s">
-        <x:v>2101</x:v>
+        <x:v>2107</x:v>
       </x:c>
       <x:c r="H177" s="116"/>
       <x:c r="I177" s="320" t="s">
-        <x:v>2102</x:v>
+        <x:v>2108</x:v>
       </x:c>
       <x:c r="J177" s="134"/>
       <x:c r="K177" s="134"/>
@@ -52246,11 +52290,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G178" s="320" t="s">
-        <x:v>2103</x:v>
+        <x:v>2109</x:v>
       </x:c>
       <x:c r="H178" s="116"/>
       <x:c r="I178" s="320" t="s">
-        <x:v>2104</x:v>
+        <x:v>2110</x:v>
       </x:c>
       <x:c r="J178" s="134"/>
       <x:c r="K178" s="134"/>
@@ -52267,22 +52311,22 @@
         <x:v>677</x:v>
       </x:c>
       <x:c r="D179" s="116" t="s">
-        <x:v>2105</x:v>
+        <x:v>2111</x:v>
       </x:c>
       <x:c r="E179" s="116" t="s">
-        <x:v>2106</x:v>
+        <x:v>2112</x:v>
       </x:c>
       <x:c r="F179" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G179" s="320" t="s">
-        <x:v>2107</x:v>
+        <x:v>2113</x:v>
       </x:c>
       <x:c r="H179" s="116" t="s">
         <x:v>681</x:v>
       </x:c>
       <x:c r="I179" s="320" t="s">
-        <x:v>2108</x:v>
+        <x:v>2114</x:v>
       </x:c>
       <x:c r="J179" s="116"/>
       <x:c r="K179" s="134"/>
@@ -52298,13 +52342,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G180" s="321" t="s">
-        <x:v>2109</x:v>
+        <x:v>2115</x:v>
       </x:c>
       <x:c r="H180" s="115" t="s">
-        <x:v>2110</x:v>
+        <x:v>2116</x:v>
       </x:c>
       <x:c r="I180" s="321" t="s">
-        <x:v>2111</x:v>
+        <x:v>2117</x:v>
       </x:c>
       <x:c r="J180" s="115"/>
       <x:c r="K180" s="137"/>
@@ -52321,22 +52365,22 @@
         <x:v>686</x:v>
       </x:c>
       <x:c r="D181" s="116" t="s">
-        <x:v>2112</x:v>
+        <x:v>2118</x:v>
       </x:c>
       <x:c r="E181" s="116" t="s">
-        <x:v>2113</x:v>
+        <x:v>2119</x:v>
       </x:c>
       <x:c r="F181" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G181" s="320" t="s">
-        <x:v>2114</x:v>
+        <x:v>2120</x:v>
       </x:c>
       <x:c r="H181" s="116" t="s">
-        <x:v>2115</x:v>
+        <x:v>2121</x:v>
       </x:c>
       <x:c r="I181" s="320" t="s">
-        <x:v>2116</x:v>
+        <x:v>2122</x:v>
       </x:c>
       <x:c r="J181" s="134"/>
       <x:c r="K181" s="134"/>
@@ -52352,13 +52396,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G182" s="320" t="s">
-        <x:v>2117</x:v>
+        <x:v>2123</x:v>
       </x:c>
       <x:c r="H182" s="116" t="s">
-        <x:v>2118</x:v>
+        <x:v>2124</x:v>
       </x:c>
       <x:c r="I182" s="320" t="s">
-        <x:v>2119</x:v>
+        <x:v>2125</x:v>
       </x:c>
       <x:c r="J182" s="134"/>
       <x:c r="K182" s="134"/>
@@ -52374,11 +52418,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G183" s="320" t="s">
-        <x:v>2120</x:v>
+        <x:v>2126</x:v>
       </x:c>
       <x:c r="H183" s="116"/>
       <x:c r="I183" s="320" t="s">
-        <x:v>2121</x:v>
+        <x:v>2127</x:v>
       </x:c>
       <x:c r="J183" s="134"/>
       <x:c r="K183" s="134"/>
@@ -52395,20 +52439,20 @@
         <x:v>696</x:v>
       </x:c>
       <x:c r="D184" s="116" t="s">
-        <x:v>2122</x:v>
+        <x:v>2128</x:v>
       </x:c>
       <x:c r="E184" s="116" t="s">
-        <x:v>2123</x:v>
+        <x:v>2129</x:v>
       </x:c>
       <x:c r="F184" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G184" s="320" t="s">
-        <x:v>2124</x:v>
+        <x:v>2130</x:v>
       </x:c>
       <x:c r="H184" s="116"/>
       <x:c r="I184" s="320" t="s">
-        <x:v>2125</x:v>
+        <x:v>2131</x:v>
       </x:c>
       <x:c r="J184" s="134"/>
       <x:c r="K184" s="134"/>
@@ -52424,13 +52468,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G185" s="320" t="s">
-        <x:v>2126</x:v>
+        <x:v>2132</x:v>
       </x:c>
       <x:c r="H185" s="116" t="s">
-        <x:v>2127</x:v>
+        <x:v>2133</x:v>
       </x:c>
       <x:c r="I185" s="320" t="s">
-        <x:v>2128</x:v>
+        <x:v>2134</x:v>
       </x:c>
       <x:c r="J185" s="134"/>
       <x:c r="K185" s="134"/>
@@ -52446,11 +52490,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G186" s="320" t="s">
-        <x:v>2129</x:v>
+        <x:v>2135</x:v>
       </x:c>
       <x:c r="H186" s="116"/>
       <x:c r="I186" s="320" t="s">
-        <x:v>2130</x:v>
+        <x:v>2136</x:v>
       </x:c>
       <x:c r="J186" s="134"/>
       <x:c r="K186" s="134"/>
@@ -52466,11 +52510,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G187" s="320" t="s">
-        <x:v>2131</x:v>
+        <x:v>2137</x:v>
       </x:c>
       <x:c r="H187" s="116"/>
       <x:c r="I187" s="320" t="s">
-        <x:v>2132</x:v>
+        <x:v>2138</x:v>
       </x:c>
       <x:c r="J187" s="134"/>
       <x:c r="K187" s="134"/>
@@ -52487,22 +52531,22 @@
         <x:v>932</x:v>
       </x:c>
       <x:c r="D188" s="114" t="s">
-        <x:v>2133</x:v>
+        <x:v>2139</x:v>
       </x:c>
       <x:c r="E188" s="114" t="s">
-        <x:v>2134</x:v>
+        <x:v>2140</x:v>
       </x:c>
       <x:c r="F188" s="329">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G188" s="324" t="s">
-        <x:v>2135</x:v>
+        <x:v>2141</x:v>
       </x:c>
       <x:c r="H188" s="324" t="s">
-        <x:v>2136</x:v>
+        <x:v>2142</x:v>
       </x:c>
       <x:c r="I188" s="325" t="s">
-        <x:v>2137</x:v>
+        <x:v>2143</x:v>
       </x:c>
       <x:c r="J188" s="61"/>
       <x:c r="K188" s="133"/>
@@ -52518,13 +52562,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G189" s="324" t="s">
-        <x:v>2138</x:v>
+        <x:v>2144</x:v>
       </x:c>
       <x:c r="H189" s="324" t="s">
-        <x:v>2139</x:v>
+        <x:v>2145</x:v>
       </x:c>
       <x:c r="I189" s="325" t="s">
-        <x:v>2140</x:v>
+        <x:v>2146</x:v>
       </x:c>
       <x:c r="J189" s="61"/>
       <x:c r="K189" s="124"/>
@@ -52540,11 +52584,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G190" s="324" t="s">
-        <x:v>2141</x:v>
+        <x:v>2147</x:v>
       </x:c>
       <x:c r="H190" s="324"/>
       <x:c r="I190" s="325" t="s">
-        <x:v>2142</x:v>
+        <x:v>2148</x:v>
       </x:c>
       <x:c r="J190" s="61"/>
       <x:c r="K190" s="111"/>
@@ -52561,20 +52605,20 @@
         <x:v>947</x:v>
       </x:c>
       <x:c r="D191" s="114" t="s">
-        <x:v>2143</x:v>
+        <x:v>2149</x:v>
       </x:c>
       <x:c r="E191" s="114" t="s">
-        <x:v>2144</x:v>
+        <x:v>2150</x:v>
       </x:c>
       <x:c r="F191" s="329">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G191" s="324" t="s">
-        <x:v>2145</x:v>
+        <x:v>2151</x:v>
       </x:c>
       <x:c r="H191" s="324"/>
       <x:c r="I191" s="325" t="s">
-        <x:v>2146</x:v>
+        <x:v>2152</x:v>
       </x:c>
       <x:c r="J191" s="61"/>
       <x:c r="K191" s="133"/>
@@ -52590,11 +52634,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G192" s="324" t="s">
-        <x:v>2147</x:v>
+        <x:v>2153</x:v>
       </x:c>
       <x:c r="H192" s="324"/>
       <x:c r="I192" s="325" t="s">
-        <x:v>2148</x:v>
+        <x:v>2154</x:v>
       </x:c>
       <x:c r="J192" s="61"/>
       <x:c r="K192" s="124"/>
@@ -52610,13 +52654,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G193" s="324" t="s">
-        <x:v>2149</x:v>
+        <x:v>2155</x:v>
       </x:c>
       <x:c r="H193" s="324" t="s">
-        <x:v>2150</x:v>
+        <x:v>2156</x:v>
       </x:c>
       <x:c r="I193" s="325" t="s">
-        <x:v>2151</x:v>
+        <x:v>2157</x:v>
       </x:c>
       <x:c r="J193" s="61"/>
       <x:c r="K193" s="111"/>
@@ -52961,16 +53005,16 @@
     <x:mergeCell ref="L191:L193"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H49" r:id="rId185"/>
-    <x:hyperlink ref="H67" r:id="rId186"/>
-    <x:hyperlink ref="H76" r:id="rId187"/>
-    <x:hyperlink ref="H85" r:id="rId188"/>
-    <x:hyperlink ref="H94" r:id="rId189"/>
-    <x:hyperlink ref="H103" r:id="rId190"/>
-    <x:hyperlink ref="H112" r:id="rId191"/>
-    <x:hyperlink ref="H4" r:id="rId192"/>
-    <x:hyperlink ref="H54" r:id="rId193"/>
-    <x:hyperlink ref="H58" r:id="rId194"/>
+    <x:hyperlink ref="H49" r:id="rId140"/>
+    <x:hyperlink ref="H67" r:id="rId141"/>
+    <x:hyperlink ref="H76" r:id="rId142"/>
+    <x:hyperlink ref="H85" r:id="rId143"/>
+    <x:hyperlink ref="H94" r:id="rId144"/>
+    <x:hyperlink ref="H103" r:id="rId145"/>
+    <x:hyperlink ref="H112" r:id="rId146"/>
+    <x:hyperlink ref="H4" r:id="rId147"/>
+    <x:hyperlink ref="H54" r:id="rId148"/>
+    <x:hyperlink ref="H58" r:id="rId149"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -53063,7 +53107,7 @@
         <x:v>1270</x:v>
       </x:c>
       <x:c r="H2" s="288" t="s">
-        <x:v>2152</x:v>
+        <x:v>2158</x:v>
       </x:c>
       <x:c r="I2" s="134" t="s">
         <x:v>1272</x:v>
@@ -53110,7 +53154,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="297" t="s">
-        <x:v>2153</x:v>
+        <x:v>2159</x:v>
       </x:c>
       <x:c r="H4" s="297" t="s">
         <x:v>1277</x:v>
@@ -53190,7 +53234,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="297" t="s">
-        <x:v>2154</x:v>
+        <x:v>2160</x:v>
       </x:c>
       <x:c r="H7" s="297"/>
       <x:c r="I7" s="298" t="s">
@@ -53223,7 +53267,7 @@
         <x:v>1297</x:v>
       </x:c>
       <x:c r="H8" s="297" t="s">
-        <x:v>2155</x:v>
+        <x:v>2161</x:v>
       </x:c>
       <x:c r="I8" s="134" t="s">
         <x:v>1299</x:v>
@@ -53242,7 +53286,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G9" s="319" t="s">
-        <x:v>2156</x:v>
+        <x:v>2162</x:v>
       </x:c>
       <x:c r="H9" s="297"/>
       <x:c r="I9" s="134"/>
@@ -53331,7 +53375,7 @@
         <x:v>1297</x:v>
       </x:c>
       <x:c r="H13" s="297" t="s">
-        <x:v>2157</x:v>
+        <x:v>2163</x:v>
       </x:c>
       <x:c r="I13" s="134" t="s">
         <x:v>1307</x:v>
@@ -53350,7 +53394,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="319" t="s">
-        <x:v>2156</x:v>
+        <x:v>2162</x:v>
       </x:c>
       <x:c r="H14" s="297"/>
       <x:c r="I14" s="134"/>
@@ -53436,7 +53480,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="61" t="s">
-        <x:v>2158</x:v>
+        <x:v>2164</x:v>
       </x:c>
       <x:c r="H18" s="140"/>
       <x:c r="I18" s="140" t="s">
@@ -53456,7 +53500,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="61" t="s">
-        <x:v>2159</x:v>
+        <x:v>2165</x:v>
       </x:c>
       <x:c r="H19" s="140" t="s">
         <x:v>965</x:v>
@@ -53476,7 +53520,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="61" t="s">
-        <x:v>2160</x:v>
+        <x:v>2166</x:v>
       </x:c>
       <x:c r="H20" s="140"/>
       <x:c r="I20" s="140"/>
@@ -53494,7 +53538,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G21" s="61" t="s">
-        <x:v>2161</x:v>
+        <x:v>2167</x:v>
       </x:c>
       <x:c r="H21" s="140" t="s">
         <x:v>968</x:v>
@@ -53514,7 +53558,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G22" s="61" t="s">
-        <x:v>2162</x:v>
+        <x:v>2168</x:v>
       </x:c>
       <x:c r="H22" s="314" t="s">
         <x:v>970</x:v>
@@ -53534,7 +53578,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G23" s="61" t="s">
-        <x:v>2163</x:v>
+        <x:v>2169</x:v>
       </x:c>
       <x:c r="H23" s="140">
         <x:v>1</x:v>
@@ -53554,7 +53598,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G24" s="61" t="s">
-        <x:v>2164</x:v>
+        <x:v>2170</x:v>
       </x:c>
       <x:c r="H24" s="140" t="s">
         <x:v>973</x:v>
@@ -53574,7 +53618,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G25" s="61" t="s">
-        <x:v>2165</x:v>
+        <x:v>2171</x:v>
       </x:c>
       <x:c r="H25" s="140"/>
       <x:c r="I25" s="140"/>
@@ -53602,7 +53646,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G26" s="61" t="s">
-        <x:v>2166</x:v>
+        <x:v>2172</x:v>
       </x:c>
       <x:c r="H26" s="140"/>
       <x:c r="I26" s="133" t="s">
@@ -53642,7 +53686,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G28" s="61" t="s">
-        <x:v>2167</x:v>
+        <x:v>2173</x:v>
       </x:c>
       <x:c r="H28" s="239" t="s">
         <x:v>970</x:v>
@@ -53662,7 +53706,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G29" s="61" t="s">
-        <x:v>2168</x:v>
+        <x:v>2174</x:v>
       </x:c>
       <x:c r="H29" s="140">
         <x:v>1</x:v>
@@ -53682,7 +53726,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G30" s="61" t="s">
-        <x:v>2169</x:v>
+        <x:v>2175</x:v>
       </x:c>
       <x:c r="H30" s="140"/>
       <x:c r="I30" s="111"/>
@@ -53710,7 +53754,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="61" t="s">
-        <x:v>2170</x:v>
+        <x:v>2176</x:v>
       </x:c>
       <x:c r="H31" s="140"/>
       <x:c r="I31" s="133" t="s">
@@ -53809,7 +53853,7 @@
         <x:v>1309</x:v>
       </x:c>
       <x:c r="D36" s="134" t="s">
-        <x:v>2171</x:v>
+        <x:v>2177</x:v>
       </x:c>
       <x:c r="E36" s="134" t="s">
         <x:v>1311</x:v>
@@ -53821,7 +53865,7 @@
         <x:v>988</x:v>
       </x:c>
       <x:c r="H36" s="297" t="s">
-        <x:v>2172</x:v>
+        <x:v>2178</x:v>
       </x:c>
       <x:c r="I36" s="134" t="s">
         <x:v>1312</x:v>
@@ -53843,7 +53887,7 @@
         <x:v>990</x:v>
       </x:c>
       <x:c r="H37" s="314" t="s">
-        <x:v>2173</x:v>
+        <x:v>2179</x:v>
       </x:c>
       <x:c r="I37" s="134"/>
       <x:c r="J37" s="9"/>
@@ -53879,7 +53923,7 @@
         <x:v>1314</x:v>
       </x:c>
       <x:c r="D39" s="134" t="s">
-        <x:v>2174</x:v>
+        <x:v>2180</x:v>
       </x:c>
       <x:c r="E39" s="134" t="s">
         <x:v>1311</x:v>
@@ -53888,10 +53932,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G39" s="319" t="s">
-        <x:v>2175</x:v>
+        <x:v>2181</x:v>
       </x:c>
       <x:c r="H39" s="297" t="s">
-        <x:v>2176</x:v>
+        <x:v>2182</x:v>
       </x:c>
       <x:c r="I39" s="134" t="s">
         <x:v>1317</x:v>
@@ -53913,7 +53957,7 @@
         <x:v>990</x:v>
       </x:c>
       <x:c r="H40" s="314" t="s">
-        <x:v>2173</x:v>
+        <x:v>2179</x:v>
       </x:c>
       <x:c r="I40" s="134"/>
       <x:c r="J40" s="9"/>
@@ -56849,17 +56893,17 @@
     <x:mergeCell ref="J168:J171"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H22" r:id="rId195"/>
-    <x:hyperlink ref="H28" r:id="rId196"/>
-    <x:hyperlink ref="H11" r:id="rId197"/>
-    <x:hyperlink ref="H16" r:id="rId198"/>
-    <x:hyperlink ref="H37" r:id="rId199"/>
-    <x:hyperlink ref="H40" r:id="rId200"/>
-    <x:hyperlink ref="H130" r:id="rId201"/>
-    <x:hyperlink ref="H136" r:id="rId202"/>
-    <x:hyperlink ref="H142" r:id="rId203"/>
-    <x:hyperlink ref="H148" r:id="rId204"/>
-    <x:hyperlink ref="H154" r:id="rId205"/>
+    <x:hyperlink ref="H22" r:id="rId150"/>
+    <x:hyperlink ref="H28" r:id="rId151"/>
+    <x:hyperlink ref="H11" r:id="rId152"/>
+    <x:hyperlink ref="H16" r:id="rId153"/>
+    <x:hyperlink ref="H37" r:id="rId154"/>
+    <x:hyperlink ref="H40" r:id="rId155"/>
+    <x:hyperlink ref="H130" r:id="rId156"/>
+    <x:hyperlink ref="H136" r:id="rId157"/>
+    <x:hyperlink ref="H142" r:id="rId158"/>
+    <x:hyperlink ref="H148" r:id="rId159"/>
+    <x:hyperlink ref="H154" r:id="rId160"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -56944,19 +56988,19 @@
         <x:v>705</x:v>
       </x:c>
       <x:c r="E2" s="116" t="s">
-        <x:v>2177</x:v>
+        <x:v>2183</x:v>
       </x:c>
       <x:c r="F2" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G2" s="327" t="s">
-        <x:v>2178</x:v>
+        <x:v>2184</x:v>
       </x:c>
       <x:c r="H2" s="116" t="s">
-        <x:v>2179</x:v>
+        <x:v>2185</x:v>
       </x:c>
       <x:c r="I2" s="289" t="s">
-        <x:v>2180</x:v>
+        <x:v>2186</x:v>
       </x:c>
       <x:c r="J2" s="1"/>
       <x:c r="K2" s="1"/>
@@ -56972,11 +57016,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G3" s="327" t="s">
-        <x:v>2181</x:v>
+        <x:v>2187</x:v>
       </x:c>
       <x:c r="H3" s="116"/>
       <x:c r="I3" s="289" t="s">
-        <x:v>2182</x:v>
+        <x:v>2188</x:v>
       </x:c>
       <x:c r="J3" s="1"/>
       <x:c r="K3" s="1"/>
@@ -56996,19 +57040,19 @@
         <x:v>707</x:v>
       </x:c>
       <x:c r="E4" s="116" t="s">
-        <x:v>2177</x:v>
+        <x:v>2183</x:v>
       </x:c>
       <x:c r="F4" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="327" t="s">
-        <x:v>2183</x:v>
+        <x:v>2189</x:v>
       </x:c>
       <x:c r="H4" s="116" t="s">
-        <x:v>2184</x:v>
+        <x:v>2190</x:v>
       </x:c>
       <x:c r="I4" s="289" t="s">
-        <x:v>2185</x:v>
+        <x:v>2191</x:v>
       </x:c>
       <x:c r="J4" s="61"/>
       <x:c r="K4" s="1"/>
@@ -57024,11 +57068,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G5" s="327" t="s">
-        <x:v>2186</x:v>
+        <x:v>2192</x:v>
       </x:c>
       <x:c r="H5" s="116"/>
       <x:c r="I5" s="289" t="s">
-        <x:v>2187</x:v>
+        <x:v>2193</x:v>
       </x:c>
       <x:c r="J5" s="61"/>
       <x:c r="K5" s="1"/>
@@ -57044,11 +57088,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G6" s="327" t="s">
-        <x:v>2080</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="H6" s="116"/>
       <x:c r="I6" s="289" t="s">
-        <x:v>2188</x:v>
+        <x:v>2194</x:v>
       </x:c>
       <x:c r="J6" s="61"/>
       <x:c r="K6" s="1"/>
@@ -57068,19 +57112,19 @@
         <x:v>709</x:v>
       </x:c>
       <x:c r="E7" s="116" t="s">
-        <x:v>2189</x:v>
+        <x:v>2195</x:v>
       </x:c>
       <x:c r="F7" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="327" t="s">
-        <x:v>2190</x:v>
+        <x:v>2196</x:v>
       </x:c>
       <x:c r="H7" s="116" t="s">
-        <x:v>2191</x:v>
+        <x:v>2197</x:v>
       </x:c>
       <x:c r="I7" s="289" t="s">
-        <x:v>2192</x:v>
+        <x:v>2198</x:v>
       </x:c>
       <x:c r="J7" s="61"/>
       <x:c r="K7" s="1"/>
@@ -57096,11 +57140,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G8" s="327" t="s">
-        <x:v>2080</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="H8" s="116"/>
       <x:c r="I8" s="289" t="s">
-        <x:v>2193</x:v>
+        <x:v>2199</x:v>
       </x:c>
       <x:c r="J8" s="61"/>
       <x:c r="K8" s="1"/>
@@ -57116,11 +57160,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G9" s="327" t="s">
-        <x:v>2194</x:v>
+        <x:v>2200</x:v>
       </x:c>
       <x:c r="H9" s="116"/>
       <x:c r="I9" s="289" t="s">
-        <x:v>2195</x:v>
+        <x:v>2201</x:v>
       </x:c>
       <x:c r="J9" s="61"/>
       <x:c r="K9" s="1"/>
@@ -57137,20 +57181,20 @@
         <x:v>717</x:v>
       </x:c>
       <x:c r="D10" s="116" t="s">
-        <x:v>2196</x:v>
+        <x:v>2202</x:v>
       </x:c>
       <x:c r="E10" s="116" t="s">
-        <x:v>2197</x:v>
+        <x:v>2203</x:v>
       </x:c>
       <x:c r="F10" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="327" t="s">
-        <x:v>2101</x:v>
+        <x:v>2107</x:v>
       </x:c>
       <x:c r="H10" s="116"/>
       <x:c r="I10" s="289" t="s">
-        <x:v>2198</x:v>
+        <x:v>2204</x:v>
       </x:c>
       <x:c r="J10" s="61"/>
       <x:c r="K10" s="1"/>
@@ -57166,11 +57210,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G11" s="327" t="s">
-        <x:v>2199</x:v>
+        <x:v>2205</x:v>
       </x:c>
       <x:c r="H11" s="116"/>
       <x:c r="I11" s="289" t="s">
-        <x:v>2200</x:v>
+        <x:v>2206</x:v>
       </x:c>
       <x:c r="J11" s="61"/>
       <x:c r="K11" s="1"/>
@@ -57186,11 +57230,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G12" s="327" t="s">
-        <x:v>2201</x:v>
+        <x:v>2207</x:v>
       </x:c>
       <x:c r="H12" s="116"/>
       <x:c r="I12" s="289" t="s">
-        <x:v>2202</x:v>
+        <x:v>2208</x:v>
       </x:c>
       <x:c r="J12" s="61"/>
       <x:c r="K12" s="1"/>
@@ -57207,20 +57251,20 @@
         <x:v>722</x:v>
       </x:c>
       <x:c r="D13" s="116" t="s">
-        <x:v>2203</x:v>
+        <x:v>2209</x:v>
       </x:c>
       <x:c r="E13" s="116" t="s">
-        <x:v>2204</x:v>
+        <x:v>2210</x:v>
       </x:c>
       <x:c r="F13" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="327" t="s">
-        <x:v>2080</x:v>
+        <x:v>2086</x:v>
       </x:c>
       <x:c r="H13" s="116"/>
       <x:c r="I13" s="289" t="s">
-        <x:v>2205</x:v>
+        <x:v>2211</x:v>
       </x:c>
       <x:c r="J13" s="61"/>
       <x:c r="K13" s="1"/>
@@ -57236,11 +57280,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="327" t="s">
-        <x:v>2206</x:v>
+        <x:v>2212</x:v>
       </x:c>
       <x:c r="H14" s="116"/>
       <x:c r="I14" s="289" t="s">
-        <x:v>2207</x:v>
+        <x:v>2213</x:v>
       </x:c>
       <x:c r="J14" s="61"/>
       <x:c r="K14" s="1"/>
@@ -57257,22 +57301,22 @@
         <x:v>724</x:v>
       </x:c>
       <x:c r="D15" s="116" t="s">
-        <x:v>2208</x:v>
+        <x:v>2214</x:v>
       </x:c>
       <x:c r="E15" s="116" t="s">
-        <x:v>2209</x:v>
+        <x:v>2215</x:v>
       </x:c>
       <x:c r="F15" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G15" s="327" t="s">
-        <x:v>2210</x:v>
+        <x:v>2216</x:v>
       </x:c>
       <x:c r="H15" s="116" t="s">
-        <x:v>2211</x:v>
+        <x:v>2217</x:v>
       </x:c>
       <x:c r="I15" s="289" t="s">
-        <x:v>2212</x:v>
+        <x:v>2218</x:v>
       </x:c>
       <x:c r="J15" s="61"/>
       <x:c r="K15" s="1"/>
@@ -57288,11 +57332,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G16" s="327" t="s">
-        <x:v>2213</x:v>
+        <x:v>2219</x:v>
       </x:c>
       <x:c r="H16" s="116"/>
       <x:c r="I16" s="289" t="s">
-        <x:v>2214</x:v>
+        <x:v>2220</x:v>
       </x:c>
       <x:c r="J16" s="61"/>
       <x:c r="K16" s="1"/>
@@ -57308,11 +57352,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G17" s="327" t="s">
-        <x:v>2215</x:v>
+        <x:v>2221</x:v>
       </x:c>
       <x:c r="H17" s="116"/>
       <x:c r="I17" s="289" t="s">
-        <x:v>2216</x:v>
+        <x:v>2222</x:v>
       </x:c>
       <x:c r="J17" s="61"/>
       <x:c r="K17" s="1"/>
@@ -57329,20 +57373,20 @@
         <x:v>726</x:v>
       </x:c>
       <x:c r="D18" s="116" t="s">
-        <x:v>2217</x:v>
+        <x:v>2223</x:v>
       </x:c>
       <x:c r="E18" s="116" t="s">
-        <x:v>2218</x:v>
+        <x:v>2224</x:v>
       </x:c>
       <x:c r="F18" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="327" t="s">
-        <x:v>2219</x:v>
+        <x:v>2225</x:v>
       </x:c>
       <x:c r="H18" s="116"/>
       <x:c r="I18" s="289" t="s">
-        <x:v>2220</x:v>
+        <x:v>2226</x:v>
       </x:c>
       <x:c r="J18" s="61"/>
       <x:c r="K18" s="1"/>
@@ -57358,13 +57402,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="327" t="s">
-        <x:v>2221</x:v>
+        <x:v>2227</x:v>
       </x:c>
       <x:c r="H19" s="116" t="s">
-        <x:v>2222</x:v>
+        <x:v>2228</x:v>
       </x:c>
       <x:c r="I19" s="289" t="s">
-        <x:v>2223</x:v>
+        <x:v>2229</x:v>
       </x:c>
       <x:c r="J19" s="61"/>
       <x:c r="K19" s="1"/>
@@ -57380,11 +57424,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="327" t="s">
-        <x:v>2224</x:v>
+        <x:v>2230</x:v>
       </x:c>
       <x:c r="H20" s="116"/>
       <x:c r="I20" s="289" t="s">
-        <x:v>2225</x:v>
+        <x:v>2231</x:v>
       </x:c>
       <x:c r="J20" s="61"/>
       <x:c r="K20" s="1"/>
@@ -57395,7 +57439,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B21" s="116" t="s">
-        <x:v>2226</x:v>
+        <x:v>2232</x:v>
       </x:c>
       <x:c r="C21" s="116" t="s">
         <x:v>732</x:v>
@@ -57404,19 +57448,19 @@
         <x:v>733</x:v>
       </x:c>
       <x:c r="E21" s="116" t="s">
-        <x:v>2227</x:v>
+        <x:v>2233</x:v>
       </x:c>
       <x:c r="F21" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G21" s="327" t="s">
-        <x:v>2228</x:v>
+        <x:v>2234</x:v>
       </x:c>
       <x:c r="H21" s="116" t="s">
         <x:v>741</x:v>
       </x:c>
       <x:c r="I21" s="289" t="s">
-        <x:v>2229</x:v>
+        <x:v>2235</x:v>
       </x:c>
       <x:c r="J21" s="61"/>
       <x:c r="K21" s="1"/>
@@ -57432,11 +57476,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G22" s="327" t="s">
-        <x:v>2230</x:v>
+        <x:v>2236</x:v>
       </x:c>
       <x:c r="H22" s="116"/>
       <x:c r="I22" s="289" t="s">
-        <x:v>2231</x:v>
+        <x:v>2237</x:v>
       </x:c>
       <x:c r="J22" s="61"/>
       <x:c r="K22" s="1"/>
@@ -57452,11 +57496,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G23" s="327" t="s">
-        <x:v>2232</x:v>
+        <x:v>2238</x:v>
       </x:c>
       <x:c r="H23" s="116"/>
       <x:c r="I23" s="289" t="s">
-        <x:v>2233</x:v>
+        <x:v>2239</x:v>
       </x:c>
       <x:c r="J23" s="61"/>
       <x:c r="K23" s="1"/>
@@ -57473,20 +57517,20 @@
         <x:v>737</x:v>
       </x:c>
       <x:c r="D24" s="116" t="s">
-        <x:v>2234</x:v>
+        <x:v>2240</x:v>
       </x:c>
       <x:c r="E24" s="116" t="s">
-        <x:v>2235</x:v>
+        <x:v>2241</x:v>
       </x:c>
       <x:c r="F24" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G24" s="327" t="s">
-        <x:v>2236</x:v>
+        <x:v>2242</x:v>
       </x:c>
       <x:c r="H24" s="116"/>
       <x:c r="I24" s="289" t="s">
-        <x:v>2237</x:v>
+        <x:v>2243</x:v>
       </x:c>
       <x:c r="J24" s="61"/>
       <x:c r="K24" s="35"/>
@@ -57502,11 +57546,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G25" s="327" t="s">
-        <x:v>2238</x:v>
+        <x:v>2244</x:v>
       </x:c>
       <x:c r="H25" s="116"/>
       <x:c r="I25" s="289" t="s">
-        <x:v>2239</x:v>
+        <x:v>2245</x:v>
       </x:c>
       <x:c r="J25" s="61"/>
       <x:c r="K25" s="35"/>
@@ -57522,11 +57566,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G26" s="327" t="s">
-        <x:v>2131</x:v>
+        <x:v>2137</x:v>
       </x:c>
       <x:c r="H26" s="116"/>
       <x:c r="I26" s="289" t="s">
-        <x:v>2240</x:v>
+        <x:v>2246</x:v>
       </x:c>
       <x:c r="J26" s="61"/>
       <x:c r="K26" s="35"/>
@@ -57543,20 +57587,20 @@
         <x:v>751</x:v>
       </x:c>
       <x:c r="D27" s="116" t="s">
-        <x:v>2241</x:v>
+        <x:v>2247</x:v>
       </x:c>
       <x:c r="E27" s="116" t="s">
-        <x:v>2242</x:v>
+        <x:v>2248</x:v>
       </x:c>
       <x:c r="F27" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G27" s="327" t="s">
-        <x:v>2243</x:v>
+        <x:v>2249</x:v>
       </x:c>
       <x:c r="H27" s="116"/>
       <x:c r="I27" s="327" t="s">
-        <x:v>2086</x:v>
+        <x:v>2092</x:v>
       </x:c>
       <x:c r="J27" s="61"/>
       <x:c r="K27" s="35"/>
@@ -57572,11 +57616,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G28" s="327" t="s">
-        <x:v>2244</x:v>
+        <x:v>2250</x:v>
       </x:c>
       <x:c r="H28" s="116"/>
       <x:c r="I28" s="289" t="s">
-        <x:v>2245</x:v>
+        <x:v>2251</x:v>
       </x:c>
       <x:c r="J28" s="61"/>
       <x:c r="K28" s="35"/>
@@ -57593,20 +57637,20 @@
         <x:v>753</x:v>
       </x:c>
       <x:c r="D29" s="116" t="s">
-        <x:v>2246</x:v>
+        <x:v>2252</x:v>
       </x:c>
       <x:c r="E29" s="116" t="s">
-        <x:v>2242</x:v>
+        <x:v>2248</x:v>
       </x:c>
       <x:c r="F29" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G29" s="327" t="s">
-        <x:v>2247</x:v>
+        <x:v>2253</x:v>
       </x:c>
       <x:c r="H29" s="116"/>
       <x:c r="I29" s="327" t="s">
-        <x:v>2086</x:v>
+        <x:v>2092</x:v>
       </x:c>
       <x:c r="J29" s="61"/>
       <x:c r="K29" s="35"/>
@@ -57622,11 +57666,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G30" s="327" t="s">
-        <x:v>2248</x:v>
+        <x:v>2254</x:v>
       </x:c>
       <x:c r="H30" s="116"/>
       <x:c r="I30" s="289" t="s">
-        <x:v>2249</x:v>
+        <x:v>2255</x:v>
       </x:c>
       <x:c r="J30" s="61"/>
       <x:c r="K30" s="35"/>
@@ -57646,19 +57690,19 @@
         <x:v>793</x:v>
       </x:c>
       <x:c r="E31" s="116" t="s">
-        <x:v>2250</x:v>
+        <x:v>2256</x:v>
       </x:c>
       <x:c r="F31" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="327" t="s">
-        <x:v>2251</x:v>
+        <x:v>2257</x:v>
       </x:c>
       <x:c r="H31" s="116" t="s">
-        <x:v>2252</x:v>
+        <x:v>2258</x:v>
       </x:c>
       <x:c r="I31" s="289" t="s">
-        <x:v>2253</x:v>
+        <x:v>2259</x:v>
       </x:c>
       <x:c r="J31" s="61"/>
       <x:c r="K31" s="35"/>
@@ -57674,11 +57718,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G32" s="327" t="s">
-        <x:v>2254</x:v>
+        <x:v>2260</x:v>
       </x:c>
       <x:c r="H32" s="116"/>
       <x:c r="I32" s="289" t="s">
-        <x:v>2255</x:v>
+        <x:v>2261</x:v>
       </x:c>
       <x:c r="J32" s="61"/>
       <x:c r="K32" s="35"/>
@@ -57698,19 +57742,19 @@
         <x:v>798</x:v>
       </x:c>
       <x:c r="E33" s="116" t="s">
-        <x:v>2256</x:v>
+        <x:v>2262</x:v>
       </x:c>
       <x:c r="F33" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G33" s="327" t="s">
-        <x:v>2257</x:v>
+        <x:v>2263</x:v>
       </x:c>
       <x:c r="H33" s="116" t="s">
-        <x:v>2252</x:v>
+        <x:v>2258</x:v>
       </x:c>
       <x:c r="I33" s="327" t="s">
-        <x:v>2086</x:v>
+        <x:v>2092</x:v>
       </x:c>
       <x:c r="J33" s="61"/>
       <x:c r="K33" s="35"/>
@@ -57726,11 +57770,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G34" s="327" t="s">
-        <x:v>2258</x:v>
+        <x:v>2264</x:v>
       </x:c>
       <x:c r="H34" s="116"/>
       <x:c r="I34" s="289" t="s">
-        <x:v>2259</x:v>
+        <x:v>2265</x:v>
       </x:c>
       <x:c r="J34" s="292"/>
       <x:c r="K34" s="35"/>
@@ -57747,20 +57791,20 @@
         <x:v>802</x:v>
       </x:c>
       <x:c r="D35" s="116" t="s">
-        <x:v>2260</x:v>
+        <x:v>2266</x:v>
       </x:c>
       <x:c r="E35" s="116" t="s">
-        <x:v>2261</x:v>
+        <x:v>2267</x:v>
       </x:c>
       <x:c r="F35" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G35" s="327" t="s">
-        <x:v>2262</x:v>
+        <x:v>2268</x:v>
       </x:c>
       <x:c r="H35" s="116"/>
       <x:c r="I35" s="289" t="s">
-        <x:v>2263</x:v>
+        <x:v>2269</x:v>
       </x:c>
       <x:c r="J35" s="61"/>
       <x:c r="K35" s="35"/>
@@ -57776,11 +57820,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G36" s="327" t="s">
-        <x:v>2264</x:v>
+        <x:v>2270</x:v>
       </x:c>
       <x:c r="H36" s="116"/>
       <x:c r="I36" s="289" t="s">
-        <x:v>2265</x:v>
+        <x:v>2271</x:v>
       </x:c>
       <x:c r="J36" s="61"/>
       <x:c r="K36" s="35"/>
@@ -57796,13 +57840,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G37" s="327" t="s">
-        <x:v>2266</x:v>
+        <x:v>2272</x:v>
       </x:c>
       <x:c r="H37" s="116" t="s">
-        <x:v>2267</x:v>
+        <x:v>2273</x:v>
       </x:c>
       <x:c r="I37" s="289" t="s">
-        <x:v>2268</x:v>
+        <x:v>2274</x:v>
       </x:c>
       <x:c r="J37" s="61"/>
       <x:c r="K37" s="35"/>
@@ -57819,20 +57863,20 @@
         <x:v>814</x:v>
       </x:c>
       <x:c r="D38" s="116" t="s">
-        <x:v>2269</x:v>
+        <x:v>2275</x:v>
       </x:c>
       <x:c r="E38" s="116" t="s">
-        <x:v>2270</x:v>
+        <x:v>2276</x:v>
       </x:c>
       <x:c r="F38" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G38" s="327" t="s">
-        <x:v>2271</x:v>
+        <x:v>2277</x:v>
       </x:c>
       <x:c r="H38" s="116"/>
       <x:c r="I38" s="289" t="s">
-        <x:v>2272</x:v>
+        <x:v>2278</x:v>
       </x:c>
       <x:c r="J38" s="61"/>
       <x:c r="K38" s="35"/>
@@ -57848,11 +57892,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G39" s="327" t="s">
-        <x:v>2273</x:v>
+        <x:v>2279</x:v>
       </x:c>
       <x:c r="H39" s="116"/>
       <x:c r="I39" s="289" t="s">
-        <x:v>2274</x:v>
+        <x:v>2280</x:v>
       </x:c>
       <x:c r="J39" s="61"/>
       <x:c r="K39" s="35"/>
@@ -57868,13 +57912,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G40" s="327" t="s">
-        <x:v>2275</x:v>
+        <x:v>2281</x:v>
       </x:c>
       <x:c r="H40" s="116" t="s">
-        <x:v>2267</x:v>
+        <x:v>2273</x:v>
       </x:c>
       <x:c r="I40" s="289" t="s">
-        <x:v>2276</x:v>
+        <x:v>2282</x:v>
       </x:c>
       <x:c r="J40" s="61"/>
       <x:c r="K40" s="35"/>
@@ -57890,11 +57934,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G41" s="327" t="s">
-        <x:v>2277</x:v>
+        <x:v>2283</x:v>
       </x:c>
       <x:c r="H41" s="116"/>
       <x:c r="I41" s="289" t="s">
-        <x:v>2278</x:v>
+        <x:v>2284</x:v>
       </x:c>
       <x:c r="J41" s="61"/>
       <x:c r="K41" s="35"/>
@@ -57911,20 +57955,20 @@
         <x:v>824</x:v>
       </x:c>
       <x:c r="D42" s="116" t="s">
-        <x:v>2279</x:v>
+        <x:v>2285</x:v>
       </x:c>
       <x:c r="E42" s="116" t="s">
-        <x:v>2280</x:v>
+        <x:v>2286</x:v>
       </x:c>
       <x:c r="F42" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G42" s="327" t="s">
-        <x:v>2281</x:v>
+        <x:v>2287</x:v>
       </x:c>
       <x:c r="H42" s="116"/>
       <x:c r="I42" s="289" t="s">
-        <x:v>2282</x:v>
+        <x:v>2288</x:v>
       </x:c>
       <x:c r="J42" s="61"/>
       <x:c r="K42" s="35"/>
@@ -57940,11 +57984,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G43" s="327" t="s">
-        <x:v>2283</x:v>
+        <x:v>2289</x:v>
       </x:c>
       <x:c r="H43" s="116"/>
       <x:c r="I43" s="289" t="s">
-        <x:v>2284</x:v>
+        <x:v>2290</x:v>
       </x:c>
       <x:c r="J43" s="61"/>
       <x:c r="K43" s="35"/>
@@ -57960,11 +58004,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G44" s="327" t="s">
-        <x:v>2285</x:v>
+        <x:v>2291</x:v>
       </x:c>
       <x:c r="H44" s="116"/>
       <x:c r="I44" s="289" t="s">
-        <x:v>2286</x:v>
+        <x:v>2292</x:v>
       </x:c>
       <x:c r="J44" s="61"/>
       <x:c r="K44" s="35"/>
@@ -57980,11 +58024,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G45" s="327" t="s">
-        <x:v>2287</x:v>
+        <x:v>2293</x:v>
       </x:c>
       <x:c r="H45" s="116"/>
       <x:c r="I45" s="289" t="s">
-        <x:v>2288</x:v>
+        <x:v>2294</x:v>
       </x:c>
       <x:c r="J45" s="61"/>
       <x:c r="K45" s="35"/>
@@ -58001,20 +58045,20 @@
         <x:v>835</x:v>
       </x:c>
       <x:c r="D46" s="116" t="s">
-        <x:v>2289</x:v>
+        <x:v>2295</x:v>
       </x:c>
       <x:c r="E46" s="116" t="s">
-        <x:v>2290</x:v>
+        <x:v>2296</x:v>
       </x:c>
       <x:c r="F46" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G46" s="327" t="s">
-        <x:v>2281</x:v>
+        <x:v>2287</x:v>
       </x:c>
       <x:c r="H46" s="116"/>
       <x:c r="I46" s="289" t="s">
-        <x:v>2291</x:v>
+        <x:v>2297</x:v>
       </x:c>
       <x:c r="J46" s="61"/>
       <x:c r="K46" s="35"/>
@@ -58030,13 +58074,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G47" s="327" t="s">
-        <x:v>2292</x:v>
+        <x:v>2298</x:v>
       </x:c>
       <x:c r="H47" s="116" t="s">
-        <x:v>2267</x:v>
+        <x:v>2273</x:v>
       </x:c>
       <x:c r="I47" s="289" t="s">
-        <x:v>2293</x:v>
+        <x:v>2299</x:v>
       </x:c>
       <x:c r="J47" s="61"/>
       <x:c r="K47" s="35"/>
@@ -58052,11 +58096,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G48" s="327" t="s">
-        <x:v>2294</x:v>
+        <x:v>2300</x:v>
       </x:c>
       <x:c r="H48" s="116"/>
       <x:c r="I48" s="289" t="s">
-        <x:v>2295</x:v>
+        <x:v>2301</x:v>
       </x:c>
       <x:c r="J48" s="61"/>
       <x:c r="K48" s="35"/>
@@ -58155,10 +58199,10 @@
         <x:v>999</x:v>
       </x:c>
       <x:c r="H52" s="334" t="s">
-        <x:v>2296</x:v>
+        <x:v>2302</x:v>
       </x:c>
       <x:c r="I52" s="51" t="s">
-        <x:v>2297</x:v>
+        <x:v>2303</x:v>
       </x:c>
       <x:c r="J52" s="51"/>
       <x:c r="K52" s="35"/>
@@ -58177,7 +58221,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H53" s="314" t="s">
-        <x:v>2298</x:v>
+        <x:v>2304</x:v>
       </x:c>
       <x:c r="I53" s="51"/>
       <x:c r="J53" s="51"/>
@@ -58228,7 +58272,7 @@
         <x:v>1000</x:v>
       </x:c>
       <x:c r="I55" s="51" t="s">
-        <x:v>2299</x:v>
+        <x:v>2305</x:v>
       </x:c>
       <x:c r="J55" s="51"/>
       <x:c r="K55" s="35"/>
@@ -58247,7 +58291,7 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="H56" s="314" t="s">
-        <x:v>2300</x:v>
+        <x:v>2306</x:v>
       </x:c>
       <x:c r="I56" s="51"/>
       <x:c r="J56" s="51"/>
@@ -58366,7 +58410,7 @@
         <x:v>422</x:v>
       </x:c>
       <x:c r="I61" s="51" t="s">
-        <x:v>2301</x:v>
+        <x:v>2307</x:v>
       </x:c>
       <x:c r="J61" s="51"/>
       <x:c r="K61" s="35"/>
@@ -58664,7 +58708,7 @@
         <x:v>1037</x:v>
       </x:c>
       <x:c r="I74" s="51" t="s">
-        <x:v>2302</x:v>
+        <x:v>2308</x:v>
       </x:c>
       <x:c r="J74" s="51"/>
       <x:c r="K74" s="35"/>
@@ -59360,19 +59404,19 @@
         <x:v>843</x:v>
       </x:c>
       <x:c r="E106" s="116" t="s">
-        <x:v>2303</x:v>
+        <x:v>2309</x:v>
       </x:c>
       <x:c r="F106" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G106" s="327" t="s">
-        <x:v>2304</x:v>
+        <x:v>2310</x:v>
       </x:c>
       <x:c r="H106" s="116" t="s">
-        <x:v>2305</x:v>
+        <x:v>2311</x:v>
       </x:c>
       <x:c r="I106" s="289" t="s">
-        <x:v>2306</x:v>
+        <x:v>2312</x:v>
       </x:c>
       <x:c r="J106" s="61"/>
       <x:c r="K106" s="140"/>
@@ -59388,11 +59432,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G107" s="327" t="s">
-        <x:v>2307</x:v>
+        <x:v>2313</x:v>
       </x:c>
       <x:c r="H107" s="116"/>
       <x:c r="I107" s="289" t="s">
-        <x:v>2308</x:v>
+        <x:v>2314</x:v>
       </x:c>
       <x:c r="J107" s="61"/>
       <x:c r="K107" s="140"/>
@@ -59408,13 +59452,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G108" s="327" t="s">
-        <x:v>2309</x:v>
+        <x:v>2315</x:v>
       </x:c>
       <x:c r="H108" s="116" t="s">
-        <x:v>2310</x:v>
+        <x:v>2316</x:v>
       </x:c>
       <x:c r="I108" s="289" t="s">
-        <x:v>2311</x:v>
+        <x:v>2317</x:v>
       </x:c>
       <x:c r="J108" s="61"/>
       <x:c r="K108" s="140"/>
@@ -59430,11 +59474,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G109" s="327" t="s">
-        <x:v>2312</x:v>
+        <x:v>2318</x:v>
       </x:c>
       <x:c r="H109" s="116"/>
       <x:c r="I109" s="289" t="s">
-        <x:v>2313</x:v>
+        <x:v>2319</x:v>
       </x:c>
       <x:c r="J109" s="61"/>
       <x:c r="K109" s="140"/>
@@ -59454,19 +59498,19 @@
         <x:v>854</x:v>
       </x:c>
       <x:c r="E110" s="116" t="s">
-        <x:v>2314</x:v>
+        <x:v>2320</x:v>
       </x:c>
       <x:c r="F110" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G110" s="327" t="s">
-        <x:v>2315</x:v>
+        <x:v>2321</x:v>
       </x:c>
       <x:c r="H110" s="116" t="s">
-        <x:v>2316</x:v>
+        <x:v>2322</x:v>
       </x:c>
       <x:c r="I110" s="289" t="s">
-        <x:v>2317</x:v>
+        <x:v>2323</x:v>
       </x:c>
       <x:c r="J110" s="61"/>
       <x:c r="K110" s="140"/>
@@ -59482,11 +59526,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G111" s="327" t="s">
-        <x:v>2307</x:v>
+        <x:v>2313</x:v>
       </x:c>
       <x:c r="H111" s="116"/>
       <x:c r="I111" s="289" t="s">
-        <x:v>2318</x:v>
+        <x:v>2324</x:v>
       </x:c>
       <x:c r="J111" s="61"/>
       <x:c r="K111" s="140"/>
@@ -59502,13 +59546,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G112" s="327" t="s">
-        <x:v>2319</x:v>
+        <x:v>2325</x:v>
       </x:c>
       <x:c r="H112" s="116" t="s">
-        <x:v>2320</x:v>
+        <x:v>2326</x:v>
       </x:c>
       <x:c r="I112" s="289" t="s">
-        <x:v>2321</x:v>
+        <x:v>2327</x:v>
       </x:c>
       <x:c r="J112" s="61"/>
       <x:c r="K112" s="140"/>
@@ -59524,11 +59568,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G113" s="327" t="s">
-        <x:v>2322</x:v>
+        <x:v>2328</x:v>
       </x:c>
       <x:c r="H113" s="116"/>
       <x:c r="I113" s="289" t="s">
-        <x:v>2323</x:v>
+        <x:v>2329</x:v>
       </x:c>
       <x:c r="J113" s="61"/>
       <x:c r="K113" s="140"/>
@@ -59545,7 +59589,7 @@
         <x:v>863</x:v>
       </x:c>
       <x:c r="D114" s="140" t="s">
-        <x:v>2324</x:v>
+        <x:v>2330</x:v>
       </x:c>
       <x:c r="E114" s="140" t="s">
         <x:v>865</x:v>
@@ -59554,7 +59598,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G114" s="61" t="s">
-        <x:v>2325</x:v>
+        <x:v>2331</x:v>
       </x:c>
       <x:c r="H114" s="140"/>
       <x:c r="I114" s="61" t="s">
@@ -59574,7 +59618,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G115" s="61" t="s">
-        <x:v>2326</x:v>
+        <x:v>2332</x:v>
       </x:c>
       <x:c r="H115" s="140"/>
       <x:c r="I115" s="61" t="s">
@@ -59594,10 +59638,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G116" s="61" t="s">
-        <x:v>2327</x:v>
+        <x:v>2333</x:v>
       </x:c>
       <x:c r="H116" s="140" t="s">
-        <x:v>2328</x:v>
+        <x:v>2334</x:v>
       </x:c>
       <x:c r="I116" s="61"/>
       <x:c r="J116" s="140"/>
@@ -59614,10 +59658,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G117" s="61" t="s">
-        <x:v>2329</x:v>
+        <x:v>2335</x:v>
       </x:c>
       <x:c r="H117" s="140" t="s">
-        <x:v>2330</x:v>
+        <x:v>2336</x:v>
       </x:c>
       <x:c r="I117" s="61"/>
       <x:c r="J117" s="140"/>
@@ -59652,7 +59696,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G119" s="61" t="s">
-        <x:v>2331</x:v>
+        <x:v>2337</x:v>
       </x:c>
       <x:c r="H119" s="140" t="s">
         <x:v>877</x:v>
@@ -59672,7 +59716,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G120" s="61" t="s">
-        <x:v>2332</x:v>
+        <x:v>2338</x:v>
       </x:c>
       <x:c r="H120" s="251">
         <x:v>0.375</x:v>
@@ -59692,7 +59736,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G121" s="61" t="s">
-        <x:v>2333</x:v>
+        <x:v>2339</x:v>
       </x:c>
       <x:c r="H121" s="140">
         <x:v>100000</x:v>
@@ -59712,7 +59756,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="G122" s="61" t="s">
-        <x:v>2334</x:v>
+        <x:v>2340</x:v>
       </x:c>
       <x:c r="H122" s="140">
         <x:v>1</x:v>
@@ -59732,7 +59776,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G123" s="61" t="s">
-        <x:v>2335</x:v>
+        <x:v>2341</x:v>
       </x:c>
       <x:c r="H123" s="140"/>
       <x:c r="I123" s="61" t="s">
@@ -59753,7 +59797,7 @@
         <x:v>884</x:v>
       </x:c>
       <x:c r="D124" s="140" t="s">
-        <x:v>2336</x:v>
+        <x:v>2342</x:v>
       </x:c>
       <x:c r="E124" s="140" t="s">
         <x:v>886</x:v>
@@ -59762,7 +59806,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G124" s="61" t="s">
-        <x:v>2337</x:v>
+        <x:v>2343</x:v>
       </x:c>
       <x:c r="H124" s="140"/>
       <x:c r="I124" s="140" t="s">
@@ -59782,7 +59826,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G125" s="61" t="s">
-        <x:v>2338</x:v>
+        <x:v>2344</x:v>
       </x:c>
       <x:c r="H125" s="140"/>
       <x:c r="I125" s="140"/>
@@ -59800,10 +59844,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G126" s="61" t="s">
-        <x:v>2339</x:v>
+        <x:v>2345</x:v>
       </x:c>
       <x:c r="H126" s="140" t="s">
-        <x:v>2340</x:v>
+        <x:v>2346</x:v>
       </x:c>
       <x:c r="I126" s="140"/>
       <x:c r="J126" s="140"/>
@@ -59820,10 +59864,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G127" s="61" t="s">
-        <x:v>2341</x:v>
+        <x:v>2347</x:v>
       </x:c>
       <x:c r="H127" s="140" t="s">
-        <x:v>2342</x:v>
+        <x:v>2348</x:v>
       </x:c>
       <x:c r="I127" s="140"/>
       <x:c r="J127" s="140"/>
@@ -59840,7 +59884,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G128" s="61" t="s">
-        <x:v>2343</x:v>
+        <x:v>2349</x:v>
       </x:c>
       <x:c r="H128" s="140" t="s">
         <x:v>877</x:v>
@@ -59878,7 +59922,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G130" s="61" t="s">
-        <x:v>2344</x:v>
+        <x:v>2350</x:v>
       </x:c>
       <x:c r="H130" s="140">
         <x:v>100000</x:v>
@@ -59898,7 +59942,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="G131" s="61" t="s">
-        <x:v>2345</x:v>
+        <x:v>2351</x:v>
       </x:c>
       <x:c r="H131" s="140">
         <x:v>1</x:v>
@@ -59918,7 +59962,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G132" s="61" t="s">
-        <x:v>2346</x:v>
+        <x:v>2352</x:v>
       </x:c>
       <x:c r="H132" s="140"/>
       <x:c r="I132" s="140"/>
@@ -59937,7 +59981,7 @@
         <x:v>900</x:v>
       </x:c>
       <x:c r="D133" s="140" t="s">
-        <x:v>2347</x:v>
+        <x:v>2353</x:v>
       </x:c>
       <x:c r="E133" s="140" t="s">
         <x:v>886</x:v>
@@ -59946,7 +59990,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G133" s="61" t="s">
-        <x:v>2348</x:v>
+        <x:v>2354</x:v>
       </x:c>
       <x:c r="H133" s="140"/>
       <x:c r="I133" s="140" t="s">
@@ -59966,7 +60010,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G134" s="61" t="s">
-        <x:v>2349</x:v>
+        <x:v>2355</x:v>
       </x:c>
       <x:c r="H134" s="140"/>
       <x:c r="I134" s="140"/>
@@ -59984,7 +60028,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G135" s="61" t="s">
-        <x:v>2350</x:v>
+        <x:v>2356</x:v>
       </x:c>
       <x:c r="H135" s="140" t="s">
         <x:v>891</x:v>
@@ -60062,7 +60106,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G139" s="61" t="s">
-        <x:v>2351</x:v>
+        <x:v>2357</x:v>
       </x:c>
       <x:c r="H139" s="140">
         <x:f>1</x:f>
@@ -60082,7 +60126,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G140" s="61" t="s">
-        <x:v>2352</x:v>
+        <x:v>2358</x:v>
       </x:c>
       <x:c r="H140" s="140"/>
       <x:c r="I140" s="140"/>
@@ -60101,7 +60145,7 @@
         <x:v>911</x:v>
       </x:c>
       <x:c r="D141" s="140" t="s">
-        <x:v>2353</x:v>
+        <x:v>2359</x:v>
       </x:c>
       <x:c r="E141" s="140" t="s">
         <x:v>886</x:v>
@@ -60110,7 +60154,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G141" s="61" t="s">
-        <x:v>2354</x:v>
+        <x:v>2360</x:v>
       </x:c>
       <x:c r="H141" s="140"/>
       <x:c r="I141" s="140" t="s">
@@ -60130,7 +60174,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G142" s="61" t="s">
-        <x:v>2355</x:v>
+        <x:v>2361</x:v>
       </x:c>
       <x:c r="H142" s="140"/>
       <x:c r="I142" s="140"/>
@@ -60148,7 +60192,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G143" s="61" t="s">
-        <x:v>2356</x:v>
+        <x:v>2362</x:v>
       </x:c>
       <x:c r="H143" s="140" t="s">
         <x:v>891</x:v>
@@ -60246,7 +60290,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G148" s="61" t="s">
-        <x:v>2357</x:v>
+        <x:v>2363</x:v>
       </x:c>
       <x:c r="H148" s="140"/>
       <x:c r="I148" s="140"/>
@@ -60265,22 +60309,22 @@
         <x:v>921</x:v>
       </x:c>
       <x:c r="D149" s="116" t="s">
-        <x:v>2358</x:v>
+        <x:v>2364</x:v>
       </x:c>
       <x:c r="E149" s="116" t="s">
-        <x:v>2359</x:v>
+        <x:v>2365</x:v>
       </x:c>
       <x:c r="F149" s="116">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G149" s="327" t="s">
-        <x:v>2360</x:v>
+        <x:v>2366</x:v>
       </x:c>
       <x:c r="H149" s="116" t="s">
-        <x:v>2361</x:v>
+        <x:v>2367</x:v>
       </x:c>
       <x:c r="I149" s="289" t="s">
-        <x:v>2362</x:v>
+        <x:v>2368</x:v>
       </x:c>
       <x:c r="J149" s="61"/>
       <x:c r="K149" s="140"/>
@@ -60296,11 +60340,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G150" s="327" t="s">
-        <x:v>2363</x:v>
+        <x:v>2369</x:v>
       </x:c>
       <x:c r="H150" s="116"/>
       <x:c r="I150" s="289" t="s">
-        <x:v>2364</x:v>
+        <x:v>2370</x:v>
       </x:c>
       <x:c r="J150" s="61"/>
       <x:c r="K150" s="140"/>
@@ -60316,13 +60360,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G151" s="327" t="s">
-        <x:v>2365</x:v>
+        <x:v>2371</x:v>
       </x:c>
       <x:c r="H151" s="116" t="s">
-        <x:v>2366</x:v>
+        <x:v>2372</x:v>
       </x:c>
       <x:c r="I151" s="289" t="s">
-        <x:v>2367</x:v>
+        <x:v>2373</x:v>
       </x:c>
       <x:c r="J151" s="61"/>
       <x:c r="K151" s="140"/>
@@ -60338,11 +60382,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G152" s="327" t="s">
-        <x:v>2368</x:v>
+        <x:v>2374</x:v>
       </x:c>
       <x:c r="H152" s="116"/>
       <x:c r="I152" s="289" t="s">
-        <x:v>2369</x:v>
+        <x:v>2375</x:v>
       </x:c>
       <x:c r="J152" s="61"/>
       <x:c r="K152" s="140"/>
@@ -60358,11 +60402,11 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G153" s="327" t="s">
-        <x:v>2370</x:v>
+        <x:v>2376</x:v>
       </x:c>
       <x:c r="H153" s="116"/>
       <x:c r="I153" s="289" t="s">
-        <x:v>2371</x:v>
+        <x:v>2377</x:v>
       </x:c>
       <x:c r="J153" s="61"/>
       <x:c r="K153" s="140"/>
@@ -60699,17 +60743,17 @@
     <x:mergeCell ref="L149:L153"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H49" r:id="rId206"/>
-    <x:hyperlink ref="H50" r:id="rId207"/>
-    <x:hyperlink ref="H55" r:id="rId208"/>
-    <x:hyperlink ref="H56" r:id="rId209"/>
-    <x:hyperlink ref="H59" r:id="rId210"/>
-    <x:hyperlink ref="H64" r:id="rId211"/>
-    <x:hyperlink ref="H65" r:id="rId212"/>
-    <x:hyperlink ref="H67" r:id="rId213"/>
-    <x:hyperlink ref="H68" r:id="rId214"/>
-    <x:hyperlink ref="H52" r:id="rId215"/>
-    <x:hyperlink ref="H61" r:id="rId216"/>
+    <x:hyperlink ref="H49" r:id="rId161"/>
+    <x:hyperlink ref="H50" r:id="rId162"/>
+    <x:hyperlink ref="H55" r:id="rId163"/>
+    <x:hyperlink ref="H56" r:id="rId164"/>
+    <x:hyperlink ref="H59" r:id="rId165"/>
+    <x:hyperlink ref="H64" r:id="rId166"/>
+    <x:hyperlink ref="H65" r:id="rId167"/>
+    <x:hyperlink ref="H67" r:id="rId168"/>
+    <x:hyperlink ref="H68" r:id="rId169"/>
+    <x:hyperlink ref="H52" r:id="rId170"/>
+    <x:hyperlink ref="H61" r:id="rId171"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -60803,7 +60847,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H2" s="340" t="s">
-        <x:v>2372</x:v>
+        <x:v>2378</x:v>
       </x:c>
       <x:c r="I2" s="51" t="s">
         <x:v>1102</x:v>
@@ -61042,7 +61086,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G14" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H14" s="292"/>
       <x:c r="I14" s="51"/>
@@ -61312,7 +61356,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G27" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H27" s="292"/>
       <x:c r="I27" s="51"/>
@@ -61343,7 +61387,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H28" s="340" t="s">
-        <x:v>2374</x:v>
+        <x:v>2380</x:v>
       </x:c>
       <x:c r="I28" s="51" t="s">
         <x:v>1127</x:v>
@@ -61582,7 +61626,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G40" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H40" s="292"/>
       <x:c r="I40" s="51"/>
@@ -61613,7 +61657,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H41" s="340" t="s">
-        <x:v>2375</x:v>
+        <x:v>2381</x:v>
       </x:c>
       <x:c r="I41" s="51" t="s">
         <x:v>1130</x:v>
@@ -61852,7 +61896,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G53" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H53" s="292"/>
       <x:c r="I53" s="51"/>
@@ -61883,7 +61927,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H54" s="340" t="s">
-        <x:v>2376</x:v>
+        <x:v>2382</x:v>
       </x:c>
       <x:c r="I54" s="51" t="s">
         <x:v>1134</x:v>
@@ -62122,7 +62166,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G66" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H66" s="292"/>
       <x:c r="I66" s="51"/>
@@ -62153,7 +62197,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H67" s="340" t="s">
-        <x:v>2377</x:v>
+        <x:v>2383</x:v>
       </x:c>
       <x:c r="I67" s="51" t="s">
         <x:v>1138</x:v>
@@ -62392,7 +62436,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G79" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H79" s="292"/>
       <x:c r="I79" s="51"/>
@@ -62423,7 +62467,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H80" s="340" t="s">
-        <x:v>2378</x:v>
+        <x:v>2384</x:v>
       </x:c>
       <x:c r="I80" s="51" t="s">
         <x:v>1141</x:v>
@@ -62662,7 +62706,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G92" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H92" s="292"/>
       <x:c r="I92" s="51"/>
@@ -62693,7 +62737,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H93" s="340" t="s">
-        <x:v>2379</x:v>
+        <x:v>2385</x:v>
       </x:c>
       <x:c r="I93" s="51" t="s">
         <x:v>1145</x:v>
@@ -62932,7 +62976,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G105" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H105" s="292"/>
       <x:c r="I105" s="51"/>
@@ -62963,7 +63007,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H106" s="340" t="s">
-        <x:v>2379</x:v>
+        <x:v>2385</x:v>
       </x:c>
       <x:c r="I106" s="51" t="s">
         <x:v>1149</x:v>
@@ -63202,7 +63246,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G118" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H118" s="292"/>
       <x:c r="I118" s="51"/>
@@ -63233,7 +63277,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H119" s="340" t="s">
-        <x:v>2380</x:v>
+        <x:v>2386</x:v>
       </x:c>
       <x:c r="I119" s="51" t="s">
         <x:v>1149</x:v>
@@ -63472,7 +63516,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G131" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H131" s="292"/>
       <x:c r="I131" s="51"/>
@@ -63503,7 +63547,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H132" s="340" t="s">
-        <x:v>2381</x:v>
+        <x:v>2387</x:v>
       </x:c>
       <x:c r="I132" s="51" t="s">
         <x:v>1160</x:v>
@@ -63742,7 +63786,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G144" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H144" s="292"/>
       <x:c r="I144" s="51"/>
@@ -63773,7 +63817,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H145" s="340" t="s">
-        <x:v>2382</x:v>
+        <x:v>2388</x:v>
       </x:c>
       <x:c r="I145" s="51" t="s">
         <x:v>1160</x:v>
@@ -64012,7 +64056,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G157" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H157" s="292"/>
       <x:c r="I157" s="51"/>
@@ -64043,7 +64087,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H158" s="340" t="s">
-        <x:v>2383</x:v>
+        <x:v>2389</x:v>
       </x:c>
       <x:c r="I158" s="51" t="s">
         <x:v>1160</x:v>
@@ -64282,7 +64326,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G170" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H170" s="292"/>
       <x:c r="I170" s="51"/>
@@ -64313,7 +64357,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H171" s="340" t="s">
-        <x:v>2384</x:v>
+        <x:v>2390</x:v>
       </x:c>
       <x:c r="I171" s="51" t="s">
         <x:v>1160</x:v>
@@ -64552,7 +64596,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G183" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H183" s="292"/>
       <x:c r="I183" s="51"/>
@@ -64822,7 +64866,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G196" s="292" t="s">
-        <x:v>2373</x:v>
+        <x:v>2379</x:v>
       </x:c>
       <x:c r="H196" s="340"/>
       <x:c r="I196" s="51"/>
@@ -64853,7 +64897,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H197" s="340" t="s">
-        <x:v>2385</x:v>
+        <x:v>2391</x:v>
       </x:c>
       <x:c r="I197" s="134" t="s">
         <x:v>1178</x:v>
@@ -65123,7 +65167,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H210" s="340" t="s">
-        <x:v>2386</x:v>
+        <x:v>2392</x:v>
       </x:c>
       <x:c r="I210" s="134" t="s">
         <x:v>1187</x:v>
@@ -65381,7 +65425,7 @@
         <x:v>1189</x:v>
       </x:c>
       <x:c r="D223" s="134" t="s">
-        <x:v>2387</x:v>
+        <x:v>2393</x:v>
       </x:c>
       <x:c r="E223" s="35" t="s">
         <x:v>1176</x:v>
@@ -65393,7 +65437,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H223" s="340" t="s">
-        <x:v>2388</x:v>
+        <x:v>2394</x:v>
       </x:c>
       <x:c r="I223" s="10" t="s">
         <x:v>1192</x:v>
@@ -65663,7 +65707,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H236" s="340" t="s">
-        <x:v>2389</x:v>
+        <x:v>2395</x:v>
       </x:c>
       <x:c r="I236" s="10" t="s">
         <x:v>1197</x:v>
@@ -65933,7 +65977,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H249" s="340" t="s">
-        <x:v>2390</x:v>
+        <x:v>2396</x:v>
       </x:c>
       <x:c r="I249" s="10" t="s">
         <x:v>1203</x:v>
@@ -66115,7 +66159,7 @@
         <x:v>1115</x:v>
       </x:c>
       <x:c r="H258" s="292" t="s">
-        <x:v>2391</x:v>
+        <x:v>2397</x:v>
       </x:c>
       <x:c r="I258" s="9"/>
       <x:c r="J258" s="9"/>
@@ -66461,7 +66505,7 @@
         <x:v>1212</x:v>
       </x:c>
       <x:c r="D275" s="35" t="s">
-        <x:v>2392</x:v>
+        <x:v>2398</x:v>
       </x:c>
       <x:c r="E275" s="35" t="s">
         <x:v>1214</x:v>
@@ -66470,10 +66514,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G275" s="297" t="s">
-        <x:v>2393</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="I275" s="10" t="s">
-        <x:v>2394</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="J275" s="10"/>
       <x:c r="K275" s="35"/>
@@ -66489,7 +66533,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G276" s="297" t="s">
-        <x:v>2395</x:v>
+        <x:v>2401</x:v>
       </x:c>
       <x:c r="I276" s="9"/>
       <x:c r="J276" s="9"/>
@@ -66506,10 +66550,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G277" s="297" t="s">
-        <x:v>2396</x:v>
+        <x:v>2402</x:v>
       </x:c>
       <x:c r="H277" s="297" t="s">
-        <x:v>2397</x:v>
+        <x:v>2403</x:v>
       </x:c>
       <x:c r="I277" s="9"/>
       <x:c r="J277" s="9"/>
@@ -66548,13 +66592,13 @@
         <x:v>1220</x:v>
       </x:c>
       <x:c r="E279" s="35" t="s">
-        <x:v>2398</x:v>
+        <x:v>2404</x:v>
       </x:c>
       <x:c r="F279" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G279" s="297" t="s">
-        <x:v>2393</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="I279" s="10" t="s">
         <x:v>1223</x:v>
@@ -66573,7 +66617,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G280" s="297" t="s">
-        <x:v>2399</x:v>
+        <x:v>2405</x:v>
       </x:c>
       <x:c r="H280" s="297" t="s">
         <x:v>1117</x:v>
@@ -66615,17 +66659,17 @@
         <x:v>1226</x:v>
       </x:c>
       <x:c r="E282" s="35" t="s">
-        <x:v>2400</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="F282" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G282" s="297" t="s">
-        <x:v>2393</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H282" s="297"/>
       <x:c r="I282" s="10" t="s">
-        <x:v>2401</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="J282" s="10"/>
       <x:c r="K282" s="35"/>
@@ -66641,7 +66685,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G283" s="297" t="s">
-        <x:v>2395</x:v>
+        <x:v>2401</x:v>
       </x:c>
       <x:c r="H283" s="297"/>
       <x:c r="I283" s="9"/>
@@ -66659,10 +66703,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G284" s="297" t="s">
-        <x:v>2402</x:v>
+        <x:v>2408</x:v>
       </x:c>
       <x:c r="H284" s="323" t="s">
-        <x:v>2403</x:v>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="I284" s="9"/>
       <x:c r="J284" s="9"/>
@@ -66701,17 +66745,17 @@
         <x:v>1233</x:v>
       </x:c>
       <x:c r="E286" s="35" t="s">
-        <x:v>2400</x:v>
+        <x:v>2406</x:v>
       </x:c>
       <x:c r="F286" s="35">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G286" s="297" t="s">
-        <x:v>2393</x:v>
+        <x:v>2399</x:v>
       </x:c>
       <x:c r="H286" s="297"/>
       <x:c r="I286" s="10" t="s">
-        <x:v>2401</x:v>
+        <x:v>2407</x:v>
       </x:c>
       <x:c r="J286" s="10"/>
       <x:c r="K286" s="35"/>
@@ -66727,7 +66771,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G287" s="297" t="s">
-        <x:v>2395</x:v>
+        <x:v>2401</x:v>
       </x:c>
       <x:c r="H287" s="297"/>
       <x:c r="I287" s="9"/>
@@ -66745,10 +66789,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G288" s="297" t="s">
-        <x:v>2404</x:v>
+        <x:v>2410</x:v>
       </x:c>
       <x:c r="H288" s="297" t="s">
-        <x:v>2405</x:v>
+        <x:v>2411</x:v>
       </x:c>
       <x:c r="I288" s="9"/>
       <x:c r="J288" s="9"/>
@@ -66796,7 +66840,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H290" s="340" t="s">
-        <x:v>2406</x:v>
+        <x:v>2412</x:v>
       </x:c>
       <x:c r="I290" s="51" t="s">
         <x:v>1102</x:v>
@@ -66875,7 +66919,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G294" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H294" s="312" t="s">
         <x:v>1117</x:v>
@@ -66895,7 +66939,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G295" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H295" s="312">
         <x:v>45758</x:v>
@@ -67015,7 +67059,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G301" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="H301" s="297"/>
       <x:c r="I301" s="51"/>
@@ -67125,7 +67169,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G306" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H306" s="312" t="s">
         <x:v>1117</x:v>
@@ -67145,7 +67189,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G307" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H307" s="312">
         <x:v>45758</x:v>
@@ -67265,7 +67309,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G313" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I313" s="51"/>
       <x:c r="J313" s="48"/>
@@ -67295,7 +67339,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H314" s="340" t="s">
-        <x:v>2410</x:v>
+        <x:v>2416</x:v>
       </x:c>
       <x:c r="I314" s="51" t="s">
         <x:v>1127</x:v>
@@ -67372,7 +67416,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G318" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H318" s="312" t="s">
         <x:v>1117</x:v>
@@ -67392,7 +67436,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G319" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H319" s="312">
         <x:v>45758</x:v>
@@ -67512,7 +67556,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G325" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I325" s="51"/>
       <x:c r="J325" s="48"/>
@@ -67542,7 +67586,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H326" s="340" t="s">
-        <x:v>2411</x:v>
+        <x:v>2417</x:v>
       </x:c>
       <x:c r="I326" s="51" t="s">
         <x:v>1130</x:v>
@@ -67619,7 +67663,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G330" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H330" s="312" t="s">
         <x:v>1117</x:v>
@@ -67639,7 +67683,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G331" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H331" s="312">
         <x:v>45758</x:v>
@@ -67759,7 +67803,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G337" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I337" s="51"/>
       <x:c r="J337" s="48"/>
@@ -67789,7 +67833,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H338" s="340" t="s">
-        <x:v>2412</x:v>
+        <x:v>2418</x:v>
       </x:c>
       <x:c r="I338" s="51" t="s">
         <x:v>1134</x:v>
@@ -67868,7 +67912,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G342" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H342" s="312"/>
       <x:c r="I342" s="51"/>
@@ -67886,7 +67930,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G343" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H343" s="312">
         <x:v>45758</x:v>
@@ -68006,7 +68050,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G349" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I349" s="51"/>
       <x:c r="J349" s="48"/>
@@ -68036,7 +68080,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H350" s="340" t="s">
-        <x:v>2412</x:v>
+        <x:v>2418</x:v>
       </x:c>
       <x:c r="I350" s="51" t="s">
         <x:v>1138</x:v>
@@ -68115,7 +68159,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G354" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H354" s="312" t="s">
         <x:v>1117</x:v>
@@ -68135,7 +68179,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G355" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H355" s="312"/>
       <x:c r="I355" s="51"/>
@@ -68253,7 +68297,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G361" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I361" s="51"/>
       <x:c r="J361" s="48"/>
@@ -68271,7 +68315,7 @@
         <x:v>1254</x:v>
       </x:c>
       <x:c r="D362" s="51" t="s">
-        <x:v>2413</x:v>
+        <x:v>2419</x:v>
       </x:c>
       <x:c r="E362" s="51" t="s">
         <x:v>1099</x:v>
@@ -68283,10 +68327,10 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H362" s="340" t="s">
-        <x:v>2414</x:v>
+        <x:v>2420</x:v>
       </x:c>
       <x:c r="I362" s="51" t="s">
-        <x:v>2415</x:v>
+        <x:v>2421</x:v>
       </x:c>
       <x:c r="J362" s="50"/>
       <x:c r="K362" s="51"/>
@@ -68360,7 +68404,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G366" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H366" s="312" t="s">
         <x:v>1117</x:v>
@@ -68380,7 +68424,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G367" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H367" s="312">
         <x:v>49410</x:v>
@@ -68498,7 +68542,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G373" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="H373" s="292"/>
       <x:c r="I373" s="51"/>
@@ -68529,7 +68573,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H374" s="340" t="s">
-        <x:v>2416</x:v>
+        <x:v>2422</x:v>
       </x:c>
       <x:c r="I374" s="51" t="s">
         <x:v>1145</x:v>
@@ -68608,7 +68652,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G378" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H378" s="312" t="s">
         <x:v>1117</x:v>
@@ -68628,7 +68672,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G379" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H379" s="312">
         <x:v>45758</x:v>
@@ -68746,7 +68790,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G385" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I385" s="51"/>
       <x:c r="J385" s="48"/>
@@ -68776,7 +68820,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H386" s="340" t="s">
-        <x:v>2417</x:v>
+        <x:v>2423</x:v>
       </x:c>
       <x:c r="I386" s="51" t="s">
         <x:v>1149</x:v>
@@ -68855,7 +68899,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G390" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H390" s="312" t="s">
         <x:v>1117</x:v>
@@ -68875,7 +68919,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G391" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H391" s="312">
         <x:v>45758</x:v>
@@ -68993,7 +69037,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G397" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I397" s="51"/>
       <x:c r="J397" s="48"/>
@@ -69023,7 +69067,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H398" s="340" t="s">
-        <x:v>2418</x:v>
+        <x:v>2424</x:v>
       </x:c>
       <x:c r="I398" s="51" t="s">
         <x:v>1149</x:v>
@@ -69100,7 +69144,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G402" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H402" s="312" t="s">
         <x:v>1117</x:v>
@@ -69120,7 +69164,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G403" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H403" s="312">
         <x:v>45758</x:v>
@@ -69240,7 +69284,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G409" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I409" s="51"/>
       <x:c r="J409" s="48"/>
@@ -69270,7 +69314,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H410" s="340" t="s">
-        <x:v>2419</x:v>
+        <x:v>2425</x:v>
       </x:c>
       <x:c r="I410" s="51" t="s">
         <x:v>1160</x:v>
@@ -69349,7 +69393,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G414" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H414" s="312" t="s">
         <x:v>1117</x:v>
@@ -69369,7 +69413,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G415" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H415" s="312">
         <x:v>45758</x:v>
@@ -69487,7 +69531,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G421" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I421" s="51"/>
       <x:c r="J421" s="48"/>
@@ -69505,7 +69549,7 @@
         <x:v>1260</x:v>
       </x:c>
       <x:c r="D422" s="51" t="s">
-        <x:v>2420</x:v>
+        <x:v>2426</x:v>
       </x:c>
       <x:c r="E422" s="51" t="s">
         <x:v>1099</x:v>
@@ -69517,10 +69561,10 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H422" s="340" t="s">
-        <x:v>2421</x:v>
+        <x:v>2427</x:v>
       </x:c>
       <x:c r="I422" s="51" t="s">
-        <x:v>2422</x:v>
+        <x:v>2428</x:v>
       </x:c>
       <x:c r="J422" s="50"/>
       <x:c r="K422" s="51"/>
@@ -69596,7 +69640,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G426" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H426" s="312" t="s">
         <x:v>1117</x:v>
@@ -69616,7 +69660,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G427" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H427" s="312">
         <x:v>45758</x:v>
@@ -69736,7 +69780,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G433" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I433" s="51"/>
       <x:c r="J433" s="48"/>
@@ -69766,7 +69810,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H434" s="340" t="s">
-        <x:v>2423</x:v>
+        <x:v>2429</x:v>
       </x:c>
       <x:c r="I434" s="51" t="s">
         <x:v>1160</x:v>
@@ -69845,7 +69889,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G438" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H438" s="312" t="s">
         <x:v>1117</x:v>
@@ -69865,7 +69909,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G439" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H439" s="312">
         <x:v>45758</x:v>
@@ -69983,7 +70027,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G445" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I445" s="51"/>
       <x:c r="J445" s="48"/>
@@ -70013,7 +70057,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="H446" s="340" t="s">
-        <x:v>2424</x:v>
+        <x:v>2430</x:v>
       </x:c>
       <x:c r="I446" s="51" t="s">
         <x:v>1160</x:v>
@@ -70092,7 +70136,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G450" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H450" s="312" t="s">
         <x:v>1117</x:v>
@@ -70112,7 +70156,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G451" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H451" s="312">
         <x:v>45758</x:v>
@@ -70230,7 +70274,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G457" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="I457" s="51"/>
       <x:c r="J457" s="48"/>
@@ -70339,7 +70383,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G462" s="292" t="s">
-        <x:v>2407</x:v>
+        <x:v>2413</x:v>
       </x:c>
       <x:c r="H462" s="340" t="s">
         <x:v>437</x:v>
@@ -70359,7 +70403,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G463" s="292" t="s">
-        <x:v>2408</x:v>
+        <x:v>2414</x:v>
       </x:c>
       <x:c r="H463" s="340" t="s">
         <x:v>437</x:v>
@@ -70479,7 +70523,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G469" s="288" t="s">
-        <x:v>2409</x:v>
+        <x:v>2415</x:v>
       </x:c>
       <x:c r="H469" s="340" t="s">
         <x:v>437</x:v>
@@ -70813,7 +70857,7 @@
     <x:mergeCell ref="K458:K469"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="H284" r:id="rId217"/>
+    <x:hyperlink ref="H284" r:id="rId172"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -70837,13 +70881,13 @@
   <x:sheetData>
     <x:row r="2" spans="1:7">
       <x:c r="A2" s="196" t="s">
-        <x:v>2425</x:v>
+        <x:v>2431</x:v>
       </x:c>
       <x:c r="D2" s="196" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="G2" s="196" t="s">
-        <x:v>2426</x:v>
+        <x:v>2432</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
@@ -70851,7 +70895,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>2427</x:v>
+        <x:v>2433</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
         <x:v>244</x:v>
@@ -70862,7 +70906,7 @@
         <x:v>245</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>2428</x:v>
+        <x:v>2434</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
         <x:v>234</x:v>
@@ -70870,10 +70914,10 @@
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="A5" s="0" t="s">
-        <x:v>2429</x:v>
+        <x:v>2435</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>2430</x:v>
+        <x:v>2436</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
         <x:v>239</x:v>

</xml_diff>

<commit_message>
Complete test cases TC_TICKET_01, TC_TICKET_02, TC_TICKET_06, TC_TICKET_08
</commit_message>
<xml_diff>
--- a/sqa-testing-report/Data/DataTest.xlsx
+++ b/sqa-testing-report/Data/DataTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\sqa-testing-report\sqa-testing-report\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DB785FC-3576-4D78-B0B6-C7E252A678DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39365BB6-7F52-4125-866A-1C18EBEA7970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="664" activeTab="5" xr2:uid="{DC4DB269-603C-4B5B-A498-B166C8A18B92}"/>
   </bookViews>
@@ -164,7 +164,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7172" uniqueCount="2600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7190" uniqueCount="2612">
   <si>
     <t>GUI &amp; FUNCTIONAL TEST CASES</t>
   </si>
@@ -8869,21 +8869,30 @@
     <t>Hiển thị đúng: Tên phim, Rạp, Phòng chiếu, Suất chiếu, Danh sách ghế, Mã vé, Tổng tiền.</t>
   </si>
   <si>
+    <t>Hiển thị đủ thông tin: Phim, Rạp, Phòng, Suất, Ghế, Tổng tiền.</t>
+  </si>
+  <si>
     <t>Quan sát mã QR Code trên vé.</t>
   </si>
   <si>
     <t>Mã QR hiển thị rõ nét ở trung tâm vé, không bị mất nét hay biến dạng.</t>
   </si>
   <si>
+    <t>Mã QR hiển thị rõ nét ở trung tâm vé.</t>
+  </si>
+  <si>
     <t>Dùng thiết bị quét mã QR chuyên dụng (hoặc App quét).</t>
   </si>
   <si>
-    <t>Mã vé: 1224</t>
+    <t>Mã vé: 1280</t>
   </si>
   <si>
     <t>Kết quả quét trả về đúng thông tin hoặc mã định danh trùng khớp với Mã vé.</t>
   </si>
   <si>
+    <t>Kết quả quét QR trả về đúng định danh mã vé (1281).</t>
+  </si>
+  <si>
     <t>Kiểm tra tính năng xem lại vé điện tử từ Lịch sử giao dịch.</t>
   </si>
   <si>
@@ -8896,22 +8905,34 @@
     <t>Hệ thống chuyển hướng vào trang Profile (Account/Profile).</t>
   </si>
   <si>
+    <t>Đã vào trang Profile.</t>
+  </si>
+  <si>
     <t>Cuộn xuống mục "Lịch sử giao dịch gần đây" và nhấn nút "Chi tiết" của vé mới nhất.</t>
   </si>
   <si>
     <t>Hiển thị Popup vé điện tử với đầy đủ thông tin phim, rạp, suất chiếu, số ghế.</t>
   </si>
   <si>
+    <t>Mở Popup vé thành công.</t>
+  </si>
+  <si>
     <t>Kiểm tra mã QR và Mã vé hiển thị trên Popup.</t>
   </si>
   <si>
     <t>Mã vé khớp với giao dịch; Mã QR hiển thị rõ ràng, không bị lỗi UI.</t>
   </si>
   <si>
+    <t>Mã vé khớp với giao dịch; Mã QR hiển thị rõ ràng (Mã vé: 1281).</t>
+  </si>
+  <si>
     <t>Thực hiện quét mã QR bằng thiết bị quét.</t>
   </si>
   <si>
-    <t>Kết quả quét trả về thông tin định danh chính xác của vé 1224.</t>
+    <t>Kết quả quét trả về thông tin định danh chính xác của vé 1280.</t>
+  </si>
+  <si>
+    <t>Kết quả quét trả về thông tin định danh chính xác của vé 1281.</t>
   </si>
   <si>
     <t>Kiểm tra hiển thị danh sách vé trong Lịch sử giao dịch.</t>
@@ -8926,10 +8947,16 @@
     <t>Hiển thị mục "Lịch sử giao dịch gần đây".</t>
   </si>
   <si>
+    <t>Đang ở trang Profile.</t>
+  </si>
+  <si>
     <t>Quan sát thứ tự sắp xếp của các vé trong danh sách.</t>
   </si>
   <si>
-    <t>Vé mới nhất (Mã 1224) hiển thị ở vị trí đầu tiên (Sắp xếp giảm dần theo thời gian).</t>
+    <t>Vé mới nhất (Mã 1280) hiển thị ở vị trí đầu tiên (Sắp xếp giảm dần theo thời gian).</t>
+  </si>
+  <si>
+    <t>Danh sách vé hiển thị thành công.</t>
   </si>
   <si>
     <t>Kiểm tra các thông tin tóm tắt hiển thị trên mỗi dòng vé.</t>
@@ -8938,12 +8965,18 @@
     <t>Hiển thị đủ: Ảnh phim, Tên phim, Rạp, Phòng chiếu, Suất chiếu.</t>
   </si>
   <si>
+    <t>Hiển thị đủ thông tin vé.</t>
+  </si>
+  <si>
     <t>Nhấn nút "Thu gọn" / "Xem thêm" ở cuối danh sách.</t>
   </si>
   <si>
     <t>Danh sách mở rộng hoặc thu hẹp số lượng vé hiển thị chính xác.</t>
   </si>
   <si>
+    <t>Nút Xem thêm/Thu gọn hoạt động tốt.</t>
+  </si>
+  <si>
     <t>Kiểm tra thứ tự hiển thị của danh sách lịch sử vé.</t>
   </si>
   <si>
@@ -8956,13 +8989,16 @@
     <t>Quan sát vị trí của vé vừa đặt thành công.</t>
   </si>
   <si>
-    <t>Vé mới nhất (1224) hiển thị ở vị trí cuối cùng của danh sách.</t>
+    <t>Vé mới nhất (1280) hiển thị ở vị trí cuối cùng của danh sách.</t>
+  </si>
+  <si>
+    <t>Vé mới nhất đang nằm cuối danh sách.</t>
   </si>
   <si>
     <t>Cuộn xuống cuối danh sách và nhấn nút "Chi tiết" của vé đó.</t>
   </si>
   <si>
-    <t>Popup hiển thị đúng thông tin chi tiết của vé 1224.</t>
+    <t>Popup hiển thị đúng thông tin chi tiết của vé 1280.</t>
   </si>
   <si>
     <t>Hệ thống báo lỗi "Tên đăng nhập hoặc mật khẩu không đúng".</t>
@@ -57875,7 +57911,7 @@
       <c r="K32" s="136"/>
       <c r="L32" s="136"/>
     </row>
-    <row r="33" spans="1:12" ht="52.8" customHeight="1">
+    <row r="33" spans="1:12" ht="84" customHeight="1">
       <c r="A33" s="138">
         <v>13</v>
       </c>
@@ -57901,11 +57937,15 @@
       <c r="I33" s="285" t="s">
         <v>2353</v>
       </c>
-      <c r="J33" s="166"/>
-      <c r="K33" s="136"/>
+      <c r="J33" s="166" t="s">
+        <v>2354</v>
+      </c>
+      <c r="K33" s="136" t="s">
+        <v>2008</v>
+      </c>
       <c r="L33" s="136"/>
     </row>
-    <row r="34" spans="1:12" ht="39.6" customHeight="1">
+    <row r="34" spans="1:12" ht="49.8" customHeight="1">
       <c r="A34" s="138"/>
       <c r="B34" s="138"/>
       <c r="C34" s="138"/>
@@ -57915,17 +57955,19 @@
         <v>2</v>
       </c>
       <c r="G34" s="285" t="s">
-        <v>2354</v>
+        <v>2355</v>
       </c>
       <c r="H34" s="178"/>
       <c r="I34" s="285" t="s">
-        <v>2355</v>
-      </c>
-      <c r="J34" s="166"/>
+        <v>2356</v>
+      </c>
+      <c r="J34" s="166" t="s">
+        <v>2357</v>
+      </c>
       <c r="K34" s="136"/>
       <c r="L34" s="136"/>
     </row>
-    <row r="35" spans="1:12" ht="52.8" customHeight="1">
+    <row r="35" spans="1:12" ht="65.400000000000006" customHeight="1">
       <c r="A35" s="138"/>
       <c r="B35" s="138"/>
       <c r="C35" s="138"/>
@@ -57935,19 +57977,21 @@
         <v>3</v>
       </c>
       <c r="G35" s="285" t="s">
-        <v>2356</v>
+        <v>2358</v>
       </c>
       <c r="H35" s="178" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="I35" s="285" t="s">
-        <v>2358</v>
-      </c>
-      <c r="J35" s="166"/>
+        <v>2360</v>
+      </c>
+      <c r="J35" s="166" t="s">
+        <v>2361</v>
+      </c>
       <c r="K35" s="136"/>
       <c r="L35" s="136"/>
     </row>
-    <row r="36" spans="1:12" ht="39.6" customHeight="1">
+    <row r="36" spans="1:12" ht="51" customHeight="1">
       <c r="A36" s="138">
         <v>14</v>
       </c>
@@ -57958,23 +58002,27 @@
         <v>814</v>
       </c>
       <c r="D36" s="138" t="s">
-        <v>2359</v>
+        <v>2362</v>
       </c>
       <c r="E36" s="138" t="s">
-        <v>2360</v>
+        <v>2363</v>
       </c>
       <c r="F36" s="178">
         <v>1</v>
       </c>
       <c r="G36" s="285" t="s">
-        <v>2361</v>
+        <v>2364</v>
       </c>
       <c r="H36" s="178"/>
       <c r="I36" s="285" t="s">
-        <v>2362</v>
-      </c>
-      <c r="J36" s="166"/>
-      <c r="K36" s="136"/>
+        <v>2365</v>
+      </c>
+      <c r="J36" s="166" t="s">
+        <v>2366</v>
+      </c>
+      <c r="K36" s="136" t="s">
+        <v>2008</v>
+      </c>
       <c r="L36" s="136"/>
     </row>
     <row r="37" spans="1:12" ht="69.599999999999994" customHeight="1">
@@ -57987,17 +58035,19 @@
         <v>2</v>
       </c>
       <c r="G37" s="285" t="s">
-        <v>2363</v>
+        <v>2367</v>
       </c>
       <c r="H37" s="178"/>
       <c r="I37" s="285" t="s">
-        <v>2364</v>
-      </c>
-      <c r="J37" s="166"/>
+        <v>2368</v>
+      </c>
+      <c r="J37" s="166" t="s">
+        <v>2369</v>
+      </c>
       <c r="K37" s="136"/>
       <c r="L37" s="136"/>
     </row>
-    <row r="38" spans="1:12" ht="48" customHeight="1">
+    <row r="38" spans="1:12" ht="73.2" customHeight="1">
       <c r="A38" s="138"/>
       <c r="B38" s="138"/>
       <c r="C38" s="138"/>
@@ -58007,19 +58057,21 @@
         <v>3</v>
       </c>
       <c r="G38" s="285" t="s">
-        <v>2365</v>
+        <v>2370</v>
       </c>
       <c r="H38" s="178" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="I38" s="285" t="s">
-        <v>2366</v>
-      </c>
-      <c r="J38" s="166"/>
+        <v>2371</v>
+      </c>
+      <c r="J38" s="166" t="s">
+        <v>2372</v>
+      </c>
       <c r="K38" s="136"/>
       <c r="L38" s="136"/>
     </row>
-    <row r="39" spans="1:12" ht="39.6" customHeight="1">
+    <row r="39" spans="1:12" ht="79.2" customHeight="1">
       <c r="A39" s="138"/>
       <c r="B39" s="138"/>
       <c r="C39" s="138"/>
@@ -58029,13 +58081,15 @@
         <v>4</v>
       </c>
       <c r="G39" s="285" t="s">
-        <v>2367</v>
+        <v>2373</v>
       </c>
       <c r="H39" s="178"/>
       <c r="I39" s="285" t="s">
-        <v>2368</v>
-      </c>
-      <c r="J39" s="166"/>
+        <v>2374</v>
+      </c>
+      <c r="J39" s="166" t="s">
+        <v>2375</v>
+      </c>
       <c r="K39" s="136"/>
       <c r="L39" s="136"/>
     </row>
@@ -58050,23 +58104,27 @@
         <v>824</v>
       </c>
       <c r="D40" s="138" t="s">
-        <v>2369</v>
+        <v>2376</v>
       </c>
       <c r="E40" s="138" t="s">
-        <v>2370</v>
+        <v>2377</v>
       </c>
       <c r="F40" s="178">
         <v>1</v>
       </c>
       <c r="G40" s="285" t="s">
-        <v>2371</v>
+        <v>2378</v>
       </c>
       <c r="H40" s="178"/>
       <c r="I40" s="285" t="s">
-        <v>2372</v>
-      </c>
-      <c r="J40" s="166"/>
-      <c r="K40" s="136"/>
+        <v>2379</v>
+      </c>
+      <c r="J40" s="166" t="s">
+        <v>2380</v>
+      </c>
+      <c r="K40" s="136" t="s">
+        <v>2008</v>
+      </c>
       <c r="L40" s="136"/>
     </row>
     <row r="41" spans="1:12" ht="52.8" customHeight="1">
@@ -58079,13 +58137,15 @@
         <v>2</v>
       </c>
       <c r="G41" s="285" t="s">
-        <v>2373</v>
+        <v>2381</v>
       </c>
       <c r="H41" s="178"/>
       <c r="I41" s="285" t="s">
-        <v>2374</v>
-      </c>
-      <c r="J41" s="166"/>
+        <v>2382</v>
+      </c>
+      <c r="J41" s="166" t="s">
+        <v>2383</v>
+      </c>
       <c r="K41" s="136"/>
       <c r="L41" s="136"/>
     </row>
@@ -58099,13 +58159,15 @@
         <v>3</v>
       </c>
       <c r="G42" s="285" t="s">
-        <v>2375</v>
+        <v>2384</v>
       </c>
       <c r="H42" s="178"/>
       <c r="I42" s="285" t="s">
-        <v>2376</v>
-      </c>
-      <c r="J42" s="166"/>
+        <v>2385</v>
+      </c>
+      <c r="J42" s="166" t="s">
+        <v>2386</v>
+      </c>
       <c r="K42" s="136"/>
       <c r="L42" s="136"/>
     </row>
@@ -58119,13 +58181,15 @@
         <v>4</v>
       </c>
       <c r="G43" s="285" t="s">
-        <v>2377</v>
+        <v>2387</v>
       </c>
       <c r="H43" s="178"/>
       <c r="I43" s="285" t="s">
-        <v>2378</v>
-      </c>
-      <c r="J43" s="166"/>
+        <v>2388</v>
+      </c>
+      <c r="J43" s="166" t="s">
+        <v>2389</v>
+      </c>
       <c r="K43" s="136"/>
       <c r="L43" s="136"/>
     </row>
@@ -58140,26 +58204,30 @@
         <v>835</v>
       </c>
       <c r="D44" s="138" t="s">
-        <v>2379</v>
+        <v>2390</v>
       </c>
       <c r="E44" s="138" t="s">
-        <v>2380</v>
+        <v>2391</v>
       </c>
       <c r="F44" s="178">
         <v>1</v>
       </c>
       <c r="G44" s="285" t="s">
-        <v>2371</v>
+        <v>2378</v>
       </c>
       <c r="H44" s="178"/>
       <c r="I44" s="285" t="s">
-        <v>2381</v>
-      </c>
-      <c r="J44" s="166"/>
-      <c r="K44" s="136"/>
+        <v>2392</v>
+      </c>
+      <c r="J44" s="166" t="s">
+        <v>2380</v>
+      </c>
+      <c r="K44" s="136" t="s">
+        <v>2008</v>
+      </c>
       <c r="L44" s="136"/>
     </row>
-    <row r="45" spans="1:12" ht="39.6" customHeight="1">
+    <row r="45" spans="1:12" ht="52.2" customHeight="1">
       <c r="A45" s="138"/>
       <c r="B45" s="138"/>
       <c r="C45" s="138"/>
@@ -58169,19 +58237,21 @@
         <v>2</v>
       </c>
       <c r="G45" s="285" t="s">
-        <v>2382</v>
+        <v>2393</v>
       </c>
       <c r="H45" s="178" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="I45" s="285" t="s">
-        <v>2383</v>
-      </c>
-      <c r="J45" s="166"/>
+        <v>2394</v>
+      </c>
+      <c r="J45" s="166" t="s">
+        <v>2395</v>
+      </c>
       <c r="K45" s="136"/>
       <c r="L45" s="136"/>
     </row>
-    <row r="46" spans="1:12" ht="40.200000000000003" customHeight="1">
+    <row r="46" spans="1:12" ht="52.8" customHeight="1">
       <c r="A46" s="138"/>
       <c r="B46" s="138"/>
       <c r="C46" s="138"/>
@@ -58191,13 +58261,15 @@
         <v>3</v>
       </c>
       <c r="G46" s="285" t="s">
-        <v>2384</v>
+        <v>2396</v>
       </c>
       <c r="H46" s="178"/>
       <c r="I46" s="285" t="s">
-        <v>2385</v>
-      </c>
-      <c r="J46" s="166"/>
+        <v>2397</v>
+      </c>
+      <c r="J46" s="166" t="s">
+        <v>2395</v>
+      </c>
       <c r="K46" s="136"/>
       <c r="L46" s="136"/>
     </row>
@@ -58297,7 +58369,7 @@
         <v>2029</v>
       </c>
       <c r="I50" s="135" t="s">
-        <v>2386</v>
+        <v>2398</v>
       </c>
       <c r="J50" s="135"/>
       <c r="K50" s="136"/>
@@ -58367,7 +58439,7 @@
         <v>1000</v>
       </c>
       <c r="I53" s="135" t="s">
-        <v>2387</v>
+        <v>2399</v>
       </c>
       <c r="J53" s="135"/>
       <c r="K53" s="136"/>
@@ -58386,7 +58458,7 @@
         <v>444</v>
       </c>
       <c r="H54" s="140" t="s">
-        <v>2388</v>
+        <v>2400</v>
       </c>
       <c r="I54" s="135"/>
       <c r="J54" s="135"/>
@@ -58505,7 +58577,7 @@
         <v>422</v>
       </c>
       <c r="I59" s="135" t="s">
-        <v>2389</v>
+        <v>2401</v>
       </c>
       <c r="J59" s="135"/>
       <c r="K59" s="136"/>
@@ -58803,7 +58875,7 @@
         <v>1037</v>
       </c>
       <c r="I72" s="135" t="s">
-        <v>2390</v>
+        <v>2402</v>
       </c>
       <c r="J72" s="135"/>
       <c r="K72" s="136"/>
@@ -59499,19 +59571,19 @@
         <v>843</v>
       </c>
       <c r="E104" s="138" t="s">
-        <v>2391</v>
+        <v>2403</v>
       </c>
       <c r="F104" s="178">
         <v>1</v>
       </c>
       <c r="G104" s="285" t="s">
-        <v>2392</v>
+        <v>2404</v>
       </c>
       <c r="H104" s="178" t="s">
-        <v>2393</v>
+        <v>2405</v>
       </c>
       <c r="I104" s="285" t="s">
-        <v>2394</v>
+        <v>2406</v>
       </c>
       <c r="J104" s="166"/>
       <c r="K104" s="133"/>
@@ -59527,11 +59599,11 @@
         <v>2</v>
       </c>
       <c r="G105" s="285" t="s">
-        <v>2395</v>
+        <v>2407</v>
       </c>
       <c r="H105" s="178"/>
       <c r="I105" s="285" t="s">
-        <v>2396</v>
+        <v>2408</v>
       </c>
       <c r="J105" s="166"/>
       <c r="K105" s="133"/>
@@ -59547,13 +59619,13 @@
         <v>3</v>
       </c>
       <c r="G106" s="285" t="s">
-        <v>2397</v>
+        <v>2409</v>
       </c>
       <c r="H106" s="178" t="s">
-        <v>2398</v>
+        <v>2410</v>
       </c>
       <c r="I106" s="285" t="s">
-        <v>2399</v>
+        <v>2411</v>
       </c>
       <c r="J106" s="166"/>
       <c r="K106" s="133"/>
@@ -59569,11 +59641,11 @@
         <v>4</v>
       </c>
       <c r="G107" s="285" t="s">
-        <v>2400</v>
+        <v>2412</v>
       </c>
       <c r="H107" s="178"/>
       <c r="I107" s="285" t="s">
-        <v>2401</v>
+        <v>2413</v>
       </c>
       <c r="J107" s="166"/>
       <c r="K107" s="133"/>
@@ -59593,19 +59665,19 @@
         <v>854</v>
       </c>
       <c r="E108" s="138" t="s">
-        <v>2402</v>
+        <v>2414</v>
       </c>
       <c r="F108" s="178">
         <v>1</v>
       </c>
       <c r="G108" s="285" t="s">
-        <v>2403</v>
+        <v>2415</v>
       </c>
       <c r="H108" s="178" t="s">
-        <v>2404</v>
+        <v>2416</v>
       </c>
       <c r="I108" s="285" t="s">
-        <v>2405</v>
+        <v>2417</v>
       </c>
       <c r="J108" s="166"/>
       <c r="K108" s="133"/>
@@ -59621,11 +59693,11 @@
         <v>2</v>
       </c>
       <c r="G109" s="285" t="s">
-        <v>2395</v>
+        <v>2407</v>
       </c>
       <c r="H109" s="178"/>
       <c r="I109" s="285" t="s">
-        <v>2406</v>
+        <v>2418</v>
       </c>
       <c r="J109" s="166"/>
       <c r="K109" s="133"/>
@@ -59641,13 +59713,13 @@
         <v>3</v>
       </c>
       <c r="G110" s="285" t="s">
-        <v>2407</v>
+        <v>2419</v>
       </c>
       <c r="H110" s="178" t="s">
-        <v>2408</v>
+        <v>2420</v>
       </c>
       <c r="I110" s="285" t="s">
-        <v>2409</v>
+        <v>2421</v>
       </c>
       <c r="J110" s="166"/>
       <c r="K110" s="133"/>
@@ -59663,11 +59735,11 @@
         <v>4</v>
       </c>
       <c r="G111" s="285" t="s">
-        <v>2410</v>
+        <v>2422</v>
       </c>
       <c r="H111" s="178"/>
       <c r="I111" s="285" t="s">
-        <v>2411</v>
+        <v>2423</v>
       </c>
       <c r="J111" s="166"/>
       <c r="K111" s="133"/>
@@ -59684,7 +59756,7 @@
         <v>863</v>
       </c>
       <c r="D112" s="133" t="s">
-        <v>2412</v>
+        <v>2424</v>
       </c>
       <c r="E112" s="133" t="s">
         <v>865</v>
@@ -59693,7 +59765,7 @@
         <v>1</v>
       </c>
       <c r="G112" s="166" t="s">
-        <v>2413</v>
+        <v>2425</v>
       </c>
       <c r="H112" s="175"/>
       <c r="I112" s="166" t="s">
@@ -59713,7 +59785,7 @@
         <v>2</v>
       </c>
       <c r="G113" s="166" t="s">
-        <v>2414</v>
+        <v>2426</v>
       </c>
       <c r="H113" s="175"/>
       <c r="I113" s="166" t="s">
@@ -59733,10 +59805,10 @@
         <v>3</v>
       </c>
       <c r="G114" s="166" t="s">
-        <v>2415</v>
+        <v>2427</v>
       </c>
       <c r="H114" s="175" t="s">
-        <v>2416</v>
+        <v>2428</v>
       </c>
       <c r="I114" s="166"/>
       <c r="J114" s="133"/>
@@ -59753,10 +59825,10 @@
         <v>4</v>
       </c>
       <c r="G115" s="166" t="s">
-        <v>2417</v>
+        <v>2429</v>
       </c>
       <c r="H115" s="175" t="s">
-        <v>2418</v>
+        <v>2430</v>
       </c>
       <c r="I115" s="166"/>
       <c r="J115" s="133"/>
@@ -59791,7 +59863,7 @@
         <v>6</v>
       </c>
       <c r="G117" s="166" t="s">
-        <v>2419</v>
+        <v>2431</v>
       </c>
       <c r="H117" s="175" t="s">
         <v>877</v>
@@ -59811,7 +59883,7 @@
         <v>7</v>
       </c>
       <c r="G118" s="166" t="s">
-        <v>2420</v>
+        <v>2432</v>
       </c>
       <c r="H118" s="247">
         <v>0.375</v>
@@ -59831,7 +59903,7 @@
         <v>8</v>
       </c>
       <c r="G119" s="166" t="s">
-        <v>2421</v>
+        <v>2433</v>
       </c>
       <c r="H119" s="175">
         <v>100000</v>
@@ -59851,7 +59923,7 @@
         <v>9</v>
       </c>
       <c r="G120" s="166" t="s">
-        <v>2422</v>
+        <v>2434</v>
       </c>
       <c r="H120" s="175">
         <v>1</v>
@@ -59871,7 +59943,7 @@
         <v>10</v>
       </c>
       <c r="G121" s="166" t="s">
-        <v>2423</v>
+        <v>2435</v>
       </c>
       <c r="H121" s="175"/>
       <c r="I121" s="166" t="s">
@@ -59892,7 +59964,7 @@
         <v>884</v>
       </c>
       <c r="D122" s="133" t="s">
-        <v>2424</v>
+        <v>2436</v>
       </c>
       <c r="E122" s="133" t="s">
         <v>886</v>
@@ -59901,7 +59973,7 @@
         <v>1</v>
       </c>
       <c r="G122" s="166" t="s">
-        <v>2425</v>
+        <v>2437</v>
       </c>
       <c r="H122" s="175"/>
       <c r="I122" s="133" t="s">
@@ -59921,7 +59993,7 @@
         <v>2</v>
       </c>
       <c r="G123" s="166" t="s">
-        <v>2426</v>
+        <v>2438</v>
       </c>
       <c r="H123" s="175"/>
       <c r="I123" s="133"/>
@@ -59939,10 +60011,10 @@
         <v>3</v>
       </c>
       <c r="G124" s="166" t="s">
-        <v>2427</v>
+        <v>2439</v>
       </c>
       <c r="H124" s="175" t="s">
-        <v>2428</v>
+        <v>2440</v>
       </c>
       <c r="I124" s="133"/>
       <c r="J124" s="133"/>
@@ -59959,10 +60031,10 @@
         <v>4</v>
       </c>
       <c r="G125" s="166" t="s">
-        <v>2429</v>
+        <v>2441</v>
       </c>
       <c r="H125" s="175" t="s">
-        <v>2430</v>
+        <v>2442</v>
       </c>
       <c r="I125" s="133"/>
       <c r="J125" s="133"/>
@@ -59979,7 +60051,7 @@
         <v>5</v>
       </c>
       <c r="G126" s="166" t="s">
-        <v>2431</v>
+        <v>2443</v>
       </c>
       <c r="H126" s="175" t="s">
         <v>877</v>
@@ -60017,7 +60089,7 @@
         <v>8</v>
       </c>
       <c r="G128" s="166" t="s">
-        <v>2432</v>
+        <v>2444</v>
       </c>
       <c r="H128" s="175">
         <v>100000</v>
@@ -60037,7 +60109,7 @@
         <v>9</v>
       </c>
       <c r="G129" s="166" t="s">
-        <v>2433</v>
+        <v>2445</v>
       </c>
       <c r="H129" s="175">
         <v>1</v>
@@ -60057,7 +60129,7 @@
         <v>10</v>
       </c>
       <c r="G130" s="166" t="s">
-        <v>2434</v>
+        <v>2446</v>
       </c>
       <c r="H130" s="175"/>
       <c r="I130" s="133"/>
@@ -60076,7 +60148,7 @@
         <v>900</v>
       </c>
       <c r="D131" s="133" t="s">
-        <v>2435</v>
+        <v>2447</v>
       </c>
       <c r="E131" s="133" t="s">
         <v>886</v>
@@ -60085,7 +60157,7 @@
         <v>1</v>
       </c>
       <c r="G131" s="166" t="s">
-        <v>2436</v>
+        <v>2448</v>
       </c>
       <c r="H131" s="175"/>
       <c r="I131" s="133" t="s">
@@ -60105,7 +60177,7 @@
         <v>2</v>
       </c>
       <c r="G132" s="166" t="s">
-        <v>2437</v>
+        <v>2449</v>
       </c>
       <c r="H132" s="175"/>
       <c r="I132" s="133"/>
@@ -60123,7 +60195,7 @@
         <v>3</v>
       </c>
       <c r="G133" s="166" t="s">
-        <v>2438</v>
+        <v>2450</v>
       </c>
       <c r="H133" s="175" t="s">
         <v>891</v>
@@ -60201,7 +60273,7 @@
         <v>7</v>
       </c>
       <c r="G137" s="166" t="s">
-        <v>2439</v>
+        <v>2451</v>
       </c>
       <c r="H137" s="175">
         <f>1</f>
@@ -60222,7 +60294,7 @@
         <v>8</v>
       </c>
       <c r="G138" s="166" t="s">
-        <v>2440</v>
+        <v>2452</v>
       </c>
       <c r="H138" s="175"/>
       <c r="I138" s="133"/>
@@ -60241,7 +60313,7 @@
         <v>911</v>
       </c>
       <c r="D139" s="133" t="s">
-        <v>2441</v>
+        <v>2453</v>
       </c>
       <c r="E139" s="133" t="s">
         <v>886</v>
@@ -60250,7 +60322,7 @@
         <v>1</v>
       </c>
       <c r="G139" s="166" t="s">
-        <v>2442</v>
+        <v>2454</v>
       </c>
       <c r="H139" s="175"/>
       <c r="I139" s="133" t="s">
@@ -60270,7 +60342,7 @@
         <v>2</v>
       </c>
       <c r="G140" s="166" t="s">
-        <v>2443</v>
+        <v>2455</v>
       </c>
       <c r="H140" s="175"/>
       <c r="I140" s="133"/>
@@ -60288,7 +60360,7 @@
         <v>3</v>
       </c>
       <c r="G141" s="166" t="s">
-        <v>2444</v>
+        <v>2456</v>
       </c>
       <c r="H141" s="175" t="s">
         <v>891</v>
@@ -60387,7 +60459,7 @@
         <v>8</v>
       </c>
       <c r="G146" s="166" t="s">
-        <v>2445</v>
+        <v>2457</v>
       </c>
       <c r="H146" s="175"/>
       <c r="I146" s="133"/>
@@ -60406,22 +60478,22 @@
         <v>921</v>
       </c>
       <c r="D147" s="138" t="s">
-        <v>2446</v>
+        <v>2458</v>
       </c>
       <c r="E147" s="138" t="s">
-        <v>2447</v>
+        <v>2459</v>
       </c>
       <c r="F147" s="178">
         <v>1</v>
       </c>
       <c r="G147" s="285" t="s">
-        <v>2448</v>
+        <v>2460</v>
       </c>
       <c r="H147" s="178" t="s">
-        <v>2449</v>
+        <v>2461</v>
       </c>
       <c r="I147" s="285" t="s">
-        <v>2450</v>
+        <v>2462</v>
       </c>
       <c r="J147" s="166"/>
       <c r="K147" s="133"/>
@@ -60437,11 +60509,11 @@
         <v>2</v>
       </c>
       <c r="G148" s="285" t="s">
-        <v>2451</v>
+        <v>2463</v>
       </c>
       <c r="H148" s="178"/>
       <c r="I148" s="285" t="s">
-        <v>2452</v>
+        <v>2464</v>
       </c>
       <c r="J148" s="166"/>
       <c r="K148" s="133"/>
@@ -60457,13 +60529,13 @@
         <v>3</v>
       </c>
       <c r="G149" s="285" t="s">
-        <v>2453</v>
+        <v>2465</v>
       </c>
       <c r="H149" s="178" t="s">
-        <v>2454</v>
+        <v>2466</v>
       </c>
       <c r="I149" s="285" t="s">
-        <v>2455</v>
+        <v>2467</v>
       </c>
       <c r="J149" s="166"/>
       <c r="K149" s="133"/>
@@ -60479,11 +60551,11 @@
         <v>4</v>
       </c>
       <c r="G150" s="285" t="s">
-        <v>2456</v>
+        <v>2468</v>
       </c>
       <c r="H150" s="178"/>
       <c r="I150" s="285" t="s">
-        <v>2457</v>
+        <v>2469</v>
       </c>
       <c r="J150" s="166"/>
       <c r="K150" s="133"/>
@@ -60499,11 +60571,11 @@
         <v>5</v>
       </c>
       <c r="G151" s="285" t="s">
-        <v>2458</v>
+        <v>2470</v>
       </c>
       <c r="H151" s="178"/>
       <c r="I151" s="285" t="s">
-        <v>2459</v>
+        <v>2471</v>
       </c>
       <c r="J151" s="166"/>
       <c r="K151" s="133"/>
@@ -60520,22 +60592,22 @@
         <v>932</v>
       </c>
       <c r="D152" s="138" t="s">
-        <v>2460</v>
+        <v>2472</v>
       </c>
       <c r="E152" s="138" t="s">
-        <v>2461</v>
+        <v>2473</v>
       </c>
       <c r="F152" s="178">
         <v>1</v>
       </c>
       <c r="G152" s="285" t="s">
-        <v>2462</v>
+        <v>2474</v>
       </c>
       <c r="H152" s="320" t="s">
-        <v>2463</v>
+        <v>2475</v>
       </c>
       <c r="I152" s="285" t="s">
-        <v>2464</v>
+        <v>2476</v>
       </c>
       <c r="J152" s="166"/>
       <c r="K152" s="133"/>
@@ -60551,13 +60623,13 @@
         <v>2</v>
       </c>
       <c r="G153" s="285" t="s">
-        <v>2465</v>
+        <v>2477</v>
       </c>
       <c r="H153" s="320" t="s">
-        <v>2466</v>
+        <v>2478</v>
       </c>
       <c r="I153" s="285" t="s">
-        <v>2467</v>
+        <v>2479</v>
       </c>
       <c r="J153" s="166"/>
       <c r="K153" s="133"/>
@@ -60573,11 +60645,11 @@
         <v>3</v>
       </c>
       <c r="G154" s="285" t="s">
-        <v>2468</v>
+        <v>2480</v>
       </c>
       <c r="H154" s="320"/>
       <c r="I154" s="285" t="s">
-        <v>2469</v>
+        <v>2481</v>
       </c>
       <c r="J154" s="166"/>
       <c r="K154" s="133"/>
@@ -61004,13 +61076,13 @@
         <v>1100</v>
       </c>
       <c r="H2" s="332" t="s">
-        <v>2470</v>
+        <v>2482</v>
       </c>
       <c r="I2" s="67" t="s">
         <v>1102</v>
       </c>
       <c r="J2" s="67" t="s">
-        <v>2471</v>
+        <v>2483</v>
       </c>
       <c r="K2" s="67" t="s">
         <v>2008</v>
@@ -61247,7 +61319,7 @@
         <v>13</v>
       </c>
       <c r="G14" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H14" s="288"/>
       <c r="I14" s="65"/>
@@ -61282,7 +61354,7 @@
         <v>1122</v>
       </c>
       <c r="J15" s="67" t="s">
-        <v>2473</v>
+        <v>2485</v>
       </c>
       <c r="K15" s="67" t="s">
         <v>2008</v>
@@ -61519,7 +61591,7 @@
         <v>13</v>
       </c>
       <c r="G27" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H27" s="288"/>
       <c r="I27" s="65"/>
@@ -61550,13 +61622,13 @@
         <v>1100</v>
       </c>
       <c r="H28" s="332" t="s">
-        <v>2474</v>
+        <v>2486</v>
       </c>
       <c r="I28" s="67" t="s">
         <v>1127</v>
       </c>
       <c r="J28" s="67" t="s">
-        <v>2475</v>
+        <v>2487</v>
       </c>
       <c r="K28" s="67" t="s">
         <v>2008</v>
@@ -61791,7 +61863,7 @@
         <v>13</v>
       </c>
       <c r="G40" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H40" s="288"/>
       <c r="I40" s="65"/>
@@ -61822,19 +61894,19 @@
         <v>1100</v>
       </c>
       <c r="H41" s="332" t="s">
-        <v>2476</v>
+        <v>2488</v>
       </c>
       <c r="I41" s="67" t="s">
         <v>1130</v>
       </c>
       <c r="J41" s="67" t="s">
-        <v>2477</v>
+        <v>2489</v>
       </c>
       <c r="K41" s="67" t="s">
         <v>2015</v>
       </c>
       <c r="L41" s="25" t="s">
-        <v>2478</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="14.4" customHeight="1">
@@ -62065,7 +62137,7 @@
         <v>13</v>
       </c>
       <c r="G53" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H53" s="288"/>
       <c r="I53" s="65"/>
@@ -62096,13 +62168,13 @@
         <v>1100</v>
       </c>
       <c r="H54" s="332" t="s">
-        <v>2479</v>
+        <v>2491</v>
       </c>
       <c r="I54" s="67" t="s">
         <v>1134</v>
       </c>
       <c r="J54" s="67" t="s">
-        <v>2480</v>
+        <v>2492</v>
       </c>
       <c r="K54" s="67" t="s">
         <v>2008</v>
@@ -62337,7 +62409,7 @@
         <v>13</v>
       </c>
       <c r="G66" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H66" s="288"/>
       <c r="I66" s="65"/>
@@ -62368,19 +62440,19 @@
         <v>1100</v>
       </c>
       <c r="H67" s="332" t="s">
-        <v>2481</v>
+        <v>2493</v>
       </c>
       <c r="I67" s="67" t="s">
         <v>1138</v>
       </c>
       <c r="J67" s="67" t="s">
-        <v>2482</v>
+        <v>2494</v>
       </c>
       <c r="K67" s="67" t="s">
         <v>2015</v>
       </c>
       <c r="L67" s="25" t="s">
-        <v>2483</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="68" spans="1:12" ht="14.4" customHeight="1">
@@ -62611,7 +62683,7 @@
         <v>13</v>
       </c>
       <c r="G79" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H79" s="288"/>
       <c r="I79" s="65"/>
@@ -62642,19 +62714,19 @@
         <v>1100</v>
       </c>
       <c r="H80" s="332" t="s">
-        <v>2484</v>
+        <v>2496</v>
       </c>
       <c r="I80" s="67" t="s">
         <v>1141</v>
       </c>
       <c r="J80" s="67" t="s">
-        <v>2485</v>
+        <v>2497</v>
       </c>
       <c r="K80" s="67" t="s">
         <v>2015</v>
       </c>
       <c r="L80" s="25" t="s">
-        <v>2486</v>
+        <v>2498</v>
       </c>
     </row>
     <row r="81" spans="1:12" ht="14.4" customHeight="1">
@@ -62885,7 +62957,7 @@
         <v>13</v>
       </c>
       <c r="G92" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H92" s="288"/>
       <c r="I92" s="65"/>
@@ -62916,13 +62988,13 @@
         <v>1100</v>
       </c>
       <c r="H93" s="332" t="s">
-        <v>2487</v>
+        <v>2499</v>
       </c>
       <c r="I93" s="67" t="s">
         <v>1145</v>
       </c>
       <c r="J93" s="67" t="s">
-        <v>2488</v>
+        <v>2500</v>
       </c>
       <c r="K93" s="67" t="s">
         <v>2008</v>
@@ -63157,7 +63229,7 @@
         <v>13</v>
       </c>
       <c r="G105" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H105" s="288"/>
       <c r="I105" s="65"/>
@@ -63188,13 +63260,13 @@
         <v>1100</v>
       </c>
       <c r="H106" s="332" t="s">
-        <v>2487</v>
+        <v>2499</v>
       </c>
       <c r="I106" s="67" t="s">
         <v>1149</v>
       </c>
       <c r="J106" s="67" t="s">
-        <v>2489</v>
+        <v>2501</v>
       </c>
       <c r="K106" s="67" t="s">
         <v>2008</v>
@@ -63429,7 +63501,7 @@
         <v>13</v>
       </c>
       <c r="G118" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H118" s="288"/>
       <c r="I118" s="65"/>
@@ -63460,13 +63532,13 @@
         <v>1100</v>
       </c>
       <c r="H119" s="332" t="s">
-        <v>2490</v>
+        <v>2502</v>
       </c>
       <c r="I119" s="67" t="s">
-        <v>2491</v>
+        <v>2503</v>
       </c>
       <c r="J119" s="67" t="s">
-        <v>2492</v>
+        <v>2504</v>
       </c>
       <c r="K119" s="67" t="s">
         <v>2008</v>
@@ -63701,7 +63773,7 @@
         <v>13</v>
       </c>
       <c r="G131" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H131" s="288"/>
       <c r="I131" s="65"/>
@@ -63732,13 +63804,13 @@
         <v>1100</v>
       </c>
       <c r="H132" s="332" t="s">
-        <v>2493</v>
+        <v>2505</v>
       </c>
       <c r="I132" s="67" t="s">
         <v>1160</v>
       </c>
       <c r="J132" s="67" t="s">
-        <v>2494</v>
+        <v>2506</v>
       </c>
       <c r="K132" s="67" t="s">
         <v>2008</v>
@@ -63973,7 +64045,7 @@
         <v>13</v>
       </c>
       <c r="G144" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H144" s="288"/>
       <c r="I144" s="65"/>
@@ -63992,7 +64064,7 @@
         <v>1164</v>
       </c>
       <c r="D145" s="67" t="s">
-        <v>2495</v>
+        <v>2507</v>
       </c>
       <c r="E145" s="67" t="s">
         <v>1099</v>
@@ -64004,19 +64076,19 @@
         <v>1100</v>
       </c>
       <c r="H145" s="332" t="s">
-        <v>2496</v>
+        <v>2508</v>
       </c>
       <c r="I145" s="67" t="s">
-        <v>2497</v>
+        <v>2509</v>
       </c>
       <c r="J145" s="67" t="s">
-        <v>2498</v>
+        <v>2510</v>
       </c>
       <c r="K145" s="67" t="s">
         <v>2015</v>
       </c>
       <c r="L145" s="25" t="s">
-        <v>2499</v>
+        <v>2511</v>
       </c>
     </row>
     <row r="146" spans="1:12" ht="14.4" customHeight="1">
@@ -64249,7 +64321,7 @@
         <v>13</v>
       </c>
       <c r="G157" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H157" s="288"/>
       <c r="I157" s="65"/>
@@ -64280,13 +64352,13 @@
         <v>1100</v>
       </c>
       <c r="H158" s="332" t="s">
-        <v>2500</v>
+        <v>2512</v>
       </c>
       <c r="I158" s="67" t="s">
-        <v>2501</v>
+        <v>2513</v>
       </c>
       <c r="J158" s="67" t="s">
-        <v>2502</v>
+        <v>2514</v>
       </c>
       <c r="K158" s="67" t="s">
         <v>2008</v>
@@ -64521,7 +64593,7 @@
         <v>13</v>
       </c>
       <c r="G170" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H170" s="288"/>
       <c r="I170" s="65"/>
@@ -64552,13 +64624,13 @@
         <v>1100</v>
       </c>
       <c r="H171" s="332" t="s">
-        <v>2503</v>
+        <v>2515</v>
       </c>
       <c r="I171" s="67" t="s">
-        <v>2504</v>
+        <v>2516</v>
       </c>
       <c r="J171" s="67" t="s">
-        <v>2505</v>
+        <v>2517</v>
       </c>
       <c r="K171" s="67" t="s">
         <v>2008</v>
@@ -64793,7 +64865,7 @@
         <v>13</v>
       </c>
       <c r="G183" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H183" s="288"/>
       <c r="I183" s="65"/>
@@ -64825,16 +64897,16 @@
       </c>
       <c r="H184" s="332"/>
       <c r="I184" s="67" t="s">
-        <v>2506</v>
+        <v>2518</v>
       </c>
       <c r="J184" s="67" t="s">
-        <v>2507</v>
+        <v>2519</v>
       </c>
       <c r="K184" s="67" t="s">
         <v>2015</v>
       </c>
       <c r="L184" s="25" t="s">
-        <v>2508</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="185" spans="1:12" ht="14.4" customHeight="1">
@@ -65045,7 +65117,7 @@
         <v>13</v>
       </c>
       <c r="G196" s="288" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H196" s="332"/>
       <c r="I196" s="65"/>
@@ -65076,19 +65148,19 @@
         <v>1100</v>
       </c>
       <c r="H197" s="332" t="s">
-        <v>2509</v>
+        <v>2521</v>
       </c>
       <c r="I197" s="56" t="s">
         <v>1178</v>
       </c>
       <c r="J197" s="25" t="s">
-        <v>2510</v>
+        <v>2522</v>
       </c>
       <c r="K197" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L197" s="25" t="s">
-        <v>2511</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="198" spans="1:12">
@@ -65321,7 +65393,7 @@
         <v>13</v>
       </c>
       <c r="G209" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H209" s="293"/>
       <c r="I209" s="56"/>
@@ -65352,19 +65424,19 @@
         <v>1100</v>
       </c>
       <c r="H210" s="332" t="s">
-        <v>2512</v>
+        <v>2524</v>
       </c>
       <c r="I210" s="56" t="s">
         <v>1187</v>
       </c>
       <c r="J210" s="25" t="s">
-        <v>2513</v>
+        <v>2525</v>
       </c>
       <c r="K210" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L210" s="25" t="s">
-        <v>2514</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="211" spans="1:12">
@@ -65597,7 +65669,7 @@
         <v>13</v>
       </c>
       <c r="G222" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H222" s="293"/>
       <c r="I222" s="56"/>
@@ -65616,7 +65688,7 @@
         <v>1189</v>
       </c>
       <c r="D223" s="56" t="s">
-        <v>2515</v>
+        <v>2527</v>
       </c>
       <c r="E223" s="136" t="s">
         <v>1176</v>
@@ -65628,19 +65700,19 @@
         <v>1100</v>
       </c>
       <c r="H223" s="332" t="s">
-        <v>2516</v>
+        <v>2528</v>
       </c>
       <c r="I223" s="25" t="s">
-        <v>2517</v>
+        <v>2529</v>
       </c>
       <c r="J223" s="25" t="s">
-        <v>2518</v>
+        <v>2530</v>
       </c>
       <c r="K223" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L223" s="25" t="s">
-        <v>2519</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="224" spans="1:12" ht="31.2" customHeight="1">
@@ -65873,7 +65945,7 @@
         <v>13</v>
       </c>
       <c r="G235" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H235" s="293"/>
       <c r="I235" s="23"/>
@@ -65904,19 +65976,19 @@
         <v>1100</v>
       </c>
       <c r="H236" s="332" t="s">
-        <v>2520</v>
+        <v>2532</v>
       </c>
       <c r="I236" s="25" t="s">
         <v>1197</v>
       </c>
       <c r="J236" s="25" t="s">
-        <v>2521</v>
+        <v>2533</v>
       </c>
       <c r="K236" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L236" s="25" t="s">
-        <v>2522</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="237" spans="1:12" ht="26.4" customHeight="1">
@@ -66149,7 +66221,7 @@
         <v>13</v>
       </c>
       <c r="G248" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H248" s="293"/>
       <c r="I248" s="23"/>
@@ -66180,19 +66252,19 @@
         <v>1100</v>
       </c>
       <c r="H249" s="332" t="s">
-        <v>2523</v>
+        <v>2535</v>
       </c>
       <c r="I249" s="25" t="s">
         <v>1203</v>
       </c>
       <c r="J249" s="25" t="s">
-        <v>2524</v>
+        <v>2536</v>
       </c>
       <c r="K249" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L249" s="25" t="s">
-        <v>2525</v>
+        <v>2537</v>
       </c>
     </row>
     <row r="250" spans="1:12" ht="30" customHeight="1">
@@ -66368,7 +66440,7 @@
         <v>1115</v>
       </c>
       <c r="H258" s="288" t="s">
-        <v>2526</v>
+        <v>2538</v>
       </c>
       <c r="I258" s="24"/>
       <c r="J258" s="24"/>
@@ -66425,7 +66497,7 @@
         <v>13</v>
       </c>
       <c r="G261" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H261" s="293"/>
       <c r="I261" s="23"/>
@@ -66447,7 +66519,7 @@
         <v>1207</v>
       </c>
       <c r="E262" s="136" t="s">
-        <v>2527</v>
+        <v>2539</v>
       </c>
       <c r="F262" s="176">
         <v>1</v>
@@ -66462,13 +66534,13 @@
         <v>1210</v>
       </c>
       <c r="J262" s="25" t="s">
-        <v>2528</v>
+        <v>2540</v>
       </c>
       <c r="K262" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L262" s="25" t="s">
-        <v>2529</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="263" spans="1:12" ht="29.4" customHeight="1">
@@ -66701,7 +66773,7 @@
         <v>13</v>
       </c>
       <c r="G274" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H274" s="293"/>
       <c r="I274" s="23"/>
@@ -66732,19 +66804,19 @@
         <v>1100</v>
       </c>
       <c r="H275" s="332" t="s">
-        <v>2530</v>
+        <v>2542</v>
       </c>
       <c r="I275" s="135" t="s">
-        <v>2531</v>
+        <v>2543</v>
       </c>
       <c r="J275" s="67" t="s">
-        <v>2532</v>
+        <v>2544</v>
       </c>
       <c r="K275" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L275" s="25" t="s">
-        <v>2533</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="276" spans="1:12">
@@ -66817,7 +66889,7 @@
         <v>5</v>
       </c>
       <c r="G279" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H279" s="308" t="s">
         <v>1117</v>
@@ -66837,7 +66909,7 @@
         <v>6</v>
       </c>
       <c r="G280" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H280" s="308">
         <v>46123</v>
@@ -66957,7 +67029,7 @@
         <v>12</v>
       </c>
       <c r="G286" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H286" s="293"/>
       <c r="I286" s="135"/>
@@ -66992,13 +67064,13 @@
         <v>1122</v>
       </c>
       <c r="J287" s="67" t="s">
-        <v>2473</v>
+        <v>2485</v>
       </c>
       <c r="K287" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L287" s="25" t="s">
-        <v>2536</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="288" spans="1:12">
@@ -67071,7 +67143,7 @@
         <v>5</v>
       </c>
       <c r="G291" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H291" s="308" t="s">
         <v>1117</v>
@@ -67091,7 +67163,7 @@
         <v>6</v>
       </c>
       <c r="G292" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H292" s="308">
         <v>46123</v>
@@ -67211,7 +67283,7 @@
         <v>12</v>
       </c>
       <c r="G298" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I298" s="135"/>
       <c r="J298" s="65"/>
@@ -67241,19 +67313,19 @@
         <v>1100</v>
       </c>
       <c r="H299" s="332" t="s">
-        <v>2537</v>
+        <v>2549</v>
       </c>
       <c r="I299" s="135" t="s">
         <v>1127</v>
       </c>
       <c r="J299" s="67" t="s">
-        <v>2475</v>
+        <v>2487</v>
       </c>
       <c r="K299" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L299" s="25" t="s">
-        <v>2538</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="300" spans="1:12">
@@ -67324,7 +67396,7 @@
         <v>5</v>
       </c>
       <c r="G303" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H303" s="308" t="s">
         <v>1117</v>
@@ -67344,7 +67416,7 @@
         <v>6</v>
       </c>
       <c r="G304" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H304" s="308">
         <v>46123</v>
@@ -67464,7 +67536,7 @@
         <v>12</v>
       </c>
       <c r="G310" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I310" s="135"/>
       <c r="J310" s="65"/>
@@ -67494,19 +67566,19 @@
         <v>1100</v>
       </c>
       <c r="H311" s="332" t="s">
-        <v>2539</v>
+        <v>2551</v>
       </c>
       <c r="I311" s="135" t="s">
         <v>1130</v>
       </c>
       <c r="J311" s="67" t="s">
-        <v>2540</v>
+        <v>2552</v>
       </c>
       <c r="K311" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L311" s="25" t="s">
-        <v>2541</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="312" spans="1:12">
@@ -67577,7 +67649,7 @@
         <v>5</v>
       </c>
       <c r="G315" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H315" s="308" t="s">
         <v>1117</v>
@@ -67597,7 +67669,7 @@
         <v>6</v>
       </c>
       <c r="G316" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H316" s="308">
         <v>46123</v>
@@ -67717,7 +67789,7 @@
         <v>12</v>
       </c>
       <c r="G322" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I322" s="135"/>
       <c r="J322" s="65"/>
@@ -67747,13 +67819,13 @@
         <v>1100</v>
       </c>
       <c r="H323" s="332" t="s">
-        <v>2542</v>
+        <v>2554</v>
       </c>
       <c r="I323" s="135" t="s">
         <v>1134</v>
       </c>
       <c r="J323" s="67" t="s">
-        <v>2480</v>
+        <v>2492</v>
       </c>
       <c r="K323" s="135" t="s">
         <v>2008</v>
@@ -67830,7 +67902,7 @@
         <v>5</v>
       </c>
       <c r="G327" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H327" s="308"/>
       <c r="I327" s="135"/>
@@ -67848,7 +67920,7 @@
         <v>6</v>
       </c>
       <c r="G328" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H328" s="308">
         <v>46123</v>
@@ -67968,7 +68040,7 @@
         <v>12</v>
       </c>
       <c r="G334" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I334" s="135"/>
       <c r="J334" s="65"/>
@@ -67998,19 +68070,19 @@
         <v>1100</v>
       </c>
       <c r="H335" s="332" t="s">
-        <v>2542</v>
+        <v>2554</v>
       </c>
       <c r="I335" s="135" t="s">
         <v>1138</v>
       </c>
       <c r="J335" s="67" t="s">
-        <v>2543</v>
+        <v>2555</v>
       </c>
       <c r="K335" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L335" s="25" t="s">
-        <v>2544</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="336" spans="1:12">
@@ -68083,7 +68155,7 @@
         <v>5</v>
       </c>
       <c r="G339" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H339" s="308" t="s">
         <v>1117</v>
@@ -68103,7 +68175,7 @@
         <v>6</v>
       </c>
       <c r="G340" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H340" s="308"/>
       <c r="I340" s="135"/>
@@ -68221,7 +68293,7 @@
         <v>12</v>
       </c>
       <c r="G346" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I346" s="135"/>
       <c r="J346" s="65"/>
@@ -68239,7 +68311,7 @@
         <v>1254</v>
       </c>
       <c r="D347" s="135" t="s">
-        <v>2545</v>
+        <v>2557</v>
       </c>
       <c r="E347" s="135" t="s">
         <v>1099</v>
@@ -68251,19 +68323,19 @@
         <v>1100</v>
       </c>
       <c r="H347" s="332" t="s">
-        <v>2546</v>
+        <v>2558</v>
       </c>
       <c r="I347" s="135" t="s">
-        <v>2547</v>
+        <v>2559</v>
       </c>
       <c r="J347" s="67" t="s">
-        <v>2548</v>
+        <v>2560</v>
       </c>
       <c r="K347" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L347" s="25" t="s">
-        <v>2549</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="348" spans="1:12">
@@ -68336,7 +68408,7 @@
         <v>5</v>
       </c>
       <c r="G351" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H351" s="308" t="s">
         <v>1117</v>
@@ -68356,7 +68428,7 @@
         <v>6</v>
       </c>
       <c r="G352" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H352" s="308">
         <v>49410</v>
@@ -68474,7 +68546,7 @@
         <v>12</v>
       </c>
       <c r="G358" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H358" s="288"/>
       <c r="I358" s="135"/>
@@ -68505,13 +68577,13 @@
         <v>1100</v>
       </c>
       <c r="H359" s="332" t="s">
-        <v>2550</v>
+        <v>2562</v>
       </c>
       <c r="I359" s="135" t="s">
         <v>1145</v>
       </c>
       <c r="J359" s="67" t="s">
-        <v>2488</v>
+        <v>2500</v>
       </c>
       <c r="K359" s="135" t="s">
         <v>2008</v>
@@ -68588,7 +68660,7 @@
         <v>5</v>
       </c>
       <c r="G363" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H363" s="308" t="s">
         <v>1117</v>
@@ -68608,7 +68680,7 @@
         <v>6</v>
       </c>
       <c r="G364" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H364" s="308">
         <v>46123</v>
@@ -68726,7 +68798,7 @@
         <v>12</v>
       </c>
       <c r="G370" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I370" s="135"/>
       <c r="J370" s="65"/>
@@ -68756,13 +68828,13 @@
         <v>1100</v>
       </c>
       <c r="H371" s="332" t="s">
-        <v>2551</v>
+        <v>2563</v>
       </c>
       <c r="I371" s="135" t="s">
         <v>1149</v>
       </c>
       <c r="J371" s="67" t="s">
-        <v>2489</v>
+        <v>2501</v>
       </c>
       <c r="K371" s="135" t="s">
         <v>2008</v>
@@ -68839,7 +68911,7 @@
         <v>5</v>
       </c>
       <c r="G375" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H375" s="308" t="s">
         <v>1117</v>
@@ -68859,7 +68931,7 @@
         <v>6</v>
       </c>
       <c r="G376" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H376" s="308">
         <v>46123</v>
@@ -68977,7 +69049,7 @@
         <v>12</v>
       </c>
       <c r="G382" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I382" s="135"/>
       <c r="J382" s="65"/>
@@ -68995,7 +69067,7 @@
         <v>1257</v>
       </c>
       <c r="D383" s="135" t="s">
-        <v>2552</v>
+        <v>2564</v>
       </c>
       <c r="E383" s="135" t="s">
         <v>1099</v>
@@ -69007,19 +69079,19 @@
         <v>1100</v>
       </c>
       <c r="H383" s="332" t="s">
-        <v>2553</v>
+        <v>2565</v>
       </c>
       <c r="I383" s="135" t="s">
-        <v>2491</v>
+        <v>2503</v>
       </c>
       <c r="J383" s="67" t="s">
-        <v>2492</v>
+        <v>2504</v>
       </c>
       <c r="K383" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L383" s="25" t="s">
-        <v>2554</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="384" spans="1:12">
@@ -69090,7 +69162,7 @@
         <v>5</v>
       </c>
       <c r="G387" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H387" s="308" t="s">
         <v>1117</v>
@@ -69110,7 +69182,7 @@
         <v>6</v>
       </c>
       <c r="G388" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H388" s="308">
         <v>46123</v>
@@ -69230,7 +69302,7 @@
         <v>12</v>
       </c>
       <c r="G394" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I394" s="135"/>
       <c r="J394" s="65"/>
@@ -69260,13 +69332,13 @@
         <v>1100</v>
       </c>
       <c r="H395" s="332" t="s">
-        <v>2555</v>
+        <v>2567</v>
       </c>
       <c r="I395" s="135" t="s">
         <v>1160</v>
       </c>
       <c r="J395" s="67" t="s">
-        <v>2494</v>
+        <v>2506</v>
       </c>
       <c r="K395" s="135" t="s">
         <v>2008</v>
@@ -69343,7 +69415,7 @@
         <v>5</v>
       </c>
       <c r="G399" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H399" s="308" t="s">
         <v>1117</v>
@@ -69363,7 +69435,7 @@
         <v>6</v>
       </c>
       <c r="G400" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H400" s="308">
         <v>46123</v>
@@ -69481,7 +69553,7 @@
         <v>12</v>
       </c>
       <c r="G406" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I406" s="135"/>
       <c r="J406" s="65"/>
@@ -69499,7 +69571,7 @@
         <v>1260</v>
       </c>
       <c r="D407" s="135" t="s">
-        <v>2556</v>
+        <v>2568</v>
       </c>
       <c r="E407" s="135" t="s">
         <v>1099</v>
@@ -69511,19 +69583,19 @@
         <v>1100</v>
       </c>
       <c r="H407" s="332" t="s">
-        <v>2557</v>
+        <v>2569</v>
       </c>
       <c r="I407" s="135" t="s">
-        <v>2558</v>
+        <v>2570</v>
       </c>
       <c r="J407" s="67" t="s">
-        <v>2559</v>
+        <v>2571</v>
       </c>
       <c r="K407" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L407" s="25" t="s">
-        <v>2560</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="408" spans="1:12">
@@ -69596,7 +69668,7 @@
         <v>5</v>
       </c>
       <c r="G411" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H411" s="308" t="s">
         <v>1117</v>
@@ -69616,7 +69688,7 @@
         <v>6</v>
       </c>
       <c r="G412" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H412" s="308">
         <v>46123</v>
@@ -69736,7 +69808,7 @@
         <v>12</v>
       </c>
       <c r="G418" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I418" s="135"/>
       <c r="J418" s="65"/>
@@ -69766,19 +69838,19 @@
         <v>1100</v>
       </c>
       <c r="H419" s="332" t="s">
-        <v>2561</v>
+        <v>2573</v>
       </c>
       <c r="I419" s="135" t="s">
-        <v>2501</v>
+        <v>2513</v>
       </c>
       <c r="J419" s="67" t="s">
-        <v>2502</v>
+        <v>2514</v>
       </c>
       <c r="K419" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L419" s="25" t="s">
-        <v>2562</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="420" spans="1:12">
@@ -69851,7 +69923,7 @@
         <v>5</v>
       </c>
       <c r="G423" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H423" s="308" t="s">
         <v>1117</v>
@@ -69871,7 +69943,7 @@
         <v>6</v>
       </c>
       <c r="G424" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H424" s="308">
         <v>46123</v>
@@ -69989,7 +70061,7 @@
         <v>12</v>
       </c>
       <c r="G430" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I430" s="135"/>
       <c r="J430" s="65"/>
@@ -70019,19 +70091,19 @@
         <v>1100</v>
       </c>
       <c r="H431" s="332" t="s">
-        <v>2563</v>
+        <v>2575</v>
       </c>
       <c r="I431" s="135" t="s">
-        <v>2504</v>
+        <v>2516</v>
       </c>
       <c r="J431" s="67" t="s">
-        <v>2505</v>
+        <v>2517</v>
       </c>
       <c r="K431" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L431" s="25" t="s">
-        <v>2564</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="432" spans="1:12">
@@ -70104,7 +70176,7 @@
         <v>5</v>
       </c>
       <c r="G435" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H435" s="308" t="s">
         <v>1117</v>
@@ -70124,7 +70196,7 @@
         <v>6</v>
       </c>
       <c r="G436" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H436" s="308">
         <v>46123</v>
@@ -70242,7 +70314,7 @@
         <v>12</v>
       </c>
       <c r="G442" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I442" s="135"/>
       <c r="J442" s="65"/>
@@ -70260,7 +70332,7 @@
         <v>1265</v>
       </c>
       <c r="D443" s="135" t="s">
-        <v>2565</v>
+        <v>2577</v>
       </c>
       <c r="E443" s="135" t="s">
         <v>1099</v>
@@ -70272,19 +70344,19 @@
         <v>1100</v>
       </c>
       <c r="H443" s="332" t="s">
-        <v>2557</v>
+        <v>2569</v>
       </c>
       <c r="I443" s="135" t="s">
-        <v>2566</v>
+        <v>2578</v>
       </c>
       <c r="J443" s="67" t="s">
-        <v>2567</v>
+        <v>2579</v>
       </c>
       <c r="K443" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L443" s="25" t="s">
-        <v>2568</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="444" spans="1:12">
@@ -70357,7 +70429,7 @@
         <v>5</v>
       </c>
       <c r="G447" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H447" s="308" t="s">
         <v>1117</v>
@@ -70377,7 +70449,7 @@
         <v>6</v>
       </c>
       <c r="G448" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H448" s="308">
         <v>46123</v>
@@ -70497,7 +70569,7 @@
         <v>12</v>
       </c>
       <c r="G454" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="I454" s="135"/>
       <c r="J454" s="65"/>
@@ -70515,10 +70587,10 @@
         <v>1212</v>
       </c>
       <c r="D455" s="136" t="s">
-        <v>2569</v>
+        <v>2581</v>
       </c>
       <c r="E455" s="136" t="s">
-        <v>2570</v>
+        <v>2582</v>
       </c>
       <c r="F455" s="176">
         <v>1</v>
@@ -70527,19 +70599,19 @@
         <v>1100</v>
       </c>
       <c r="H455" s="332" t="s">
-        <v>2571</v>
+        <v>2583</v>
       </c>
       <c r="I455" s="25" t="s">
-        <v>2572</v>
+        <v>2584</v>
       </c>
       <c r="J455" s="25" t="s">
-        <v>2573</v>
+        <v>2585</v>
       </c>
       <c r="K455" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L455" s="25" t="s">
-        <v>2574</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="456" spans="1:12">
@@ -70612,7 +70684,7 @@
         <v>5</v>
       </c>
       <c r="G459" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H459" s="308" t="s">
         <v>1117</v>
@@ -70632,7 +70704,7 @@
         <v>6</v>
       </c>
       <c r="G460" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H460" s="308">
         <v>46123</v>
@@ -70695,7 +70767,7 @@
         <v>1115</v>
       </c>
       <c r="H463" s="318" t="s">
-        <v>2575</v>
+        <v>2587</v>
       </c>
       <c r="I463" s="24"/>
       <c r="J463" s="24"/>
@@ -70752,7 +70824,7 @@
         <v>12</v>
       </c>
       <c r="G466" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H466" s="293"/>
       <c r="I466" s="23"/>
@@ -70771,10 +70843,10 @@
         <v>1219</v>
       </c>
       <c r="D467" s="136" t="s">
-        <v>2576</v>
+        <v>2588</v>
       </c>
       <c r="E467" s="136" t="s">
-        <v>2577</v>
+        <v>2589</v>
       </c>
       <c r="F467" s="176">
         <v>1</v>
@@ -70783,19 +70855,19 @@
         <v>1100</v>
       </c>
       <c r="H467" s="332" t="s">
-        <v>2578</v>
+        <v>2590</v>
       </c>
       <c r="I467" s="25" t="s">
-        <v>2517</v>
+        <v>2529</v>
       </c>
       <c r="J467" s="25" t="s">
-        <v>2579</v>
+        <v>2591</v>
       </c>
       <c r="K467" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L467" s="25" t="s">
-        <v>2580</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="468" spans="1:12">
@@ -70868,7 +70940,7 @@
         <v>5</v>
       </c>
       <c r="G471" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H471" s="308" t="s">
         <v>1117</v>
@@ -70888,7 +70960,7 @@
         <v>6</v>
       </c>
       <c r="G472" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H472" s="308">
         <v>46123</v>
@@ -71008,7 +71080,7 @@
         <v>12</v>
       </c>
       <c r="G478" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H478" s="293"/>
       <c r="I478" s="23"/>
@@ -71027,10 +71099,10 @@
         <v>1225</v>
       </c>
       <c r="D479" s="136" t="s">
-        <v>2581</v>
+        <v>2593</v>
       </c>
       <c r="E479" s="136" t="s">
-        <v>2582</v>
+        <v>2594</v>
       </c>
       <c r="F479" s="176">
         <v>1</v>
@@ -71039,19 +71111,19 @@
         <v>1100</v>
       </c>
       <c r="H479" s="332" t="s">
-        <v>2583</v>
+        <v>2595</v>
       </c>
       <c r="I479" s="25" t="s">
-        <v>2584</v>
+        <v>2596</v>
       </c>
       <c r="J479" s="25" t="s">
-        <v>2585</v>
+        <v>2597</v>
       </c>
       <c r="K479" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L479" s="25" t="s">
-        <v>2586</v>
+        <v>2598</v>
       </c>
     </row>
     <row r="480" spans="1:12">
@@ -71067,7 +71139,7 @@
         <v>1103</v>
       </c>
       <c r="H480" s="332" t="s">
-        <v>2587</v>
+        <v>2599</v>
       </c>
       <c r="I480" s="24"/>
       <c r="J480" s="24"/>
@@ -71124,7 +71196,7 @@
         <v>5</v>
       </c>
       <c r="G483" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H483" s="308" t="s">
         <v>1117</v>
@@ -71144,7 +71216,7 @@
         <v>6</v>
       </c>
       <c r="G484" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H484" s="308">
         <v>46123</v>
@@ -71264,7 +71336,7 @@
         <v>12</v>
       </c>
       <c r="G490" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H490" s="293"/>
       <c r="I490" s="23"/>
@@ -71283,10 +71355,10 @@
         <v>1232</v>
       </c>
       <c r="D491" s="136" t="s">
-        <v>2588</v>
+        <v>2600</v>
       </c>
       <c r="E491" s="136" t="s">
-        <v>2582</v>
+        <v>2594</v>
       </c>
       <c r="F491" s="176">
         <v>1</v>
@@ -71295,19 +71367,19 @@
         <v>1100</v>
       </c>
       <c r="H491" s="292" t="s">
-        <v>2589</v>
+        <v>2601</v>
       </c>
       <c r="I491" s="25" t="s">
-        <v>2590</v>
+        <v>2602</v>
       </c>
       <c r="J491" s="25" t="s">
-        <v>2591</v>
+        <v>2603</v>
       </c>
       <c r="K491" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L491" s="25" t="s">
-        <v>2592</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="492" spans="1:12" ht="15" customHeight="1">
@@ -71323,7 +71395,7 @@
         <v>1103</v>
       </c>
       <c r="H492" s="332" t="s">
-        <v>2593</v>
+        <v>2605</v>
       </c>
       <c r="I492" s="24"/>
       <c r="J492" s="24"/>
@@ -71380,7 +71452,7 @@
         <v>5</v>
       </c>
       <c r="G495" s="288" t="s">
-        <v>2534</v>
+        <v>2546</v>
       </c>
       <c r="H495" s="308" t="s">
         <v>1117</v>
@@ -71400,7 +71472,7 @@
         <v>6</v>
       </c>
       <c r="G496" s="288" t="s">
-        <v>2535</v>
+        <v>2547</v>
       </c>
       <c r="H496" s="308">
         <v>46123</v>
@@ -71520,7 +71592,7 @@
         <v>12</v>
       </c>
       <c r="G502" s="293" t="s">
-        <v>2472</v>
+        <v>2484</v>
       </c>
       <c r="H502" s="293"/>
       <c r="I502" s="23"/>
@@ -71911,13 +71983,13 @@
   <sheetData>
     <row r="2" spans="1:7">
       <c r="A2" s="192" t="s">
-        <v>2594</v>
+        <v>2606</v>
       </c>
       <c r="D2" s="192" t="s">
         <v>29</v>
       </c>
       <c r="G2" s="192" t="s">
-        <v>2595</v>
+        <v>2607</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -71925,7 +71997,7 @@
         <v>229</v>
       </c>
       <c r="D3" t="s">
-        <v>2596</v>
+        <v>2608</v>
       </c>
       <c r="G3" t="s">
         <v>244</v>
@@ -71936,7 +72008,7 @@
         <v>245</v>
       </c>
       <c r="D4" t="s">
-        <v>2597</v>
+        <v>2609</v>
       </c>
       <c r="G4" t="s">
         <v>234</v>
@@ -71944,10 +72016,10 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>2598</v>
+        <v>2610</v>
       </c>
       <c r="D5" t="s">
-        <v>2599</v>
+        <v>2611</v>
       </c>
       <c r="G5" t="s">
         <v>239</v>

</xml_diff>

<commit_message>
Test: Complete testcase TC_SHOW_02
</commit_message>
<xml_diff>
--- a/sqa-testing-report/Data/DataTest.xlsx
+++ b/sqa-testing-report/Data/DataTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\sqa-testing-report\sqa-testing-report\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C70A8AA5-DE9A-44B5-A106-0A58CBBA34AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF902E4F-A249-4A8F-897B-2EC8CCD165BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="664" activeTab="5" xr2:uid="{DC4DB269-603C-4B5B-A498-B166C8A18B92}"/>
   </bookViews>
@@ -164,7 +164,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7224" uniqueCount="2621">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7229" uniqueCount="2624">
   <si>
     <t>GUI &amp; FUNCTIONAL TEST CASES</t>
   </si>
@@ -9055,9 +9055,15 @@
     <t>Tại màn hình Timeline, chọn Rạp và chọn Ngày muốn tạo lịch.</t>
   </si>
   <si>
+    <t>Rạp: Galaxy Bến Tre; Ngày: 15/04/2026</t>
+  </si>
+  <si>
     <t>Hệ thống tải dữ liệu của rạp và ngày đã chọn.</t>
   </si>
   <si>
+    <t>Đã check và tìm được phòng trống: Phòng 1 vào ngày 15/04/2026. Modal Thêm lịch chiếu đang mở.</t>
+  </si>
+  <si>
     <t>Nhấn nút "+ Thêm lịch chiếu".</t>
   </si>
   <si>
@@ -9073,10 +9079,19 @@
     <t>Thông báo "Thêm thành công" và Modal đóng lại.</t>
   </si>
   <si>
+    <t>Đã nhập đủ thông tin cho phòng Phòng 1, loại suất chiếu 1. Nhấn Lưu và Modal đóng lại.</t>
+  </si>
+  <si>
     <t>Nhấn nút "Tải lịch chiếu" (Nút xanh dương).</t>
   </si>
   <si>
     <t>Lịch chiếu vừa tạo (Phim Khá, 08:00 AM) hiển thị đúng trên Timeline của phòng 3.</t>
+  </si>
+  <si>
+    <t>Lịch chiếu vừa tạo hiển thị chính xác trên Timeline của Phòng 1 lúc 08:00 AM.</t>
+  </si>
+  <si>
+    <t>Đăng nhập Admin; Đã có sẵn 01 suất chiếu tại Phòng 3 (khung giờ 08:00 AM - 11:51 PM).</t>
   </si>
   <si>
     <t>Tại màn hình Timeline, chọn đúng Rạp và Ngày có suất chiếu đã tồn tại.</t>
@@ -10298,12 +10313,6 @@
   </si>
   <si>
     <t>Failed</t>
-  </si>
-  <si>
-    <t>Rạp: Galaxy Bến Tre; Ngày: 15/04/2026</t>
-  </si>
-  <si>
-    <t>Đăng nhập Admin; Đã có sẵn 01 suất chiếu tại Phòng 3 (khung giờ 08:00 AM - 11:51 PM).</t>
   </si>
 </sst>
 </file>
@@ -59655,7 +59664,7 @@
       <c r="K103" s="135"/>
       <c r="L103" s="135"/>
     </row>
-    <row r="104" spans="1:12" ht="40.200000000000003" customHeight="1">
+    <row r="104" spans="1:12" ht="143.4" customHeight="1">
       <c r="A104" s="138">
         <v>33</v>
       </c>
@@ -59678,16 +59687,20 @@
         <v>2414</v>
       </c>
       <c r="H104" s="178" t="s">
-        <v>2619</v>
+        <v>2415</v>
       </c>
       <c r="I104" s="285" t="s">
-        <v>2415</v>
-      </c>
-      <c r="J104" s="166"/>
-      <c r="K104" s="130"/>
+        <v>2416</v>
+      </c>
+      <c r="J104" s="166" t="s">
+        <v>2417</v>
+      </c>
+      <c r="K104" s="130" t="s">
+        <v>2008</v>
+      </c>
       <c r="L104" s="130"/>
     </row>
-    <row r="105" spans="1:12" ht="52.8" customHeight="1">
+    <row r="105" spans="1:12" ht="132" customHeight="1">
       <c r="A105" s="138"/>
       <c r="B105" s="138"/>
       <c r="C105" s="138"/>
@@ -59697,17 +59710,19 @@
         <v>2</v>
       </c>
       <c r="G105" s="285" t="s">
-        <v>2416</v>
+        <v>2418</v>
       </c>
       <c r="H105" s="178"/>
       <c r="I105" s="285" t="s">
+        <v>2419</v>
+      </c>
+      <c r="J105" s="166" t="s">
         <v>2417</v>
       </c>
-      <c r="J105" s="166"/>
       <c r="K105" s="130"/>
       <c r="L105" s="130"/>
     </row>
-    <row r="106" spans="1:12" ht="64.2" customHeight="1">
+    <row r="106" spans="1:12" ht="114.6" customHeight="1">
       <c r="A106" s="138"/>
       <c r="B106" s="138"/>
       <c r="C106" s="138"/>
@@ -59717,19 +59732,21 @@
         <v>3</v>
       </c>
       <c r="G106" s="285" t="s">
-        <v>2418</v>
+        <v>2420</v>
       </c>
       <c r="H106" s="178" t="s">
-        <v>2419</v>
+        <v>2421</v>
       </c>
       <c r="I106" s="285" t="s">
-        <v>2420</v>
-      </c>
-      <c r="J106" s="166"/>
+        <v>2422</v>
+      </c>
+      <c r="J106" s="166" t="s">
+        <v>2423</v>
+      </c>
       <c r="K106" s="130"/>
       <c r="L106" s="130"/>
     </row>
-    <row r="107" spans="1:12" ht="72" customHeight="1">
+    <row r="107" spans="1:12" ht="100.8" customHeight="1">
       <c r="A107" s="138"/>
       <c r="B107" s="138"/>
       <c r="C107" s="138"/>
@@ -59739,13 +59756,15 @@
         <v>4</v>
       </c>
       <c r="G107" s="285" t="s">
-        <v>2421</v>
+        <v>2424</v>
       </c>
       <c r="H107" s="178"/>
       <c r="I107" s="285" t="s">
-        <v>2422</v>
-      </c>
-      <c r="J107" s="166"/>
+        <v>2425</v>
+      </c>
+      <c r="J107" s="166" t="s">
+        <v>2426</v>
+      </c>
       <c r="K107" s="130"/>
       <c r="L107" s="130"/>
     </row>
@@ -59763,19 +59782,19 @@
         <v>854</v>
       </c>
       <c r="E108" s="138" t="s">
-        <v>2620</v>
+        <v>2427</v>
       </c>
       <c r="F108" s="178">
         <v>1</v>
       </c>
       <c r="G108" s="285" t="s">
-        <v>2423</v>
+        <v>2428</v>
       </c>
       <c r="H108" s="178" t="s">
-        <v>2619</v>
+        <v>2415</v>
       </c>
       <c r="I108" s="285" t="s">
-        <v>2424</v>
+        <v>2429</v>
       </c>
       <c r="J108" s="166"/>
       <c r="K108" s="130"/>
@@ -59791,11 +59810,11 @@
         <v>2</v>
       </c>
       <c r="G109" s="285" t="s">
-        <v>2416</v>
+        <v>2418</v>
       </c>
       <c r="H109" s="178"/>
       <c r="I109" s="285" t="s">
-        <v>2425</v>
+        <v>2430</v>
       </c>
       <c r="J109" s="166"/>
       <c r="K109" s="130"/>
@@ -59811,13 +59830,13 @@
         <v>3</v>
       </c>
       <c r="G110" s="285" t="s">
-        <v>2426</v>
+        <v>2431</v>
       </c>
       <c r="H110" s="178" t="s">
-        <v>2427</v>
+        <v>2432</v>
       </c>
       <c r="I110" s="285" t="s">
-        <v>2428</v>
+        <v>2433</v>
       </c>
       <c r="J110" s="166"/>
       <c r="K110" s="130"/>
@@ -59833,11 +59852,11 @@
         <v>4</v>
       </c>
       <c r="G111" s="285" t="s">
-        <v>2429</v>
+        <v>2434</v>
       </c>
       <c r="H111" s="178"/>
       <c r="I111" s="285" t="s">
-        <v>2430</v>
+        <v>2435</v>
       </c>
       <c r="J111" s="166"/>
       <c r="K111" s="130"/>
@@ -59854,7 +59873,7 @@
         <v>863</v>
       </c>
       <c r="D112" s="130" t="s">
-        <v>2431</v>
+        <v>2436</v>
       </c>
       <c r="E112" s="130" t="s">
         <v>865</v>
@@ -59863,7 +59882,7 @@
         <v>1</v>
       </c>
       <c r="G112" s="166" t="s">
-        <v>2432</v>
+        <v>2437</v>
       </c>
       <c r="H112" s="175"/>
       <c r="I112" s="166" t="s">
@@ -59883,7 +59902,7 @@
         <v>2</v>
       </c>
       <c r="G113" s="166" t="s">
-        <v>2433</v>
+        <v>2438</v>
       </c>
       <c r="H113" s="175"/>
       <c r="I113" s="166" t="s">
@@ -59903,10 +59922,10 @@
         <v>3</v>
       </c>
       <c r="G114" s="166" t="s">
-        <v>2434</v>
+        <v>2439</v>
       </c>
       <c r="H114" s="175" t="s">
-        <v>2435</v>
+        <v>2440</v>
       </c>
       <c r="I114" s="166"/>
       <c r="J114" s="130"/>
@@ -59923,10 +59942,10 @@
         <v>4</v>
       </c>
       <c r="G115" s="166" t="s">
-        <v>2436</v>
+        <v>2441</v>
       </c>
       <c r="H115" s="175" t="s">
-        <v>2437</v>
+        <v>2442</v>
       </c>
       <c r="I115" s="166"/>
       <c r="J115" s="130"/>
@@ -59961,7 +59980,7 @@
         <v>6</v>
       </c>
       <c r="G117" s="166" t="s">
-        <v>2438</v>
+        <v>2443</v>
       </c>
       <c r="H117" s="175" t="s">
         <v>877</v>
@@ -59981,7 +60000,7 @@
         <v>7</v>
       </c>
       <c r="G118" s="166" t="s">
-        <v>2439</v>
+        <v>2444</v>
       </c>
       <c r="H118" s="247">
         <v>0.375</v>
@@ -60001,7 +60020,7 @@
         <v>8</v>
       </c>
       <c r="G119" s="166" t="s">
-        <v>2440</v>
+        <v>2445</v>
       </c>
       <c r="H119" s="175">
         <v>100000</v>
@@ -60021,7 +60040,7 @@
         <v>9</v>
       </c>
       <c r="G120" s="166" t="s">
-        <v>2441</v>
+        <v>2446</v>
       </c>
       <c r="H120" s="175">
         <v>1</v>
@@ -60041,7 +60060,7 @@
         <v>10</v>
       </c>
       <c r="G121" s="166" t="s">
-        <v>2442</v>
+        <v>2447</v>
       </c>
       <c r="H121" s="175"/>
       <c r="I121" s="166" t="s">
@@ -60062,7 +60081,7 @@
         <v>884</v>
       </c>
       <c r="D122" s="130" t="s">
-        <v>2443</v>
+        <v>2448</v>
       </c>
       <c r="E122" s="130" t="s">
         <v>886</v>
@@ -60071,7 +60090,7 @@
         <v>1</v>
       </c>
       <c r="G122" s="166" t="s">
-        <v>2444</v>
+        <v>2449</v>
       </c>
       <c r="H122" s="175"/>
       <c r="I122" s="130" t="s">
@@ -60091,7 +60110,7 @@
         <v>2</v>
       </c>
       <c r="G123" s="166" t="s">
-        <v>2445</v>
+        <v>2450</v>
       </c>
       <c r="H123" s="175"/>
       <c r="I123" s="130"/>
@@ -60109,10 +60128,10 @@
         <v>3</v>
       </c>
       <c r="G124" s="166" t="s">
-        <v>2446</v>
+        <v>2451</v>
       </c>
       <c r="H124" s="175" t="s">
-        <v>2447</v>
+        <v>2452</v>
       </c>
       <c r="I124" s="130"/>
       <c r="J124" s="130"/>
@@ -60129,10 +60148,10 @@
         <v>4</v>
       </c>
       <c r="G125" s="166" t="s">
-        <v>2448</v>
+        <v>2453</v>
       </c>
       <c r="H125" s="175" t="s">
-        <v>2449</v>
+        <v>2454</v>
       </c>
       <c r="I125" s="130"/>
       <c r="J125" s="130"/>
@@ -60149,7 +60168,7 @@
         <v>5</v>
       </c>
       <c r="G126" s="166" t="s">
-        <v>2450</v>
+        <v>2455</v>
       </c>
       <c r="H126" s="175" t="s">
         <v>877</v>
@@ -60187,7 +60206,7 @@
         <v>8</v>
       </c>
       <c r="G128" s="166" t="s">
-        <v>2451</v>
+        <v>2456</v>
       </c>
       <c r="H128" s="175">
         <v>100000</v>
@@ -60207,7 +60226,7 @@
         <v>9</v>
       </c>
       <c r="G129" s="166" t="s">
-        <v>2452</v>
+        <v>2457</v>
       </c>
       <c r="H129" s="175">
         <v>1</v>
@@ -60227,7 +60246,7 @@
         <v>10</v>
       </c>
       <c r="G130" s="166" t="s">
-        <v>2453</v>
+        <v>2458</v>
       </c>
       <c r="H130" s="175"/>
       <c r="I130" s="130"/>
@@ -60246,7 +60265,7 @@
         <v>900</v>
       </c>
       <c r="D131" s="130" t="s">
-        <v>2454</v>
+        <v>2459</v>
       </c>
       <c r="E131" s="130" t="s">
         <v>886</v>
@@ -60255,7 +60274,7 @@
         <v>1</v>
       </c>
       <c r="G131" s="166" t="s">
-        <v>2455</v>
+        <v>2460</v>
       </c>
       <c r="H131" s="175"/>
       <c r="I131" s="130" t="s">
@@ -60275,7 +60294,7 @@
         <v>2</v>
       </c>
       <c r="G132" s="166" t="s">
-        <v>2456</v>
+        <v>2461</v>
       </c>
       <c r="H132" s="175"/>
       <c r="I132" s="130"/>
@@ -60293,7 +60312,7 @@
         <v>3</v>
       </c>
       <c r="G133" s="166" t="s">
-        <v>2457</v>
+        <v>2462</v>
       </c>
       <c r="H133" s="175" t="s">
         <v>891</v>
@@ -60371,7 +60390,7 @@
         <v>7</v>
       </c>
       <c r="G137" s="166" t="s">
-        <v>2458</v>
+        <v>2463</v>
       </c>
       <c r="H137" s="175">
         <f>1</f>
@@ -60392,7 +60411,7 @@
         <v>8</v>
       </c>
       <c r="G138" s="166" t="s">
-        <v>2459</v>
+        <v>2464</v>
       </c>
       <c r="H138" s="175"/>
       <c r="I138" s="130"/>
@@ -60411,7 +60430,7 @@
         <v>911</v>
       </c>
       <c r="D139" s="130" t="s">
-        <v>2460</v>
+        <v>2465</v>
       </c>
       <c r="E139" s="130" t="s">
         <v>886</v>
@@ -60420,7 +60439,7 @@
         <v>1</v>
       </c>
       <c r="G139" s="166" t="s">
-        <v>2461</v>
+        <v>2466</v>
       </c>
       <c r="H139" s="175"/>
       <c r="I139" s="130" t="s">
@@ -60440,7 +60459,7 @@
         <v>2</v>
       </c>
       <c r="G140" s="166" t="s">
-        <v>2462</v>
+        <v>2467</v>
       </c>
       <c r="H140" s="175"/>
       <c r="I140" s="130"/>
@@ -60458,7 +60477,7 @@
         <v>3</v>
       </c>
       <c r="G141" s="166" t="s">
-        <v>2463</v>
+        <v>2468</v>
       </c>
       <c r="H141" s="175" t="s">
         <v>891</v>
@@ -60557,7 +60576,7 @@
         <v>8</v>
       </c>
       <c r="G146" s="166" t="s">
-        <v>2464</v>
+        <v>2469</v>
       </c>
       <c r="H146" s="175"/>
       <c r="I146" s="130"/>
@@ -60576,22 +60595,22 @@
         <v>921</v>
       </c>
       <c r="D147" s="138" t="s">
-        <v>2465</v>
+        <v>2470</v>
       </c>
       <c r="E147" s="138" t="s">
-        <v>2466</v>
+        <v>2471</v>
       </c>
       <c r="F147" s="178">
         <v>1</v>
       </c>
       <c r="G147" s="285" t="s">
-        <v>2467</v>
+        <v>2472</v>
       </c>
       <c r="H147" s="178" t="s">
-        <v>2468</v>
+        <v>2473</v>
       </c>
       <c r="I147" s="285" t="s">
-        <v>2469</v>
+        <v>2474</v>
       </c>
       <c r="J147" s="166"/>
       <c r="K147" s="130"/>
@@ -60607,11 +60626,11 @@
         <v>2</v>
       </c>
       <c r="G148" s="285" t="s">
-        <v>2470</v>
+        <v>2475</v>
       </c>
       <c r="H148" s="178"/>
       <c r="I148" s="285" t="s">
-        <v>2471</v>
+        <v>2476</v>
       </c>
       <c r="J148" s="166"/>
       <c r="K148" s="130"/>
@@ -60627,13 +60646,13 @@
         <v>3</v>
       </c>
       <c r="G149" s="285" t="s">
-        <v>2472</v>
+        <v>2477</v>
       </c>
       <c r="H149" s="178" t="s">
-        <v>2473</v>
+        <v>2478</v>
       </c>
       <c r="I149" s="285" t="s">
-        <v>2474</v>
+        <v>2479</v>
       </c>
       <c r="J149" s="166"/>
       <c r="K149" s="130"/>
@@ -60649,11 +60668,11 @@
         <v>4</v>
       </c>
       <c r="G150" s="285" t="s">
-        <v>2475</v>
+        <v>2480</v>
       </c>
       <c r="H150" s="178"/>
       <c r="I150" s="285" t="s">
-        <v>2476</v>
+        <v>2481</v>
       </c>
       <c r="J150" s="166"/>
       <c r="K150" s="130"/>
@@ -60669,11 +60688,11 @@
         <v>5</v>
       </c>
       <c r="G151" s="285" t="s">
-        <v>2477</v>
+        <v>2482</v>
       </c>
       <c r="H151" s="178"/>
       <c r="I151" s="285" t="s">
-        <v>2478</v>
+        <v>2483</v>
       </c>
       <c r="J151" s="166"/>
       <c r="K151" s="130"/>
@@ -60690,22 +60709,22 @@
         <v>932</v>
       </c>
       <c r="D152" s="138" t="s">
-        <v>2479</v>
+        <v>2484</v>
       </c>
       <c r="E152" s="138" t="s">
-        <v>2480</v>
+        <v>2485</v>
       </c>
       <c r="F152" s="178">
         <v>1</v>
       </c>
       <c r="G152" s="285" t="s">
-        <v>2481</v>
+        <v>2486</v>
       </c>
       <c r="H152" s="320" t="s">
-        <v>2482</v>
+        <v>2487</v>
       </c>
       <c r="I152" s="285" t="s">
-        <v>2483</v>
+        <v>2488</v>
       </c>
       <c r="J152" s="166"/>
       <c r="K152" s="130"/>
@@ -60721,13 +60740,13 @@
         <v>2</v>
       </c>
       <c r="G153" s="285" t="s">
-        <v>2484</v>
+        <v>2489</v>
       </c>
       <c r="H153" s="320" t="s">
-        <v>2485</v>
+        <v>2490</v>
       </c>
       <c r="I153" s="285" t="s">
-        <v>2486</v>
+        <v>2491</v>
       </c>
       <c r="J153" s="166"/>
       <c r="K153" s="130"/>
@@ -60743,11 +60762,11 @@
         <v>3</v>
       </c>
       <c r="G154" s="285" t="s">
-        <v>2487</v>
+        <v>2492</v>
       </c>
       <c r="H154" s="320"/>
       <c r="I154" s="285" t="s">
-        <v>2488</v>
+        <v>2493</v>
       </c>
       <c r="J154" s="166"/>
       <c r="K154" s="130"/>
@@ -61174,13 +61193,13 @@
         <v>1100</v>
       </c>
       <c r="H2" s="332" t="s">
-        <v>2489</v>
+        <v>2494</v>
       </c>
       <c r="I2" s="64" t="s">
         <v>1102</v>
       </c>
       <c r="J2" s="64" t="s">
-        <v>2490</v>
+        <v>2495</v>
       </c>
       <c r="K2" s="64" t="s">
         <v>2008</v>
@@ -61417,7 +61436,7 @@
         <v>13</v>
       </c>
       <c r="G14" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H14" s="288"/>
       <c r="I14" s="62"/>
@@ -61452,7 +61471,7 @@
         <v>1122</v>
       </c>
       <c r="J15" s="64" t="s">
-        <v>2492</v>
+        <v>2497</v>
       </c>
       <c r="K15" s="64" t="s">
         <v>2008</v>
@@ -61689,7 +61708,7 @@
         <v>13</v>
       </c>
       <c r="G27" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H27" s="288"/>
       <c r="I27" s="62"/>
@@ -61720,13 +61739,13 @@
         <v>1100</v>
       </c>
       <c r="H28" s="332" t="s">
-        <v>2493</v>
+        <v>2498</v>
       </c>
       <c r="I28" s="64" t="s">
         <v>1127</v>
       </c>
       <c r="J28" s="64" t="s">
-        <v>2494</v>
+        <v>2499</v>
       </c>
       <c r="K28" s="64" t="s">
         <v>2008</v>
@@ -61961,7 +61980,7 @@
         <v>13</v>
       </c>
       <c r="G40" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H40" s="288"/>
       <c r="I40" s="62"/>
@@ -61992,19 +62011,19 @@
         <v>1100</v>
       </c>
       <c r="H41" s="332" t="s">
-        <v>2495</v>
+        <v>2500</v>
       </c>
       <c r="I41" s="64" t="s">
         <v>1130</v>
       </c>
       <c r="J41" s="64" t="s">
-        <v>2496</v>
+        <v>2501</v>
       </c>
       <c r="K41" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L41" s="134" t="s">
-        <v>2497</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="14.4" customHeight="1">
@@ -62235,7 +62254,7 @@
         <v>13</v>
       </c>
       <c r="G53" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H53" s="288"/>
       <c r="I53" s="62"/>
@@ -62266,13 +62285,13 @@
         <v>1100</v>
       </c>
       <c r="H54" s="332" t="s">
-        <v>2498</v>
+        <v>2503</v>
       </c>
       <c r="I54" s="64" t="s">
         <v>1134</v>
       </c>
       <c r="J54" s="64" t="s">
-        <v>2499</v>
+        <v>2504</v>
       </c>
       <c r="K54" s="64" t="s">
         <v>2008</v>
@@ -62507,7 +62526,7 @@
         <v>13</v>
       </c>
       <c r="G66" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H66" s="288"/>
       <c r="I66" s="62"/>
@@ -62538,19 +62557,19 @@
         <v>1100</v>
       </c>
       <c r="H67" s="332" t="s">
-        <v>2500</v>
+        <v>2505</v>
       </c>
       <c r="I67" s="64" t="s">
         <v>1138</v>
       </c>
       <c r="J67" s="64" t="s">
-        <v>2501</v>
+        <v>2506</v>
       </c>
       <c r="K67" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L67" s="134" t="s">
-        <v>2502</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="68" spans="1:12" ht="14.4" customHeight="1">
@@ -62781,7 +62800,7 @@
         <v>13</v>
       </c>
       <c r="G79" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H79" s="288"/>
       <c r="I79" s="62"/>
@@ -62812,19 +62831,19 @@
         <v>1100</v>
       </c>
       <c r="H80" s="332" t="s">
-        <v>2503</v>
+        <v>2508</v>
       </c>
       <c r="I80" s="64" t="s">
         <v>1141</v>
       </c>
       <c r="J80" s="64" t="s">
-        <v>2504</v>
+        <v>2509</v>
       </c>
       <c r="K80" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L80" s="134" t="s">
-        <v>2505</v>
+        <v>2510</v>
       </c>
     </row>
     <row r="81" spans="1:12" ht="14.4" customHeight="1">
@@ -63055,7 +63074,7 @@
         <v>13</v>
       </c>
       <c r="G92" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H92" s="288"/>
       <c r="I92" s="62"/>
@@ -63086,13 +63105,13 @@
         <v>1100</v>
       </c>
       <c r="H93" s="332" t="s">
-        <v>2506</v>
+        <v>2511</v>
       </c>
       <c r="I93" s="64" t="s">
         <v>1145</v>
       </c>
       <c r="J93" s="64" t="s">
-        <v>2507</v>
+        <v>2512</v>
       </c>
       <c r="K93" s="64" t="s">
         <v>2008</v>
@@ -63327,7 +63346,7 @@
         <v>13</v>
       </c>
       <c r="G105" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H105" s="288"/>
       <c r="I105" s="62"/>
@@ -63358,13 +63377,13 @@
         <v>1100</v>
       </c>
       <c r="H106" s="332" t="s">
-        <v>2506</v>
+        <v>2511</v>
       </c>
       <c r="I106" s="64" t="s">
         <v>1149</v>
       </c>
       <c r="J106" s="64" t="s">
-        <v>2508</v>
+        <v>2513</v>
       </c>
       <c r="K106" s="64" t="s">
         <v>2008</v>
@@ -63599,7 +63618,7 @@
         <v>13</v>
       </c>
       <c r="G118" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H118" s="288"/>
       <c r="I118" s="62"/>
@@ -63630,13 +63649,13 @@
         <v>1100</v>
       </c>
       <c r="H119" s="332" t="s">
-        <v>2509</v>
+        <v>2514</v>
       </c>
       <c r="I119" s="64" t="s">
-        <v>2510</v>
+        <v>2515</v>
       </c>
       <c r="J119" s="64" t="s">
-        <v>2511</v>
+        <v>2516</v>
       </c>
       <c r="K119" s="64" t="s">
         <v>2008</v>
@@ -63871,7 +63890,7 @@
         <v>13</v>
       </c>
       <c r="G131" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H131" s="288"/>
       <c r="I131" s="62"/>
@@ -63902,13 +63921,13 @@
         <v>1100</v>
       </c>
       <c r="H132" s="332" t="s">
-        <v>2512</v>
+        <v>2517</v>
       </c>
       <c r="I132" s="64" t="s">
         <v>1160</v>
       </c>
       <c r="J132" s="64" t="s">
-        <v>2513</v>
+        <v>2518</v>
       </c>
       <c r="K132" s="64" t="s">
         <v>2008</v>
@@ -64143,7 +64162,7 @@
         <v>13</v>
       </c>
       <c r="G144" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H144" s="288"/>
       <c r="I144" s="62"/>
@@ -64162,7 +64181,7 @@
         <v>1164</v>
       </c>
       <c r="D145" s="64" t="s">
-        <v>2514</v>
+        <v>2519</v>
       </c>
       <c r="E145" s="64" t="s">
         <v>1099</v>
@@ -64174,19 +64193,19 @@
         <v>1100</v>
       </c>
       <c r="H145" s="332" t="s">
-        <v>2515</v>
+        <v>2520</v>
       </c>
       <c r="I145" s="64" t="s">
-        <v>2516</v>
+        <v>2521</v>
       </c>
       <c r="J145" s="64" t="s">
-        <v>2517</v>
+        <v>2522</v>
       </c>
       <c r="K145" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L145" s="134" t="s">
-        <v>2518</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="146" spans="1:12" ht="14.4" customHeight="1">
@@ -64419,7 +64438,7 @@
         <v>13</v>
       </c>
       <c r="G157" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H157" s="288"/>
       <c r="I157" s="62"/>
@@ -64450,13 +64469,13 @@
         <v>1100</v>
       </c>
       <c r="H158" s="332" t="s">
-        <v>2519</v>
+        <v>2524</v>
       </c>
       <c r="I158" s="64" t="s">
-        <v>2520</v>
+        <v>2525</v>
       </c>
       <c r="J158" s="64" t="s">
-        <v>2521</v>
+        <v>2526</v>
       </c>
       <c r="K158" s="64" t="s">
         <v>2008</v>
@@ -64691,7 +64710,7 @@
         <v>13</v>
       </c>
       <c r="G170" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H170" s="288"/>
       <c r="I170" s="62"/>
@@ -64722,13 +64741,13 @@
         <v>1100</v>
       </c>
       <c r="H171" s="332" t="s">
-        <v>2522</v>
+        <v>2527</v>
       </c>
       <c r="I171" s="64" t="s">
-        <v>2523</v>
+        <v>2528</v>
       </c>
       <c r="J171" s="64" t="s">
-        <v>2524</v>
+        <v>2529</v>
       </c>
       <c r="K171" s="64" t="s">
         <v>2008</v>
@@ -64963,7 +64982,7 @@
         <v>13</v>
       </c>
       <c r="G183" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H183" s="288"/>
       <c r="I183" s="62"/>
@@ -64995,16 +65014,16 @@
       </c>
       <c r="H184" s="332"/>
       <c r="I184" s="64" t="s">
-        <v>2525</v>
+        <v>2530</v>
       </c>
       <c r="J184" s="64" t="s">
-        <v>2526</v>
+        <v>2531</v>
       </c>
       <c r="K184" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L184" s="134" t="s">
-        <v>2527</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="185" spans="1:12" ht="14.4" customHeight="1">
@@ -65215,7 +65234,7 @@
         <v>13</v>
       </c>
       <c r="G196" s="288" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H196" s="332"/>
       <c r="I196" s="62"/>
@@ -65246,19 +65265,19 @@
         <v>1100</v>
       </c>
       <c r="H197" s="332" t="s">
-        <v>2528</v>
+        <v>2533</v>
       </c>
       <c r="I197" s="53" t="s">
         <v>1178</v>
       </c>
       <c r="J197" s="134" t="s">
-        <v>2529</v>
+        <v>2534</v>
       </c>
       <c r="K197" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L197" s="134" t="s">
-        <v>2530</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="198" spans="1:12">
@@ -65491,7 +65510,7 @@
         <v>13</v>
       </c>
       <c r="G209" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H209" s="293"/>
       <c r="I209" s="53"/>
@@ -65522,19 +65541,19 @@
         <v>1100</v>
       </c>
       <c r="H210" s="332" t="s">
-        <v>2531</v>
+        <v>2536</v>
       </c>
       <c r="I210" s="53" t="s">
         <v>1187</v>
       </c>
       <c r="J210" s="134" t="s">
-        <v>2532</v>
+        <v>2537</v>
       </c>
       <c r="K210" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L210" s="134" t="s">
-        <v>2533</v>
+        <v>2538</v>
       </c>
     </row>
     <row r="211" spans="1:12">
@@ -65767,7 +65786,7 @@
         <v>13</v>
       </c>
       <c r="G222" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H222" s="293"/>
       <c r="I222" s="53"/>
@@ -65786,7 +65805,7 @@
         <v>1189</v>
       </c>
       <c r="D223" s="53" t="s">
-        <v>2534</v>
+        <v>2539</v>
       </c>
       <c r="E223" s="136" t="s">
         <v>1176</v>
@@ -65798,19 +65817,19 @@
         <v>1100</v>
       </c>
       <c r="H223" s="332" t="s">
-        <v>2535</v>
+        <v>2540</v>
       </c>
       <c r="I223" s="134" t="s">
-        <v>2536</v>
+        <v>2541</v>
       </c>
       <c r="J223" s="134" t="s">
-        <v>2537</v>
+        <v>2542</v>
       </c>
       <c r="K223" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L223" s="134" t="s">
-        <v>2538</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="224" spans="1:12" ht="31.2" customHeight="1">
@@ -66043,7 +66062,7 @@
         <v>13</v>
       </c>
       <c r="G235" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H235" s="293"/>
       <c r="I235" s="132"/>
@@ -66074,19 +66093,19 @@
         <v>1100</v>
       </c>
       <c r="H236" s="332" t="s">
-        <v>2539</v>
+        <v>2544</v>
       </c>
       <c r="I236" s="134" t="s">
         <v>1197</v>
       </c>
       <c r="J236" s="134" t="s">
-        <v>2540</v>
+        <v>2545</v>
       </c>
       <c r="K236" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L236" s="134" t="s">
-        <v>2541</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="237" spans="1:12" ht="26.4" customHeight="1">
@@ -66319,7 +66338,7 @@
         <v>13</v>
       </c>
       <c r="G248" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H248" s="293"/>
       <c r="I248" s="132"/>
@@ -66350,19 +66369,19 @@
         <v>1100</v>
       </c>
       <c r="H249" s="332" t="s">
-        <v>2542</v>
+        <v>2547</v>
       </c>
       <c r="I249" s="134" t="s">
         <v>1203</v>
       </c>
       <c r="J249" s="134" t="s">
-        <v>2543</v>
+        <v>2548</v>
       </c>
       <c r="K249" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L249" s="134" t="s">
-        <v>2544</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="250" spans="1:12" ht="30" customHeight="1">
@@ -66538,7 +66557,7 @@
         <v>1115</v>
       </c>
       <c r="H258" s="288" t="s">
-        <v>2545</v>
+        <v>2550</v>
       </c>
       <c r="I258" s="133"/>
       <c r="J258" s="133"/>
@@ -66595,7 +66614,7 @@
         <v>13</v>
       </c>
       <c r="G261" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H261" s="293"/>
       <c r="I261" s="132"/>
@@ -66617,7 +66636,7 @@
         <v>1207</v>
       </c>
       <c r="E262" s="136" t="s">
-        <v>2546</v>
+        <v>2551</v>
       </c>
       <c r="F262" s="176">
         <v>1</v>
@@ -66632,13 +66651,13 @@
         <v>1210</v>
       </c>
       <c r="J262" s="134" t="s">
-        <v>2547</v>
+        <v>2552</v>
       </c>
       <c r="K262" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L262" s="134" t="s">
-        <v>2548</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="263" spans="1:12" ht="29.4" customHeight="1">
@@ -66871,7 +66890,7 @@
         <v>13</v>
       </c>
       <c r="G274" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H274" s="293"/>
       <c r="I274" s="132"/>
@@ -66902,19 +66921,19 @@
         <v>1100</v>
       </c>
       <c r="H275" s="332" t="s">
-        <v>2549</v>
+        <v>2554</v>
       </c>
       <c r="I275" s="135" t="s">
-        <v>2550</v>
+        <v>2555</v>
       </c>
       <c r="J275" s="64" t="s">
-        <v>2551</v>
+        <v>2556</v>
       </c>
       <c r="K275" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L275" s="134" t="s">
-        <v>2552</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="276" spans="1:12">
@@ -66987,7 +67006,7 @@
         <v>5</v>
       </c>
       <c r="G279" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H279" s="308" t="s">
         <v>1117</v>
@@ -67007,7 +67026,7 @@
         <v>6</v>
       </c>
       <c r="G280" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H280" s="308">
         <v>46123</v>
@@ -67127,7 +67146,7 @@
         <v>12</v>
       </c>
       <c r="G286" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H286" s="293"/>
       <c r="I286" s="135"/>
@@ -67162,13 +67181,13 @@
         <v>1122</v>
       </c>
       <c r="J287" s="64" t="s">
-        <v>2492</v>
+        <v>2497</v>
       </c>
       <c r="K287" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L287" s="134" t="s">
-        <v>2555</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="288" spans="1:12">
@@ -67241,7 +67260,7 @@
         <v>5</v>
       </c>
       <c r="G291" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H291" s="308" t="s">
         <v>1117</v>
@@ -67261,7 +67280,7 @@
         <v>6</v>
       </c>
       <c r="G292" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H292" s="308">
         <v>46123</v>
@@ -67381,7 +67400,7 @@
         <v>12</v>
       </c>
       <c r="G298" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I298" s="135"/>
       <c r="J298" s="62"/>
@@ -67411,19 +67430,19 @@
         <v>1100</v>
       </c>
       <c r="H299" s="332" t="s">
-        <v>2556</v>
+        <v>2561</v>
       </c>
       <c r="I299" s="135" t="s">
         <v>1127</v>
       </c>
       <c r="J299" s="64" t="s">
-        <v>2494</v>
+        <v>2499</v>
       </c>
       <c r="K299" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L299" s="134" t="s">
-        <v>2557</v>
+        <v>2562</v>
       </c>
     </row>
     <row r="300" spans="1:12">
@@ -67494,7 +67513,7 @@
         <v>5</v>
       </c>
       <c r="G303" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H303" s="308" t="s">
         <v>1117</v>
@@ -67514,7 +67533,7 @@
         <v>6</v>
       </c>
       <c r="G304" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H304" s="308">
         <v>46123</v>
@@ -67634,7 +67653,7 @@
         <v>12</v>
       </c>
       <c r="G310" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I310" s="135"/>
       <c r="J310" s="62"/>
@@ -67664,19 +67683,19 @@
         <v>1100</v>
       </c>
       <c r="H311" s="332" t="s">
-        <v>2558</v>
+        <v>2563</v>
       </c>
       <c r="I311" s="135" t="s">
         <v>1130</v>
       </c>
       <c r="J311" s="64" t="s">
-        <v>2559</v>
+        <v>2564</v>
       </c>
       <c r="K311" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L311" s="134" t="s">
-        <v>2560</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="312" spans="1:12">
@@ -67747,7 +67766,7 @@
         <v>5</v>
       </c>
       <c r="G315" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H315" s="308" t="s">
         <v>1117</v>
@@ -67767,7 +67786,7 @@
         <v>6</v>
       </c>
       <c r="G316" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H316" s="308">
         <v>46123</v>
@@ -67887,7 +67906,7 @@
         <v>12</v>
       </c>
       <c r="G322" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I322" s="135"/>
       <c r="J322" s="62"/>
@@ -67917,13 +67936,13 @@
         <v>1100</v>
       </c>
       <c r="H323" s="332" t="s">
-        <v>2561</v>
+        <v>2566</v>
       </c>
       <c r="I323" s="135" t="s">
         <v>1134</v>
       </c>
       <c r="J323" s="64" t="s">
-        <v>2499</v>
+        <v>2504</v>
       </c>
       <c r="K323" s="135" t="s">
         <v>2008</v>
@@ -68000,7 +68019,7 @@
         <v>5</v>
       </c>
       <c r="G327" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H327" s="308"/>
       <c r="I327" s="135"/>
@@ -68018,7 +68037,7 @@
         <v>6</v>
       </c>
       <c r="G328" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H328" s="308">
         <v>46123</v>
@@ -68138,7 +68157,7 @@
         <v>12</v>
       </c>
       <c r="G334" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I334" s="135"/>
       <c r="J334" s="62"/>
@@ -68168,19 +68187,19 @@
         <v>1100</v>
       </c>
       <c r="H335" s="332" t="s">
-        <v>2561</v>
+        <v>2566</v>
       </c>
       <c r="I335" s="135" t="s">
         <v>1138</v>
       </c>
       <c r="J335" s="64" t="s">
-        <v>2562</v>
+        <v>2567</v>
       </c>
       <c r="K335" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L335" s="134" t="s">
-        <v>2563</v>
+        <v>2568</v>
       </c>
     </row>
     <row r="336" spans="1:12">
@@ -68253,7 +68272,7 @@
         <v>5</v>
       </c>
       <c r="G339" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H339" s="308" t="s">
         <v>1117</v>
@@ -68273,7 +68292,7 @@
         <v>6</v>
       </c>
       <c r="G340" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H340" s="308"/>
       <c r="I340" s="135"/>
@@ -68391,7 +68410,7 @@
         <v>12</v>
       </c>
       <c r="G346" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I346" s="135"/>
       <c r="J346" s="62"/>
@@ -68409,7 +68428,7 @@
         <v>1254</v>
       </c>
       <c r="D347" s="135" t="s">
-        <v>2564</v>
+        <v>2569</v>
       </c>
       <c r="E347" s="135" t="s">
         <v>1099</v>
@@ -68421,19 +68440,19 @@
         <v>1100</v>
       </c>
       <c r="H347" s="332" t="s">
-        <v>2565</v>
+        <v>2570</v>
       </c>
       <c r="I347" s="135" t="s">
-        <v>2566</v>
+        <v>2571</v>
       </c>
       <c r="J347" s="64" t="s">
-        <v>2567</v>
+        <v>2572</v>
       </c>
       <c r="K347" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L347" s="134" t="s">
-        <v>2568</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="348" spans="1:12">
@@ -68506,7 +68525,7 @@
         <v>5</v>
       </c>
       <c r="G351" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H351" s="308" t="s">
         <v>1117</v>
@@ -68526,7 +68545,7 @@
         <v>6</v>
       </c>
       <c r="G352" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H352" s="308">
         <v>49410</v>
@@ -68644,7 +68663,7 @@
         <v>12</v>
       </c>
       <c r="G358" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H358" s="288"/>
       <c r="I358" s="135"/>
@@ -68675,13 +68694,13 @@
         <v>1100</v>
       </c>
       <c r="H359" s="332" t="s">
-        <v>2569</v>
+        <v>2574</v>
       </c>
       <c r="I359" s="135" t="s">
         <v>1145</v>
       </c>
       <c r="J359" s="64" t="s">
-        <v>2507</v>
+        <v>2512</v>
       </c>
       <c r="K359" s="135" t="s">
         <v>2008</v>
@@ -68758,7 +68777,7 @@
         <v>5</v>
       </c>
       <c r="G363" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H363" s="308" t="s">
         <v>1117</v>
@@ -68778,7 +68797,7 @@
         <v>6</v>
       </c>
       <c r="G364" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H364" s="308">
         <v>46123</v>
@@ -68896,7 +68915,7 @@
         <v>12</v>
       </c>
       <c r="G370" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I370" s="135"/>
       <c r="J370" s="62"/>
@@ -68926,13 +68945,13 @@
         <v>1100</v>
       </c>
       <c r="H371" s="332" t="s">
-        <v>2570</v>
+        <v>2575</v>
       </c>
       <c r="I371" s="135" t="s">
         <v>1149</v>
       </c>
       <c r="J371" s="64" t="s">
-        <v>2508</v>
+        <v>2513</v>
       </c>
       <c r="K371" s="135" t="s">
         <v>2008</v>
@@ -69009,7 +69028,7 @@
         <v>5</v>
       </c>
       <c r="G375" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H375" s="308" t="s">
         <v>1117</v>
@@ -69029,7 +69048,7 @@
         <v>6</v>
       </c>
       <c r="G376" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H376" s="308">
         <v>46123</v>
@@ -69147,7 +69166,7 @@
         <v>12</v>
       </c>
       <c r="G382" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I382" s="135"/>
       <c r="J382" s="62"/>
@@ -69165,7 +69184,7 @@
         <v>1257</v>
       </c>
       <c r="D383" s="135" t="s">
-        <v>2571</v>
+        <v>2576</v>
       </c>
       <c r="E383" s="135" t="s">
         <v>1099</v>
@@ -69177,19 +69196,19 @@
         <v>1100</v>
       </c>
       <c r="H383" s="332" t="s">
-        <v>2572</v>
+        <v>2577</v>
       </c>
       <c r="I383" s="135" t="s">
-        <v>2510</v>
+        <v>2515</v>
       </c>
       <c r="J383" s="64" t="s">
-        <v>2511</v>
+        <v>2516</v>
       </c>
       <c r="K383" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L383" s="134" t="s">
-        <v>2573</v>
+        <v>2578</v>
       </c>
     </row>
     <row r="384" spans="1:12">
@@ -69260,7 +69279,7 @@
         <v>5</v>
       </c>
       <c r="G387" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H387" s="308" t="s">
         <v>1117</v>
@@ -69280,7 +69299,7 @@
         <v>6</v>
       </c>
       <c r="G388" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H388" s="308">
         <v>46123</v>
@@ -69400,7 +69419,7 @@
         <v>12</v>
       </c>
       <c r="G394" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I394" s="135"/>
       <c r="J394" s="62"/>
@@ -69430,13 +69449,13 @@
         <v>1100</v>
       </c>
       <c r="H395" s="332" t="s">
-        <v>2574</v>
+        <v>2579</v>
       </c>
       <c r="I395" s="135" t="s">
         <v>1160</v>
       </c>
       <c r="J395" s="64" t="s">
-        <v>2513</v>
+        <v>2518</v>
       </c>
       <c r="K395" s="135" t="s">
         <v>2008</v>
@@ -69513,7 +69532,7 @@
         <v>5</v>
       </c>
       <c r="G399" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H399" s="308" t="s">
         <v>1117</v>
@@ -69533,7 +69552,7 @@
         <v>6</v>
       </c>
       <c r="G400" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H400" s="308">
         <v>46123</v>
@@ -69651,7 +69670,7 @@
         <v>12</v>
       </c>
       <c r="G406" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I406" s="135"/>
       <c r="J406" s="62"/>
@@ -69669,7 +69688,7 @@
         <v>1260</v>
       </c>
       <c r="D407" s="135" t="s">
-        <v>2575</v>
+        <v>2580</v>
       </c>
       <c r="E407" s="135" t="s">
         <v>1099</v>
@@ -69681,19 +69700,19 @@
         <v>1100</v>
       </c>
       <c r="H407" s="332" t="s">
-        <v>2576</v>
+        <v>2581</v>
       </c>
       <c r="I407" s="135" t="s">
-        <v>2577</v>
+        <v>2582</v>
       </c>
       <c r="J407" s="64" t="s">
-        <v>2578</v>
+        <v>2583</v>
       </c>
       <c r="K407" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L407" s="134" t="s">
-        <v>2579</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="408" spans="1:12">
@@ -69766,7 +69785,7 @@
         <v>5</v>
       </c>
       <c r="G411" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H411" s="308" t="s">
         <v>1117</v>
@@ -69786,7 +69805,7 @@
         <v>6</v>
       </c>
       <c r="G412" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H412" s="308">
         <v>46123</v>
@@ -69906,7 +69925,7 @@
         <v>12</v>
       </c>
       <c r="G418" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I418" s="135"/>
       <c r="J418" s="62"/>
@@ -69936,19 +69955,19 @@
         <v>1100</v>
       </c>
       <c r="H419" s="332" t="s">
-        <v>2580</v>
+        <v>2585</v>
       </c>
       <c r="I419" s="135" t="s">
-        <v>2520</v>
+        <v>2525</v>
       </c>
       <c r="J419" s="64" t="s">
-        <v>2521</v>
+        <v>2526</v>
       </c>
       <c r="K419" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L419" s="134" t="s">
-        <v>2581</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="420" spans="1:12">
@@ -70021,7 +70040,7 @@
         <v>5</v>
       </c>
       <c r="G423" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H423" s="308" t="s">
         <v>1117</v>
@@ -70041,7 +70060,7 @@
         <v>6</v>
       </c>
       <c r="G424" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H424" s="308">
         <v>46123</v>
@@ -70159,7 +70178,7 @@
         <v>12</v>
       </c>
       <c r="G430" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I430" s="135"/>
       <c r="J430" s="62"/>
@@ -70189,19 +70208,19 @@
         <v>1100</v>
       </c>
       <c r="H431" s="332" t="s">
-        <v>2582</v>
+        <v>2587</v>
       </c>
       <c r="I431" s="135" t="s">
-        <v>2523</v>
+        <v>2528</v>
       </c>
       <c r="J431" s="64" t="s">
-        <v>2524</v>
+        <v>2529</v>
       </c>
       <c r="K431" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L431" s="134" t="s">
-        <v>2583</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="432" spans="1:12">
@@ -70274,7 +70293,7 @@
         <v>5</v>
       </c>
       <c r="G435" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H435" s="308" t="s">
         <v>1117</v>
@@ -70294,7 +70313,7 @@
         <v>6</v>
       </c>
       <c r="G436" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H436" s="308">
         <v>46123</v>
@@ -70412,7 +70431,7 @@
         <v>12</v>
       </c>
       <c r="G442" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I442" s="135"/>
       <c r="J442" s="62"/>
@@ -70430,7 +70449,7 @@
         <v>1265</v>
       </c>
       <c r="D443" s="135" t="s">
-        <v>2584</v>
+        <v>2589</v>
       </c>
       <c r="E443" s="135" t="s">
         <v>1099</v>
@@ -70442,19 +70461,19 @@
         <v>1100</v>
       </c>
       <c r="H443" s="332" t="s">
-        <v>2576</v>
+        <v>2581</v>
       </c>
       <c r="I443" s="135" t="s">
-        <v>2585</v>
+        <v>2590</v>
       </c>
       <c r="J443" s="64" t="s">
-        <v>2586</v>
+        <v>2591</v>
       </c>
       <c r="K443" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L443" s="134" t="s">
-        <v>2587</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="444" spans="1:12">
@@ -70527,7 +70546,7 @@
         <v>5</v>
       </c>
       <c r="G447" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H447" s="308" t="s">
         <v>1117</v>
@@ -70547,7 +70566,7 @@
         <v>6</v>
       </c>
       <c r="G448" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H448" s="308">
         <v>46123</v>
@@ -70667,7 +70686,7 @@
         <v>12</v>
       </c>
       <c r="G454" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="I454" s="135"/>
       <c r="J454" s="62"/>
@@ -70685,10 +70704,10 @@
         <v>1212</v>
       </c>
       <c r="D455" s="136" t="s">
-        <v>2588</v>
+        <v>2593</v>
       </c>
       <c r="E455" s="136" t="s">
-        <v>2589</v>
+        <v>2594</v>
       </c>
       <c r="F455" s="176">
         <v>1</v>
@@ -70697,19 +70716,19 @@
         <v>1100</v>
       </c>
       <c r="H455" s="332" t="s">
-        <v>2590</v>
+        <v>2595</v>
       </c>
       <c r="I455" s="134" t="s">
-        <v>2591</v>
+        <v>2596</v>
       </c>
       <c r="J455" s="134" t="s">
-        <v>2592</v>
+        <v>2597</v>
       </c>
       <c r="K455" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L455" s="134" t="s">
-        <v>2593</v>
+        <v>2598</v>
       </c>
     </row>
     <row r="456" spans="1:12">
@@ -70782,7 +70801,7 @@
         <v>5</v>
       </c>
       <c r="G459" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H459" s="308" t="s">
         <v>1117</v>
@@ -70802,7 +70821,7 @@
         <v>6</v>
       </c>
       <c r="G460" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H460" s="308">
         <v>46123</v>
@@ -70865,7 +70884,7 @@
         <v>1115</v>
       </c>
       <c r="H463" s="318" t="s">
-        <v>2594</v>
+        <v>2599</v>
       </c>
       <c r="I463" s="133"/>
       <c r="J463" s="133"/>
@@ -70922,7 +70941,7 @@
         <v>12</v>
       </c>
       <c r="G466" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H466" s="293"/>
       <c r="I466" s="132"/>
@@ -70941,10 +70960,10 @@
         <v>1219</v>
       </c>
       <c r="D467" s="136" t="s">
-        <v>2595</v>
+        <v>2600</v>
       </c>
       <c r="E467" s="136" t="s">
-        <v>2596</v>
+        <v>2601</v>
       </c>
       <c r="F467" s="176">
         <v>1</v>
@@ -70953,19 +70972,19 @@
         <v>1100</v>
       </c>
       <c r="H467" s="332" t="s">
-        <v>2597</v>
+        <v>2602</v>
       </c>
       <c r="I467" s="134" t="s">
-        <v>2536</v>
+        <v>2541</v>
       </c>
       <c r="J467" s="134" t="s">
-        <v>2598</v>
+        <v>2603</v>
       </c>
       <c r="K467" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L467" s="134" t="s">
-        <v>2599</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="468" spans="1:12">
@@ -71038,7 +71057,7 @@
         <v>5</v>
       </c>
       <c r="G471" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H471" s="308" t="s">
         <v>1117</v>
@@ -71058,7 +71077,7 @@
         <v>6</v>
       </c>
       <c r="G472" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H472" s="308">
         <v>46123</v>
@@ -71178,7 +71197,7 @@
         <v>12</v>
       </c>
       <c r="G478" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H478" s="293"/>
       <c r="I478" s="132"/>
@@ -71197,10 +71216,10 @@
         <v>1225</v>
       </c>
       <c r="D479" s="136" t="s">
-        <v>2600</v>
+        <v>2605</v>
       </c>
       <c r="E479" s="136" t="s">
-        <v>2601</v>
+        <v>2606</v>
       </c>
       <c r="F479" s="176">
         <v>1</v>
@@ -71209,19 +71228,19 @@
         <v>1100</v>
       </c>
       <c r="H479" s="332" t="s">
-        <v>2602</v>
+        <v>2607</v>
       </c>
       <c r="I479" s="134" t="s">
-        <v>2603</v>
+        <v>2608</v>
       </c>
       <c r="J479" s="134" t="s">
-        <v>2604</v>
+        <v>2609</v>
       </c>
       <c r="K479" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L479" s="134" t="s">
-        <v>2605</v>
+        <v>2610</v>
       </c>
     </row>
     <row r="480" spans="1:12">
@@ -71237,7 +71256,7 @@
         <v>1103</v>
       </c>
       <c r="H480" s="332" t="s">
-        <v>2606</v>
+        <v>2611</v>
       </c>
       <c r="I480" s="133"/>
       <c r="J480" s="133"/>
@@ -71294,7 +71313,7 @@
         <v>5</v>
       </c>
       <c r="G483" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H483" s="308" t="s">
         <v>1117</v>
@@ -71314,7 +71333,7 @@
         <v>6</v>
       </c>
       <c r="G484" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H484" s="308">
         <v>46123</v>
@@ -71434,7 +71453,7 @@
         <v>12</v>
       </c>
       <c r="G490" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H490" s="293"/>
       <c r="I490" s="132"/>
@@ -71453,10 +71472,10 @@
         <v>1232</v>
       </c>
       <c r="D491" s="136" t="s">
-        <v>2607</v>
+        <v>2612</v>
       </c>
       <c r="E491" s="136" t="s">
-        <v>2601</v>
+        <v>2606</v>
       </c>
       <c r="F491" s="176">
         <v>1</v>
@@ -71465,19 +71484,19 @@
         <v>1100</v>
       </c>
       <c r="H491" s="292" t="s">
-        <v>2608</v>
+        <v>2613</v>
       </c>
       <c r="I491" s="134" t="s">
-        <v>2609</v>
+        <v>2614</v>
       </c>
       <c r="J491" s="134" t="s">
-        <v>2610</v>
+        <v>2615</v>
       </c>
       <c r="K491" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L491" s="134" t="s">
-        <v>2611</v>
+        <v>2616</v>
       </c>
     </row>
     <row r="492" spans="1:12" ht="15" customHeight="1">
@@ -71493,7 +71512,7 @@
         <v>1103</v>
       </c>
       <c r="H492" s="332" t="s">
-        <v>2612</v>
+        <v>2617</v>
       </c>
       <c r="I492" s="133"/>
       <c r="J492" s="133"/>
@@ -71550,7 +71569,7 @@
         <v>5</v>
       </c>
       <c r="G495" s="288" t="s">
-        <v>2553</v>
+        <v>2558</v>
       </c>
       <c r="H495" s="308" t="s">
         <v>1117</v>
@@ -71570,7 +71589,7 @@
         <v>6</v>
       </c>
       <c r="G496" s="288" t="s">
-        <v>2554</v>
+        <v>2559</v>
       </c>
       <c r="H496" s="308">
         <v>46123</v>
@@ -71690,7 +71709,7 @@
         <v>12</v>
       </c>
       <c r="G502" s="293" t="s">
-        <v>2491</v>
+        <v>2496</v>
       </c>
       <c r="H502" s="293"/>
       <c r="I502" s="132"/>
@@ -72081,13 +72100,13 @@
   <sheetData>
     <row r="2" spans="1:7">
       <c r="A2" s="192" t="s">
-        <v>2613</v>
+        <v>2618</v>
       </c>
       <c r="D2" s="192" t="s">
         <v>29</v>
       </c>
       <c r="G2" s="192" t="s">
-        <v>2614</v>
+        <v>2619</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -72095,7 +72114,7 @@
         <v>229</v>
       </c>
       <c r="D3" t="s">
-        <v>2615</v>
+        <v>2620</v>
       </c>
       <c r="G3" t="s">
         <v>244</v>
@@ -72106,7 +72125,7 @@
         <v>245</v>
       </c>
       <c r="D4" t="s">
-        <v>2616</v>
+        <v>2621</v>
       </c>
       <c r="G4" t="s">
         <v>234</v>
@@ -72114,10 +72133,10 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>2617</v>
+        <v>2622</v>
       </c>
       <c r="D5" t="s">
-        <v>2618</v>
+        <v>2623</v>
       </c>
       <c r="G5" t="s">
         <v>239</v>

</xml_diff>

<commit_message>
Edit the message is write in the actual result of TC_SHOW_02.
</commit_message>
<xml_diff>
--- a/sqa-testing-report/Data/DataTest.xlsx
+++ b/sqa-testing-report/Data/DataTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\sqa-testing-report\sqa-testing-report\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF902E4F-A249-4A8F-897B-2EC8CCD165BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{624B7ADA-E173-4879-989C-AF278ECCBDFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="664" activeTab="5" xr2:uid="{DC4DB269-603C-4B5B-A498-B166C8A18B92}"/>
   </bookViews>
@@ -9061,7 +9061,7 @@
     <t>Hệ thống tải dữ liệu của rạp và ngày đã chọn.</t>
   </si>
   <si>
-    <t>Đã check và tìm được phòng trống: Phòng 1 vào ngày 15/04/2026. Modal Thêm lịch chiếu đang mở.</t>
+    <t>Đã mở Modal, chọn ngày 16/04/2026 và phòng Phòng 1.</t>
   </si>
   <si>
     <t>Nhấn nút "+ Thêm lịch chiếu".</t>
@@ -9073,13 +9073,13 @@
     <t>Nhập đầy đủ thông tin hợp lệ vào Modal và nhấn "Lưu".</t>
   </si>
   <si>
-    <t>Phim: Khá; Phòng: phòng 3; Bắt đầu: 08:00 AM; Chi phí: 15000; Loại: 2 (Suất chiếu khuya)</t>
+    <t>Phim: Khá; Phòng: phòng 3; Bắt đầu: 08:00 AM; Chi phí: 15000; Loại: 1 (Suất chiếu thường)</t>
   </si>
   <si>
     <t>Thông báo "Thêm thành công" và Modal đóng lại.</t>
   </si>
   <si>
-    <t>Đã nhập đủ thông tin cho phòng Phòng 1, loại suất chiếu 1. Nhấn Lưu và Modal đóng lại.</t>
+    <t>Đã nhập thông tin và lưu thành công.</t>
   </si>
   <si>
     <t>Nhấn nút "Tải lịch chiếu" (Nút xanh dương).</t>
@@ -9088,10 +9088,7 @@
     <t>Lịch chiếu vừa tạo (Phim Khá, 08:00 AM) hiển thị đúng trên Timeline của phòng 3.</t>
   </si>
   <si>
-    <t>Lịch chiếu vừa tạo hiển thị chính xác trên Timeline của Phòng 1 lúc 08:00 AM.</t>
-  </si>
-  <si>
-    <t>Đăng nhập Admin; Đã có sẵn 01 suất chiếu tại Phòng 3 (khung giờ 08:00 AM - 11:51 PM).</t>
+    <t>Lịch chiếu hiển thị đúng trên Timeline.</t>
   </si>
   <si>
     <t>Tại màn hình Timeline, chọn đúng Rạp và Ngày có suất chiếu đã tồn tại.</t>
@@ -9104,9 +9101,6 @@
   </si>
   <si>
     <t>Nhập thông tin suất chiếu mới có thời gian bắt đầu trùng hoặc nằm trong khung giờ của suất chiếu cũ.</t>
-  </si>
-  <si>
-    <t>Phim: Conan; Phòng: Phòng 1; Bắt đầu: 10:00 PM; Chi phí: 100000; Loại: 1</t>
   </si>
   <si>
     <t>Các thông tin được điền vào Form thành công.</t>
@@ -10313,6 +10307,12 @@
   </si>
   <si>
     <t>Failed</t>
+  </si>
+  <si>
+    <t>Phim: Khá; Phòng: Phòng 1; Bắt đầu: 08:00 AM; Chi phí: 10000; Loại: 1</t>
+  </si>
+  <si>
+    <t>Đăng nhập Admin; Đã có sẵn 01 suất chiếu tại Phòng 1 (khung giờ 08:00 AM - 10:00 AM).</t>
   </si>
 </sst>
 </file>
@@ -59664,7 +59664,7 @@
       <c r="K103" s="135"/>
       <c r="L103" s="135"/>
     </row>
-    <row r="104" spans="1:12" ht="143.4" customHeight="1">
+    <row r="104" spans="1:12" ht="76.2" customHeight="1">
       <c r="A104" s="138">
         <v>33</v>
       </c>
@@ -59700,7 +59700,7 @@
       </c>
       <c r="L104" s="130"/>
     </row>
-    <row r="105" spans="1:12" ht="132" customHeight="1">
+    <row r="105" spans="1:12" ht="84" customHeight="1">
       <c r="A105" s="138"/>
       <c r="B105" s="138"/>
       <c r="C105" s="138"/>
@@ -59722,7 +59722,7 @@
       <c r="K105" s="130"/>
       <c r="L105" s="130"/>
     </row>
-    <row r="106" spans="1:12" ht="114.6" customHeight="1">
+    <row r="106" spans="1:12" ht="62.4" customHeight="1">
       <c r="A106" s="138"/>
       <c r="B106" s="138"/>
       <c r="C106" s="138"/>
@@ -59782,25 +59782,25 @@
         <v>854</v>
       </c>
       <c r="E108" s="138" t="s">
-        <v>2427</v>
+        <v>2623</v>
       </c>
       <c r="F108" s="178">
         <v>1</v>
       </c>
       <c r="G108" s="285" t="s">
-        <v>2428</v>
+        <v>2427</v>
       </c>
       <c r="H108" s="178" t="s">
         <v>2415</v>
       </c>
       <c r="I108" s="285" t="s">
-        <v>2429</v>
+        <v>2428</v>
       </c>
       <c r="J108" s="166"/>
       <c r="K108" s="130"/>
       <c r="L108" s="130"/>
     </row>
-    <row r="109" spans="1:12" ht="27" customHeight="1">
+    <row r="109" spans="1:12" ht="38.4" customHeight="1">
       <c r="A109" s="138"/>
       <c r="B109" s="138"/>
       <c r="C109" s="138"/>
@@ -59814,7 +59814,7 @@
       </c>
       <c r="H109" s="178"/>
       <c r="I109" s="285" t="s">
-        <v>2430</v>
+        <v>2429</v>
       </c>
       <c r="J109" s="166"/>
       <c r="K109" s="130"/>
@@ -59830,13 +59830,13 @@
         <v>3</v>
       </c>
       <c r="G110" s="285" t="s">
+        <v>2430</v>
+      </c>
+      <c r="H110" s="178" t="s">
+        <v>2622</v>
+      </c>
+      <c r="I110" s="285" t="s">
         <v>2431</v>
-      </c>
-      <c r="H110" s="178" t="s">
-        <v>2432</v>
-      </c>
-      <c r="I110" s="285" t="s">
-        <v>2433</v>
       </c>
       <c r="J110" s="166"/>
       <c r="K110" s="130"/>
@@ -59852,11 +59852,11 @@
         <v>4</v>
       </c>
       <c r="G111" s="285" t="s">
-        <v>2434</v>
+        <v>2432</v>
       </c>
       <c r="H111" s="178"/>
       <c r="I111" s="285" t="s">
-        <v>2435</v>
+        <v>2433</v>
       </c>
       <c r="J111" s="166"/>
       <c r="K111" s="130"/>
@@ -59873,7 +59873,7 @@
         <v>863</v>
       </c>
       <c r="D112" s="130" t="s">
-        <v>2436</v>
+        <v>2434</v>
       </c>
       <c r="E112" s="130" t="s">
         <v>865</v>
@@ -59882,7 +59882,7 @@
         <v>1</v>
       </c>
       <c r="G112" s="166" t="s">
-        <v>2437</v>
+        <v>2435</v>
       </c>
       <c r="H112" s="175"/>
       <c r="I112" s="166" t="s">
@@ -59902,7 +59902,7 @@
         <v>2</v>
       </c>
       <c r="G113" s="166" t="s">
-        <v>2438</v>
+        <v>2436</v>
       </c>
       <c r="H113" s="175"/>
       <c r="I113" s="166" t="s">
@@ -59922,10 +59922,10 @@
         <v>3</v>
       </c>
       <c r="G114" s="166" t="s">
-        <v>2439</v>
+        <v>2437</v>
       </c>
       <c r="H114" s="175" t="s">
-        <v>2440</v>
+        <v>2438</v>
       </c>
       <c r="I114" s="166"/>
       <c r="J114" s="130"/>
@@ -59942,10 +59942,10 @@
         <v>4</v>
       </c>
       <c r="G115" s="166" t="s">
-        <v>2441</v>
+        <v>2439</v>
       </c>
       <c r="H115" s="175" t="s">
-        <v>2442</v>
+        <v>2440</v>
       </c>
       <c r="I115" s="166"/>
       <c r="J115" s="130"/>
@@ -59980,7 +59980,7 @@
         <v>6</v>
       </c>
       <c r="G117" s="166" t="s">
-        <v>2443</v>
+        <v>2441</v>
       </c>
       <c r="H117" s="175" t="s">
         <v>877</v>
@@ -60000,7 +60000,7 @@
         <v>7</v>
       </c>
       <c r="G118" s="166" t="s">
-        <v>2444</v>
+        <v>2442</v>
       </c>
       <c r="H118" s="247">
         <v>0.375</v>
@@ -60020,7 +60020,7 @@
         <v>8</v>
       </c>
       <c r="G119" s="166" t="s">
-        <v>2445</v>
+        <v>2443</v>
       </c>
       <c r="H119" s="175">
         <v>100000</v>
@@ -60040,7 +60040,7 @@
         <v>9</v>
       </c>
       <c r="G120" s="166" t="s">
-        <v>2446</v>
+        <v>2444</v>
       </c>
       <c r="H120" s="175">
         <v>1</v>
@@ -60060,7 +60060,7 @@
         <v>10</v>
       </c>
       <c r="G121" s="166" t="s">
-        <v>2447</v>
+        <v>2445</v>
       </c>
       <c r="H121" s="175"/>
       <c r="I121" s="166" t="s">
@@ -60081,7 +60081,7 @@
         <v>884</v>
       </c>
       <c r="D122" s="130" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="E122" s="130" t="s">
         <v>886</v>
@@ -60090,7 +60090,7 @@
         <v>1</v>
       </c>
       <c r="G122" s="166" t="s">
-        <v>2449</v>
+        <v>2447</v>
       </c>
       <c r="H122" s="175"/>
       <c r="I122" s="130" t="s">
@@ -60110,7 +60110,7 @@
         <v>2</v>
       </c>
       <c r="G123" s="166" t="s">
-        <v>2450</v>
+        <v>2448</v>
       </c>
       <c r="H123" s="175"/>
       <c r="I123" s="130"/>
@@ -60128,10 +60128,10 @@
         <v>3</v>
       </c>
       <c r="G124" s="166" t="s">
-        <v>2451</v>
+        <v>2449</v>
       </c>
       <c r="H124" s="175" t="s">
-        <v>2452</v>
+        <v>2450</v>
       </c>
       <c r="I124" s="130"/>
       <c r="J124" s="130"/>
@@ -60148,10 +60148,10 @@
         <v>4</v>
       </c>
       <c r="G125" s="166" t="s">
-        <v>2453</v>
+        <v>2451</v>
       </c>
       <c r="H125" s="175" t="s">
-        <v>2454</v>
+        <v>2452</v>
       </c>
       <c r="I125" s="130"/>
       <c r="J125" s="130"/>
@@ -60168,7 +60168,7 @@
         <v>5</v>
       </c>
       <c r="G126" s="166" t="s">
-        <v>2455</v>
+        <v>2453</v>
       </c>
       <c r="H126" s="175" t="s">
         <v>877</v>
@@ -60206,7 +60206,7 @@
         <v>8</v>
       </c>
       <c r="G128" s="166" t="s">
-        <v>2456</v>
+        <v>2454</v>
       </c>
       <c r="H128" s="175">
         <v>100000</v>
@@ -60226,7 +60226,7 @@
         <v>9</v>
       </c>
       <c r="G129" s="166" t="s">
-        <v>2457</v>
+        <v>2455</v>
       </c>
       <c r="H129" s="175">
         <v>1</v>
@@ -60246,7 +60246,7 @@
         <v>10</v>
       </c>
       <c r="G130" s="166" t="s">
-        <v>2458</v>
+        <v>2456</v>
       </c>
       <c r="H130" s="175"/>
       <c r="I130" s="130"/>
@@ -60265,7 +60265,7 @@
         <v>900</v>
       </c>
       <c r="D131" s="130" t="s">
-        <v>2459</v>
+        <v>2457</v>
       </c>
       <c r="E131" s="130" t="s">
         <v>886</v>
@@ -60274,7 +60274,7 @@
         <v>1</v>
       </c>
       <c r="G131" s="166" t="s">
-        <v>2460</v>
+        <v>2458</v>
       </c>
       <c r="H131" s="175"/>
       <c r="I131" s="130" t="s">
@@ -60294,7 +60294,7 @@
         <v>2</v>
       </c>
       <c r="G132" s="166" t="s">
-        <v>2461</v>
+        <v>2459</v>
       </c>
       <c r="H132" s="175"/>
       <c r="I132" s="130"/>
@@ -60312,7 +60312,7 @@
         <v>3</v>
       </c>
       <c r="G133" s="166" t="s">
-        <v>2462</v>
+        <v>2460</v>
       </c>
       <c r="H133" s="175" t="s">
         <v>891</v>
@@ -60390,7 +60390,7 @@
         <v>7</v>
       </c>
       <c r="G137" s="166" t="s">
-        <v>2463</v>
+        <v>2461</v>
       </c>
       <c r="H137" s="175">
         <f>1</f>
@@ -60411,7 +60411,7 @@
         <v>8</v>
       </c>
       <c r="G138" s="166" t="s">
-        <v>2464</v>
+        <v>2462</v>
       </c>
       <c r="H138" s="175"/>
       <c r="I138" s="130"/>
@@ -60430,7 +60430,7 @@
         <v>911</v>
       </c>
       <c r="D139" s="130" t="s">
-        <v>2465</v>
+        <v>2463</v>
       </c>
       <c r="E139" s="130" t="s">
         <v>886</v>
@@ -60439,7 +60439,7 @@
         <v>1</v>
       </c>
       <c r="G139" s="166" t="s">
-        <v>2466</v>
+        <v>2464</v>
       </c>
       <c r="H139" s="175"/>
       <c r="I139" s="130" t="s">
@@ -60459,7 +60459,7 @@
         <v>2</v>
       </c>
       <c r="G140" s="166" t="s">
-        <v>2467</v>
+        <v>2465</v>
       </c>
       <c r="H140" s="175"/>
       <c r="I140" s="130"/>
@@ -60477,7 +60477,7 @@
         <v>3</v>
       </c>
       <c r="G141" s="166" t="s">
-        <v>2468</v>
+        <v>2466</v>
       </c>
       <c r="H141" s="175" t="s">
         <v>891</v>
@@ -60576,7 +60576,7 @@
         <v>8</v>
       </c>
       <c r="G146" s="166" t="s">
-        <v>2469</v>
+        <v>2467</v>
       </c>
       <c r="H146" s="175"/>
       <c r="I146" s="130"/>
@@ -60595,22 +60595,22 @@
         <v>921</v>
       </c>
       <c r="D147" s="138" t="s">
-        <v>2470</v>
+        <v>2468</v>
       </c>
       <c r="E147" s="138" t="s">
-        <v>2471</v>
+        <v>2469</v>
       </c>
       <c r="F147" s="178">
         <v>1</v>
       </c>
       <c r="G147" s="285" t="s">
+        <v>2470</v>
+      </c>
+      <c r="H147" s="178" t="s">
+        <v>2471</v>
+      </c>
+      <c r="I147" s="285" t="s">
         <v>2472</v>
-      </c>
-      <c r="H147" s="178" t="s">
-        <v>2473</v>
-      </c>
-      <c r="I147" s="285" t="s">
-        <v>2474</v>
       </c>
       <c r="J147" s="166"/>
       <c r="K147" s="130"/>
@@ -60626,11 +60626,11 @@
         <v>2</v>
       </c>
       <c r="G148" s="285" t="s">
-        <v>2475</v>
+        <v>2473</v>
       </c>
       <c r="H148" s="178"/>
       <c r="I148" s="285" t="s">
-        <v>2476</v>
+        <v>2474</v>
       </c>
       <c r="J148" s="166"/>
       <c r="K148" s="130"/>
@@ -60646,13 +60646,13 @@
         <v>3</v>
       </c>
       <c r="G149" s="285" t="s">
+        <v>2475</v>
+      </c>
+      <c r="H149" s="178" t="s">
+        <v>2476</v>
+      </c>
+      <c r="I149" s="285" t="s">
         <v>2477</v>
-      </c>
-      <c r="H149" s="178" t="s">
-        <v>2478</v>
-      </c>
-      <c r="I149" s="285" t="s">
-        <v>2479</v>
       </c>
       <c r="J149" s="166"/>
       <c r="K149" s="130"/>
@@ -60668,11 +60668,11 @@
         <v>4</v>
       </c>
       <c r="G150" s="285" t="s">
-        <v>2480</v>
+        <v>2478</v>
       </c>
       <c r="H150" s="178"/>
       <c r="I150" s="285" t="s">
-        <v>2481</v>
+        <v>2479</v>
       </c>
       <c r="J150" s="166"/>
       <c r="K150" s="130"/>
@@ -60688,11 +60688,11 @@
         <v>5</v>
       </c>
       <c r="G151" s="285" t="s">
-        <v>2482</v>
+        <v>2480</v>
       </c>
       <c r="H151" s="178"/>
       <c r="I151" s="285" t="s">
-        <v>2483</v>
+        <v>2481</v>
       </c>
       <c r="J151" s="166"/>
       <c r="K151" s="130"/>
@@ -60709,22 +60709,22 @@
         <v>932</v>
       </c>
       <c r="D152" s="138" t="s">
-        <v>2484</v>
+        <v>2482</v>
       </c>
       <c r="E152" s="138" t="s">
-        <v>2485</v>
+        <v>2483</v>
       </c>
       <c r="F152" s="178">
         <v>1</v>
       </c>
       <c r="G152" s="285" t="s">
+        <v>2484</v>
+      </c>
+      <c r="H152" s="320" t="s">
+        <v>2485</v>
+      </c>
+      <c r="I152" s="285" t="s">
         <v>2486</v>
-      </c>
-      <c r="H152" s="320" t="s">
-        <v>2487</v>
-      </c>
-      <c r="I152" s="285" t="s">
-        <v>2488</v>
       </c>
       <c r="J152" s="166"/>
       <c r="K152" s="130"/>
@@ -60740,13 +60740,13 @@
         <v>2</v>
       </c>
       <c r="G153" s="285" t="s">
+        <v>2487</v>
+      </c>
+      <c r="H153" s="320" t="s">
+        <v>2488</v>
+      </c>
+      <c r="I153" s="285" t="s">
         <v>2489</v>
-      </c>
-      <c r="H153" s="320" t="s">
-        <v>2490</v>
-      </c>
-      <c r="I153" s="285" t="s">
-        <v>2491</v>
       </c>
       <c r="J153" s="166"/>
       <c r="K153" s="130"/>
@@ -60762,11 +60762,11 @@
         <v>3</v>
       </c>
       <c r="G154" s="285" t="s">
-        <v>2492</v>
+        <v>2490</v>
       </c>
       <c r="H154" s="320"/>
       <c r="I154" s="285" t="s">
-        <v>2493</v>
+        <v>2491</v>
       </c>
       <c r="J154" s="166"/>
       <c r="K154" s="130"/>
@@ -61193,13 +61193,13 @@
         <v>1100</v>
       </c>
       <c r="H2" s="332" t="s">
-        <v>2494</v>
+        <v>2492</v>
       </c>
       <c r="I2" s="64" t="s">
         <v>1102</v>
       </c>
       <c r="J2" s="64" t="s">
-        <v>2495</v>
+        <v>2493</v>
       </c>
       <c r="K2" s="64" t="s">
         <v>2008</v>
@@ -61436,7 +61436,7 @@
         <v>13</v>
       </c>
       <c r="G14" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H14" s="288"/>
       <c r="I14" s="62"/>
@@ -61471,7 +61471,7 @@
         <v>1122</v>
       </c>
       <c r="J15" s="64" t="s">
-        <v>2497</v>
+        <v>2495</v>
       </c>
       <c r="K15" s="64" t="s">
         <v>2008</v>
@@ -61708,7 +61708,7 @@
         <v>13</v>
       </c>
       <c r="G27" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H27" s="288"/>
       <c r="I27" s="62"/>
@@ -61739,13 +61739,13 @@
         <v>1100</v>
       </c>
       <c r="H28" s="332" t="s">
-        <v>2498</v>
+        <v>2496</v>
       </c>
       <c r="I28" s="64" t="s">
         <v>1127</v>
       </c>
       <c r="J28" s="64" t="s">
-        <v>2499</v>
+        <v>2497</v>
       </c>
       <c r="K28" s="64" t="s">
         <v>2008</v>
@@ -61980,7 +61980,7 @@
         <v>13</v>
       </c>
       <c r="G40" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H40" s="288"/>
       <c r="I40" s="62"/>
@@ -62011,19 +62011,19 @@
         <v>1100</v>
       </c>
       <c r="H41" s="332" t="s">
-        <v>2500</v>
+        <v>2498</v>
       </c>
       <c r="I41" s="64" t="s">
         <v>1130</v>
       </c>
       <c r="J41" s="64" t="s">
-        <v>2501</v>
+        <v>2499</v>
       </c>
       <c r="K41" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L41" s="134" t="s">
-        <v>2502</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="14.4" customHeight="1">
@@ -62254,7 +62254,7 @@
         <v>13</v>
       </c>
       <c r="G53" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H53" s="288"/>
       <c r="I53" s="62"/>
@@ -62285,13 +62285,13 @@
         <v>1100</v>
       </c>
       <c r="H54" s="332" t="s">
-        <v>2503</v>
+        <v>2501</v>
       </c>
       <c r="I54" s="64" t="s">
         <v>1134</v>
       </c>
       <c r="J54" s="64" t="s">
-        <v>2504</v>
+        <v>2502</v>
       </c>
       <c r="K54" s="64" t="s">
         <v>2008</v>
@@ -62526,7 +62526,7 @@
         <v>13</v>
       </c>
       <c r="G66" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H66" s="288"/>
       <c r="I66" s="62"/>
@@ -62557,19 +62557,19 @@
         <v>1100</v>
       </c>
       <c r="H67" s="332" t="s">
-        <v>2505</v>
+        <v>2503</v>
       </c>
       <c r="I67" s="64" t="s">
         <v>1138</v>
       </c>
       <c r="J67" s="64" t="s">
-        <v>2506</v>
+        <v>2504</v>
       </c>
       <c r="K67" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L67" s="134" t="s">
-        <v>2507</v>
+        <v>2505</v>
       </c>
     </row>
     <row r="68" spans="1:12" ht="14.4" customHeight="1">
@@ -62800,7 +62800,7 @@
         <v>13</v>
       </c>
       <c r="G79" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H79" s="288"/>
       <c r="I79" s="62"/>
@@ -62831,19 +62831,19 @@
         <v>1100</v>
       </c>
       <c r="H80" s="332" t="s">
-        <v>2508</v>
+        <v>2506</v>
       </c>
       <c r="I80" s="64" t="s">
         <v>1141</v>
       </c>
       <c r="J80" s="64" t="s">
-        <v>2509</v>
+        <v>2507</v>
       </c>
       <c r="K80" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L80" s="134" t="s">
-        <v>2510</v>
+        <v>2508</v>
       </c>
     </row>
     <row r="81" spans="1:12" ht="14.4" customHeight="1">
@@ -63074,7 +63074,7 @@
         <v>13</v>
       </c>
       <c r="G92" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H92" s="288"/>
       <c r="I92" s="62"/>
@@ -63105,13 +63105,13 @@
         <v>1100</v>
       </c>
       <c r="H93" s="332" t="s">
-        <v>2511</v>
+        <v>2509</v>
       </c>
       <c r="I93" s="64" t="s">
         <v>1145</v>
       </c>
       <c r="J93" s="64" t="s">
-        <v>2512</v>
+        <v>2510</v>
       </c>
       <c r="K93" s="64" t="s">
         <v>2008</v>
@@ -63346,7 +63346,7 @@
         <v>13</v>
       </c>
       <c r="G105" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H105" s="288"/>
       <c r="I105" s="62"/>
@@ -63377,13 +63377,13 @@
         <v>1100</v>
       </c>
       <c r="H106" s="332" t="s">
-        <v>2511</v>
+        <v>2509</v>
       </c>
       <c r="I106" s="64" t="s">
         <v>1149</v>
       </c>
       <c r="J106" s="64" t="s">
-        <v>2513</v>
+        <v>2511</v>
       </c>
       <c r="K106" s="64" t="s">
         <v>2008</v>
@@ -63618,7 +63618,7 @@
         <v>13</v>
       </c>
       <c r="G118" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H118" s="288"/>
       <c r="I118" s="62"/>
@@ -63649,13 +63649,13 @@
         <v>1100</v>
       </c>
       <c r="H119" s="332" t="s">
+        <v>2512</v>
+      </c>
+      <c r="I119" s="64" t="s">
+        <v>2513</v>
+      </c>
+      <c r="J119" s="64" t="s">
         <v>2514</v>
-      </c>
-      <c r="I119" s="64" t="s">
-        <v>2515</v>
-      </c>
-      <c r="J119" s="64" t="s">
-        <v>2516</v>
       </c>
       <c r="K119" s="64" t="s">
         <v>2008</v>
@@ -63890,7 +63890,7 @@
         <v>13</v>
       </c>
       <c r="G131" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H131" s="288"/>
       <c r="I131" s="62"/>
@@ -63921,13 +63921,13 @@
         <v>1100</v>
       </c>
       <c r="H132" s="332" t="s">
-        <v>2517</v>
+        <v>2515</v>
       </c>
       <c r="I132" s="64" t="s">
         <v>1160</v>
       </c>
       <c r="J132" s="64" t="s">
-        <v>2518</v>
+        <v>2516</v>
       </c>
       <c r="K132" s="64" t="s">
         <v>2008</v>
@@ -64162,7 +64162,7 @@
         <v>13</v>
       </c>
       <c r="G144" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H144" s="288"/>
       <c r="I144" s="62"/>
@@ -64181,7 +64181,7 @@
         <v>1164</v>
       </c>
       <c r="D145" s="64" t="s">
-        <v>2519</v>
+        <v>2517</v>
       </c>
       <c r="E145" s="64" t="s">
         <v>1099</v>
@@ -64193,19 +64193,19 @@
         <v>1100</v>
       </c>
       <c r="H145" s="332" t="s">
+        <v>2518</v>
+      </c>
+      <c r="I145" s="64" t="s">
+        <v>2519</v>
+      </c>
+      <c r="J145" s="64" t="s">
         <v>2520</v>
-      </c>
-      <c r="I145" s="64" t="s">
-        <v>2521</v>
-      </c>
-      <c r="J145" s="64" t="s">
-        <v>2522</v>
       </c>
       <c r="K145" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L145" s="134" t="s">
-        <v>2523</v>
+        <v>2521</v>
       </c>
     </row>
     <row r="146" spans="1:12" ht="14.4" customHeight="1">
@@ -64438,7 +64438,7 @@
         <v>13</v>
       </c>
       <c r="G157" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H157" s="288"/>
       <c r="I157" s="62"/>
@@ -64469,13 +64469,13 @@
         <v>1100</v>
       </c>
       <c r="H158" s="332" t="s">
+        <v>2522</v>
+      </c>
+      <c r="I158" s="64" t="s">
+        <v>2523</v>
+      </c>
+      <c r="J158" s="64" t="s">
         <v>2524</v>
-      </c>
-      <c r="I158" s="64" t="s">
-        <v>2525</v>
-      </c>
-      <c r="J158" s="64" t="s">
-        <v>2526</v>
       </c>
       <c r="K158" s="64" t="s">
         <v>2008</v>
@@ -64710,7 +64710,7 @@
         <v>13</v>
       </c>
       <c r="G170" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H170" s="288"/>
       <c r="I170" s="62"/>
@@ -64741,13 +64741,13 @@
         <v>1100</v>
       </c>
       <c r="H171" s="332" t="s">
+        <v>2525</v>
+      </c>
+      <c r="I171" s="64" t="s">
+        <v>2526</v>
+      </c>
+      <c r="J171" s="64" t="s">
         <v>2527</v>
-      </c>
-      <c r="I171" s="64" t="s">
-        <v>2528</v>
-      </c>
-      <c r="J171" s="64" t="s">
-        <v>2529</v>
       </c>
       <c r="K171" s="64" t="s">
         <v>2008</v>
@@ -64982,7 +64982,7 @@
         <v>13</v>
       </c>
       <c r="G183" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H183" s="288"/>
       <c r="I183" s="62"/>
@@ -65014,16 +65014,16 @@
       </c>
       <c r="H184" s="332"/>
       <c r="I184" s="64" t="s">
-        <v>2530</v>
+        <v>2528</v>
       </c>
       <c r="J184" s="64" t="s">
-        <v>2531</v>
+        <v>2529</v>
       </c>
       <c r="K184" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L184" s="134" t="s">
-        <v>2532</v>
+        <v>2530</v>
       </c>
     </row>
     <row r="185" spans="1:12" ht="14.4" customHeight="1">
@@ -65234,7 +65234,7 @@
         <v>13</v>
       </c>
       <c r="G196" s="288" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H196" s="332"/>
       <c r="I196" s="62"/>
@@ -65265,19 +65265,19 @@
         <v>1100</v>
       </c>
       <c r="H197" s="332" t="s">
-        <v>2533</v>
+        <v>2531</v>
       </c>
       <c r="I197" s="53" t="s">
         <v>1178</v>
       </c>
       <c r="J197" s="134" t="s">
-        <v>2534</v>
+        <v>2532</v>
       </c>
       <c r="K197" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L197" s="134" t="s">
-        <v>2535</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="198" spans="1:12">
@@ -65510,7 +65510,7 @@
         <v>13</v>
       </c>
       <c r="G209" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H209" s="293"/>
       <c r="I209" s="53"/>
@@ -65541,19 +65541,19 @@
         <v>1100</v>
       </c>
       <c r="H210" s="332" t="s">
-        <v>2536</v>
+        <v>2534</v>
       </c>
       <c r="I210" s="53" t="s">
         <v>1187</v>
       </c>
       <c r="J210" s="134" t="s">
-        <v>2537</v>
+        <v>2535</v>
       </c>
       <c r="K210" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L210" s="134" t="s">
-        <v>2538</v>
+        <v>2536</v>
       </c>
     </row>
     <row r="211" spans="1:12">
@@ -65786,7 +65786,7 @@
         <v>13</v>
       </c>
       <c r="G222" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H222" s="293"/>
       <c r="I222" s="53"/>
@@ -65805,7 +65805,7 @@
         <v>1189</v>
       </c>
       <c r="D223" s="53" t="s">
-        <v>2539</v>
+        <v>2537</v>
       </c>
       <c r="E223" s="136" t="s">
         <v>1176</v>
@@ -65817,19 +65817,19 @@
         <v>1100</v>
       </c>
       <c r="H223" s="332" t="s">
+        <v>2538</v>
+      </c>
+      <c r="I223" s="134" t="s">
+        <v>2539</v>
+      </c>
+      <c r="J223" s="134" t="s">
         <v>2540</v>
-      </c>
-      <c r="I223" s="134" t="s">
-        <v>2541</v>
-      </c>
-      <c r="J223" s="134" t="s">
-        <v>2542</v>
       </c>
       <c r="K223" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L223" s="134" t="s">
-        <v>2543</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="224" spans="1:12" ht="31.2" customHeight="1">
@@ -66062,7 +66062,7 @@
         <v>13</v>
       </c>
       <c r="G235" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H235" s="293"/>
       <c r="I235" s="132"/>
@@ -66093,19 +66093,19 @@
         <v>1100</v>
       </c>
       <c r="H236" s="332" t="s">
-        <v>2544</v>
+        <v>2542</v>
       </c>
       <c r="I236" s="134" t="s">
         <v>1197</v>
       </c>
       <c r="J236" s="134" t="s">
-        <v>2545</v>
+        <v>2543</v>
       </c>
       <c r="K236" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L236" s="134" t="s">
-        <v>2546</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="237" spans="1:12" ht="26.4" customHeight="1">
@@ -66338,7 +66338,7 @@
         <v>13</v>
       </c>
       <c r="G248" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H248" s="293"/>
       <c r="I248" s="132"/>
@@ -66369,19 +66369,19 @@
         <v>1100</v>
       </c>
       <c r="H249" s="332" t="s">
-        <v>2547</v>
+        <v>2545</v>
       </c>
       <c r="I249" s="134" t="s">
         <v>1203</v>
       </c>
       <c r="J249" s="134" t="s">
-        <v>2548</v>
+        <v>2546</v>
       </c>
       <c r="K249" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L249" s="134" t="s">
-        <v>2549</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="250" spans="1:12" ht="30" customHeight="1">
@@ -66557,7 +66557,7 @@
         <v>1115</v>
       </c>
       <c r="H258" s="288" t="s">
-        <v>2550</v>
+        <v>2548</v>
       </c>
       <c r="I258" s="133"/>
       <c r="J258" s="133"/>
@@ -66614,7 +66614,7 @@
         <v>13</v>
       </c>
       <c r="G261" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H261" s="293"/>
       <c r="I261" s="132"/>
@@ -66636,7 +66636,7 @@
         <v>1207</v>
       </c>
       <c r="E262" s="136" t="s">
-        <v>2551</v>
+        <v>2549</v>
       </c>
       <c r="F262" s="176">
         <v>1</v>
@@ -66651,13 +66651,13 @@
         <v>1210</v>
       </c>
       <c r="J262" s="134" t="s">
-        <v>2552</v>
+        <v>2550</v>
       </c>
       <c r="K262" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L262" s="134" t="s">
-        <v>2553</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="263" spans="1:12" ht="29.4" customHeight="1">
@@ -66890,7 +66890,7 @@
         <v>13</v>
       </c>
       <c r="G274" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H274" s="293"/>
       <c r="I274" s="132"/>
@@ -66921,19 +66921,19 @@
         <v>1100</v>
       </c>
       <c r="H275" s="332" t="s">
+        <v>2552</v>
+      </c>
+      <c r="I275" s="135" t="s">
+        <v>2553</v>
+      </c>
+      <c r="J275" s="64" t="s">
         <v>2554</v>
-      </c>
-      <c r="I275" s="135" t="s">
-        <v>2555</v>
-      </c>
-      <c r="J275" s="64" t="s">
-        <v>2556</v>
       </c>
       <c r="K275" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L275" s="134" t="s">
-        <v>2557</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="276" spans="1:12">
@@ -67006,7 +67006,7 @@
         <v>5</v>
       </c>
       <c r="G279" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H279" s="308" t="s">
         <v>1117</v>
@@ -67026,7 +67026,7 @@
         <v>6</v>
       </c>
       <c r="G280" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H280" s="308">
         <v>46123</v>
@@ -67146,7 +67146,7 @@
         <v>12</v>
       </c>
       <c r="G286" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H286" s="293"/>
       <c r="I286" s="135"/>
@@ -67181,13 +67181,13 @@
         <v>1122</v>
       </c>
       <c r="J287" s="64" t="s">
-        <v>2497</v>
+        <v>2495</v>
       </c>
       <c r="K287" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L287" s="134" t="s">
-        <v>2560</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="288" spans="1:12">
@@ -67260,7 +67260,7 @@
         <v>5</v>
       </c>
       <c r="G291" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H291" s="308" t="s">
         <v>1117</v>
@@ -67280,7 +67280,7 @@
         <v>6</v>
       </c>
       <c r="G292" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H292" s="308">
         <v>46123</v>
@@ -67400,7 +67400,7 @@
         <v>12</v>
       </c>
       <c r="G298" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I298" s="135"/>
       <c r="J298" s="62"/>
@@ -67430,19 +67430,19 @@
         <v>1100</v>
       </c>
       <c r="H299" s="332" t="s">
-        <v>2561</v>
+        <v>2559</v>
       </c>
       <c r="I299" s="135" t="s">
         <v>1127</v>
       </c>
       <c r="J299" s="64" t="s">
-        <v>2499</v>
+        <v>2497</v>
       </c>
       <c r="K299" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L299" s="134" t="s">
-        <v>2562</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="300" spans="1:12">
@@ -67513,7 +67513,7 @@
         <v>5</v>
       </c>
       <c r="G303" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H303" s="308" t="s">
         <v>1117</v>
@@ -67533,7 +67533,7 @@
         <v>6</v>
       </c>
       <c r="G304" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H304" s="308">
         <v>46123</v>
@@ -67653,7 +67653,7 @@
         <v>12</v>
       </c>
       <c r="G310" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I310" s="135"/>
       <c r="J310" s="62"/>
@@ -67683,19 +67683,19 @@
         <v>1100</v>
       </c>
       <c r="H311" s="332" t="s">
-        <v>2563</v>
+        <v>2561</v>
       </c>
       <c r="I311" s="135" t="s">
         <v>1130</v>
       </c>
       <c r="J311" s="64" t="s">
-        <v>2564</v>
+        <v>2562</v>
       </c>
       <c r="K311" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L311" s="134" t="s">
-        <v>2565</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="312" spans="1:12">
@@ -67766,7 +67766,7 @@
         <v>5</v>
       </c>
       <c r="G315" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H315" s="308" t="s">
         <v>1117</v>
@@ -67786,7 +67786,7 @@
         <v>6</v>
       </c>
       <c r="G316" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H316" s="308">
         <v>46123</v>
@@ -67906,7 +67906,7 @@
         <v>12</v>
       </c>
       <c r="G322" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I322" s="135"/>
       <c r="J322" s="62"/>
@@ -67936,13 +67936,13 @@
         <v>1100</v>
       </c>
       <c r="H323" s="332" t="s">
-        <v>2566</v>
+        <v>2564</v>
       </c>
       <c r="I323" s="135" t="s">
         <v>1134</v>
       </c>
       <c r="J323" s="64" t="s">
-        <v>2504</v>
+        <v>2502</v>
       </c>
       <c r="K323" s="135" t="s">
         <v>2008</v>
@@ -68019,7 +68019,7 @@
         <v>5</v>
       </c>
       <c r="G327" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H327" s="308"/>
       <c r="I327" s="135"/>
@@ -68037,7 +68037,7 @@
         <v>6</v>
       </c>
       <c r="G328" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H328" s="308">
         <v>46123</v>
@@ -68157,7 +68157,7 @@
         <v>12</v>
       </c>
       <c r="G334" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I334" s="135"/>
       <c r="J334" s="62"/>
@@ -68187,19 +68187,19 @@
         <v>1100</v>
       </c>
       <c r="H335" s="332" t="s">
-        <v>2566</v>
+        <v>2564</v>
       </c>
       <c r="I335" s="135" t="s">
         <v>1138</v>
       </c>
       <c r="J335" s="64" t="s">
-        <v>2567</v>
+        <v>2565</v>
       </c>
       <c r="K335" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L335" s="134" t="s">
-        <v>2568</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="336" spans="1:12">
@@ -68272,7 +68272,7 @@
         <v>5</v>
       </c>
       <c r="G339" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H339" s="308" t="s">
         <v>1117</v>
@@ -68292,7 +68292,7 @@
         <v>6</v>
       </c>
       <c r="G340" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H340" s="308"/>
       <c r="I340" s="135"/>
@@ -68410,7 +68410,7 @@
         <v>12</v>
       </c>
       <c r="G346" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I346" s="135"/>
       <c r="J346" s="62"/>
@@ -68428,7 +68428,7 @@
         <v>1254</v>
       </c>
       <c r="D347" s="135" t="s">
-        <v>2569</v>
+        <v>2567</v>
       </c>
       <c r="E347" s="135" t="s">
         <v>1099</v>
@@ -68440,19 +68440,19 @@
         <v>1100</v>
       </c>
       <c r="H347" s="332" t="s">
+        <v>2568</v>
+      </c>
+      <c r="I347" s="135" t="s">
+        <v>2569</v>
+      </c>
+      <c r="J347" s="64" t="s">
         <v>2570</v>
-      </c>
-      <c r="I347" s="135" t="s">
-        <v>2571</v>
-      </c>
-      <c r="J347" s="64" t="s">
-        <v>2572</v>
       </c>
       <c r="K347" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L347" s="134" t="s">
-        <v>2573</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="348" spans="1:12">
@@ -68525,7 +68525,7 @@
         <v>5</v>
       </c>
       <c r="G351" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H351" s="308" t="s">
         <v>1117</v>
@@ -68545,7 +68545,7 @@
         <v>6</v>
       </c>
       <c r="G352" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H352" s="308">
         <v>49410</v>
@@ -68663,7 +68663,7 @@
         <v>12</v>
       </c>
       <c r="G358" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H358" s="288"/>
       <c r="I358" s="135"/>
@@ -68694,13 +68694,13 @@
         <v>1100</v>
       </c>
       <c r="H359" s="332" t="s">
-        <v>2574</v>
+        <v>2572</v>
       </c>
       <c r="I359" s="135" t="s">
         <v>1145</v>
       </c>
       <c r="J359" s="64" t="s">
-        <v>2512</v>
+        <v>2510</v>
       </c>
       <c r="K359" s="135" t="s">
         <v>2008</v>
@@ -68777,7 +68777,7 @@
         <v>5</v>
       </c>
       <c r="G363" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H363" s="308" t="s">
         <v>1117</v>
@@ -68797,7 +68797,7 @@
         <v>6</v>
       </c>
       <c r="G364" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H364" s="308">
         <v>46123</v>
@@ -68915,7 +68915,7 @@
         <v>12</v>
       </c>
       <c r="G370" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I370" s="135"/>
       <c r="J370" s="62"/>
@@ -68945,13 +68945,13 @@
         <v>1100</v>
       </c>
       <c r="H371" s="332" t="s">
-        <v>2575</v>
+        <v>2573</v>
       </c>
       <c r="I371" s="135" t="s">
         <v>1149</v>
       </c>
       <c r="J371" s="64" t="s">
-        <v>2513</v>
+        <v>2511</v>
       </c>
       <c r="K371" s="135" t="s">
         <v>2008</v>
@@ -69028,7 +69028,7 @@
         <v>5</v>
       </c>
       <c r="G375" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H375" s="308" t="s">
         <v>1117</v>
@@ -69048,7 +69048,7 @@
         <v>6</v>
       </c>
       <c r="G376" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H376" s="308">
         <v>46123</v>
@@ -69166,7 +69166,7 @@
         <v>12</v>
       </c>
       <c r="G382" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I382" s="135"/>
       <c r="J382" s="62"/>
@@ -69184,7 +69184,7 @@
         <v>1257</v>
       </c>
       <c r="D383" s="135" t="s">
-        <v>2576</v>
+        <v>2574</v>
       </c>
       <c r="E383" s="135" t="s">
         <v>1099</v>
@@ -69196,19 +69196,19 @@
         <v>1100</v>
       </c>
       <c r="H383" s="332" t="s">
-        <v>2577</v>
+        <v>2575</v>
       </c>
       <c r="I383" s="135" t="s">
-        <v>2515</v>
+        <v>2513</v>
       </c>
       <c r="J383" s="64" t="s">
-        <v>2516</v>
+        <v>2514</v>
       </c>
       <c r="K383" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L383" s="134" t="s">
-        <v>2578</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="384" spans="1:12">
@@ -69279,7 +69279,7 @@
         <v>5</v>
       </c>
       <c r="G387" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H387" s="308" t="s">
         <v>1117</v>
@@ -69299,7 +69299,7 @@
         <v>6</v>
       </c>
       <c r="G388" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H388" s="308">
         <v>46123</v>
@@ -69419,7 +69419,7 @@
         <v>12</v>
       </c>
       <c r="G394" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I394" s="135"/>
       <c r="J394" s="62"/>
@@ -69449,13 +69449,13 @@
         <v>1100</v>
       </c>
       <c r="H395" s="332" t="s">
-        <v>2579</v>
+        <v>2577</v>
       </c>
       <c r="I395" s="135" t="s">
         <v>1160</v>
       </c>
       <c r="J395" s="64" t="s">
-        <v>2518</v>
+        <v>2516</v>
       </c>
       <c r="K395" s="135" t="s">
         <v>2008</v>
@@ -69532,7 +69532,7 @@
         <v>5</v>
       </c>
       <c r="G399" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H399" s="308" t="s">
         <v>1117</v>
@@ -69552,7 +69552,7 @@
         <v>6</v>
       </c>
       <c r="G400" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H400" s="308">
         <v>46123</v>
@@ -69670,7 +69670,7 @@
         <v>12</v>
       </c>
       <c r="G406" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I406" s="135"/>
       <c r="J406" s="62"/>
@@ -69688,7 +69688,7 @@
         <v>1260</v>
       </c>
       <c r="D407" s="135" t="s">
-        <v>2580</v>
+        <v>2578</v>
       </c>
       <c r="E407" s="135" t="s">
         <v>1099</v>
@@ -69700,19 +69700,19 @@
         <v>1100</v>
       </c>
       <c r="H407" s="332" t="s">
+        <v>2579</v>
+      </c>
+      <c r="I407" s="135" t="s">
+        <v>2580</v>
+      </c>
+      <c r="J407" s="64" t="s">
         <v>2581</v>
-      </c>
-      <c r="I407" s="135" t="s">
-        <v>2582</v>
-      </c>
-      <c r="J407" s="64" t="s">
-        <v>2583</v>
       </c>
       <c r="K407" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L407" s="134" t="s">
-        <v>2584</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="408" spans="1:12">
@@ -69785,7 +69785,7 @@
         <v>5</v>
       </c>
       <c r="G411" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H411" s="308" t="s">
         <v>1117</v>
@@ -69805,7 +69805,7 @@
         <v>6</v>
       </c>
       <c r="G412" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H412" s="308">
         <v>46123</v>
@@ -69925,7 +69925,7 @@
         <v>12</v>
       </c>
       <c r="G418" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I418" s="135"/>
       <c r="J418" s="62"/>
@@ -69955,19 +69955,19 @@
         <v>1100</v>
       </c>
       <c r="H419" s="332" t="s">
-        <v>2585</v>
+        <v>2583</v>
       </c>
       <c r="I419" s="135" t="s">
-        <v>2525</v>
+        <v>2523</v>
       </c>
       <c r="J419" s="64" t="s">
-        <v>2526</v>
+        <v>2524</v>
       </c>
       <c r="K419" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L419" s="134" t="s">
-        <v>2586</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="420" spans="1:12">
@@ -70040,7 +70040,7 @@
         <v>5</v>
       </c>
       <c r="G423" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H423" s="308" t="s">
         <v>1117</v>
@@ -70060,7 +70060,7 @@
         <v>6</v>
       </c>
       <c r="G424" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H424" s="308">
         <v>46123</v>
@@ -70178,7 +70178,7 @@
         <v>12</v>
       </c>
       <c r="G430" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I430" s="135"/>
       <c r="J430" s="62"/>
@@ -70208,19 +70208,19 @@
         <v>1100</v>
       </c>
       <c r="H431" s="332" t="s">
-        <v>2587</v>
+        <v>2585</v>
       </c>
       <c r="I431" s="135" t="s">
-        <v>2528</v>
+        <v>2526</v>
       </c>
       <c r="J431" s="64" t="s">
-        <v>2529</v>
+        <v>2527</v>
       </c>
       <c r="K431" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L431" s="134" t="s">
-        <v>2588</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="432" spans="1:12">
@@ -70293,7 +70293,7 @@
         <v>5</v>
       </c>
       <c r="G435" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H435" s="308" t="s">
         <v>1117</v>
@@ -70313,7 +70313,7 @@
         <v>6</v>
       </c>
       <c r="G436" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H436" s="308">
         <v>46123</v>
@@ -70431,7 +70431,7 @@
         <v>12</v>
       </c>
       <c r="G442" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I442" s="135"/>
       <c r="J442" s="62"/>
@@ -70449,7 +70449,7 @@
         <v>1265</v>
       </c>
       <c r="D443" s="135" t="s">
-        <v>2589</v>
+        <v>2587</v>
       </c>
       <c r="E443" s="135" t="s">
         <v>1099</v>
@@ -70461,19 +70461,19 @@
         <v>1100</v>
       </c>
       <c r="H443" s="332" t="s">
-        <v>2581</v>
+        <v>2579</v>
       </c>
       <c r="I443" s="135" t="s">
-        <v>2590</v>
+        <v>2588</v>
       </c>
       <c r="J443" s="64" t="s">
-        <v>2591</v>
+        <v>2589</v>
       </c>
       <c r="K443" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L443" s="134" t="s">
-        <v>2592</v>
+        <v>2590</v>
       </c>
     </row>
     <row r="444" spans="1:12">
@@ -70546,7 +70546,7 @@
         <v>5</v>
       </c>
       <c r="G447" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H447" s="308" t="s">
         <v>1117</v>
@@ -70566,7 +70566,7 @@
         <v>6</v>
       </c>
       <c r="G448" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H448" s="308">
         <v>46123</v>
@@ -70686,7 +70686,7 @@
         <v>12</v>
       </c>
       <c r="G454" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="I454" s="135"/>
       <c r="J454" s="62"/>
@@ -70704,10 +70704,10 @@
         <v>1212</v>
       </c>
       <c r="D455" s="136" t="s">
-        <v>2593</v>
+        <v>2591</v>
       </c>
       <c r="E455" s="136" t="s">
-        <v>2594</v>
+        <v>2592</v>
       </c>
       <c r="F455" s="176">
         <v>1</v>
@@ -70716,19 +70716,19 @@
         <v>1100</v>
       </c>
       <c r="H455" s="332" t="s">
+        <v>2593</v>
+      </c>
+      <c r="I455" s="134" t="s">
+        <v>2594</v>
+      </c>
+      <c r="J455" s="134" t="s">
         <v>2595</v>
-      </c>
-      <c r="I455" s="134" t="s">
-        <v>2596</v>
-      </c>
-      <c r="J455" s="134" t="s">
-        <v>2597</v>
       </c>
       <c r="K455" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L455" s="134" t="s">
-        <v>2598</v>
+        <v>2596</v>
       </c>
     </row>
     <row r="456" spans="1:12">
@@ -70801,7 +70801,7 @@
         <v>5</v>
       </c>
       <c r="G459" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H459" s="308" t="s">
         <v>1117</v>
@@ -70821,7 +70821,7 @@
         <v>6</v>
       </c>
       <c r="G460" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H460" s="308">
         <v>46123</v>
@@ -70884,7 +70884,7 @@
         <v>1115</v>
       </c>
       <c r="H463" s="318" t="s">
-        <v>2599</v>
+        <v>2597</v>
       </c>
       <c r="I463" s="133"/>
       <c r="J463" s="133"/>
@@ -70941,7 +70941,7 @@
         <v>12</v>
       </c>
       <c r="G466" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H466" s="293"/>
       <c r="I466" s="132"/>
@@ -70960,10 +70960,10 @@
         <v>1219</v>
       </c>
       <c r="D467" s="136" t="s">
-        <v>2600</v>
+        <v>2598</v>
       </c>
       <c r="E467" s="136" t="s">
-        <v>2601</v>
+        <v>2599</v>
       </c>
       <c r="F467" s="176">
         <v>1</v>
@@ -70972,19 +70972,19 @@
         <v>1100</v>
       </c>
       <c r="H467" s="332" t="s">
-        <v>2602</v>
+        <v>2600</v>
       </c>
       <c r="I467" s="134" t="s">
-        <v>2541</v>
+        <v>2539</v>
       </c>
       <c r="J467" s="134" t="s">
-        <v>2603</v>
+        <v>2601</v>
       </c>
       <c r="K467" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L467" s="134" t="s">
-        <v>2604</v>
+        <v>2602</v>
       </c>
     </row>
     <row r="468" spans="1:12">
@@ -71057,7 +71057,7 @@
         <v>5</v>
       </c>
       <c r="G471" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H471" s="308" t="s">
         <v>1117</v>
@@ -71077,7 +71077,7 @@
         <v>6</v>
       </c>
       <c r="G472" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H472" s="308">
         <v>46123</v>
@@ -71197,7 +71197,7 @@
         <v>12</v>
       </c>
       <c r="G478" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H478" s="293"/>
       <c r="I478" s="132"/>
@@ -71216,10 +71216,10 @@
         <v>1225</v>
       </c>
       <c r="D479" s="136" t="s">
-        <v>2605</v>
+        <v>2603</v>
       </c>
       <c r="E479" s="136" t="s">
-        <v>2606</v>
+        <v>2604</v>
       </c>
       <c r="F479" s="176">
         <v>1</v>
@@ -71228,19 +71228,19 @@
         <v>1100</v>
       </c>
       <c r="H479" s="332" t="s">
+        <v>2605</v>
+      </c>
+      <c r="I479" s="134" t="s">
+        <v>2606</v>
+      </c>
+      <c r="J479" s="134" t="s">
         <v>2607</v>
-      </c>
-      <c r="I479" s="134" t="s">
-        <v>2608</v>
-      </c>
-      <c r="J479" s="134" t="s">
-        <v>2609</v>
       </c>
       <c r="K479" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L479" s="134" t="s">
-        <v>2610</v>
+        <v>2608</v>
       </c>
     </row>
     <row r="480" spans="1:12">
@@ -71256,7 +71256,7 @@
         <v>1103</v>
       </c>
       <c r="H480" s="332" t="s">
-        <v>2611</v>
+        <v>2609</v>
       </c>
       <c r="I480" s="133"/>
       <c r="J480" s="133"/>
@@ -71313,7 +71313,7 @@
         <v>5</v>
       </c>
       <c r="G483" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H483" s="308" t="s">
         <v>1117</v>
@@ -71333,7 +71333,7 @@
         <v>6</v>
       </c>
       <c r="G484" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H484" s="308">
         <v>46123</v>
@@ -71453,7 +71453,7 @@
         <v>12</v>
       </c>
       <c r="G490" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H490" s="293"/>
       <c r="I490" s="132"/>
@@ -71472,10 +71472,10 @@
         <v>1232</v>
       </c>
       <c r="D491" s="136" t="s">
-        <v>2612</v>
+        <v>2610</v>
       </c>
       <c r="E491" s="136" t="s">
-        <v>2606</v>
+        <v>2604</v>
       </c>
       <c r="F491" s="176">
         <v>1</v>
@@ -71484,19 +71484,19 @@
         <v>1100</v>
       </c>
       <c r="H491" s="292" t="s">
+        <v>2611</v>
+      </c>
+      <c r="I491" s="134" t="s">
+        <v>2612</v>
+      </c>
+      <c r="J491" s="134" t="s">
         <v>2613</v>
-      </c>
-      <c r="I491" s="134" t="s">
-        <v>2614</v>
-      </c>
-      <c r="J491" s="134" t="s">
-        <v>2615</v>
       </c>
       <c r="K491" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L491" s="134" t="s">
-        <v>2616</v>
+        <v>2614</v>
       </c>
     </row>
     <row r="492" spans="1:12" ht="15" customHeight="1">
@@ -71512,7 +71512,7 @@
         <v>1103</v>
       </c>
       <c r="H492" s="332" t="s">
-        <v>2617</v>
+        <v>2615</v>
       </c>
       <c r="I492" s="133"/>
       <c r="J492" s="133"/>
@@ -71569,7 +71569,7 @@
         <v>5</v>
       </c>
       <c r="G495" s="288" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
       <c r="H495" s="308" t="s">
         <v>1117</v>
@@ -71589,7 +71589,7 @@
         <v>6</v>
       </c>
       <c r="G496" s="288" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
       <c r="H496" s="308">
         <v>46123</v>
@@ -71709,7 +71709,7 @@
         <v>12</v>
       </c>
       <c r="G502" s="293" t="s">
-        <v>2496</v>
+        <v>2494</v>
       </c>
       <c r="H502" s="293"/>
       <c r="I502" s="132"/>
@@ -72100,13 +72100,13 @@
   <sheetData>
     <row r="2" spans="1:7">
       <c r="A2" s="192" t="s">
-        <v>2618</v>
+        <v>2616</v>
       </c>
       <c r="D2" s="192" t="s">
         <v>29</v>
       </c>
       <c r="G2" s="192" t="s">
-        <v>2619</v>
+        <v>2617</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -72114,7 +72114,7 @@
         <v>229</v>
       </c>
       <c r="D3" t="s">
-        <v>2620</v>
+        <v>2618</v>
       </c>
       <c r="G3" t="s">
         <v>244</v>
@@ -72125,7 +72125,7 @@
         <v>245</v>
       </c>
       <c r="D4" t="s">
-        <v>2621</v>
+        <v>2619</v>
       </c>
       <c r="G4" t="s">
         <v>234</v>
@@ -72133,10 +72133,10 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>2622</v>
+        <v>2620</v>
       </c>
       <c r="D5" t="s">
-        <v>2623</v>
+        <v>2621</v>
       </c>
       <c r="G5" t="s">
         <v>239</v>

</xml_diff>

<commit_message>
Test: Complete testcase TC_SHOW_03
</commit_message>
<xml_diff>
--- a/sqa-testing-report/Data/DataTest.xlsx
+++ b/sqa-testing-report/Data/DataTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\sqa-testing-report\sqa-testing-report\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{624B7ADA-E173-4879-989C-AF278ECCBDFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A37C33B-4B6A-45E9-92C9-59EB536566FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="664" activeTab="5" xr2:uid="{DC4DB269-603C-4B5B-A498-B166C8A18B92}"/>
   </bookViews>
@@ -164,7 +164,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7229" uniqueCount="2624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7234" uniqueCount="2628">
   <si>
     <t>GUI &amp; FUNCTIONAL TEST CASES</t>
   </si>
@@ -9091,25 +9091,43 @@
     <t>Lịch chiếu hiển thị đúng trên Timeline.</t>
   </si>
   <si>
+    <t>Đăng nhập Admin; Đã có sẵn 01 suất chiếu tại Phòng 3 (khung giờ 08:00 AM - 10:00 AM).</t>
+  </si>
+  <si>
     <t>Tại màn hình Timeline, chọn đúng Rạp và Ngày có suất chiếu đã tồn tại.</t>
   </si>
   <si>
+    <t>Rạp: Galaxy Bến Tre; Ngày: 16/04/2026</t>
+  </si>
+  <si>
     <t>Hệ thống tải dữ liệu Timeline của rạp và ngày đã chọn.</t>
   </si>
   <si>
+    <t>Mở Modal, chọn ngày 16/04/2026 và phòng đã có lịch (Phòng 1).</t>
+  </si>
+  <si>
     <t>Hiển thị Modal "Thêm lịch chiếu".</t>
   </si>
   <si>
     <t>Nhập thông tin suất chiếu mới có thời gian bắt đầu trùng hoặc nằm trong khung giờ của suất chiếu cũ.</t>
   </si>
   <si>
+    <t>Phim: Khá; Phòng: Phòng 3; Bắt đầu: 08:00 AM; Chi phí: 10000; Loại: 1</t>
+  </si>
+  <si>
     <t>Các thông tin được điền vào Form thành công.</t>
   </si>
   <si>
+    <t>Đã nhập thông tin trùng lặp và lưu thành công.</t>
+  </si>
+  <si>
     <t>Nhấn nút "Lưu".</t>
   </si>
   <si>
     <t>Hiển thị thông báo lỗi: "Trùng lịch chiếu" (hoặc cảnh báo khung giờ đã có suất chiếu); Modal không đóng.</t>
+  </si>
+  <si>
+    <t>Không tạo thêm suất chiếu trùng. Số lượng giữ nguyên.</t>
   </si>
   <si>
     <r>
@@ -10307,12 +10325,6 @@
   </si>
   <si>
     <t>Failed</t>
-  </si>
-  <si>
-    <t>Phim: Khá; Phòng: Phòng 1; Bắt đầu: 08:00 AM; Chi phí: 10000; Loại: 1</t>
-  </si>
-  <si>
-    <t>Đăng nhập Admin; Đã có sẵn 01 suất chiếu tại Phòng 1 (khung giờ 08:00 AM - 10:00 AM).</t>
   </si>
 </sst>
 </file>
@@ -59768,7 +59780,7 @@
       <c r="K107" s="130"/>
       <c r="L107" s="130"/>
     </row>
-    <row r="108" spans="1:12" ht="40.200000000000003" customHeight="1">
+    <row r="108" spans="1:12" ht="80.400000000000006" customHeight="1">
       <c r="A108" s="138">
         <v>34</v>
       </c>
@@ -59782,25 +59794,29 @@
         <v>854</v>
       </c>
       <c r="E108" s="138" t="s">
-        <v>2623</v>
+        <v>2427</v>
       </c>
       <c r="F108" s="178">
         <v>1</v>
       </c>
       <c r="G108" s="285" t="s">
-        <v>2427</v>
+        <v>2428</v>
       </c>
       <c r="H108" s="178" t="s">
-        <v>2415</v>
+        <v>2429</v>
       </c>
       <c r="I108" s="285" t="s">
-        <v>2428</v>
-      </c>
-      <c r="J108" s="166"/>
-      <c r="K108" s="130"/>
+        <v>2430</v>
+      </c>
+      <c r="J108" s="166" t="s">
+        <v>2431</v>
+      </c>
+      <c r="K108" s="130" t="s">
+        <v>2008</v>
+      </c>
       <c r="L108" s="130"/>
     </row>
-    <row r="109" spans="1:12" ht="38.4" customHeight="1">
+    <row r="109" spans="1:12" ht="89.4" customHeight="1">
       <c r="A109" s="138"/>
       <c r="B109" s="138"/>
       <c r="C109" s="138"/>
@@ -59814,9 +59830,11 @@
       </c>
       <c r="H109" s="178"/>
       <c r="I109" s="285" t="s">
-        <v>2429</v>
-      </c>
-      <c r="J109" s="166"/>
+        <v>2432</v>
+      </c>
+      <c r="J109" s="166" t="s">
+        <v>2431</v>
+      </c>
       <c r="K109" s="130"/>
       <c r="L109" s="130"/>
     </row>
@@ -59830,15 +59848,17 @@
         <v>3</v>
       </c>
       <c r="G110" s="285" t="s">
-        <v>2430</v>
+        <v>2433</v>
       </c>
       <c r="H110" s="178" t="s">
-        <v>2622</v>
+        <v>2434</v>
       </c>
       <c r="I110" s="285" t="s">
-        <v>2431</v>
-      </c>
-      <c r="J110" s="166"/>
+        <v>2435</v>
+      </c>
+      <c r="J110" s="166" t="s">
+        <v>2436</v>
+      </c>
       <c r="K110" s="130"/>
       <c r="L110" s="130"/>
     </row>
@@ -59852,13 +59872,15 @@
         <v>4</v>
       </c>
       <c r="G111" s="285" t="s">
-        <v>2432</v>
+        <v>2437</v>
       </c>
       <c r="H111" s="178"/>
       <c r="I111" s="285" t="s">
-        <v>2433</v>
-      </c>
-      <c r="J111" s="166"/>
+        <v>2438</v>
+      </c>
+      <c r="J111" s="166" t="s">
+        <v>2439</v>
+      </c>
       <c r="K111" s="130"/>
       <c r="L111" s="130"/>
     </row>
@@ -59873,7 +59895,7 @@
         <v>863</v>
       </c>
       <c r="D112" s="130" t="s">
-        <v>2434</v>
+        <v>2440</v>
       </c>
       <c r="E112" s="130" t="s">
         <v>865</v>
@@ -59882,7 +59904,7 @@
         <v>1</v>
       </c>
       <c r="G112" s="166" t="s">
-        <v>2435</v>
+        <v>2441</v>
       </c>
       <c r="H112" s="175"/>
       <c r="I112" s="166" t="s">
@@ -59902,7 +59924,7 @@
         <v>2</v>
       </c>
       <c r="G113" s="166" t="s">
-        <v>2436</v>
+        <v>2442</v>
       </c>
       <c r="H113" s="175"/>
       <c r="I113" s="166" t="s">
@@ -59922,10 +59944,10 @@
         <v>3</v>
       </c>
       <c r="G114" s="166" t="s">
-        <v>2437</v>
+        <v>2443</v>
       </c>
       <c r="H114" s="175" t="s">
-        <v>2438</v>
+        <v>2444</v>
       </c>
       <c r="I114" s="166"/>
       <c r="J114" s="130"/>
@@ -59942,10 +59964,10 @@
         <v>4</v>
       </c>
       <c r="G115" s="166" t="s">
-        <v>2439</v>
+        <v>2445</v>
       </c>
       <c r="H115" s="175" t="s">
-        <v>2440</v>
+        <v>2446</v>
       </c>
       <c r="I115" s="166"/>
       <c r="J115" s="130"/>
@@ -59980,7 +60002,7 @@
         <v>6</v>
       </c>
       <c r="G117" s="166" t="s">
-        <v>2441</v>
+        <v>2447</v>
       </c>
       <c r="H117" s="175" t="s">
         <v>877</v>
@@ -60000,7 +60022,7 @@
         <v>7</v>
       </c>
       <c r="G118" s="166" t="s">
-        <v>2442</v>
+        <v>2448</v>
       </c>
       <c r="H118" s="247">
         <v>0.375</v>
@@ -60020,7 +60042,7 @@
         <v>8</v>
       </c>
       <c r="G119" s="166" t="s">
-        <v>2443</v>
+        <v>2449</v>
       </c>
       <c r="H119" s="175">
         <v>100000</v>
@@ -60040,7 +60062,7 @@
         <v>9</v>
       </c>
       <c r="G120" s="166" t="s">
-        <v>2444</v>
+        <v>2450</v>
       </c>
       <c r="H120" s="175">
         <v>1</v>
@@ -60060,7 +60082,7 @@
         <v>10</v>
       </c>
       <c r="G121" s="166" t="s">
-        <v>2445</v>
+        <v>2451</v>
       </c>
       <c r="H121" s="175"/>
       <c r="I121" s="166" t="s">
@@ -60081,7 +60103,7 @@
         <v>884</v>
       </c>
       <c r="D122" s="130" t="s">
-        <v>2446</v>
+        <v>2452</v>
       </c>
       <c r="E122" s="130" t="s">
         <v>886</v>
@@ -60090,7 +60112,7 @@
         <v>1</v>
       </c>
       <c r="G122" s="166" t="s">
-        <v>2447</v>
+        <v>2453</v>
       </c>
       <c r="H122" s="175"/>
       <c r="I122" s="130" t="s">
@@ -60110,7 +60132,7 @@
         <v>2</v>
       </c>
       <c r="G123" s="166" t="s">
-        <v>2448</v>
+        <v>2454</v>
       </c>
       <c r="H123" s="175"/>
       <c r="I123" s="130"/>
@@ -60128,10 +60150,10 @@
         <v>3</v>
       </c>
       <c r="G124" s="166" t="s">
-        <v>2449</v>
+        <v>2455</v>
       </c>
       <c r="H124" s="175" t="s">
-        <v>2450</v>
+        <v>2456</v>
       </c>
       <c r="I124" s="130"/>
       <c r="J124" s="130"/>
@@ -60148,10 +60170,10 @@
         <v>4</v>
       </c>
       <c r="G125" s="166" t="s">
-        <v>2451</v>
+        <v>2457</v>
       </c>
       <c r="H125" s="175" t="s">
-        <v>2452</v>
+        <v>2458</v>
       </c>
       <c r="I125" s="130"/>
       <c r="J125" s="130"/>
@@ -60168,7 +60190,7 @@
         <v>5</v>
       </c>
       <c r="G126" s="166" t="s">
-        <v>2453</v>
+        <v>2459</v>
       </c>
       <c r="H126" s="175" t="s">
         <v>877</v>
@@ -60206,7 +60228,7 @@
         <v>8</v>
       </c>
       <c r="G128" s="166" t="s">
-        <v>2454</v>
+        <v>2460</v>
       </c>
       <c r="H128" s="175">
         <v>100000</v>
@@ -60226,7 +60248,7 @@
         <v>9</v>
       </c>
       <c r="G129" s="166" t="s">
-        <v>2455</v>
+        <v>2461</v>
       </c>
       <c r="H129" s="175">
         <v>1</v>
@@ -60246,7 +60268,7 @@
         <v>10</v>
       </c>
       <c r="G130" s="166" t="s">
-        <v>2456</v>
+        <v>2462</v>
       </c>
       <c r="H130" s="175"/>
       <c r="I130" s="130"/>
@@ -60265,7 +60287,7 @@
         <v>900</v>
       </c>
       <c r="D131" s="130" t="s">
-        <v>2457</v>
+        <v>2463</v>
       </c>
       <c r="E131" s="130" t="s">
         <v>886</v>
@@ -60274,7 +60296,7 @@
         <v>1</v>
       </c>
       <c r="G131" s="166" t="s">
-        <v>2458</v>
+        <v>2464</v>
       </c>
       <c r="H131" s="175"/>
       <c r="I131" s="130" t="s">
@@ -60294,7 +60316,7 @@
         <v>2</v>
       </c>
       <c r="G132" s="166" t="s">
-        <v>2459</v>
+        <v>2465</v>
       </c>
       <c r="H132" s="175"/>
       <c r="I132" s="130"/>
@@ -60312,7 +60334,7 @@
         <v>3</v>
       </c>
       <c r="G133" s="166" t="s">
-        <v>2460</v>
+        <v>2466</v>
       </c>
       <c r="H133" s="175" t="s">
         <v>891</v>
@@ -60390,7 +60412,7 @@
         <v>7</v>
       </c>
       <c r="G137" s="166" t="s">
-        <v>2461</v>
+        <v>2467</v>
       </c>
       <c r="H137" s="175">
         <f>1</f>
@@ -60411,7 +60433,7 @@
         <v>8</v>
       </c>
       <c r="G138" s="166" t="s">
-        <v>2462</v>
+        <v>2468</v>
       </c>
       <c r="H138" s="175"/>
       <c r="I138" s="130"/>
@@ -60430,7 +60452,7 @@
         <v>911</v>
       </c>
       <c r="D139" s="130" t="s">
-        <v>2463</v>
+        <v>2469</v>
       </c>
       <c r="E139" s="130" t="s">
         <v>886</v>
@@ -60439,7 +60461,7 @@
         <v>1</v>
       </c>
       <c r="G139" s="166" t="s">
-        <v>2464</v>
+        <v>2470</v>
       </c>
       <c r="H139" s="175"/>
       <c r="I139" s="130" t="s">
@@ -60459,7 +60481,7 @@
         <v>2</v>
       </c>
       <c r="G140" s="166" t="s">
-        <v>2465</v>
+        <v>2471</v>
       </c>
       <c r="H140" s="175"/>
       <c r="I140" s="130"/>
@@ -60477,7 +60499,7 @@
         <v>3</v>
       </c>
       <c r="G141" s="166" t="s">
-        <v>2466</v>
+        <v>2472</v>
       </c>
       <c r="H141" s="175" t="s">
         <v>891</v>
@@ -60576,7 +60598,7 @@
         <v>8</v>
       </c>
       <c r="G146" s="166" t="s">
-        <v>2467</v>
+        <v>2473</v>
       </c>
       <c r="H146" s="175"/>
       <c r="I146" s="130"/>
@@ -60595,22 +60617,22 @@
         <v>921</v>
       </c>
       <c r="D147" s="138" t="s">
-        <v>2468</v>
+        <v>2474</v>
       </c>
       <c r="E147" s="138" t="s">
-        <v>2469</v>
+        <v>2475</v>
       </c>
       <c r="F147" s="178">
         <v>1</v>
       </c>
       <c r="G147" s="285" t="s">
-        <v>2470</v>
+        <v>2476</v>
       </c>
       <c r="H147" s="178" t="s">
-        <v>2471</v>
+        <v>2477</v>
       </c>
       <c r="I147" s="285" t="s">
-        <v>2472</v>
+        <v>2478</v>
       </c>
       <c r="J147" s="166"/>
       <c r="K147" s="130"/>
@@ -60626,11 +60648,11 @@
         <v>2</v>
       </c>
       <c r="G148" s="285" t="s">
-        <v>2473</v>
+        <v>2479</v>
       </c>
       <c r="H148" s="178"/>
       <c r="I148" s="285" t="s">
-        <v>2474</v>
+        <v>2480</v>
       </c>
       <c r="J148" s="166"/>
       <c r="K148" s="130"/>
@@ -60646,13 +60668,13 @@
         <v>3</v>
       </c>
       <c r="G149" s="285" t="s">
-        <v>2475</v>
+        <v>2481</v>
       </c>
       <c r="H149" s="178" t="s">
-        <v>2476</v>
+        <v>2482</v>
       </c>
       <c r="I149" s="285" t="s">
-        <v>2477</v>
+        <v>2483</v>
       </c>
       <c r="J149" s="166"/>
       <c r="K149" s="130"/>
@@ -60668,11 +60690,11 @@
         <v>4</v>
       </c>
       <c r="G150" s="285" t="s">
-        <v>2478</v>
+        <v>2484</v>
       </c>
       <c r="H150" s="178"/>
       <c r="I150" s="285" t="s">
-        <v>2479</v>
+        <v>2485</v>
       </c>
       <c r="J150" s="166"/>
       <c r="K150" s="130"/>
@@ -60688,11 +60710,11 @@
         <v>5</v>
       </c>
       <c r="G151" s="285" t="s">
-        <v>2480</v>
+        <v>2486</v>
       </c>
       <c r="H151" s="178"/>
       <c r="I151" s="285" t="s">
-        <v>2481</v>
+        <v>2487</v>
       </c>
       <c r="J151" s="166"/>
       <c r="K151" s="130"/>
@@ -60709,22 +60731,22 @@
         <v>932</v>
       </c>
       <c r="D152" s="138" t="s">
-        <v>2482</v>
+        <v>2488</v>
       </c>
       <c r="E152" s="138" t="s">
-        <v>2483</v>
+        <v>2489</v>
       </c>
       <c r="F152" s="178">
         <v>1</v>
       </c>
       <c r="G152" s="285" t="s">
-        <v>2484</v>
+        <v>2490</v>
       </c>
       <c r="H152" s="320" t="s">
-        <v>2485</v>
+        <v>2491</v>
       </c>
       <c r="I152" s="285" t="s">
-        <v>2486</v>
+        <v>2492</v>
       </c>
       <c r="J152" s="166"/>
       <c r="K152" s="130"/>
@@ -60740,13 +60762,13 @@
         <v>2</v>
       </c>
       <c r="G153" s="285" t="s">
-        <v>2487</v>
+        <v>2493</v>
       </c>
       <c r="H153" s="320" t="s">
-        <v>2488</v>
+        <v>2494</v>
       </c>
       <c r="I153" s="285" t="s">
-        <v>2489</v>
+        <v>2495</v>
       </c>
       <c r="J153" s="166"/>
       <c r="K153" s="130"/>
@@ -60762,11 +60784,11 @@
         <v>3</v>
       </c>
       <c r="G154" s="285" t="s">
-        <v>2490</v>
+        <v>2496</v>
       </c>
       <c r="H154" s="320"/>
       <c r="I154" s="285" t="s">
-        <v>2491</v>
+        <v>2497</v>
       </c>
       <c r="J154" s="166"/>
       <c r="K154" s="130"/>
@@ -61193,13 +61215,13 @@
         <v>1100</v>
       </c>
       <c r="H2" s="332" t="s">
-        <v>2492</v>
+        <v>2498</v>
       </c>
       <c r="I2" s="64" t="s">
         <v>1102</v>
       </c>
       <c r="J2" s="64" t="s">
-        <v>2493</v>
+        <v>2499</v>
       </c>
       <c r="K2" s="64" t="s">
         <v>2008</v>
@@ -61436,7 +61458,7 @@
         <v>13</v>
       </c>
       <c r="G14" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H14" s="288"/>
       <c r="I14" s="62"/>
@@ -61471,7 +61493,7 @@
         <v>1122</v>
       </c>
       <c r="J15" s="64" t="s">
-        <v>2495</v>
+        <v>2501</v>
       </c>
       <c r="K15" s="64" t="s">
         <v>2008</v>
@@ -61708,7 +61730,7 @@
         <v>13</v>
       </c>
       <c r="G27" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H27" s="288"/>
       <c r="I27" s="62"/>
@@ -61739,13 +61761,13 @@
         <v>1100</v>
       </c>
       <c r="H28" s="332" t="s">
-        <v>2496</v>
+        <v>2502</v>
       </c>
       <c r="I28" s="64" t="s">
         <v>1127</v>
       </c>
       <c r="J28" s="64" t="s">
-        <v>2497</v>
+        <v>2503</v>
       </c>
       <c r="K28" s="64" t="s">
         <v>2008</v>
@@ -61980,7 +62002,7 @@
         <v>13</v>
       </c>
       <c r="G40" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H40" s="288"/>
       <c r="I40" s="62"/>
@@ -62011,19 +62033,19 @@
         <v>1100</v>
       </c>
       <c r="H41" s="332" t="s">
-        <v>2498</v>
+        <v>2504</v>
       </c>
       <c r="I41" s="64" t="s">
         <v>1130</v>
       </c>
       <c r="J41" s="64" t="s">
-        <v>2499</v>
+        <v>2505</v>
       </c>
       <c r="K41" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L41" s="134" t="s">
-        <v>2500</v>
+        <v>2506</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="14.4" customHeight="1">
@@ -62254,7 +62276,7 @@
         <v>13</v>
       </c>
       <c r="G53" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H53" s="288"/>
       <c r="I53" s="62"/>
@@ -62285,13 +62307,13 @@
         <v>1100</v>
       </c>
       <c r="H54" s="332" t="s">
-        <v>2501</v>
+        <v>2507</v>
       </c>
       <c r="I54" s="64" t="s">
         <v>1134</v>
       </c>
       <c r="J54" s="64" t="s">
-        <v>2502</v>
+        <v>2508</v>
       </c>
       <c r="K54" s="64" t="s">
         <v>2008</v>
@@ -62526,7 +62548,7 @@
         <v>13</v>
       </c>
       <c r="G66" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H66" s="288"/>
       <c r="I66" s="62"/>
@@ -62557,19 +62579,19 @@
         <v>1100</v>
       </c>
       <c r="H67" s="332" t="s">
-        <v>2503</v>
+        <v>2509</v>
       </c>
       <c r="I67" s="64" t="s">
         <v>1138</v>
       </c>
       <c r="J67" s="64" t="s">
-        <v>2504</v>
+        <v>2510</v>
       </c>
       <c r="K67" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L67" s="134" t="s">
-        <v>2505</v>
+        <v>2511</v>
       </c>
     </row>
     <row r="68" spans="1:12" ht="14.4" customHeight="1">
@@ -62800,7 +62822,7 @@
         <v>13</v>
       </c>
       <c r="G79" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H79" s="288"/>
       <c r="I79" s="62"/>
@@ -62831,19 +62853,19 @@
         <v>1100</v>
       </c>
       <c r="H80" s="332" t="s">
-        <v>2506</v>
+        <v>2512</v>
       </c>
       <c r="I80" s="64" t="s">
         <v>1141</v>
       </c>
       <c r="J80" s="64" t="s">
-        <v>2507</v>
+        <v>2513</v>
       </c>
       <c r="K80" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L80" s="134" t="s">
-        <v>2508</v>
+        <v>2514</v>
       </c>
     </row>
     <row r="81" spans="1:12" ht="14.4" customHeight="1">
@@ -63074,7 +63096,7 @@
         <v>13</v>
       </c>
       <c r="G92" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H92" s="288"/>
       <c r="I92" s="62"/>
@@ -63105,13 +63127,13 @@
         <v>1100</v>
       </c>
       <c r="H93" s="332" t="s">
-        <v>2509</v>
+        <v>2515</v>
       </c>
       <c r="I93" s="64" t="s">
         <v>1145</v>
       </c>
       <c r="J93" s="64" t="s">
-        <v>2510</v>
+        <v>2516</v>
       </c>
       <c r="K93" s="64" t="s">
         <v>2008</v>
@@ -63346,7 +63368,7 @@
         <v>13</v>
       </c>
       <c r="G105" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H105" s="288"/>
       <c r="I105" s="62"/>
@@ -63377,13 +63399,13 @@
         <v>1100</v>
       </c>
       <c r="H106" s="332" t="s">
-        <v>2509</v>
+        <v>2515</v>
       </c>
       <c r="I106" s="64" t="s">
         <v>1149</v>
       </c>
       <c r="J106" s="64" t="s">
-        <v>2511</v>
+        <v>2517</v>
       </c>
       <c r="K106" s="64" t="s">
         <v>2008</v>
@@ -63618,7 +63640,7 @@
         <v>13</v>
       </c>
       <c r="G118" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H118" s="288"/>
       <c r="I118" s="62"/>
@@ -63649,13 +63671,13 @@
         <v>1100</v>
       </c>
       <c r="H119" s="332" t="s">
-        <v>2512</v>
+        <v>2518</v>
       </c>
       <c r="I119" s="64" t="s">
-        <v>2513</v>
+        <v>2519</v>
       </c>
       <c r="J119" s="64" t="s">
-        <v>2514</v>
+        <v>2520</v>
       </c>
       <c r="K119" s="64" t="s">
         <v>2008</v>
@@ -63890,7 +63912,7 @@
         <v>13</v>
       </c>
       <c r="G131" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H131" s="288"/>
       <c r="I131" s="62"/>
@@ -63921,13 +63943,13 @@
         <v>1100</v>
       </c>
       <c r="H132" s="332" t="s">
-        <v>2515</v>
+        <v>2521</v>
       </c>
       <c r="I132" s="64" t="s">
         <v>1160</v>
       </c>
       <c r="J132" s="64" t="s">
-        <v>2516</v>
+        <v>2522</v>
       </c>
       <c r="K132" s="64" t="s">
         <v>2008</v>
@@ -64162,7 +64184,7 @@
         <v>13</v>
       </c>
       <c r="G144" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H144" s="288"/>
       <c r="I144" s="62"/>
@@ -64181,7 +64203,7 @@
         <v>1164</v>
       </c>
       <c r="D145" s="64" t="s">
-        <v>2517</v>
+        <v>2523</v>
       </c>
       <c r="E145" s="64" t="s">
         <v>1099</v>
@@ -64193,19 +64215,19 @@
         <v>1100</v>
       </c>
       <c r="H145" s="332" t="s">
-        <v>2518</v>
+        <v>2524</v>
       </c>
       <c r="I145" s="64" t="s">
-        <v>2519</v>
+        <v>2525</v>
       </c>
       <c r="J145" s="64" t="s">
-        <v>2520</v>
+        <v>2526</v>
       </c>
       <c r="K145" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L145" s="134" t="s">
-        <v>2521</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="146" spans="1:12" ht="14.4" customHeight="1">
@@ -64438,7 +64460,7 @@
         <v>13</v>
       </c>
       <c r="G157" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H157" s="288"/>
       <c r="I157" s="62"/>
@@ -64469,13 +64491,13 @@
         <v>1100</v>
       </c>
       <c r="H158" s="332" t="s">
-        <v>2522</v>
+        <v>2528</v>
       </c>
       <c r="I158" s="64" t="s">
-        <v>2523</v>
+        <v>2529</v>
       </c>
       <c r="J158" s="64" t="s">
-        <v>2524</v>
+        <v>2530</v>
       </c>
       <c r="K158" s="64" t="s">
         <v>2008</v>
@@ -64710,7 +64732,7 @@
         <v>13</v>
       </c>
       <c r="G170" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H170" s="288"/>
       <c r="I170" s="62"/>
@@ -64741,13 +64763,13 @@
         <v>1100</v>
       </c>
       <c r="H171" s="332" t="s">
-        <v>2525</v>
+        <v>2531</v>
       </c>
       <c r="I171" s="64" t="s">
-        <v>2526</v>
+        <v>2532</v>
       </c>
       <c r="J171" s="64" t="s">
-        <v>2527</v>
+        <v>2533</v>
       </c>
       <c r="K171" s="64" t="s">
         <v>2008</v>
@@ -64982,7 +65004,7 @@
         <v>13</v>
       </c>
       <c r="G183" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H183" s="288"/>
       <c r="I183" s="62"/>
@@ -65014,16 +65036,16 @@
       </c>
       <c r="H184" s="332"/>
       <c r="I184" s="64" t="s">
-        <v>2528</v>
+        <v>2534</v>
       </c>
       <c r="J184" s="64" t="s">
-        <v>2529</v>
+        <v>2535</v>
       </c>
       <c r="K184" s="64" t="s">
         <v>2015</v>
       </c>
       <c r="L184" s="134" t="s">
-        <v>2530</v>
+        <v>2536</v>
       </c>
     </row>
     <row r="185" spans="1:12" ht="14.4" customHeight="1">
@@ -65234,7 +65256,7 @@
         <v>13</v>
       </c>
       <c r="G196" s="288" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H196" s="332"/>
       <c r="I196" s="62"/>
@@ -65265,19 +65287,19 @@
         <v>1100</v>
       </c>
       <c r="H197" s="332" t="s">
-        <v>2531</v>
+        <v>2537</v>
       </c>
       <c r="I197" s="53" t="s">
         <v>1178</v>
       </c>
       <c r="J197" s="134" t="s">
-        <v>2532</v>
+        <v>2538</v>
       </c>
       <c r="K197" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L197" s="134" t="s">
-        <v>2533</v>
+        <v>2539</v>
       </c>
     </row>
     <row r="198" spans="1:12">
@@ -65510,7 +65532,7 @@
         <v>13</v>
       </c>
       <c r="G209" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H209" s="293"/>
       <c r="I209" s="53"/>
@@ -65541,19 +65563,19 @@
         <v>1100</v>
       </c>
       <c r="H210" s="332" t="s">
-        <v>2534</v>
+        <v>2540</v>
       </c>
       <c r="I210" s="53" t="s">
         <v>1187</v>
       </c>
       <c r="J210" s="134" t="s">
-        <v>2535</v>
+        <v>2541</v>
       </c>
       <c r="K210" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L210" s="134" t="s">
-        <v>2536</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="211" spans="1:12">
@@ -65786,7 +65808,7 @@
         <v>13</v>
       </c>
       <c r="G222" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H222" s="293"/>
       <c r="I222" s="53"/>
@@ -65805,7 +65827,7 @@
         <v>1189</v>
       </c>
       <c r="D223" s="53" t="s">
-        <v>2537</v>
+        <v>2543</v>
       </c>
       <c r="E223" s="136" t="s">
         <v>1176</v>
@@ -65817,19 +65839,19 @@
         <v>1100</v>
       </c>
       <c r="H223" s="332" t="s">
-        <v>2538</v>
+        <v>2544</v>
       </c>
       <c r="I223" s="134" t="s">
-        <v>2539</v>
+        <v>2545</v>
       </c>
       <c r="J223" s="134" t="s">
-        <v>2540</v>
+        <v>2546</v>
       </c>
       <c r="K223" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L223" s="134" t="s">
-        <v>2541</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="224" spans="1:12" ht="31.2" customHeight="1">
@@ -66062,7 +66084,7 @@
         <v>13</v>
       </c>
       <c r="G235" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H235" s="293"/>
       <c r="I235" s="132"/>
@@ -66093,19 +66115,19 @@
         <v>1100</v>
       </c>
       <c r="H236" s="332" t="s">
-        <v>2542</v>
+        <v>2548</v>
       </c>
       <c r="I236" s="134" t="s">
         <v>1197</v>
       </c>
       <c r="J236" s="134" t="s">
-        <v>2543</v>
+        <v>2549</v>
       </c>
       <c r="K236" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L236" s="134" t="s">
-        <v>2544</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="237" spans="1:12" ht="26.4" customHeight="1">
@@ -66338,7 +66360,7 @@
         <v>13</v>
       </c>
       <c r="G248" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H248" s="293"/>
       <c r="I248" s="132"/>
@@ -66369,19 +66391,19 @@
         <v>1100</v>
       </c>
       <c r="H249" s="332" t="s">
-        <v>2545</v>
+        <v>2551</v>
       </c>
       <c r="I249" s="134" t="s">
         <v>1203</v>
       </c>
       <c r="J249" s="134" t="s">
-        <v>2546</v>
+        <v>2552</v>
       </c>
       <c r="K249" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L249" s="134" t="s">
-        <v>2547</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="250" spans="1:12" ht="30" customHeight="1">
@@ -66557,7 +66579,7 @@
         <v>1115</v>
       </c>
       <c r="H258" s="288" t="s">
-        <v>2548</v>
+        <v>2554</v>
       </c>
       <c r="I258" s="133"/>
       <c r="J258" s="133"/>
@@ -66614,7 +66636,7 @@
         <v>13</v>
       </c>
       <c r="G261" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H261" s="293"/>
       <c r="I261" s="132"/>
@@ -66636,7 +66658,7 @@
         <v>1207</v>
       </c>
       <c r="E262" s="136" t="s">
-        <v>2549</v>
+        <v>2555</v>
       </c>
       <c r="F262" s="176">
         <v>1</v>
@@ -66651,13 +66673,13 @@
         <v>1210</v>
       </c>
       <c r="J262" s="134" t="s">
-        <v>2550</v>
+        <v>2556</v>
       </c>
       <c r="K262" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L262" s="134" t="s">
-        <v>2551</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="263" spans="1:12" ht="29.4" customHeight="1">
@@ -66890,7 +66912,7 @@
         <v>13</v>
       </c>
       <c r="G274" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H274" s="293"/>
       <c r="I274" s="132"/>
@@ -66921,19 +66943,19 @@
         <v>1100</v>
       </c>
       <c r="H275" s="332" t="s">
-        <v>2552</v>
+        <v>2558</v>
       </c>
       <c r="I275" s="135" t="s">
-        <v>2553</v>
+        <v>2559</v>
       </c>
       <c r="J275" s="64" t="s">
-        <v>2554</v>
+        <v>2560</v>
       </c>
       <c r="K275" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L275" s="134" t="s">
-        <v>2555</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="276" spans="1:12">
@@ -67006,7 +67028,7 @@
         <v>5</v>
       </c>
       <c r="G279" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H279" s="308" t="s">
         <v>1117</v>
@@ -67026,7 +67048,7 @@
         <v>6</v>
       </c>
       <c r="G280" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H280" s="308">
         <v>46123</v>
@@ -67146,7 +67168,7 @@
         <v>12</v>
       </c>
       <c r="G286" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H286" s="293"/>
       <c r="I286" s="135"/>
@@ -67181,13 +67203,13 @@
         <v>1122</v>
       </c>
       <c r="J287" s="64" t="s">
-        <v>2495</v>
+        <v>2501</v>
       </c>
       <c r="K287" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L287" s="134" t="s">
-        <v>2558</v>
+        <v>2564</v>
       </c>
     </row>
     <row r="288" spans="1:12">
@@ -67260,7 +67282,7 @@
         <v>5</v>
       </c>
       <c r="G291" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H291" s="308" t="s">
         <v>1117</v>
@@ -67280,7 +67302,7 @@
         <v>6</v>
       </c>
       <c r="G292" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H292" s="308">
         <v>46123</v>
@@ -67400,7 +67422,7 @@
         <v>12</v>
       </c>
       <c r="G298" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I298" s="135"/>
       <c r="J298" s="62"/>
@@ -67430,19 +67452,19 @@
         <v>1100</v>
       </c>
       <c r="H299" s="332" t="s">
-        <v>2559</v>
+        <v>2565</v>
       </c>
       <c r="I299" s="135" t="s">
         <v>1127</v>
       </c>
       <c r="J299" s="64" t="s">
-        <v>2497</v>
+        <v>2503</v>
       </c>
       <c r="K299" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L299" s="134" t="s">
-        <v>2560</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="300" spans="1:12">
@@ -67513,7 +67535,7 @@
         <v>5</v>
       </c>
       <c r="G303" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H303" s="308" t="s">
         <v>1117</v>
@@ -67533,7 +67555,7 @@
         <v>6</v>
       </c>
       <c r="G304" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H304" s="308">
         <v>46123</v>
@@ -67653,7 +67675,7 @@
         <v>12</v>
       </c>
       <c r="G310" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I310" s="135"/>
       <c r="J310" s="62"/>
@@ -67683,19 +67705,19 @@
         <v>1100</v>
       </c>
       <c r="H311" s="332" t="s">
-        <v>2561</v>
+        <v>2567</v>
       </c>
       <c r="I311" s="135" t="s">
         <v>1130</v>
       </c>
       <c r="J311" s="64" t="s">
-        <v>2562</v>
+        <v>2568</v>
       </c>
       <c r="K311" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L311" s="134" t="s">
-        <v>2563</v>
+        <v>2569</v>
       </c>
     </row>
     <row r="312" spans="1:12">
@@ -67766,7 +67788,7 @@
         <v>5</v>
       </c>
       <c r="G315" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H315" s="308" t="s">
         <v>1117</v>
@@ -67786,7 +67808,7 @@
         <v>6</v>
       </c>
       <c r="G316" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H316" s="308">
         <v>46123</v>
@@ -67906,7 +67928,7 @@
         <v>12</v>
       </c>
       <c r="G322" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I322" s="135"/>
       <c r="J322" s="62"/>
@@ -67936,13 +67958,13 @@
         <v>1100</v>
       </c>
       <c r="H323" s="332" t="s">
-        <v>2564</v>
+        <v>2570</v>
       </c>
       <c r="I323" s="135" t="s">
         <v>1134</v>
       </c>
       <c r="J323" s="64" t="s">
-        <v>2502</v>
+        <v>2508</v>
       </c>
       <c r="K323" s="135" t="s">
         <v>2008</v>
@@ -68019,7 +68041,7 @@
         <v>5</v>
       </c>
       <c r="G327" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H327" s="308"/>
       <c r="I327" s="135"/>
@@ -68037,7 +68059,7 @@
         <v>6</v>
       </c>
       <c r="G328" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H328" s="308">
         <v>46123</v>
@@ -68157,7 +68179,7 @@
         <v>12</v>
       </c>
       <c r="G334" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I334" s="135"/>
       <c r="J334" s="62"/>
@@ -68187,19 +68209,19 @@
         <v>1100</v>
       </c>
       <c r="H335" s="332" t="s">
-        <v>2564</v>
+        <v>2570</v>
       </c>
       <c r="I335" s="135" t="s">
         <v>1138</v>
       </c>
       <c r="J335" s="64" t="s">
-        <v>2565</v>
+        <v>2571</v>
       </c>
       <c r="K335" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L335" s="134" t="s">
-        <v>2566</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="336" spans="1:12">
@@ -68272,7 +68294,7 @@
         <v>5</v>
       </c>
       <c r="G339" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H339" s="308" t="s">
         <v>1117</v>
@@ -68292,7 +68314,7 @@
         <v>6</v>
       </c>
       <c r="G340" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H340" s="308"/>
       <c r="I340" s="135"/>
@@ -68410,7 +68432,7 @@
         <v>12</v>
       </c>
       <c r="G346" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I346" s="135"/>
       <c r="J346" s="62"/>
@@ -68428,7 +68450,7 @@
         <v>1254</v>
       </c>
       <c r="D347" s="135" t="s">
-        <v>2567</v>
+        <v>2573</v>
       </c>
       <c r="E347" s="135" t="s">
         <v>1099</v>
@@ -68440,19 +68462,19 @@
         <v>1100</v>
       </c>
       <c r="H347" s="332" t="s">
-        <v>2568</v>
+        <v>2574</v>
       </c>
       <c r="I347" s="135" t="s">
-        <v>2569</v>
+        <v>2575</v>
       </c>
       <c r="J347" s="64" t="s">
-        <v>2570</v>
+        <v>2576</v>
       </c>
       <c r="K347" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L347" s="134" t="s">
-        <v>2571</v>
+        <v>2577</v>
       </c>
     </row>
     <row r="348" spans="1:12">
@@ -68525,7 +68547,7 @@
         <v>5</v>
       </c>
       <c r="G351" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H351" s="308" t="s">
         <v>1117</v>
@@ -68545,7 +68567,7 @@
         <v>6</v>
       </c>
       <c r="G352" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H352" s="308">
         <v>49410</v>
@@ -68663,7 +68685,7 @@
         <v>12</v>
       </c>
       <c r="G358" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H358" s="288"/>
       <c r="I358" s="135"/>
@@ -68694,13 +68716,13 @@
         <v>1100</v>
       </c>
       <c r="H359" s="332" t="s">
-        <v>2572</v>
+        <v>2578</v>
       </c>
       <c r="I359" s="135" t="s">
         <v>1145</v>
       </c>
       <c r="J359" s="64" t="s">
-        <v>2510</v>
+        <v>2516</v>
       </c>
       <c r="K359" s="135" t="s">
         <v>2008</v>
@@ -68777,7 +68799,7 @@
         <v>5</v>
       </c>
       <c r="G363" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H363" s="308" t="s">
         <v>1117</v>
@@ -68797,7 +68819,7 @@
         <v>6</v>
       </c>
       <c r="G364" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H364" s="308">
         <v>46123</v>
@@ -68915,7 +68937,7 @@
         <v>12</v>
       </c>
       <c r="G370" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I370" s="135"/>
       <c r="J370" s="62"/>
@@ -68945,13 +68967,13 @@
         <v>1100</v>
       </c>
       <c r="H371" s="332" t="s">
-        <v>2573</v>
+        <v>2579</v>
       </c>
       <c r="I371" s="135" t="s">
         <v>1149</v>
       </c>
       <c r="J371" s="64" t="s">
-        <v>2511</v>
+        <v>2517</v>
       </c>
       <c r="K371" s="135" t="s">
         <v>2008</v>
@@ -69028,7 +69050,7 @@
         <v>5</v>
       </c>
       <c r="G375" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H375" s="308" t="s">
         <v>1117</v>
@@ -69048,7 +69070,7 @@
         <v>6</v>
       </c>
       <c r="G376" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H376" s="308">
         <v>46123</v>
@@ -69166,7 +69188,7 @@
         <v>12</v>
       </c>
       <c r="G382" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I382" s="135"/>
       <c r="J382" s="62"/>
@@ -69184,7 +69206,7 @@
         <v>1257</v>
       </c>
       <c r="D383" s="135" t="s">
-        <v>2574</v>
+        <v>2580</v>
       </c>
       <c r="E383" s="135" t="s">
         <v>1099</v>
@@ -69196,19 +69218,19 @@
         <v>1100</v>
       </c>
       <c r="H383" s="332" t="s">
-        <v>2575</v>
+        <v>2581</v>
       </c>
       <c r="I383" s="135" t="s">
-        <v>2513</v>
+        <v>2519</v>
       </c>
       <c r="J383" s="64" t="s">
-        <v>2514</v>
+        <v>2520</v>
       </c>
       <c r="K383" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L383" s="134" t="s">
-        <v>2576</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="384" spans="1:12">
@@ -69279,7 +69301,7 @@
         <v>5</v>
       </c>
       <c r="G387" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H387" s="308" t="s">
         <v>1117</v>
@@ -69299,7 +69321,7 @@
         <v>6</v>
       </c>
       <c r="G388" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H388" s="308">
         <v>46123</v>
@@ -69419,7 +69441,7 @@
         <v>12</v>
       </c>
       <c r="G394" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I394" s="135"/>
       <c r="J394" s="62"/>
@@ -69449,13 +69471,13 @@
         <v>1100</v>
       </c>
       <c r="H395" s="332" t="s">
-        <v>2577</v>
+        <v>2583</v>
       </c>
       <c r="I395" s="135" t="s">
         <v>1160</v>
       </c>
       <c r="J395" s="64" t="s">
-        <v>2516</v>
+        <v>2522</v>
       </c>
       <c r="K395" s="135" t="s">
         <v>2008</v>
@@ -69532,7 +69554,7 @@
         <v>5</v>
       </c>
       <c r="G399" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H399" s="308" t="s">
         <v>1117</v>
@@ -69552,7 +69574,7 @@
         <v>6</v>
       </c>
       <c r="G400" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H400" s="308">
         <v>46123</v>
@@ -69670,7 +69692,7 @@
         <v>12</v>
       </c>
       <c r="G406" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I406" s="135"/>
       <c r="J406" s="62"/>
@@ -69688,7 +69710,7 @@
         <v>1260</v>
       </c>
       <c r="D407" s="135" t="s">
-        <v>2578</v>
+        <v>2584</v>
       </c>
       <c r="E407" s="135" t="s">
         <v>1099</v>
@@ -69700,19 +69722,19 @@
         <v>1100</v>
       </c>
       <c r="H407" s="332" t="s">
-        <v>2579</v>
+        <v>2585</v>
       </c>
       <c r="I407" s="135" t="s">
-        <v>2580</v>
+        <v>2586</v>
       </c>
       <c r="J407" s="64" t="s">
-        <v>2581</v>
+        <v>2587</v>
       </c>
       <c r="K407" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L407" s="134" t="s">
-        <v>2582</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="408" spans="1:12">
@@ -69785,7 +69807,7 @@
         <v>5</v>
       </c>
       <c r="G411" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H411" s="308" t="s">
         <v>1117</v>
@@ -69805,7 +69827,7 @@
         <v>6</v>
       </c>
       <c r="G412" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H412" s="308">
         <v>46123</v>
@@ -69925,7 +69947,7 @@
         <v>12</v>
       </c>
       <c r="G418" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I418" s="135"/>
       <c r="J418" s="62"/>
@@ -69955,19 +69977,19 @@
         <v>1100</v>
       </c>
       <c r="H419" s="332" t="s">
-        <v>2583</v>
+        <v>2589</v>
       </c>
       <c r="I419" s="135" t="s">
-        <v>2523</v>
+        <v>2529</v>
       </c>
       <c r="J419" s="64" t="s">
-        <v>2524</v>
+        <v>2530</v>
       </c>
       <c r="K419" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L419" s="134" t="s">
-        <v>2584</v>
+        <v>2590</v>
       </c>
     </row>
     <row r="420" spans="1:12">
@@ -70040,7 +70062,7 @@
         <v>5</v>
       </c>
       <c r="G423" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H423" s="308" t="s">
         <v>1117</v>
@@ -70060,7 +70082,7 @@
         <v>6</v>
       </c>
       <c r="G424" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H424" s="308">
         <v>46123</v>
@@ -70178,7 +70200,7 @@
         <v>12</v>
       </c>
       <c r="G430" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I430" s="135"/>
       <c r="J430" s="62"/>
@@ -70208,19 +70230,19 @@
         <v>1100</v>
       </c>
       <c r="H431" s="332" t="s">
-        <v>2585</v>
+        <v>2591</v>
       </c>
       <c r="I431" s="135" t="s">
-        <v>2526</v>
+        <v>2532</v>
       </c>
       <c r="J431" s="64" t="s">
-        <v>2527</v>
+        <v>2533</v>
       </c>
       <c r="K431" s="135" t="s">
         <v>2008</v>
       </c>
       <c r="L431" s="134" t="s">
-        <v>2586</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="432" spans="1:12">
@@ -70293,7 +70315,7 @@
         <v>5</v>
       </c>
       <c r="G435" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H435" s="308" t="s">
         <v>1117</v>
@@ -70313,7 +70335,7 @@
         <v>6</v>
       </c>
       <c r="G436" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H436" s="308">
         <v>46123</v>
@@ -70431,7 +70453,7 @@
         <v>12</v>
       </c>
       <c r="G442" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I442" s="135"/>
       <c r="J442" s="62"/>
@@ -70449,7 +70471,7 @@
         <v>1265</v>
       </c>
       <c r="D443" s="135" t="s">
-        <v>2587</v>
+        <v>2593</v>
       </c>
       <c r="E443" s="135" t="s">
         <v>1099</v>
@@ -70461,19 +70483,19 @@
         <v>1100</v>
       </c>
       <c r="H443" s="332" t="s">
-        <v>2579</v>
+        <v>2585</v>
       </c>
       <c r="I443" s="135" t="s">
-        <v>2588</v>
+        <v>2594</v>
       </c>
       <c r="J443" s="64" t="s">
-        <v>2589</v>
+        <v>2595</v>
       </c>
       <c r="K443" s="135" t="s">
         <v>2015</v>
       </c>
       <c r="L443" s="134" t="s">
-        <v>2590</v>
+        <v>2596</v>
       </c>
     </row>
     <row r="444" spans="1:12">
@@ -70546,7 +70568,7 @@
         <v>5</v>
       </c>
       <c r="G447" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H447" s="308" t="s">
         <v>1117</v>
@@ -70566,7 +70588,7 @@
         <v>6</v>
       </c>
       <c r="G448" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H448" s="308">
         <v>46123</v>
@@ -70686,7 +70708,7 @@
         <v>12</v>
       </c>
       <c r="G454" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="I454" s="135"/>
       <c r="J454" s="62"/>
@@ -70704,10 +70726,10 @@
         <v>1212</v>
       </c>
       <c r="D455" s="136" t="s">
-        <v>2591</v>
+        <v>2597</v>
       </c>
       <c r="E455" s="136" t="s">
-        <v>2592</v>
+        <v>2598</v>
       </c>
       <c r="F455" s="176">
         <v>1</v>
@@ -70716,19 +70738,19 @@
         <v>1100</v>
       </c>
       <c r="H455" s="332" t="s">
-        <v>2593</v>
+        <v>2599</v>
       </c>
       <c r="I455" s="134" t="s">
-        <v>2594</v>
+        <v>2600</v>
       </c>
       <c r="J455" s="134" t="s">
-        <v>2595</v>
+        <v>2601</v>
       </c>
       <c r="K455" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L455" s="134" t="s">
-        <v>2596</v>
+        <v>2602</v>
       </c>
     </row>
     <row r="456" spans="1:12">
@@ -70801,7 +70823,7 @@
         <v>5</v>
       </c>
       <c r="G459" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H459" s="308" t="s">
         <v>1117</v>
@@ -70821,7 +70843,7 @@
         <v>6</v>
       </c>
       <c r="G460" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H460" s="308">
         <v>46123</v>
@@ -70884,7 +70906,7 @@
         <v>1115</v>
       </c>
       <c r="H463" s="318" t="s">
-        <v>2597</v>
+        <v>2603</v>
       </c>
       <c r="I463" s="133"/>
       <c r="J463" s="133"/>
@@ -70941,7 +70963,7 @@
         <v>12</v>
       </c>
       <c r="G466" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H466" s="293"/>
       <c r="I466" s="132"/>
@@ -70960,10 +70982,10 @@
         <v>1219</v>
       </c>
       <c r="D467" s="136" t="s">
-        <v>2598</v>
+        <v>2604</v>
       </c>
       <c r="E467" s="136" t="s">
-        <v>2599</v>
+        <v>2605</v>
       </c>
       <c r="F467" s="176">
         <v>1</v>
@@ -70972,19 +70994,19 @@
         <v>1100</v>
       </c>
       <c r="H467" s="332" t="s">
-        <v>2600</v>
+        <v>2606</v>
       </c>
       <c r="I467" s="134" t="s">
-        <v>2539</v>
+        <v>2545</v>
       </c>
       <c r="J467" s="134" t="s">
-        <v>2601</v>
+        <v>2607</v>
       </c>
       <c r="K467" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L467" s="134" t="s">
-        <v>2602</v>
+        <v>2608</v>
       </c>
     </row>
     <row r="468" spans="1:12">
@@ -71057,7 +71079,7 @@
         <v>5</v>
       </c>
       <c r="G471" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H471" s="308" t="s">
         <v>1117</v>
@@ -71077,7 +71099,7 @@
         <v>6</v>
       </c>
       <c r="G472" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H472" s="308">
         <v>46123</v>
@@ -71197,7 +71219,7 @@
         <v>12</v>
       </c>
       <c r="G478" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H478" s="293"/>
       <c r="I478" s="132"/>
@@ -71216,10 +71238,10 @@
         <v>1225</v>
       </c>
       <c r="D479" s="136" t="s">
-        <v>2603</v>
+        <v>2609</v>
       </c>
       <c r="E479" s="136" t="s">
-        <v>2604</v>
+        <v>2610</v>
       </c>
       <c r="F479" s="176">
         <v>1</v>
@@ -71228,19 +71250,19 @@
         <v>1100</v>
       </c>
       <c r="H479" s="332" t="s">
-        <v>2605</v>
+        <v>2611</v>
       </c>
       <c r="I479" s="134" t="s">
-        <v>2606</v>
+        <v>2612</v>
       </c>
       <c r="J479" s="134" t="s">
-        <v>2607</v>
+        <v>2613</v>
       </c>
       <c r="K479" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L479" s="134" t="s">
-        <v>2608</v>
+        <v>2614</v>
       </c>
     </row>
     <row r="480" spans="1:12">
@@ -71256,7 +71278,7 @@
         <v>1103</v>
       </c>
       <c r="H480" s="332" t="s">
-        <v>2609</v>
+        <v>2615</v>
       </c>
       <c r="I480" s="133"/>
       <c r="J480" s="133"/>
@@ -71313,7 +71335,7 @@
         <v>5</v>
       </c>
       <c r="G483" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H483" s="308" t="s">
         <v>1117</v>
@@ -71333,7 +71355,7 @@
         <v>6</v>
       </c>
       <c r="G484" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H484" s="308">
         <v>46123</v>
@@ -71453,7 +71475,7 @@
         <v>12</v>
       </c>
       <c r="G490" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H490" s="293"/>
       <c r="I490" s="132"/>
@@ -71472,10 +71494,10 @@
         <v>1232</v>
       </c>
       <c r="D491" s="136" t="s">
+        <v>2616</v>
+      </c>
+      <c r="E491" s="136" t="s">
         <v>2610</v>
-      </c>
-      <c r="E491" s="136" t="s">
-        <v>2604</v>
       </c>
       <c r="F491" s="176">
         <v>1</v>
@@ -71484,19 +71506,19 @@
         <v>1100</v>
       </c>
       <c r="H491" s="292" t="s">
-        <v>2611</v>
+        <v>2617</v>
       </c>
       <c r="I491" s="134" t="s">
-        <v>2612</v>
+        <v>2618</v>
       </c>
       <c r="J491" s="134" t="s">
-        <v>2613</v>
+        <v>2619</v>
       </c>
       <c r="K491" s="136" t="s">
         <v>2015</v>
       </c>
       <c r="L491" s="134" t="s">
-        <v>2614</v>
+        <v>2620</v>
       </c>
     </row>
     <row r="492" spans="1:12" ht="15" customHeight="1">
@@ -71512,7 +71534,7 @@
         <v>1103</v>
       </c>
       <c r="H492" s="332" t="s">
-        <v>2615</v>
+        <v>2621</v>
       </c>
       <c r="I492" s="133"/>
       <c r="J492" s="133"/>
@@ -71569,7 +71591,7 @@
         <v>5</v>
       </c>
       <c r="G495" s="288" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="H495" s="308" t="s">
         <v>1117</v>
@@ -71589,7 +71611,7 @@
         <v>6</v>
       </c>
       <c r="G496" s="288" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
       <c r="H496" s="308">
         <v>46123</v>
@@ -71709,7 +71731,7 @@
         <v>12</v>
       </c>
       <c r="G502" s="293" t="s">
-        <v>2494</v>
+        <v>2500</v>
       </c>
       <c r="H502" s="293"/>
       <c r="I502" s="132"/>
@@ -72100,13 +72122,13 @@
   <sheetData>
     <row r="2" spans="1:7">
       <c r="A2" s="192" t="s">
-        <v>2616</v>
+        <v>2622</v>
       </c>
       <c r="D2" s="192" t="s">
         <v>29</v>
       </c>
       <c r="G2" s="192" t="s">
-        <v>2617</v>
+        <v>2623</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -72114,7 +72136,7 @@
         <v>229</v>
       </c>
       <c r="D3" t="s">
-        <v>2618</v>
+        <v>2624</v>
       </c>
       <c r="G3" t="s">
         <v>244</v>
@@ -72125,7 +72147,7 @@
         <v>245</v>
       </c>
       <c r="D4" t="s">
-        <v>2619</v>
+        <v>2625</v>
       </c>
       <c r="G4" t="s">
         <v>234</v>
@@ -72133,10 +72155,10 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>2620</v>
+        <v>2626</v>
       </c>
       <c r="D5" t="s">
-        <v>2621</v>
+        <v>2627</v>
       </c>
       <c r="G5" t="s">
         <v>239</v>

</xml_diff>